<commit_message>
Derive energy/opex reduction from the memory+FLOP cuts (default = cost-weighted); overridable; add assumptions-derivation table
Energy splits between memory (data movement) and compute like cost does, so opex reduction now defaults to the cost-weighted reduction instead of a free 10x slider (sidebar toggle to override; xlsx Inputs!B5 = =B20, overtypable). Adds a consolidated 'how each value is derived' table to the Methodology tab + xlsx notes.
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -1900,7 +1900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A42"/>
+  <dimension ref="A1:A44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -1971,210 +1971,224 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Net AI economics (Totals + company tabs): Net AI = AI revenue - AI capex (full AI-infra) - AI opex (cash basis). With our arch: Net AI + spend cut.</t>
+          <t>Energy/opex reduction: DERIVED = cost-weighted reduction (energy splits memory/compute like cost). Inputs B5 defaults to =B20; overtype that cell to override.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>HOW EACH INPUT IS DERIVED: Inputs sheet column D notes every global assumption; Evidence sheet has the BOM cost split (mem share), accelerator-share teardowns, own-silicon TCO and filing top-lines; per-company capex/shares/revenue carry a basis + clickable Sources on each company tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Net AI economics (Totals + company tabs): Net AI = AI revenue - AI capex (full AI-infra) - AI opex (cash basis). With our arch: Net AI + spend cut.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Shows they all LOSE money on AI today. TOGGLE 'Datacenter scaling factor' (Inputs B13): 0 = accelerator-only (conservative); 1 = whole datacenter scales -&gt; net AI flips positive (~0.7 = breakeven).</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>KEY RESULTS (defaults)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>- Cost-weighted reduction ~22x (NOT 100x; range 17-38x over memory share 45-82%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>- Net AI FY25: 6 named firms spend ~$375B (capex+opex) vs ~$79B AI revenue = ~ -$295B/yr cash burn.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>- With our architecture: spend cut ~$159B -&gt; burn shrinks to ~ -$136B/yr (~42% of AI spend cut).</t>
+          <t>- Cost-weighted reduction ~22x (NOT 100x; range 17-38x over memory share 45-82%).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>- Spend-cut value (named floor): FY25 ~$159B/yr (~$1.6T capitalized); FY26 r/r ~$328B/yr (~$3.3T).</t>
+          <t>- Net AI FY25: 6 named firms spend ~$375B (capex+opex) vs ~$79B AI revenue = ~ -$295B/yr cash burn.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
+          <t>- With our architecture: spend cut ~$159B -&gt; burn shrinks to ~ -$136B/yr (~42% of AI spend cut).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>- Spend-cut value (named floor): FY25 ~$159B/yr (~$1.6T capitalized); FY26 r/r ~$328B/yr (~$3.3T).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>- GLOBAL estimate (named ~80% of world AI capex): FY25 ~$2.0T, FY26 ~$4.1T capitalized. Clearly an estimate.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>CAVEATS</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>- AI REVENUE is the softest input: MSFT $37B &amp; Amazon $15B run-rates are DISCLOSED; Google/Meta/Oracle/SpaceX are ESTIMATES. Meta's real AI payoff is indirect ad-uplift (~$20B), not direct revenue -- so its 'loss' here overstates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>- Net AI is CASH basis (capex not depreciated). On an accounting (depreciation) basis the loss is smaller; on a depreciation basis it is closer to a true P&amp;L.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>- No company reports 'accelerator capex'. Totals DISCLOSED; server/accel split ESTIMATED (server CFO-disclosed; accel-within from BOM). +/-15-20%.</t>
+          <t>- AI REVENUE is the softest input: MSFT $37B &amp; Amazon $15B run-rates are DISCLOSED; Google/Meta/Oracle/SpaceX are ESTIMATES. Meta's real AI payoff is indirect ad-uplift (~$20B), not direct revenue -- so its 'loss' here overstates.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>- FY26 is a full live chain (FY26 total-capex guidance x FY26 shares). SpaceX FY26 ~$18B is an estimate.</t>
+          <t>- Net AI is CASH basis (capex not depreciated). On an accounting (depreciation) basis the loss is smaller; on a depreciation basis it is closer to a true P&amp;L.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>- Hyperscaler market caps (company tab row 7) are approximate placeholders -- edit to current.</t>
+          <t>- No company reports 'accelerator capex'. Totals DISCLOSED; server/accel split ESTIMATED (server CFO-disclosed; accel-within from BOM). +/-15-20%.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>- Own-silicon (TPU/Trainium/MTIA) is cheaper per FLOP, but compute is valued at ACTUAL cost; CostLadder shows the buy/rent premium.</t>
+          <t>- FY26 is a full live chain (FY26 total-capex guidance x FY26 shares). SpaceX FY26 ~$18B is an estimate.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>- 1000x (=100x*10x) is NOT physical: cost is additive (Amdahl), not multiplicative.</t>
+          <t>- Hyperscaler market caps (company tab row 7) are approximate placeholders -- edit to current.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
+          <t>- Own-silicon (TPU/Trainium/MTIA) is cheaper per FLOP, but compute is valued at ACTUAL cost; CostLadder shows the buy/rent premium.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>- 1000x (=100x*10x) is NOT physical: cost is additive (Amdahl), not multiplicative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
           <t>- JEVONS: savings reinvested into more AI, not budget cuts. Capitalization is a simple perpetuity.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>SOURCES</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>SpaceX S-1 / IPO: https://www.hl.co.uk/news/inside-spacexs-ipo-filing-revenue-starlink-ai-and-key-financials</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>Microsoft FY25 capex (Q3 FY26 call): https://www.fool.com/earnings/call-transcripts/2026/04/29/microsoft-msft-q3-2026-earnings-transcript/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Alphabet FY25 $91.4B, 60/40 split (Q4'25 call): https://www.fool.com/earnings/call-transcripts/2026/02/04/alphabet-googl-q4-2025-earnings-call-transcript/</t>
+          <t>SpaceX S-1 / IPO: https://www.hl.co.uk/news/inside-spacexs-ipo-filing-revenue-starlink-ai-and-key-financials</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Amazon FY25 $128.3B + server life 6-&gt;5yr (10-K): https://www.sec.gov/Archives/edgar/data/1018724/000101872426000004/amzn-20251231.htm</t>
+          <t>Microsoft FY25 capex (Q3 FY26 call): https://www.fool.com/earnings/call-transcripts/2026/04/29/microsoft-msft-q3-2026-earnings-transcript/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Meta FY25 $72.2B (Q4/FY25 release): https://investor.atmeta.com/investor-news/press-release-details/2026/Meta-Reports-Fourth-Quarter-and-Full-Year-2025-Results/default.aspx</t>
+          <t>Alphabet FY25 $91.4B, 60/40 split (Q4'25 call): https://www.fool.com/earnings/call-transcripts/2026/02/04/alphabet-googl-q4-2025-earnings-call-transcript/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>H100/B200 BOM + margin (Silicon Analysts): https://siliconanalysts.com/analysis/nvidia-b200-blackwell-cost-breakdown</t>
+          <t>Amazon FY25 $128.3B + server life 6-&gt;5yr (10-K): https://www.sec.gov/Archives/edgar/data/1018724/000101872426000004/amzn-20251231.htm</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>TPU/Trainium TCO (SemiAnalysis): https://newsletter.semianalysis.com/p/tpuv7-google-takes-a-swing-at-the</t>
+          <t>Meta FY25 $72.2B (Q4/FY25 release): https://investor.atmeta.com/investor-news/press-release-details/2026/Meta-Reports-Fourth-Quarter-and-Full-Year-2025-Results/default.aspx</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>GPU rental prices 2026 (Spheron): https://www.spheron.network/blog/gpu-cloud-pricing-comparison-2026/</t>
+          <t>H100/B200 BOM + margin (Silicon Analysts): https://siliconanalysts.com/analysis/nvidia-b200-blackwell-cost-breakdown</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Microsoft $37B AI run-rate (Q3 FY26): https://news.alphastreet.com/microsoft-msft-q3-fy2026-azure-hits-40-growth-as-ai-business-reaches-37-billion-run-rate/</t>
+          <t>TPU/Trainium TCO (SemiAnalysis): https://newsletter.semianalysis.com/p/tpuv7-google-takes-a-swing-at-the</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Amazon &gt;$15B AWS AI run-rate (Q1 FY26): https://www.bnnbloomberg.ca/business/artificial-intelligence/2026/04/09/amazon-cloud-units-ai-revenue-run-rate-exceeds-us15-billion-in-first-quarter-ceo-says/</t>
+          <t>GPU rental prices 2026 (Spheron): https://www.spheron.network/blog/gpu-cloud-pricing-comparison-2026/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Microsoft $37B AI run-rate (Q3 FY26): https://news.alphastreet.com/microsoft-msft-q3-fy2026-azure-hits-40-growth-as-ai-business-reaches-37-billion-run-rate/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Amazon &gt;$15B AWS AI run-rate (Q1 FY26): https://www.bnnbloomberg.ca/business/artificial-intelligence/2026/04/09/amazon-cloud-units-ai-revenue-run-rate-exceeds-us15-billion-in-first-quarter-ceo-says/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>Hyperscalers losing money on AI (capex vs revenue): https://fortune.com/2026/04/15/data-centers-hyperscalers-spending-billions-on-hardware-thats-worthless-in-3-years/</t>
         </is>
@@ -6370,8 +6384,9 @@
           <t>Opex / energy reduction factor</t>
         </is>
       </c>
-      <c r="B5" s="23" t="n">
-        <v>10</v>
+      <c r="B5" s="23">
+        <f>B20</f>
+        <v/>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -6380,7 +6395,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Energy ~ total FLOPs executed -&gt; 10x floor.</t>
+          <t>DERIVED default = cost-weighted reduction (B20): energy splits memory/compute like cost. Overtype this cell to override.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Two-scenario model: Today (quality-matched x9.24) vs Ceiling (prefill x22.1)
- Scenarios cut from five presets to Today / Ceiling (2026-08-17 ruling):
  Today = measured serving blend x2.19 x equal-quality parameter ratio at the
  deployment scale (x4.22 at 1T) = x9.24 -> ~20x cost-weighted; Ceiling =
  measured prefill x4.02 x 5.5 kernel-campaign speedup = x22.1 -> ~41x.
- Deployment-scale slider trimmed to 1B-1T (default 1T).
- Discount rate 10% -> 6%; SpaceX market cap 1770 -> 1840.
- Market caps refreshed (Alphabet 4250, Amazon 2830, Meta 1490, Oracle 433);
  FY26 capex updates (Amazon 220, Oracle 55.7 actual, Meta 137.5).
- Sidebar de-verbosed; long derivations live in the Methodology tab.
- Workbook: transformer decode now uses the measured 1/context law; Inputs
  carries the Today/Ceiling scenario block; stale 10%-era numbers fixed.
- Blend crossover corrections (training share ~0.06, 100:1@8k x0.28).
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Totals" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Microsoft" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Alphabet" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Amazon" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Meta" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Oracle" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="SpaceX" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Inputs" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Sensitivity" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="CostLadder" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Evidence" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Methodology" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Totals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Microsoft" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alphabet" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amazon" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meta" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oracle" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpaceX" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CostLadder" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ServingTraining" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,10 +28,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="0.000000"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="169" formatCode="$0.0000"/>
+    <numFmt numFmtId="170" formatCode="$0.00"/>
+    <numFmt numFmtId="171" formatCode="0.0×"/>
+    <numFmt numFmtId="172" formatCode="0.00×"/>
+    <numFmt numFmtId="173" formatCode="0.000×"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -111,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -144,10 +152,40 @@
     <xf numFmtId="3" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1194,10 +1232,10 @@
           <t>Own custom silicon (TPU/Trainium)</t>
         </is>
       </c>
-      <c r="B3" s="28" t="n">
+      <c r="B3" s="30" t="n">
         <v>0.9</v>
       </c>
-      <c r="C3" s="28" t="n">
+      <c r="C3" s="30" t="n">
         <v>1.4</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1212,10 +1250,10 @@
           <t>Buy + operate NVIDIA (scale)</t>
         </is>
       </c>
-      <c r="B4" s="28" t="n">
+      <c r="B4" s="30" t="n">
         <v>1.5</v>
       </c>
-      <c r="C4" s="28" t="n">
+      <c r="C4" s="30" t="n">
         <v>2</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1230,10 +1268,10 @@
           <t>Rent NVIDIA - neocloud / committed</t>
         </is>
       </c>
-      <c r="B5" s="28" t="n">
+      <c r="B5" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="28" t="n">
+      <c r="C5" s="30" t="n">
         <v>3.5</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1248,10 +1286,10 @@
           <t>Rent NVIDIA - hyperscaler on-demand</t>
         </is>
       </c>
-      <c r="B6" s="28" t="n">
+      <c r="B6" s="30" t="n">
         <v>3</v>
       </c>
-      <c r="C6" s="28" t="n">
+      <c r="C6" s="30" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -1318,7 +1356,7 @@
           <t>DC/staff adder $/hr</t>
         </is>
       </c>
-      <c r="B12" s="29" t="n">
+      <c r="B12" s="28" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -1328,7 +1366,7 @@
           <t>Owned TCO $/hr</t>
         </is>
       </c>
-      <c r="B13" s="30">
+      <c r="B13" s="29">
         <f>B10+B11+B12</f>
         <v/>
       </c>
@@ -1391,6 +1429,1774 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F119"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SERVING &amp; TRAINING — measured 2026-08-07/08 (2/4/8 x H100), priced at the CostLadder rent mid ($2.50/GPU-hr). Source: bdm/docs/deck/build/derived.json (keys in ai_capex_model.MEASURED).</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>WORKLOAD — edit the yellow cells; every sheet recomputes</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Training, prefill and decode point in opposite directions at today's kernel maturity, so the compute lever is blended over the workload rather than fixed. Cost per GENERATED token = in:out input tokens through prefill + one token through decode. Transformer decode follows the MEASURED 1/context law at its own KV ceiling (granted no KV compression by default; raise the KV-compression cell below to grant it a mature stack).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Input : output token ratio</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>~10:1 = code / reasoning / agent traces. 50-100:1 = RAG and document QA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>E[context] (tokens)</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="n">
+        <v>65536</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Our decode cost is context-flat and the transformer's is linear, so the decode advantage is linear in this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Training share of accelerator cost</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>0 = a serving-cost claim. Training is a LOSS at short sequence today; above ~0.06 the blend drops below 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Measured constants</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Owned decode, tokens/s/box (context-flat)</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="n">
+        <v>4496.668604837461</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>KV MB per token per stream</t>
+        </is>
+      </c>
+      <c r="B13" s="31" t="n">
+        <v>0.15234375</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HBM TB/s per GPU</t>
+        </is>
+      </c>
+      <c r="B14" s="28" t="n">
+        <v>3.35</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Transformer KV compression (mature stack)</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GPUs per box</t>
+        </is>
+      </c>
+      <c r="B16" s="32" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Training advantage, short sequence (owned / transformer)</t>
+        </is>
+      </c>
+      <c r="B17" s="33" t="n">
+        <v>0.1041666666666667</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Transformer is 9.6x faster at T=2048 blocks (d1152). Crossover near T~88,000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>KV GB per stream</t>
+        </is>
+      </c>
+      <c r="B20" s="19">
+        <f>$B$8*$B$13/1024</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>KV GB per stream, compressed</t>
+        </is>
+      </c>
+      <c r="B21" s="34">
+        <f>$B$20/$B$15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Transformer decode, tokens/s/box</t>
+        </is>
+      </c>
+      <c r="B22" s="18">
+        <f>511.8416*32768/$B$8*$B$15*$B$16</f>
+        <v/>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>MEASURED 1/context law (2026-08-14 re-base): 511.84 tok/s/GPU at 32,768 ctx x 32768/E[context] x KV-compression x GPUs. Crosses our flat 562/GPU near ~30k context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Prefill table row (lookup)</t>
+        </is>
+      </c>
+      <c r="B23" s="35">
+        <f>MATCH($B$8,$A$33:$A$39,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Prefill tokens/s/box — transformer</t>
+        </is>
+      </c>
+      <c r="B24" s="18">
+        <f>IF(INDEX($B$33:$B$39,MIN($B$23+1,7))=INDEX($B$33:$B$39,$B$23),INDEX($B$33:$B$39,$B$23),EXP(LN(INDEX($B$33:$B$39,$B$23))+(LN($B$8)-LN(INDEX($A$33:$A$39,$B$23)))/(LN(INDEX($A$33:$A$39,MIN($B$23+1,7)))-LN(INDEX($A$33:$A$39,$B$23)))*(LN(INDEX($B$33:$B$39,MIN($B$23+1,7)))-LN(INDEX($B$33:$B$39,$B$23)))))*$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Prefill tokens/s/box — owned</t>
+        </is>
+      </c>
+      <c r="B25" s="18">
+        <f>IF(INDEX($C$33:$C$39,MIN($B$23+1,7))=INDEX($C$33:$C$39,$B$23),INDEX($C$33:$C$39,$B$23),EXP(LN(INDEX($C$33:$C$39,$B$23))+(LN($B$8)-LN(INDEX($A$33:$A$39,$B$23)))/(LN(INDEX($A$33:$A$39,MIN($B$23+1,7)))-LN(INDEX($A$33:$A$39,$B$23)))*(LN(INDEX($C$33:$C$39,MIN($B$23+1,7)))-LN(INDEX($C$33:$C$39,$B$23)))))*$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Transformer seconds per generated token</t>
+        </is>
+      </c>
+      <c r="B26" s="36">
+        <f>$B$7/$B$24+1/$B$22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Owned seconds per generated token</t>
+        </is>
+      </c>
+      <c r="B27" s="36">
+        <f>$B$7/$B$25+1/$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>BLENDED COMPUTE LEVER (flop_factor)</t>
+        </is>
+      </c>
+      <c r="B28" s="29">
+        <f>IF($B$9&gt;0,1/($B$9/$B$17+(1-$B$9)/($B$26/$B$27)),$B$26/$B$27)</f>
+        <v/>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Inputs!B24 (TODAY lever) = this x the equal-quality parameter ratio; Inputs!B3 follows it, so this drives the whole workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of which: prefill advantage</t>
+        </is>
+      </c>
+      <c r="B29" s="19">
+        <f>($B$7/$B$24)/($B$7/$B$25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of which: decode advantage</t>
+        </is>
+      </c>
+      <c r="B30" s="37">
+        <f>(1/$B$22)/(1/$B$12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Measured prefill throughput, tokens/s/GPU (bf16 saturated lane, d2048)</t>
+        </is>
+      </c>
+      <c r="D32" s="38" t="inlineStr">
+        <is>
+          <t>Context</t>
+        </is>
+      </c>
+      <c r="E32" s="38" t="inlineStr">
+        <is>
+          <t>Transformer</t>
+        </is>
+      </c>
+      <c r="F32" s="38" t="inlineStr">
+        <is>
+          <t>Owned</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="39" t="n">
+        <v>2048</v>
+      </c>
+      <c r="B33" s="17" t="n">
+        <v>4682606.88285999</v>
+      </c>
+      <c r="C33" s="17" t="n">
+        <v>1185825</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="39" t="n">
+        <v>8192</v>
+      </c>
+      <c r="B34" s="17" t="n">
+        <v>3450080</v>
+      </c>
+      <c r="C34" s="17" t="n">
+        <v>1183690</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="39" t="n">
+        <v>32768</v>
+      </c>
+      <c r="B35" s="17" t="n">
+        <v>1711802</v>
+      </c>
+      <c r="C35" s="17" t="n">
+        <v>1186661</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="39" t="n">
+        <v>65536</v>
+      </c>
+      <c r="B36" s="17" t="n">
+        <v>1007187</v>
+      </c>
+      <c r="C36" s="17" t="n">
+        <v>1181622</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="39" t="n">
+        <v>131072</v>
+      </c>
+      <c r="B37" s="17" t="n">
+        <v>541094</v>
+      </c>
+      <c r="C37" s="17" t="n">
+        <v>978107</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="39" t="n">
+        <v>262144</v>
+      </c>
+      <c r="B38" s="17" t="n">
+        <v>277474</v>
+      </c>
+      <c r="C38" s="17" t="n">
+        <v>726142</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="39" t="n">
+        <v>524288</v>
+      </c>
+      <c r="B39" s="17" t="n">
+        <v>140820</v>
+      </c>
+      <c r="C39" s="17" t="n">
+        <v>478522</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>SCOPE: the serving and training blocks below are component-scope systems benches (bAttention d1536 fwd+bwd h-recurrence sub-block vs transformer d2048 forward-only layer); every speedup there is each family vs its OWN 1-GPU baseline. The prefill lanes quoted further down are cross-family: bf16 parameter-matched at block scope, and fp32 at full-model scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>Serving at long context — $/1M generated tokens, one 8xH100 box</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="38" t="inlineStr">
+        <is>
+          <t>Context (tokens)</t>
+        </is>
+      </c>
+      <c r="B44" s="38" t="inlineStr">
+        <is>
+          <t>bAttention $/1M tok</t>
+        </is>
+      </c>
+      <c r="C44" s="38" t="inlineStr">
+        <is>
+          <t>Transformer $/1M tok (mature stack)</t>
+        </is>
+      </c>
+      <c r="D44" s="38" t="inlineStr">
+        <is>
+          <t>TF streams/GPU</t>
+        </is>
+      </c>
+      <c r="E44" s="38" t="inlineStr">
+        <is>
+          <t>Cost ratio</t>
+        </is>
+      </c>
+      <c r="F44" s="38" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="39" t="n">
+        <v>4096</v>
+      </c>
+      <c r="B45" s="40" t="n">
+        <v>1.235482541359387</v>
+      </c>
+      <c r="C45" s="41" t="n">
+        <v>0.1695945640120853</v>
+      </c>
+      <c r="D45" s="35" t="n">
+        <v>118</v>
+      </c>
+      <c r="E45" s="42" t="n">
+        <v>0.1372698992779634</v>
+      </c>
+      <c r="F45" s="43" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="39" t="n">
+        <v>16384</v>
+      </c>
+      <c r="B46" s="40" t="n">
+        <v>1.235482541359387</v>
+      </c>
+      <c r="C46" s="41" t="n">
+        <v>0.678378256048341</v>
+      </c>
+      <c r="D46" s="35" t="n">
+        <v>29</v>
+      </c>
+      <c r="E46" s="42" t="n">
+        <v>0.5490795971118535</v>
+      </c>
+      <c r="F46" s="43" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="39" t="n">
+        <v>32768</v>
+      </c>
+      <c r="B47" s="40" t="n">
+        <v>1.235482541359387</v>
+      </c>
+      <c r="C47" s="41" t="n">
+        <v>1.356756512096682</v>
+      </c>
+      <c r="D47" s="35" t="n">
+        <v>14</v>
+      </c>
+      <c r="E47" s="42" t="n">
+        <v>1.098159194223707</v>
+      </c>
+      <c r="F47" s="43" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="39" t="n">
+        <v>65536</v>
+      </c>
+      <c r="B48" s="40" t="n">
+        <v>1.235482541359387</v>
+      </c>
+      <c r="C48" s="41" t="n">
+        <v>2.713513024193364</v>
+      </c>
+      <c r="D48" s="35" t="n">
+        <v>7</v>
+      </c>
+      <c r="E48" s="42" t="n">
+        <v>2.196318388447414</v>
+      </c>
+      <c r="F48" s="43" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="39" t="n">
+        <v>131072</v>
+      </c>
+      <c r="B49" s="40" t="n">
+        <v>1.235482541359387</v>
+      </c>
+      <c r="C49" s="41" t="n">
+        <v>5.427026048386728</v>
+      </c>
+      <c r="D49" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" s="42" t="n">
+        <v>4.392636776894828</v>
+      </c>
+      <c r="F49" s="43" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="39" t="n">
+        <v>262144</v>
+      </c>
+      <c r="B50" s="40" t="n">
+        <v>1.235482541359387</v>
+      </c>
+      <c r="C50" s="41" t="n">
+        <v>10.85405209677346</v>
+      </c>
+      <c r="D50" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="42" t="n">
+        <v>8.785273553789656</v>
+      </c>
+      <c r="F50" s="43" t="inlineStr">
+        <is>
+          <t>a measured decode cell (64 streams/GPU against the transformer 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="39" t="n">
+        <v>1048576</v>
+      </c>
+      <c r="B51" s="44" t="n">
+        <v>1.235482541359387</v>
+      </c>
+      <c r="C51" s="41" t="n">
+        <v/>
+      </c>
+      <c r="D51" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="42" t="n">
+        <v/>
+      </c>
+      <c r="F51" s="43" t="inlineStr">
+        <is>
+          <t>bAttention rate extrapolated past 262k (flatness measured 4k-262k)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>RE-BASED 2026-08-14 on the full-model decode receipt: per-GPU aggregate throughput at each family's own concurrency ceiling, transformer granted no KV compression. Ratio ~ context/29,800, so the TRANSFORMER is ahead below ~30k context; x2.2 at 64k, x8.8 at 262k. Memory-ceiling result, not a per-token one - at one stream and 64k the transformer decodes a token faster than we do. Granting it KV /8: x1.1 at 262k.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>Training at scale — same cluster, more steps/s</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
+      <c r="E54" s="2" t="n"/>
+      <c r="F54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="38" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B55" s="38" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C55" s="38" t="inlineStr">
+        <is>
+          <t>Ratio / consequence</t>
+        </is>
+      </c>
+      <c r="D55" s="38" t="inlineStr"/>
+      <c r="E55" s="38" t="inlineStr"/>
+      <c r="F55" s="38" t="inlineStr">
+        <is>
+          <t>Status — derived.json key</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="45" t="inlineStr">
+        <is>
+          <t>8-GPU speedup, matched load (16 in flight)</t>
+        </is>
+      </c>
+      <c r="B56" s="46" t="inlineStr">
+        <is>
+          <t>x5.15 fwd+bwd vs x3.70 fwd-only Ulysses best</t>
+        </is>
+      </c>
+      <c r="C56" s="47" t="inlineStr">
+        <is>
+          <t>x1.39 cluster throughput</t>
+        </is>
+      </c>
+      <c r="F56" s="43" t="inlineStr">
+        <is>
+          <t>MEASURED — matched_load_curve</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="45" t="inlineStr">
+        <is>
+          <t>8-GPU speedup, deep load (256 in flight)</t>
+        </is>
+      </c>
+      <c r="B57" s="46" t="inlineStr">
+        <is>
+          <t>x6.27 (pipeline keeps filling; TF saturated by 16)</t>
+        </is>
+      </c>
+      <c r="C57" s="47" t="inlineStr">
+        <is>
+          <t>x1.70</t>
+        </is>
+      </c>
+      <c r="F57" s="43" t="inlineStr">
+        <is>
+          <t>MEASURED — scaling_1to8_best</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="45" t="inlineStr">
+        <is>
+          <t>GPU-hours for the same training work</t>
+        </is>
+      </c>
+      <c r="B58" s="48" t="inlineStr">
+        <is>
+          <t>-28% (matched) … -41% (deep)</t>
+        </is>
+      </c>
+      <c r="C58" s="45" t="inlineStr"/>
+      <c r="F58" s="43" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="45" t="inlineStr">
+        <is>
+          <t>64k-token sequence on one 80 GB GPU</t>
+        </is>
+      </c>
+      <c r="B59" s="46" t="inlineStr">
+        <is>
+          <t>30.9 GB fits vs OOM (78.4 GB attempted)</t>
+        </is>
+      </c>
+      <c r="C59" s="45" t="inlineStr"/>
+      <c r="F59" s="43" t="inlineStr">
+        <is>
+          <t>MEASURED — pipeline_feasibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="45" t="inlineStr">
+        <is>
+          <t>Pipeline per-GPU peak (flat in load)</t>
+        </is>
+      </c>
+      <c r="B60" s="46" t="inlineStr">
+        <is>
+          <t>9.05 GB vs 43.3 GB GPipe stage</t>
+        </is>
+      </c>
+      <c r="C60" s="47" t="inlineStr">
+        <is>
+          <t>x4.8 (component-scope, width-unmatched)</t>
+        </is>
+      </c>
+      <c r="F60" s="43" t="inlineStr">
+        <is>
+          <t>MEASURED — pipeline_memory_asymmetry</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="45" t="inlineStr">
+        <is>
+          <t>Params for equal quality at 70B</t>
+        </is>
+      </c>
+      <c r="B61" s="49" t="inlineStr">
+        <is>
+          <t>x4.1 [2.2-7.7] transformer</t>
+        </is>
+      </c>
+      <c r="C61" s="45" t="inlineStr"/>
+      <c r="F61" s="43" t="inlineStr">
+        <is>
+          <t>PROJECTION — quality_fit.ref_70B</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="45" t="inlineStr">
+        <is>
+          <t>Tokens for equal quality at 70B</t>
+        </is>
+      </c>
+      <c r="B62" s="49" t="inlineStr">
+        <is>
+          <t>x1.68 [1.33-2.10] (beta=0.28 assumption)</t>
+        </is>
+      </c>
+      <c r="C62" s="45" t="inlineStr"/>
+      <c r="F62" s="43" t="inlineStr">
+        <is>
+          <t>PROJECTION — quality_fit.ref_70B</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="45" t="inlineStr">
+        <is>
+          <t>Stepped vs scanned training</t>
+        </is>
+      </c>
+      <c r="B63" s="46" t="inlineStr">
+        <is>
+          <t>x24 cost to step the recurrence token-by-token</t>
+        </is>
+      </c>
+      <c r="C63" s="45" t="inlineStr"/>
+      <c r="F63" s="43" t="inlineStr">
+        <is>
+          <t>MEASURED — stepped_vs_scanned</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="inlineStr">
+        <is>
+          <t>The compute lever — blended over the workload (sets flop_factor)</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n"/>
+      <c r="C65" s="2" t="n"/>
+      <c r="D65" s="2" t="n"/>
+      <c r="E65" s="2" t="n"/>
+      <c r="F65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>Training, prefill and decode point in OPPOSITE directions at today's kernel maturity, so a single number cannot represent them. Training is a loss at short sequence (transformer 5.3-9.6x faster at T=2048 blocks; FLOPs near-matched at 1.07-1.19x, the gap is achieved FLOP/s 200.9 vs 21.7 TF/s; crossover near T~88,000). Prefill crosses over near 65k context. Decode crosses in our favour near ~30k context. The lever is therefore blended over the workload: per generated token, in:out input tokens through prefill plus one token through decode, using measured per-GPU throughput at each family's own concurrency ceiling, the transformer granted no KV compression. At the default operating point (10:1, 64k context, training share 0): prefill x1.17, decode x2.20, blended x2.19, with decode ~99.7% of transformer serving cost. The decode half is a MEMORY CEILING, not a per-token result - at one stream and 64k the transformer decodes a token more cheaply than we do - and it crosses 1 at ~30k context, below which the transformer wins. Granting it KV/8 divides our decode lever by 8. A training share above ~0.06 also takes the blend below 1. All are reachable in the live model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>The prefill component itself exists in two lanes, both shown below. It comes from the bf16 lane, where both families run their production attention kernels (there is no fp32 FlashAttention kernel). BF16 LANE: parameter counts exactly matched, 1 layer, batch 16, 1 x H100 80GB HBM3, 2026-07-21 — x4.02 at d512/1M, x3.83 at d1024/1M, x2.01 at d2048/262k. Receipts: experiments/paper_figures/output/matched_d{512,1024,2048}_h100.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="38" t="inlineStr">
+        <is>
+          <t>Context (tokens)</t>
+        </is>
+      </c>
+      <c r="B70" s="38" t="inlineStr">
+        <is>
+          <t>Transformer ms</t>
+        </is>
+      </c>
+      <c r="C70" s="38" t="inlineStr">
+        <is>
+          <t>bAttention ms</t>
+        </is>
+      </c>
+      <c r="D70" s="38" t="inlineStr">
+        <is>
+          <t>TF / bAttention</t>
+        </is>
+      </c>
+      <c r="E70" s="38" t="inlineStr"/>
+      <c r="F70" s="38" t="inlineStr">
+        <is>
+          <t>Lane / note</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="39" t="n">
+        <v>2048</v>
+      </c>
+      <c r="B71" s="5" t="n">
+        <v>111.229</v>
+      </c>
+      <c r="C71" s="14" t="n">
+        <v>663.1130000000001</v>
+      </c>
+      <c r="D71" s="50" t="n">
+        <v>0.16773762541226</v>
+      </c>
+      <c r="F71" s="43" t="inlineStr">
+        <is>
+          <t>bf16 (lever) — transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="39" t="n">
+        <v>4096</v>
+      </c>
+      <c r="B72" s="5" t="n">
+        <v>125.091</v>
+      </c>
+      <c r="C72" s="14" t="n">
+        <v>662.751</v>
+      </c>
+      <c r="D72" s="50" t="n">
+        <v>0.1887450943114382</v>
+      </c>
+      <c r="F72" s="43" t="inlineStr">
+        <is>
+          <t>bf16 (lever) — transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="39" t="n">
+        <v>8192</v>
+      </c>
+      <c r="B73" s="5" t="n">
+        <v>153.085</v>
+      </c>
+      <c r="C73" s="14" t="n">
+        <v>663.327</v>
+      </c>
+      <c r="D73" s="50" t="n">
+        <v>0.2307836104967836</v>
+      </c>
+      <c r="F73" s="43" t="inlineStr">
+        <is>
+          <t>bf16 (lever) — transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="39" t="n">
+        <v>16384</v>
+      </c>
+      <c r="B74" s="5" t="n">
+        <v>204.919</v>
+      </c>
+      <c r="C74" s="14" t="n">
+        <v>663.202</v>
+      </c>
+      <c r="D74" s="50" t="n">
+        <v>0.3089842913622094</v>
+      </c>
+      <c r="F74" s="43" t="inlineStr">
+        <is>
+          <t>bf16 (lever) — transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="39" t="n">
+        <v>32768</v>
+      </c>
+      <c r="B75" s="5" t="n">
+        <v>309.886</v>
+      </c>
+      <c r="C75" s="14" t="n">
+        <v>662.6180000000001</v>
+      </c>
+      <c r="D75" s="50" t="n">
+        <v>0.4676691547769605</v>
+      </c>
+      <c r="F75" s="43" t="inlineStr">
+        <is>
+          <t>bf16 (lever) — transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="39" t="n">
+        <v>65536</v>
+      </c>
+      <c r="B76" s="5" t="n">
+        <v>520.986</v>
+      </c>
+      <c r="C76" s="14" t="n">
+        <v>663.199</v>
+      </c>
+      <c r="D76" s="50" t="n">
+        <v>0.7855651169558459</v>
+      </c>
+      <c r="F76" s="43" t="inlineStr">
+        <is>
+          <t>bf16 (lever) — transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="39" t="n">
+        <v>131072</v>
+      </c>
+      <c r="B77" s="5" t="n">
+        <v>969.79</v>
+      </c>
+      <c r="C77" s="14" t="n">
+        <v>753.457</v>
+      </c>
+      <c r="D77" s="50" t="n">
+        <v>1.287120565606265</v>
+      </c>
+      <c r="F77" s="43" t="inlineStr">
+        <is>
+          <t>bf16 (lever)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="39" t="n">
+        <v>262144</v>
+      </c>
+      <c r="B78" s="5" t="n">
+        <v>1889.616</v>
+      </c>
+      <c r="C78" s="14" t="n">
+        <v>938.175</v>
+      </c>
+      <c r="D78" s="50" t="n">
+        <v>2.014140219042289</v>
+      </c>
+      <c r="F78" s="43" t="inlineStr">
+        <is>
+          <t>bf16 (lever)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="39" t="n">
+        <v>524288</v>
+      </c>
+      <c r="B79" s="5" t="n">
+        <v>3718.717</v>
+      </c>
+      <c r="C79" s="14" t="n">
+        <v>1308.837</v>
+      </c>
+      <c r="D79" s="50" t="n">
+        <v>2.841237678947035</v>
+      </c>
+      <c r="F79" s="43" t="inlineStr">
+        <is>
+          <t>bf16 (lever)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="39" t="n">
+        <v>512</v>
+      </c>
+      <c r="B80" s="5" t="n">
+        <v>6.578</v>
+      </c>
+      <c r="C80" s="15" t="n">
+        <v>61.216</v>
+      </c>
+      <c r="D80" s="50" t="n">
+        <v>0.1074555671719812</v>
+      </c>
+      <c r="F80" s="43" t="inlineStr">
+        <is>
+          <t>fp32 (full model) — transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="39" t="n">
+        <v>1024</v>
+      </c>
+      <c r="B81" s="5" t="n">
+        <v>12.611</v>
+      </c>
+      <c r="C81" s="15" t="n">
+        <v>86.66</v>
+      </c>
+      <c r="D81" s="50" t="n">
+        <v>0.145522732517886</v>
+      </c>
+      <c r="F81" s="43" t="inlineStr">
+        <is>
+          <t>fp32 (full model) — transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="39" t="n">
+        <v>2048</v>
+      </c>
+      <c r="B82" s="5" t="n">
+        <v>27.856</v>
+      </c>
+      <c r="C82" s="15" t="n">
+        <v>160.738</v>
+      </c>
+      <c r="D82" s="50" t="n">
+        <v>0.1733006507484229</v>
+      </c>
+      <c r="F82" s="43" t="inlineStr">
+        <is>
+          <t>fp32 (full model) — transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="39" t="n">
+        <v>4096</v>
+      </c>
+      <c r="B83" s="5" t="n">
+        <v>70.339</v>
+      </c>
+      <c r="C83" s="15" t="n">
+        <v>305.622</v>
+      </c>
+      <c r="D83" s="50" t="n">
+        <v>0.2301503164039238</v>
+      </c>
+      <c r="F83" s="43" t="inlineStr">
+        <is>
+          <t>fp32 (full model) — transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="39" t="n">
+        <v>8192</v>
+      </c>
+      <c r="B84" s="5" t="n">
+        <v>207.758</v>
+      </c>
+      <c r="C84" s="15" t="n">
+        <v>595.671</v>
+      </c>
+      <c r="D84" s="50" t="n">
+        <v>0.3487797794420074</v>
+      </c>
+      <c r="F84" s="43" t="inlineStr">
+        <is>
+          <t>fp32 (full model) — transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="39" t="n">
+        <v>16384</v>
+      </c>
+      <c r="B85" s="5" t="n">
+        <v>686.813</v>
+      </c>
+      <c r="C85" s="15" t="n">
+        <v>1177.361</v>
+      </c>
+      <c r="D85" s="50" t="n">
+        <v>0.5833495418992135</v>
+      </c>
+      <c r="F85" s="43" t="inlineStr">
+        <is>
+          <t>fp32 (full model) — transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="39" t="n">
+        <v>32768</v>
+      </c>
+      <c r="B86" s="5" t="n">
+        <v>2518.562</v>
+      </c>
+      <c r="C86" s="15" t="n">
+        <v>2359.638</v>
+      </c>
+      <c r="D86" s="50" t="n">
+        <v>1.067351008925945</v>
+      </c>
+      <c r="F86" s="43" t="inlineStr">
+        <is>
+          <t>fp32 (full model)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="39" t="n">
+        <v>65536</v>
+      </c>
+      <c r="B87" s="5" t="n">
+        <v>9629.459000000001</v>
+      </c>
+      <c r="C87" s="15" t="n">
+        <v>4704.054</v>
+      </c>
+      <c r="D87" s="50" t="n">
+        <v>2.047055369687508</v>
+      </c>
+      <c r="F87" s="43" t="inlineStr">
+        <is>
+          <t>fp32 (full model)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="39" t="n">
+        <v>131072</v>
+      </c>
+      <c r="B88" s="5" t="n">
+        <v>37690.932</v>
+      </c>
+      <c r="C88" s="15" t="n">
+        <v>9432.108</v>
+      </c>
+      <c r="D88" s="50" t="n">
+        <v>3.996024218552205</v>
+      </c>
+      <c r="F88" s="43" t="inlineStr">
+        <is>
+          <t>fp32 (full model)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="39" t="n">
+        <v>262144</v>
+      </c>
+      <c r="B89" s="5" t="n">
+        <v>149366.343</v>
+      </c>
+      <c r="C89" s="15" t="n">
+        <v>18888.452</v>
+      </c>
+      <c r="D89" s="50" t="n">
+        <v>7.907812826588436</v>
+      </c>
+      <c r="F89" s="43" t="inlineStr">
+        <is>
+          <t>fp32 (full model)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>Both blocks are d2048, so the lanes are directly comparable: 2.01x in bf16 against 7.91x in fp32 at 262k. The fp32 lane is full-model scope (24 layers, batch 1) and its receipt records FLASH_ATTENTION and CUDNN_ATTENTION as 'rejected: No available kernel', with the owned arm's route attestation reading dtype_mix io=fp32,bf_col=fp16; its params differ by 16.7%. Full model in bf16 has not been run. Receipt: experiments/paper_figures/output/deck_speed_scaling_d2048_h100_20260803.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="inlineStr">
+        <is>
+          <t>16-bit IO in training</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="n"/>
+      <c r="C92" s="2" t="n"/>
+      <c r="D92" s="2" t="n"/>
+      <c r="E92" s="2" t="n"/>
+      <c r="F92" s="2" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>A training step-time gate: same architecture on every row, only the IO dtype varies. d1536 / 27 layers / block 2048 / batch 32 / seed 1, 1 x GH200 480GB, GPU verified idle before each arm, steady state only. 0 skipped steps on all arms; verdict PASS_io16_SHIPS. Throughput and memory rows are d1536/L27; the val deltas come from the gate's smaller vehicle (width 512, 15 layers). This is why the production training lane is 16-bit; it is not an input to the compute lever above. Receipt: experiments/paper_figures/output/receipts/io16_gate_20260809.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="38" t="inlineStr">
+        <is>
+          <t>IO dtype</t>
+        </is>
+      </c>
+      <c r="B95" s="38" t="inlineStr">
+        <is>
+          <t>s/step</t>
+        </is>
+      </c>
+      <c r="C95" s="38" t="inlineStr">
+        <is>
+          <t>Speed vs fp32</t>
+        </is>
+      </c>
+      <c r="D95" s="38" t="inlineStr">
+        <is>
+          <t>Peak allocated (GB)</t>
+        </is>
+      </c>
+      <c r="E95" s="38" t="inlineStr">
+        <is>
+          <t>Memory vs fp32</t>
+        </is>
+      </c>
+      <c r="F95" s="38" t="inlineStr">
+        <is>
+          <t>Val cost @601 steps</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="45" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="B96" s="33" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="C96" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D96" s="26" t="n">
+        <v>70.669921875</v>
+      </c>
+      <c r="E96" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F96" s="45" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="45" t="inlineStr">
+        <is>
+          <t>fp16</t>
+        </is>
+      </c>
+      <c r="B97" s="33" t="n">
+        <v>8.827999999999999</v>
+      </c>
+      <c r="C97" s="51" t="n">
+        <v>1.185</v>
+      </c>
+      <c r="D97" s="26" t="n">
+        <v>58.2685546875</v>
+      </c>
+      <c r="E97" s="51" t="n">
+        <v>0.825</v>
+      </c>
+      <c r="F97" s="45" t="inlineStr">
+        <is>
+          <t>+0.00128</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="45" t="inlineStr">
+        <is>
+          <t>bf16</t>
+        </is>
+      </c>
+      <c r="B98" s="33" t="n">
+        <v>8.930999999999999</v>
+      </c>
+      <c r="C98" s="51" t="n">
+        <v>1.171</v>
+      </c>
+      <c r="D98" s="26" t="n">
+        <v>56.10546875</v>
+      </c>
+      <c r="E98" s="51" t="n">
+        <v>0.794</v>
+      </c>
+      <c r="F98" s="45" t="inlineStr">
+        <is>
+          <t>+0.00391</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="inlineStr">
+        <is>
+          <t>Assumptions — one row each (MEASURED / PROJECTION / ASSUMPTION)</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="n"/>
+      <c r="C100" s="2" t="n"/>
+      <c r="D100" s="2" t="n"/>
+      <c r="E100" s="2" t="n"/>
+      <c r="F100" s="2" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="38" t="inlineStr">
+        <is>
+          <t>Assumption</t>
+        </is>
+      </c>
+      <c r="B101" s="38" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C101" s="38" t="inlineStr"/>
+      <c r="D101" s="38" t="inlineStr"/>
+      <c r="E101" s="38" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F101" s="38" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="45" t="inlineStr">
+        <is>
+          <t>Compute lever (economics slide)</t>
+        </is>
+      </c>
+      <c r="B102" s="43" t="inlineStr">
+        <is>
+          <t>x9.24 = the x2.19 MEASURED serving blend x the x4.22 FIT-DERIVED equal-quality parameter ratio at trillion scale</t>
+        </is>
+      </c>
+      <c r="E102" s="52" t="inlineStr">
+        <is>
+          <t>MEASURED x PROJECTION</t>
+        </is>
+      </c>
+      <c r="F102" s="43" t="inlineStr">
+        <is>
+          <t>workload_compute_advantage() x quality_matched_compute_lever(); receipts derived.json + quality_fit_v4.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="45" t="inlineStr">
+        <is>
+          <t>Equal-quality parameter matching</t>
+        </is>
+      </c>
+      <c r="B103" s="43" t="inlineStr">
+        <is>
+          <t>sealed 2026-08-14 refit, 4 rungs per family (47M-663M params): the fits cross at 392M and bAttention then matches the transformer fit's quality on 84.2% of the params at 1B, 55.2% at 10B, 36.2% at 100B, 23.7% at 1T, 15.5% at 10T. The receipt's own words: 'a projection of the two fits, not a measurement'</t>
+        </is>
+      </c>
+      <c r="E103" s="52" t="inlineStr">
+        <is>
+          <t>PROJECTION</t>
+        </is>
+      </c>
+      <c r="F103" s="43" t="inlineStr">
+        <is>
+          <t>quality_fit_v4.json param_matching; fits over the sealed rope-convention ladder</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="45" t="inlineStr">
+        <is>
+          <t>Single-GPU training step (AGAINST us)</t>
+        </is>
+      </c>
+      <c r="B104" s="43" t="inlineStr">
+        <is>
+          <t>at 2,048-token context on one GPU a bAttention step costs x6.46 MORE (8,979 vs 1,389 ms/step, d1536/27L, fp16, 601-step protocol). At equal quality the same step costs x1.53 more, not x6.46 - the parameter ratio shrinks the gap but does not erase it. Training is excluded from the serving claim for this reason</t>
+        </is>
+      </c>
+      <c r="E104" s="53" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F104" s="43" t="inlineStr">
+        <is>
+          <t>dtype_trio_v4.json rows[fp16]</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="45" t="inlineStr">
+        <is>
+          <t>$/GPU-hour</t>
+        </is>
+      </c>
+      <c r="B105" s="43" t="inlineStr">
+        <is>
+          <t>$2.50 (H100 rent, neocloud/committed mid; ladder 2.00-3.50)</t>
+        </is>
+      </c>
+      <c r="E105" s="52" t="inlineStr">
+        <is>
+          <t>ASSUMPTION</t>
+        </is>
+      </c>
+      <c r="F105" s="43" t="inlineStr">
+        <is>
+          <t>this file's CostLadder row — unchanged rate basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="45" t="inlineStr">
+        <is>
+          <t>Utilization</t>
+        </is>
+      </c>
+      <c r="B106" s="43" t="inlineStr">
+        <is>
+          <t>85%</t>
+        </is>
+      </c>
+      <c r="E106" s="52" t="inlineStr">
+        <is>
+          <t>ASSUMPTION</t>
+        </is>
+      </c>
+      <c r="F106" s="43" t="inlineStr">
+        <is>
+          <t>same value as the ladder's owned-TCO cross-check</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="45" t="inlineStr">
+        <is>
+          <t>Context-length mix</t>
+        </is>
+      </c>
+      <c r="B107" s="43" t="inlineStr">
+        <is>
+          <t>headline quoted at 262k (a measured decode cell); table sweeps 4k-1M. The decode lever crosses 1 at ~29,800 tokens and BELOW that the transformer serves more tokens per GPU-second than we do — stated on every surface</t>
+        </is>
+      </c>
+      <c r="E107" s="52" t="inlineStr">
+        <is>
+          <t>ASSUMPTION</t>
+        </is>
+      </c>
+      <c r="F107" s="43" t="inlineStr">
+        <is>
+          <t>serving_cost_curve, decode_throughput_ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="45" t="inlineStr">
+        <is>
+          <t>Decode lever is MEMORY-CEILING, not latency (READ FIRST)</t>
+        </is>
+      </c>
+      <c r="B108" s="43" t="inlineStr">
+        <is>
+          <t>per generated token at ONE stream the transformer is AHEAD of us at 64k context — 4.92 vs 5.74 GPU-busy per token. The lever is that it cannot hold many long-context streams: it re-reads its whole KV cache per emitted token, so its aggregate throughput falls as 1/context while ours is flat. Measured: 1 stream at 262k (2 OOM — an exact ceiling) and 8 streams at 32k (16 OOM, so that ceiling is only bracketed at 8-15 and the 32k cell is a bounded x0.97-1.14, near parity) against 64 of ours in 1.62 GB</t>
+        </is>
+      </c>
+      <c r="E108" s="53" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F108" s="43" t="inlineStr">
+        <is>
+          <t>deck_decode_d2048_bf16_gh200_20260814.json; DECODE_THROUGHPUT_20260814</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="45" t="inlineStr">
+        <is>
+          <t>Transformer-stack maturity</t>
+        </is>
+      </c>
+      <c r="B109" s="43" t="inlineStr">
+        <is>
+          <t>NOT GRANTED by default since the 2026-08-14 re-base: the headline runs on the measured cells, in which neither family's decode is optimised (ours ran the unoptimised Triton per-step path at 9.5% GPU-busy while the transformer sat at 95.6%). Setting tf_kv_compression=8.0 grants it paged attention + KV quantization, divides our decode lever by 8 and puts the TRANSFORMER ahead at 64k — reported, not hidden</t>
+        </is>
+      </c>
+      <c r="E109" s="52" t="inlineStr">
+        <is>
+          <t>ASSUMPTION</t>
+        </is>
+      </c>
+      <c r="F109" s="43" t="inlineStr">
+        <is>
+          <t>SERVING['tf_kv_compression']</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="45" t="inlineStr">
+        <is>
+          <t>bAttention serving throughput</t>
+        </is>
+      </c>
+      <c r="B110" s="43" t="inlineStr">
+        <is>
+          <t>562 tok/s/GPU (4,497/box): 64 concurrent 262,144-token streams on one GPU, context-flat 32k-262k (-4.0%). The 64-stream cell is a grid cap, not a ceiling — 1.62 GB of state on a 96 GB card at 9.5% GPU-busy — so it is a LOWER bound. Supersedes a 349,880 tok/s/box figure measured on the h-carry-only proxy</t>
+        </is>
+      </c>
+      <c r="E110" s="53" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F110" s="43" t="inlineStr">
+        <is>
+          <t>deck_decode_d2048_bf16_gh200_20260814.json rows[bdm, 64 streams]</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="45" t="inlineStr">
+        <is>
+          <t>bAttention per-stream state</t>
+        </is>
+      </c>
+      <c r="B111" s="43" t="inlineStr">
+        <is>
+          <t>25.4 MB/stream, the FULL recurrent cell (h + M memory), 24.2 MiB measured, context-flat. The 0.15 MB figure previously quoted was an h-carry-only proxy with no M memory and is retired as a headline</t>
+        </is>
+      </c>
+      <c r="E111" s="53" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F111" s="43" t="inlineStr">
+        <is>
+          <t>deck_decode_d2048_bf16_gh200_20260814.json state_bytes_per_stream</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="45" t="inlineStr">
+        <is>
+          <t>Transformer KV wall</t>
+        </is>
+      </c>
+      <c r="B112" s="43" t="inlineStr">
+        <is>
+          <t>197 KB per token of context per stream — 51.5 GB for one 262,144-token stream, a 2nd stream OOMs a 96 GB card, and 16 streams OOM it at 32,768 tokens. Its retired 88.5 per-token decode cost was inflated by a growing-KV re-planning harness artifact; the traced figure is 14.92 GPU-busy at 262k</t>
+        </is>
+      </c>
+      <c r="E112" s="53" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F112" s="43" t="inlineStr">
+        <is>
+          <t>deck_decode_d2048_bf16_gh200_20260814.json rows[transformer]</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="45" t="inlineStr">
+        <is>
+          <t>Training throughput at 8 GPUs</t>
+        </is>
+      </c>
+      <c r="B113" s="43" t="inlineStr">
+        <is>
+          <t>x5.15 (bAttention, fwd+bwd) vs x3.70 (transformer Ulysses best, forward-only) at matched 16-in-flight load -&gt; x1.39; x6.27 at 256 in flight -&gt; x1.70</t>
+        </is>
+      </c>
+      <c r="E113" s="53" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F113" s="43" t="inlineStr">
+        <is>
+          <t>derived.json matched_load_curve, scaling_1to8_best</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="45" t="inlineStr">
+        <is>
+          <t>Memory walls (component scope)</t>
+        </is>
+      </c>
+      <c r="B114" s="43" t="inlineStr">
+        <is>
+          <t>64k-token sequence: 30.9 GB (fits 1 GPU) vs OOM at 78.4 GB attempted; pipeline stage 9.05 GB flat vs GPipe 43.3 GB</t>
+        </is>
+      </c>
+      <c r="E114" s="53" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F114" s="43" t="inlineStr">
+        <is>
+          <t>derived.json pipeline_feasibility, pipeline_memory_asymmetry</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="45" t="inlineStr">
+        <is>
+          <t>Compute lever (flop_factor)</t>
+        </is>
+      </c>
+      <c r="B115" s="43" t="inlineStr">
+        <is>
+          <t>cross-family prefill, bf16, 1xH100, parameter counts exactly matched, block scope (1 layer, batch 16): TF/bAttention 4.02 at d512/1M, 3.83 at d1024/1M, 2.01 at d2048/262k. Short context favours the transformer and is stated so</t>
+        </is>
+      </c>
+      <c r="E115" s="53" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F115" s="43" t="inlineStr">
+        <is>
+          <t>matched_d{512,1024,2048}_h100.json (2026-07-21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="45" t="inlineStr">
+        <is>
+          <t>Compute, fp32 lane (scope reference)</t>
+        </is>
+      </c>
+      <c r="B116" s="43" t="inlineStr">
+        <is>
+          <t>the d2048/24-layer fp32 sweep gives 7.91 at 262k at full-model scope. No fp32 FlashAttention kernel exists, so that lane runs mem-efficient attention on the transformer and the owned arm is fp16 internally; params 16.7% apart. Full model in bf16 has not been run</t>
+        </is>
+      </c>
+      <c r="E116" s="52" t="inlineStr">
+        <is>
+          <t>LABEL</t>
+        </is>
+      </c>
+      <c r="F116" s="43" t="inlineStr">
+        <is>
+          <t>deck_speed_scaling_d2048_h100_20260803.json sdpa_fp32_backend_probe + last_route_attestation</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="45" t="inlineStr">
+        <is>
+          <t>16-bit IO (training)</t>
+        </is>
+      </c>
+      <c r="B117" s="43" t="inlineStr">
+        <is>
+          <t>same-arch GH200 gate at d1536: fp16 x1.185 step time and -17.5% peak memory, bf16 x1.171 and -20.6%; quality deltas +0.001 to +0.004 from the gate's smaller vehicle. Reported on its own; not an input to the compute lever</t>
+        </is>
+      </c>
+      <c r="E117" s="53" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F117" s="43" t="inlineStr">
+        <is>
+          <t>receipts/io16_gate_20260809.md (2026-08-09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="45" t="inlineStr">
+        <is>
+          <t>Quality parity at 70B</t>
+        </is>
+      </c>
+      <c r="B118" s="43" t="inlineStr">
+        <is>
+          <t>transformer needs x4.1 params [2.2-7.7] or x1.7 tokens [1.33-2.10, beta=0.28 assumption]; crossover N* ~321M = the top measured rung</t>
+        </is>
+      </c>
+      <c r="E118" s="52" t="inlineStr">
+        <is>
+          <t>PROJECTION</t>
+        </is>
+      </c>
+      <c r="F118" s="43" t="inlineStr">
+        <is>
+          <t>derived.json quality_fit.ref_70B, parity_cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="45" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B119" s="43" t="inlineStr">
+        <is>
+          <t>systems numbers are component-scope (bAttention d1536 fwd+bwd h-recurrence sub-block vs transformer d2048 forward-only layer); every speedup is vs the family's OWN 1-GPU baseline</t>
+        </is>
+      </c>
+      <c r="E119" s="52" t="inlineStr">
+        <is>
+          <t>LABEL</t>
+        </is>
+      </c>
+      <c r="F119" s="43" t="inlineStr">
+        <is>
+          <t>derived.json scope_reconciliation; deck README</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1790,7 +3596,7 @@
       <c r="C26" t="inlineStr"/>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>live: =1/(w/100+(1-w)/10)</t>
+          <t>live: =1/(w/memfac+(1-w)/flopfac)</t>
         </is>
       </c>
     </row>
@@ -1803,7 +3609,7 @@
       <c r="B27" s="16" t="n">
         <v>0.45</v>
       </c>
-      <c r="C27" s="31">
+      <c r="C27" s="37">
         <f>1/(B27/Inputs!$B$2+(1-B27)/Inputs!$B$3)</f>
         <v/>
       </c>
@@ -1822,7 +3628,7 @@
       <c r="B28" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="C28" s="31">
+      <c r="C28" s="37">
         <f>1/(B28/Inputs!$B$2+(1-B28)/Inputs!$B$3)</f>
         <v/>
       </c>
@@ -1841,7 +3647,7 @@
       <c r="B29" s="16" t="n">
         <v>0.6</v>
       </c>
-      <c r="C29" s="31">
+      <c r="C29" s="37">
         <f>1/(B29/Inputs!$B$2+(1-B29)/Inputs!$B$3)</f>
         <v/>
       </c>
@@ -1860,7 +3666,7 @@
       <c r="B30" s="16" t="n">
         <v>0.7</v>
       </c>
-      <c r="C30" s="31">
+      <c r="C30" s="37">
         <f>1/(B30/Inputs!$B$2+(1-B30)/Inputs!$B$3)</f>
         <v/>
       </c>
@@ -1879,7 +3685,7 @@
       <c r="B31" s="16" t="n">
         <v>0.82</v>
       </c>
-      <c r="C31" s="31">
+      <c r="C31" s="37">
         <f>1/(B31/Inputs!$B$2+(1-B31)/Inputs!$B$3)</f>
         <v/>
       </c>
@@ -1894,7 +3700,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1919,14 +3725,14 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Engine: GPU cost ~60% memory / ~40% compute. Memory x100 + FLOPs x10 -&gt; residual 0.6%+4% -&gt; ~22x cost-weighted reduction (Inputs B20).</t>
+          <t>Engine: GPU cost ~60% memory / ~40% compute. TODAY (default): memory x100 + FLOPs x9.24 (blend x2.19 x equal-quality parameter ratio x4.22 at 1T) -&gt; ~20x cost-weighted (Inputs B20). CEILING: FLOPs x22.1 -&gt; ~41x.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Floored by the least-reduced part (compute, 10x). Neither alone helps (mem-only ~2.5x, FLOP-only ~1.6x).</t>
+          <t xml:space="preserve">  Floored by the least-reduced part (compute). Neither alone helps (mem-only ~2.5x, FLOP-only ~1.5x).</t>
         </is>
       </c>
     </row>
@@ -2009,7 +3815,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>- Cost-weighted reduction ~22x (NOT 100x; range 17-38x over memory share 45-82%).</t>
+          <t>- Cost-weighted reduction ~20x TODAY, ~41x at the CEILING (NOT 100x; ~16-36x over memory share 45-82% at the Today lever).</t>
         </is>
       </c>
     </row>
@@ -2030,14 +3836,14 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>- Spend-cut value (named floor): FY25 ~$159B/yr (~$1.6T capitalized); FY26 r/r ~$328B/yr (~$3.3T).</t>
+          <t>- Spend-cut value (named floor, 6% discount rate): FY25 ~$159B/yr (~$2.6T capitalized); FY26 r/r ~$337B/yr (~$5.6T). Ceiling: ~$163B FY25.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>- GLOBAL estimate (named ~80% of world AI capex): FY25 ~$2.0T, FY26 ~$4.1T capitalized. Clearly an estimate.</t>
+          <t>- GLOBAL estimate (named ~80% of world AI capex): FY25 ~$3.3T, FY26 ~$7.0T capitalized. Clearly an estimate.</t>
         </is>
       </c>
     </row>
@@ -2096,7 +3902,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>- 1000x (=100x*10x) is NOT physical: cost is additive (Amdahl), not multiplicative.</t>
+          <t>- Multiplying the levers (100x * 9.2x ~ 900x) is NOT physical: cost is additive (Amdahl), not multiplicative.</t>
         </is>
       </c>
     </row>
@@ -2260,7 +4066,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>FY25 capex incl leases ~$88B [DISCLOSED proxy]; FY26 ~$190B CY26 guide. Short-lived 'half'-&gt;'two-thirds' (CFO). Accel ~75% [BOM]. AI rev $37B run-rate (Q3 FY26).</t>
+          <t>FY25 capex incl leases ~$88B [DISCLOSED proxy]; FY26 ~$190B CY26 guide (Jul'26 restated to ~$175B capex+finance-leases on an accounting change -- the gross guide is kept here). Short-lived 'half'-&gt;'two-thirds' (CFO). Accel ~75% [BOM]. AI rev $37B run-rate (Q3 FY26).</t>
         </is>
       </c>
     </row>
@@ -3012,7 +4818,7 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>2600</v>
+        <v>4250</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
@@ -3616,11 +5422,11 @@
         <v>128.3</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>FY25 cash capex $128.3B [DISCLOSED]; FY26 ~$200B. AWS ~68-70% -&gt; strips fulfillment. Accel ~67% [BOM]. AI rev &gt;$15B AWS run-rate (Q1 FY26, Jassy).</t>
+          <t>FY25 cash capex $128.3B [DISCLOSED]; FY26 raised to ~$220B (Q2'26, 2026-07-30). AWS ~68-70% -&gt; strips fulfillment. Accel ~67% [BOM]. AI rev &gt;$15B AWS run-rate (Q1 FY26, Jassy).</t>
         </is>
       </c>
     </row>
@@ -3685,7 +5491,7 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>2400</v>
+        <v>2830</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
@@ -4289,11 +6095,11 @@
         <v>72.2</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>135</v>
+        <v>137.5</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>FY25 capex incl leases $72.2B [DISCLOSED]; FY26 $125-145B. Accel ~74% [BOM]. AI rev DIRECT est ~$4B -- Meta's real AI payoff is INDIRECT ad-uplift (~$20B), not counted.</t>
+          <t>FY25 capex incl leases $72.2B [DISCLOSED]; FY26 $130-145B guide (mid 137.5). Accel ~74% [BOM]. AI rev DIRECT est ~$4B -- Meta's real AI payoff is INDIRECT ad-uplift (~$20B), not counted.</t>
         </is>
       </c>
     </row>
@@ -4358,7 +6164,7 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>1900</v>
+        <v>1490</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
@@ -4990,11 +6796,11 @@
         <v>21.2</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>50</v>
+        <v>55.7</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>FY25 capex $21.2B [DISCLOSED 10-K]; FY26 ~$50B guide (rev $67B). Capex ~all OCI/GPU data centers. Accel ~70% [BOM]. AI rev = OCI/GPU cloud (IaaS ~$12B r/r Q4 FY25; AI subset, EST).</t>
+          <t>FY25 capex $21.2B [DISCLOSED 10-K]; FY26 ACTUAL $55.7B (reported 2026-06-10; FY27 guide ~$70B net / up to $95B gross). Capex ~all OCI/GPU data centers. Accel ~70% [BOM]. AI rev = OCI/GPU cloud (IaaS ~$12B r/r Q4 FY25; AI subset, EST).</t>
         </is>
       </c>
     </row>
@@ -5059,7 +6865,7 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>700</v>
+        <v>433</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
@@ -5667,7 +7473,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>FY25 S-1 AI capex $12.7B [DISCLOSED]; FY26 ~$18B (ESTIMATE). ~all accelerator (greenfield). AI rev ~0 (nascent; Anthropic orbital compute is future).</t>
+          <t>FY25 S-1 AI capex $12.7B [DISCLOSED]; FY26 ~$18B (ESTIMATE, likely conservative -- Q1'26 AI capex alone was $7.7B, ~$31B annualized). ~all accelerator (greenfield). AI rev ~0 (nascent; Anthropic orbital compute is future).</t>
         </is>
       </c>
     </row>
@@ -5732,7 +7538,7 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>1770</v>
+        <v>1840</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
@@ -6299,7 +8105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6344,8 +8150,9 @@
           <t>FLOPs reduction factor</t>
         </is>
       </c>
-      <c r="B3" s="23" t="n">
-        <v>10</v>
+      <c r="B3" s="23">
+        <f>$B$24</f>
+        <v/>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -6354,7 +8161,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1e-1 FLOPs = 10x fewer.</t>
+          <t>TODAY scenario (default) = x9.24: the measured workload blend x2.19 (10:1 input:output, 64k context; prefill x1.17, decode x2.20 on the memory ceiling; training excluded) x the fit-derived equal-quality parameter ratio x4.22 at 1T (rows 23-25 below). Overtype with =B25 for the CEILING scenario (x22.1 = measured prefill x4.02 x 5.5 kernel speedup), or any number. See ServingTraining for the blend.</t>
         </is>
       </c>
     </row>
@@ -6406,7 +8213,7 @@
         </is>
       </c>
       <c r="B6" s="24" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -6415,7 +8222,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Perpetuity capitalization: value = annual benefit / rate (=10x at 10%).</t>
+          <t>Perpetuity capitalization: value = annual benefit / rate (=16.7x at 6%).</t>
         </is>
       </c>
     </row>
@@ -6526,7 +8333,7 @@
         </is>
       </c>
       <c r="B12" s="26" t="n">
-        <v>1770</v>
+        <v>1840</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -6535,7 +8342,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>IPO 2026-06-12 ~$1.77T (market data; used by Sensitivity).</t>
+          <t>~$1.84T Aug 2026; IPO 2026-06-12 at ~$1.77T (market data; used by Sensitivity).</t>
         </is>
       </c>
     </row>
@@ -6671,6 +8478,77 @@
       <c r="D20" s="3" t="inlineStr">
         <is>
           <t>1 / residual. The realistic $ reduction used everywhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>SCENARIOS (2026-08-17 ruling) — TODAY (default) vs CEILING</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Equal-quality parameter ratio at 1T</t>
+        </is>
+      </c>
+      <c r="B23" s="28" t="n">
+        <v>4.2185</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>FIT-DERIVED (sealed 2026-08-14 refit): bAttention matches the transformer fit's quality on 23.7% of the params at 1T -&gt; x4.22 compute per token at equal quality. 84.2% at 1B, 55.2% at 10B, 36.2% at 100B. A projection of the two fits, not a measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>TODAY compute lever = blend x ratio</t>
+        </is>
+      </c>
+      <c r="B24" s="29">
+        <f>ServingTraining!$B$28*$B$23</f>
+        <v/>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>B3 (the FLOPs lever) points here by default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CEILING compute lever</t>
+        </is>
+      </c>
+      <c r="B25" s="28" t="n">
+        <v>22.09</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Measured prefill x4.02 (bf16 parameter-matched, d512/1M, 2026-07-21) x 5.5 kernel-campaign speedup. Overtype B3 with =B25 to run the workbook at the ceiling (~41x cost-weighted).</t>
         </is>
       </c>
     </row>
@@ -6698,7 +8576,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SENSITIVITY (SpaceX) — count-based reduction tiers vs cost-weighted</t>
+          <t>SENSITIVITY (SpaceX) — TODAY vs CEILING vs live cost-weighted</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -6714,22 +8592,17 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>10x compute-bound</t>
+          <t>TODAY (~20x)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>30x balanced</t>
+          <t>CEILING (~41x)</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>100x memory-bound</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Cost-weighted</t>
+          <t>Cost-weighted (live)</t>
         </is>
       </c>
     </row>
@@ -6740,18 +8613,14 @@
         </is>
       </c>
       <c r="B3" s="19">
-        <f>SpaceX!$B$12/(10)</f>
+        <f>SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$24))</f>
         <v/>
       </c>
       <c r="C3" s="19">
-        <f>SpaceX!$B$12/(30)</f>
+        <f>SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$25))</f>
         <v/>
       </c>
       <c r="D3" s="19">
-        <f>SpaceX!$B$12/(100)</f>
-        <v/>
-      </c>
-      <c r="E3" s="19">
         <f>SpaceX!$B$12/(Inputs!$B$20)</f>
         <v/>
       </c>
@@ -6763,18 +8632,14 @@
         </is>
       </c>
       <c r="B4" s="19">
-        <f>SpaceX!$B$12-SpaceX!$B$12/(10)</f>
+        <f>SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$24))</f>
         <v/>
       </c>
       <c r="C4" s="19">
-        <f>SpaceX!$B$12-SpaceX!$B$12/(30)</f>
+        <f>SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$25))</f>
         <v/>
       </c>
       <c r="D4" s="19">
-        <f>SpaceX!$B$12-SpaceX!$B$12/(100)</f>
-        <v/>
-      </c>
-      <c r="E4" s="19">
         <f>SpaceX!$B$12-SpaceX!$B$12/(Inputs!$B$20)</f>
         <v/>
       </c>
@@ -6797,10 +8662,6 @@
         <f>SpaceX!$B$26</f>
         <v/>
       </c>
-      <c r="E5" s="5">
-        <f>SpaceX!$B$26</f>
-        <v/>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6809,18 +8670,14 @@
         </is>
       </c>
       <c r="B6" s="19">
-        <f>(SpaceX!$B$12-SpaceX!$B$12/(10))+SpaceX!$B$26/1000</f>
+        <f>(SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$24)))+SpaceX!$B$26/1000</f>
         <v/>
       </c>
       <c r="C6" s="19">
-        <f>(SpaceX!$B$12-SpaceX!$B$12/(30))+SpaceX!$B$26/1000</f>
+        <f>(SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$25)))+SpaceX!$B$26/1000</f>
         <v/>
       </c>
       <c r="D6" s="19">
-        <f>(SpaceX!$B$12-SpaceX!$B$12/(100))+SpaceX!$B$26/1000</f>
-        <v/>
-      </c>
-      <c r="E6" s="19">
         <f>(SpaceX!$B$12-SpaceX!$B$12/(Inputs!$B$20))+SpaceX!$B$26/1000</f>
         <v/>
       </c>
@@ -6832,18 +8689,14 @@
         </is>
       </c>
       <c r="B7" s="18">
-        <f>((SpaceX!$B$12-SpaceX!$B$12/(10))+SpaceX!$B$26/1000)/Inputs!$B$6</f>
+        <f>((SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$24)))+SpaceX!$B$26/1000)/Inputs!$B$6</f>
         <v/>
       </c>
       <c r="C7" s="18">
-        <f>((SpaceX!$B$12-SpaceX!$B$12/(30))+SpaceX!$B$26/1000)/Inputs!$B$6</f>
+        <f>((SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$25)))+SpaceX!$B$26/1000)/Inputs!$B$6</f>
         <v/>
       </c>
       <c r="D7" s="18">
-        <f>((SpaceX!$B$12-SpaceX!$B$12/(100))+SpaceX!$B$26/1000)/Inputs!$B$6</f>
-        <v/>
-      </c>
-      <c r="E7" s="18">
         <f>((SpaceX!$B$12-SpaceX!$B$12/(Inputs!$B$20))+SpaceX!$B$26/1000)/Inputs!$B$6</f>
         <v/>
       </c>
@@ -6855,18 +8708,14 @@
         </is>
       </c>
       <c r="B8" s="21">
-        <f>(((SpaceX!$B$12-SpaceX!$B$12/(10))+SpaceX!$B$26/1000)/Inputs!$B$6)/Inputs!$B$12</f>
+        <f>(((SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$24)))+SpaceX!$B$26/1000)/Inputs!$B$6)/Inputs!$B$12</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>(((SpaceX!$B$12-SpaceX!$B$12/(30))+SpaceX!$B$26/1000)/Inputs!$B$6)/Inputs!$B$12</f>
+        <f>(((SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$25)))+SpaceX!$B$26/1000)/Inputs!$B$6)/Inputs!$B$12</f>
         <v/>
       </c>
       <c r="D8" s="21">
-        <f>(((SpaceX!$B$12-SpaceX!$B$12/(100))+SpaceX!$B$26/1000)/Inputs!$B$6)/Inputs!$B$12</f>
-        <v/>
-      </c>
-      <c r="E8" s="21">
         <f>(((SpaceX!$B$12-SpaceX!$B$12/(Inputs!$B$20))+SpaceX!$B$26/1000)/Inputs!$B$6)/Inputs!$B$12</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
SpaceX refresh, io16-only lane, dedup; FY26 re-based
- SpaceX: mcap 1840 -> 1950; FY26 AI capex 18 -> ~55 (H1'26 disclosed $23.5B:
  Q1 $7.7B + Q2 $15.8B, capex guided roughly flat Q3/Q4). FY26 named cut
  ~$366B (~$6.1T capitalized), global ~$7.6T.
- 16-bit is the only lane shown (competition serves in 16-bit): fp32 full-model
  sweep and the io16 training gate retired to one Evidence/assumption row each,
  in both the app and the workbook.
- Decode re-base story deduplicated: full derivation lives in Methodology,
  other surfaces carry one sentence + pointer.
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -28,7 +28,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
@@ -38,7 +38,6 @@
     <numFmt numFmtId="170" formatCode="$0.00"/>
     <numFmt numFmtId="171" formatCode="0.0×"/>
     <numFmt numFmtId="172" formatCode="0.00×"/>
-    <numFmt numFmtId="173" formatCode="0.000×"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -119,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -183,7 +182,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="172" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -1429,7 +1427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F119"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1828,7 +1826,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>SCOPE: the serving and training blocks below are component-scope systems benches (bAttention d1536 fwd+bwd h-recurrence sub-block vs transformer d2048 forward-only layer); every speedup there is each family vs its OWN 1-GPU baseline. The prefill lanes quoted further down are cross-family: bf16 parameter-matched at block scope, and fp32 at full-model scope.</t>
+          <t>SCOPE: the serving and training blocks below are component-scope systems benches (bAttention d1536 fwd+bwd h-recurrence sub-block vs transformer d2048 forward-only layer); every speedup there is each family vs its OWN 1-GPU baseline. The prefill lanes quoted further down are cross-family: 16-bit parameter-matched at block scope (the fp32 full-model sweep is retired to an assumption row).</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2229,7 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>The prefill component itself exists in two lanes, both shown below. It comes from the bf16 lane, where both families run their production attention kernels (there is no fp32 FlashAttention kernel). BF16 LANE: parameter counts exactly matched, 1 layer, batch 16, 1 x H100 80GB HBM3, 2026-07-21 — x4.02 at d512/1M, x3.83 at d1024/1M, x2.01 at d2048/262k. Receipts: experiments/paper_figures/output/matched_d{512,1024,2048}_h100.json</t>
+          <t>The prefill component, 16-bit and parameter-matched — the lane the competition serves in. Parameter counts exactly matched, 1 layer, batch 16, 1 x H100 80GB HBM3, 2026-07-21 — x4.02 at d512/1M, x3.83 at d1024/1M, x2.01 at d2048/262k. The fp32 full-model sweep and the own-baseline 16-bit-IO training gate are retired to one assumption row each below. Receipts: experiments/paper_figures/output/matched_d{512,1024,2048}_h100.json</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2257,7 @@
       <c r="E70" s="38" t="inlineStr"/>
       <c r="F70" s="38" t="inlineStr">
         <is>
-          <t>Lane / note</t>
+          <t>Note</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2276,7 @@
       </c>
       <c r="F71" s="43" t="inlineStr">
         <is>
-          <t>bf16 (lever) — transformer ahead</t>
+          <t>transformer ahead</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2295,7 @@
       </c>
       <c r="F72" s="43" t="inlineStr">
         <is>
-          <t>bf16 (lever) — transformer ahead</t>
+          <t>transformer ahead</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2314,7 @@
       </c>
       <c r="F73" s="43" t="inlineStr">
         <is>
-          <t>bf16 (lever) — transformer ahead</t>
+          <t>transformer ahead</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2333,7 @@
       </c>
       <c r="F74" s="43" t="inlineStr">
         <is>
-          <t>bf16 (lever) — transformer ahead</t>
+          <t>transformer ahead</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2352,7 @@
       </c>
       <c r="F75" s="43" t="inlineStr">
         <is>
-          <t>bf16 (lever) — transformer ahead</t>
+          <t>transformer ahead</t>
         </is>
       </c>
     </row>
@@ -2373,7 +2371,7 @@
       </c>
       <c r="F76" s="43" t="inlineStr">
         <is>
-          <t>bf16 (lever) — transformer ahead</t>
+          <t>transformer ahead</t>
         </is>
       </c>
     </row>
@@ -2390,11 +2388,7 @@
       <c r="D77" s="50" t="n">
         <v>1.287120565606265</v>
       </c>
-      <c r="F77" s="43" t="inlineStr">
-        <is>
-          <t>bf16 (lever)</t>
-        </is>
-      </c>
+      <c r="F77" s="43" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="39" t="n">
@@ -2409,11 +2403,7 @@
       <c r="D78" s="50" t="n">
         <v>2.014140219042289</v>
       </c>
-      <c r="F78" s="43" t="inlineStr">
-        <is>
-          <t>bf16 (lever)</t>
-        </is>
-      </c>
+      <c r="F78" s="43" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="39" t="n">
@@ -2428,759 +2418,435 @@
       <c r="D79" s="50" t="n">
         <v>2.841237678947035</v>
       </c>
-      <c r="F79" s="43" t="inlineStr">
-        <is>
-          <t>bf16 (lever)</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="39" t="n">
-        <v>512</v>
-      </c>
-      <c r="B80" s="5" t="n">
-        <v>6.578</v>
-      </c>
-      <c r="C80" s="15" t="n">
-        <v>61.216</v>
-      </c>
-      <c r="D80" s="50" t="n">
-        <v>0.1074555671719812</v>
-      </c>
-      <c r="F80" s="43" t="inlineStr">
-        <is>
-          <t>fp32 (full model) — transformer ahead</t>
-        </is>
-      </c>
+      <c r="F79" s="43" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="39" t="n">
-        <v>1024</v>
-      </c>
-      <c r="B81" s="5" t="n">
-        <v>12.611</v>
-      </c>
-      <c r="C81" s="15" t="n">
-        <v>86.66</v>
-      </c>
-      <c r="D81" s="50" t="n">
-        <v>0.145522732517886</v>
-      </c>
-      <c r="F81" s="43" t="inlineStr">
-        <is>
-          <t>fp32 (full model) — transformer ahead</t>
-        </is>
-      </c>
+      <c r="A81" s="1" t="inlineStr">
+        <is>
+          <t>Assumptions — one row each (MEASURED / PROJECTION / ASSUMPTION)</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="n"/>
+      <c r="C81" s="2" t="n"/>
+      <c r="D81" s="2" t="n"/>
+      <c r="E81" s="2" t="n"/>
+      <c r="F81" s="2" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="39" t="n">
-        <v>2048</v>
-      </c>
-      <c r="B82" s="5" t="n">
-        <v>27.856</v>
-      </c>
-      <c r="C82" s="15" t="n">
-        <v>160.738</v>
-      </c>
-      <c r="D82" s="50" t="n">
-        <v>0.1733006507484229</v>
-      </c>
-      <c r="F82" s="43" t="inlineStr">
-        <is>
-          <t>fp32 (full model) — transformer ahead</t>
+      <c r="A82" s="38" t="inlineStr">
+        <is>
+          <t>Assumption</t>
+        </is>
+      </c>
+      <c r="B82" s="38" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C82" s="38" t="inlineStr"/>
+      <c r="D82" s="38" t="inlineStr"/>
+      <c r="E82" s="38" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F82" s="38" t="inlineStr">
+        <is>
+          <t>Source</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="39" t="n">
-        <v>4096</v>
-      </c>
-      <c r="B83" s="5" t="n">
-        <v>70.339</v>
-      </c>
-      <c r="C83" s="15" t="n">
-        <v>305.622</v>
-      </c>
-      <c r="D83" s="50" t="n">
-        <v>0.2301503164039238</v>
+      <c r="A83" s="45" t="inlineStr">
+        <is>
+          <t>Compute lever (economics slide)</t>
+        </is>
+      </c>
+      <c r="B83" s="43" t="inlineStr">
+        <is>
+          <t>x9.24 = the x2.19 MEASURED serving blend x the x4.22 FIT-DERIVED equal-quality parameter ratio at trillion scale</t>
+        </is>
+      </c>
+      <c r="E83" s="51" t="inlineStr">
+        <is>
+          <t>MEASURED x PROJECTION</t>
+        </is>
       </c>
       <c r="F83" s="43" t="inlineStr">
         <is>
-          <t>fp32 (full model) — transformer ahead</t>
+          <t>workload_compute_advantage() x quality_matched_compute_lever(); receipts derived.json + quality_fit_v4.json</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="39" t="n">
-        <v>8192</v>
-      </c>
-      <c r="B84" s="5" t="n">
-        <v>207.758</v>
-      </c>
-      <c r="C84" s="15" t="n">
-        <v>595.671</v>
-      </c>
-      <c r="D84" s="50" t="n">
-        <v>0.3487797794420074</v>
+      <c r="A84" s="45" t="inlineStr">
+        <is>
+          <t>Equal-quality parameter matching</t>
+        </is>
+      </c>
+      <c r="B84" s="43" t="inlineStr">
+        <is>
+          <t>sealed 2026-08-14 refit, 4 rungs per family (47M-663M params): the fits cross at 392M and bAttention then matches the transformer fit's quality on 84.2% of the params at 1B, 55.2% at 10B, 36.2% at 100B, 23.7% at 1T, 15.5% at 10T. The receipt's own words: 'a projection of the two fits, not a measurement'</t>
+        </is>
+      </c>
+      <c r="E84" s="51" t="inlineStr">
+        <is>
+          <t>PROJECTION</t>
+        </is>
       </c>
       <c r="F84" s="43" t="inlineStr">
         <is>
-          <t>fp32 (full model) — transformer ahead</t>
+          <t>quality_fit_v4.json param_matching; fits over the sealed rope-convention ladder</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="39" t="n">
-        <v>16384</v>
-      </c>
-      <c r="B85" s="5" t="n">
-        <v>686.813</v>
-      </c>
-      <c r="C85" s="15" t="n">
-        <v>1177.361</v>
-      </c>
-      <c r="D85" s="50" t="n">
-        <v>0.5833495418992135</v>
+      <c r="A85" s="45" t="inlineStr">
+        <is>
+          <t>Single-GPU training step (AGAINST us)</t>
+        </is>
+      </c>
+      <c r="B85" s="43" t="inlineStr">
+        <is>
+          <t>at 2,048-token context on one GPU a bAttention step costs x6.46 MORE (8,979 vs 1,389 ms/step, d1536/27L, fp16, 601-step protocol). At equal quality the same step costs x1.53 more, not x6.46 - the parameter ratio shrinks the gap but does not erase it. Training is excluded from the serving claim for this reason</t>
+        </is>
+      </c>
+      <c r="E85" s="52" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
       </c>
       <c r="F85" s="43" t="inlineStr">
         <is>
-          <t>fp32 (full model) — transformer ahead</t>
+          <t>dtype_trio_v4.json rows[fp16]</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="39" t="n">
-        <v>32768</v>
-      </c>
-      <c r="B86" s="5" t="n">
-        <v>2518.562</v>
-      </c>
-      <c r="C86" s="15" t="n">
-        <v>2359.638</v>
-      </c>
-      <c r="D86" s="50" t="n">
-        <v>1.067351008925945</v>
+      <c r="A86" s="45" t="inlineStr">
+        <is>
+          <t>$/GPU-hour</t>
+        </is>
+      </c>
+      <c r="B86" s="43" t="inlineStr">
+        <is>
+          <t>$2.50 (H100 rent, neocloud/committed mid; ladder 2.00-3.50)</t>
+        </is>
+      </c>
+      <c r="E86" s="51" t="inlineStr">
+        <is>
+          <t>ASSUMPTION</t>
+        </is>
       </c>
       <c r="F86" s="43" t="inlineStr">
         <is>
-          <t>fp32 (full model)</t>
+          <t>this file's CostLadder row — unchanged rate basis</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="39" t="n">
-        <v>65536</v>
-      </c>
-      <c r="B87" s="5" t="n">
-        <v>9629.459000000001</v>
-      </c>
-      <c r="C87" s="15" t="n">
-        <v>4704.054</v>
-      </c>
-      <c r="D87" s="50" t="n">
-        <v>2.047055369687508</v>
+      <c r="A87" s="45" t="inlineStr">
+        <is>
+          <t>Utilization</t>
+        </is>
+      </c>
+      <c r="B87" s="43" t="inlineStr">
+        <is>
+          <t>85%</t>
+        </is>
+      </c>
+      <c r="E87" s="51" t="inlineStr">
+        <is>
+          <t>ASSUMPTION</t>
+        </is>
       </c>
       <c r="F87" s="43" t="inlineStr">
         <is>
-          <t>fp32 (full model)</t>
+          <t>same value as the ladder's owned-TCO cross-check</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="39" t="n">
-        <v>131072</v>
-      </c>
-      <c r="B88" s="5" t="n">
-        <v>37690.932</v>
-      </c>
-      <c r="C88" s="15" t="n">
-        <v>9432.108</v>
-      </c>
-      <c r="D88" s="50" t="n">
-        <v>3.996024218552205</v>
+      <c r="A88" s="45" t="inlineStr">
+        <is>
+          <t>Context-length mix</t>
+        </is>
+      </c>
+      <c r="B88" s="43" t="inlineStr">
+        <is>
+          <t>headline quoted at 262k (a measured decode cell); table sweeps 4k-1M. The decode lever crosses 1 at ~29,800 tokens and BELOW that the transformer serves more tokens per GPU-second than we do — stated on every surface</t>
+        </is>
+      </c>
+      <c r="E88" s="51" t="inlineStr">
+        <is>
+          <t>ASSUMPTION</t>
+        </is>
       </c>
       <c r="F88" s="43" t="inlineStr">
         <is>
-          <t>fp32 (full model)</t>
+          <t>serving_cost_curve, decode_throughput_ratio</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="39" t="n">
-        <v>262144</v>
-      </c>
-      <c r="B89" s="5" t="n">
-        <v>149366.343</v>
-      </c>
-      <c r="C89" s="15" t="n">
-        <v>18888.452</v>
-      </c>
-      <c r="D89" s="50" t="n">
-        <v>7.907812826588436</v>
+      <c r="A89" s="45" t="inlineStr">
+        <is>
+          <t>Decode lever is MEMORY-CEILING, not latency (READ FIRST)</t>
+        </is>
+      </c>
+      <c r="B89" s="43" t="inlineStr">
+        <is>
+          <t>per generated token at ONE stream the transformer is AHEAD of us at 64k context — 4.92 vs 5.74 GPU-busy per token. The lever is that it cannot hold many long-context streams: it re-reads its whole KV cache per emitted token, so its aggregate throughput falls as 1/context while ours is flat. Measured: 1 stream at 262k (2 OOM — an exact ceiling) and 8 streams at 32k (16 OOM, so that ceiling is only bracketed at 8-15 and the 32k cell is a bounded x0.97-1.14, near parity) against 64 of ours in 1.62 GB</t>
+        </is>
+      </c>
+      <c r="E89" s="52" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
       </c>
       <c r="F89" s="43" t="inlineStr">
         <is>
-          <t>fp32 (full model)</t>
+          <t>deck_decode_d2048_bf16_gh200_20260814.json; DECODE_THROUGHPUT_20260814</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="3" t="inlineStr">
-        <is>
-          <t>Both blocks are d2048, so the lanes are directly comparable: 2.01x in bf16 against 7.91x in fp32 at 262k. The fp32 lane is full-model scope (24 layers, batch 1) and its receipt records FLASH_ATTENTION and CUDNN_ATTENTION as 'rejected: No available kernel', with the owned arm's route attestation reading dtype_mix io=fp32,bf_col=fp16; its params differ by 16.7%. Full model in bf16 has not been run. Receipt: experiments/paper_figures/output/deck_speed_scaling_d2048_h100_20260803.json</t>
+      <c r="A90" s="45" t="inlineStr">
+        <is>
+          <t>Transformer-stack maturity</t>
+        </is>
+      </c>
+      <c r="B90" s="43" t="inlineStr">
+        <is>
+          <t>NOT GRANTED by default since the 2026-08-14 re-base: the headline runs on the measured cells, in which neither family's decode is optimised (ours ran the unoptimised Triton per-step path at 9.5% GPU-busy while the transformer sat at 95.6%). Setting tf_kv_compression=8.0 grants it paged attention + KV quantization, divides our decode lever by 8 and puts the TRANSFORMER ahead at 64k — reported, not hidden</t>
+        </is>
+      </c>
+      <c r="E90" s="51" t="inlineStr">
+        <is>
+          <t>ASSUMPTION</t>
+        </is>
+      </c>
+      <c r="F90" s="43" t="inlineStr">
+        <is>
+          <t>SERVING['tf_kv_compression']</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="45" t="inlineStr">
+        <is>
+          <t>bAttention serving throughput</t>
+        </is>
+      </c>
+      <c r="B91" s="43" t="inlineStr">
+        <is>
+          <t>562 tok/s/GPU (4,497/box): 64 concurrent 262,144-token streams on one GPU, context-flat 32k-262k (-4.0%). The 64-stream cell is a grid cap, not a ceiling — 1.62 GB of state on a 96 GB card at 9.5% GPU-busy — so it is a LOWER bound. Supersedes a 349,880 tok/s/box figure measured on the h-carry-only proxy</t>
+        </is>
+      </c>
+      <c r="E91" s="52" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F91" s="43" t="inlineStr">
+        <is>
+          <t>deck_decode_d2048_bf16_gh200_20260814.json rows[bdm, 64 streams]</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="inlineStr">
-        <is>
-          <t>16-bit IO in training</t>
-        </is>
-      </c>
-      <c r="B92" s="2" t="n"/>
-      <c r="C92" s="2" t="n"/>
-      <c r="D92" s="2" t="n"/>
-      <c r="E92" s="2" t="n"/>
-      <c r="F92" s="2" t="n"/>
+      <c r="A92" s="45" t="inlineStr">
+        <is>
+          <t>bAttention per-stream state</t>
+        </is>
+      </c>
+      <c r="B92" s="43" t="inlineStr">
+        <is>
+          <t>25.4 MB/stream, the FULL recurrent cell (h + M memory), 24.2 MiB measured, context-flat. The 0.15 MB figure previously quoted was an h-carry-only proxy with no M memory and is retired as a headline</t>
+        </is>
+      </c>
+      <c r="E92" s="52" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F92" s="43" t="inlineStr">
+        <is>
+          <t>deck_decode_d2048_bf16_gh200_20260814.json state_bytes_per_stream</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="3" t="inlineStr">
-        <is>
-          <t>A training step-time gate: same architecture on every row, only the IO dtype varies. d1536 / 27 layers / block 2048 / batch 32 / seed 1, 1 x GH200 480GB, GPU verified idle before each arm, steady state only. 0 skipped steps on all arms; verdict PASS_io16_SHIPS. Throughput and memory rows are d1536/L27; the val deltas come from the gate's smaller vehicle (width 512, 15 layers). This is why the production training lane is 16-bit; it is not an input to the compute lever above. Receipt: experiments/paper_figures/output/receipts/io16_gate_20260809.md</t>
+      <c r="A93" s="45" t="inlineStr">
+        <is>
+          <t>Transformer KV wall</t>
+        </is>
+      </c>
+      <c r="B93" s="43" t="inlineStr">
+        <is>
+          <t>197 KB per token of context per stream — 51.5 GB for one 262,144-token stream, a 2nd stream OOMs a 96 GB card, and 16 streams OOM it at 32,768 tokens. Its retired 88.5 per-token decode cost was inflated by a growing-KV re-planning harness artifact; the traced figure is 14.92 GPU-busy at 262k</t>
+        </is>
+      </c>
+      <c r="E93" s="52" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F93" s="43" t="inlineStr">
+        <is>
+          <t>deck_decode_d2048_bf16_gh200_20260814.json rows[transformer]</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="45" t="inlineStr">
+        <is>
+          <t>Training throughput at 8 GPUs</t>
+        </is>
+      </c>
+      <c r="B94" s="43" t="inlineStr">
+        <is>
+          <t>x5.15 (bAttention, fwd+bwd) vs x3.70 (transformer Ulysses best, forward-only) at matched 16-in-flight load -&gt; x1.39; x6.27 at 256 in flight -&gt; x1.70</t>
+        </is>
+      </c>
+      <c r="E94" s="52" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F94" s="43" t="inlineStr">
+        <is>
+          <t>derived.json matched_load_curve, scaling_1to8_best</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="38" t="inlineStr">
-        <is>
-          <t>IO dtype</t>
-        </is>
-      </c>
-      <c r="B95" s="38" t="inlineStr">
-        <is>
-          <t>s/step</t>
-        </is>
-      </c>
-      <c r="C95" s="38" t="inlineStr">
-        <is>
-          <t>Speed vs fp32</t>
-        </is>
-      </c>
-      <c r="D95" s="38" t="inlineStr">
-        <is>
-          <t>Peak allocated (GB)</t>
-        </is>
-      </c>
-      <c r="E95" s="38" t="inlineStr">
-        <is>
-          <t>Memory vs fp32</t>
-        </is>
-      </c>
-      <c r="F95" s="38" t="inlineStr">
-        <is>
-          <t>Val cost @601 steps</t>
+      <c r="A95" s="45" t="inlineStr">
+        <is>
+          <t>Memory walls (component scope)</t>
+        </is>
+      </c>
+      <c r="B95" s="43" t="inlineStr">
+        <is>
+          <t>64k-token sequence: 30.9 GB (fits 1 GPU) vs OOM at 78.4 GB attempted; pipeline stage 9.05 GB flat vs GPipe 43.3 GB</t>
+        </is>
+      </c>
+      <c r="E95" s="52" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F95" s="43" t="inlineStr">
+        <is>
+          <t>derived.json pipeline_feasibility, pipeline_memory_asymmetry</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="45" t="inlineStr">
         <is>
-          <t>fp32</t>
-        </is>
-      </c>
-      <c r="B96" s="33" t="n">
-        <v>10.46</v>
-      </c>
-      <c r="C96" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="D96" s="26" t="n">
-        <v>70.669921875</v>
-      </c>
-      <c r="E96" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F96" s="45" t="inlineStr">
-        <is>
-          <t>baseline</t>
+          <t>Compute lever (flop_factor)</t>
+        </is>
+      </c>
+      <c r="B96" s="43" t="inlineStr">
+        <is>
+          <t>cross-family prefill, bf16, 1xH100, parameter counts exactly matched, block scope (1 layer, batch 16): TF/bAttention 4.02 at d512/1M, 3.83 at d1024/1M, 2.01 at d2048/262k. Short context favours the transformer and is stated so</t>
+        </is>
+      </c>
+      <c r="E96" s="52" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F96" s="43" t="inlineStr">
+        <is>
+          <t>matched_d{512,1024,2048}_h100.json (2026-07-21)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="45" t="inlineStr">
         <is>
-          <t>fp16</t>
-        </is>
-      </c>
-      <c r="B97" s="33" t="n">
-        <v>8.827999999999999</v>
-      </c>
-      <c r="C97" s="51" t="n">
-        <v>1.185</v>
-      </c>
-      <c r="D97" s="26" t="n">
-        <v>58.2685546875</v>
-      </c>
-      <c r="E97" s="51" t="n">
-        <v>0.825</v>
-      </c>
-      <c r="F97" s="45" t="inlineStr">
-        <is>
-          <t>+0.00128</t>
+          <t>Compute, fp32 lane (scope reference)</t>
+        </is>
+      </c>
+      <c r="B97" s="43" t="inlineStr">
+        <is>
+          <t>the d2048/24-layer fp32 sweep gives 7.91 at 262k at full-model scope. No fp32 FlashAttention kernel exists, so that lane runs mem-efficient attention on the transformer and the owned arm is fp16 internally; params 16.7% apart. Full model in bf16 has not been run</t>
+        </is>
+      </c>
+      <c r="E97" s="51" t="inlineStr">
+        <is>
+          <t>LABEL</t>
+        </is>
+      </c>
+      <c r="F97" s="43" t="inlineStr">
+        <is>
+          <t>deck_speed_scaling_d2048_h100_20260803.json sdpa_fp32_backend_probe + last_route_attestation</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="45" t="inlineStr">
         <is>
-          <t>bf16</t>
-        </is>
-      </c>
-      <c r="B98" s="33" t="n">
-        <v>8.930999999999999</v>
-      </c>
-      <c r="C98" s="51" t="n">
-        <v>1.171</v>
-      </c>
-      <c r="D98" s="26" t="n">
-        <v>56.10546875</v>
-      </c>
-      <c r="E98" s="51" t="n">
-        <v>0.794</v>
-      </c>
-      <c r="F98" s="45" t="inlineStr">
-        <is>
-          <t>+0.00391</t>
+          <t>16-bit IO (training)</t>
+        </is>
+      </c>
+      <c r="B98" s="43" t="inlineStr">
+        <is>
+          <t>same-arch GH200 gate at d1536: fp16 x1.185 step time and -17.5% peak memory, bf16 x1.171 and -20.6%; quality deltas +0.001 to +0.004 from the gate's smaller vehicle. Reported on its own; not an input to the compute lever</t>
+        </is>
+      </c>
+      <c r="E98" s="52" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F98" s="43" t="inlineStr">
+        <is>
+          <t>receipts/io16_gate_20260809.md (2026-08-09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="45" t="inlineStr">
+        <is>
+          <t>Quality parity at 70B</t>
+        </is>
+      </c>
+      <c r="B99" s="43" t="inlineStr">
+        <is>
+          <t>transformer needs x4.1 params [2.2-7.7] or x1.7 tokens [1.33-2.10, beta=0.28 assumption]; crossover N* ~321M = the top measured rung</t>
+        </is>
+      </c>
+      <c r="E99" s="51" t="inlineStr">
+        <is>
+          <t>PROJECTION</t>
+        </is>
+      </c>
+      <c r="F99" s="43" t="inlineStr">
+        <is>
+          <t>derived.json quality_fit.ref_70B, parity_cost</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="inlineStr">
-        <is>
-          <t>Assumptions — one row each (MEASURED / PROJECTION / ASSUMPTION)</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="n"/>
-      <c r="C100" s="2" t="n"/>
-      <c r="D100" s="2" t="n"/>
-      <c r="E100" s="2" t="n"/>
-      <c r="F100" s="2" t="n"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="38" t="inlineStr">
-        <is>
-          <t>Assumption</t>
-        </is>
-      </c>
-      <c r="B101" s="38" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C101" s="38" t="inlineStr"/>
-      <c r="D101" s="38" t="inlineStr"/>
-      <c r="E101" s="38" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F101" s="38" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="45" t="inlineStr">
-        <is>
-          <t>Compute lever (economics slide)</t>
-        </is>
-      </c>
-      <c r="B102" s="43" t="inlineStr">
-        <is>
-          <t>x9.24 = the x2.19 MEASURED serving blend x the x4.22 FIT-DERIVED equal-quality parameter ratio at trillion scale</t>
-        </is>
-      </c>
-      <c r="E102" s="52" t="inlineStr">
-        <is>
-          <t>MEASURED x PROJECTION</t>
-        </is>
-      </c>
-      <c r="F102" s="43" t="inlineStr">
-        <is>
-          <t>workload_compute_advantage() x quality_matched_compute_lever(); receipts derived.json + quality_fit_v4.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="45" t="inlineStr">
-        <is>
-          <t>Equal-quality parameter matching</t>
-        </is>
-      </c>
-      <c r="B103" s="43" t="inlineStr">
-        <is>
-          <t>sealed 2026-08-14 refit, 4 rungs per family (47M-663M params): the fits cross at 392M and bAttention then matches the transformer fit's quality on 84.2% of the params at 1B, 55.2% at 10B, 36.2% at 100B, 23.7% at 1T, 15.5% at 10T. The receipt's own words: 'a projection of the two fits, not a measurement'</t>
-        </is>
-      </c>
-      <c r="E103" s="52" t="inlineStr">
-        <is>
-          <t>PROJECTION</t>
-        </is>
-      </c>
-      <c r="F103" s="43" t="inlineStr">
-        <is>
-          <t>quality_fit_v4.json param_matching; fits over the sealed rope-convention ladder</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="45" t="inlineStr">
-        <is>
-          <t>Single-GPU training step (AGAINST us)</t>
-        </is>
-      </c>
-      <c r="B104" s="43" t="inlineStr">
-        <is>
-          <t>at 2,048-token context on one GPU a bAttention step costs x6.46 MORE (8,979 vs 1,389 ms/step, d1536/27L, fp16, 601-step protocol). At equal quality the same step costs x1.53 more, not x6.46 - the parameter ratio shrinks the gap but does not erase it. Training is excluded from the serving claim for this reason</t>
-        </is>
-      </c>
-      <c r="E104" s="53" t="inlineStr">
-        <is>
-          <t>MEASURED</t>
-        </is>
-      </c>
-      <c r="F104" s="43" t="inlineStr">
-        <is>
-          <t>dtype_trio_v4.json rows[fp16]</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="45" t="inlineStr">
-        <is>
-          <t>$/GPU-hour</t>
-        </is>
-      </c>
-      <c r="B105" s="43" t="inlineStr">
-        <is>
-          <t>$2.50 (H100 rent, neocloud/committed mid; ladder 2.00-3.50)</t>
-        </is>
-      </c>
-      <c r="E105" s="52" t="inlineStr">
-        <is>
-          <t>ASSUMPTION</t>
-        </is>
-      </c>
-      <c r="F105" s="43" t="inlineStr">
-        <is>
-          <t>this file's CostLadder row — unchanged rate basis</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="45" t="inlineStr">
-        <is>
-          <t>Utilization</t>
-        </is>
-      </c>
-      <c r="B106" s="43" t="inlineStr">
-        <is>
-          <t>85%</t>
-        </is>
-      </c>
-      <c r="E106" s="52" t="inlineStr">
-        <is>
-          <t>ASSUMPTION</t>
-        </is>
-      </c>
-      <c r="F106" s="43" t="inlineStr">
-        <is>
-          <t>same value as the ladder's owned-TCO cross-check</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="45" t="inlineStr">
-        <is>
-          <t>Context-length mix</t>
-        </is>
-      </c>
-      <c r="B107" s="43" t="inlineStr">
-        <is>
-          <t>headline quoted at 262k (a measured decode cell); table sweeps 4k-1M. The decode lever crosses 1 at ~29,800 tokens and BELOW that the transformer serves more tokens per GPU-second than we do — stated on every surface</t>
-        </is>
-      </c>
-      <c r="E107" s="52" t="inlineStr">
-        <is>
-          <t>ASSUMPTION</t>
-        </is>
-      </c>
-      <c r="F107" s="43" t="inlineStr">
-        <is>
-          <t>serving_cost_curve, decode_throughput_ratio</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="45" t="inlineStr">
-        <is>
-          <t>Decode lever is MEMORY-CEILING, not latency (READ FIRST)</t>
-        </is>
-      </c>
-      <c r="B108" s="43" t="inlineStr">
-        <is>
-          <t>per generated token at ONE stream the transformer is AHEAD of us at 64k context — 4.92 vs 5.74 GPU-busy per token. The lever is that it cannot hold many long-context streams: it re-reads its whole KV cache per emitted token, so its aggregate throughput falls as 1/context while ours is flat. Measured: 1 stream at 262k (2 OOM — an exact ceiling) and 8 streams at 32k (16 OOM, so that ceiling is only bracketed at 8-15 and the 32k cell is a bounded x0.97-1.14, near parity) against 64 of ours in 1.62 GB</t>
-        </is>
-      </c>
-      <c r="E108" s="53" t="inlineStr">
-        <is>
-          <t>MEASURED</t>
-        </is>
-      </c>
-      <c r="F108" s="43" t="inlineStr">
-        <is>
-          <t>deck_decode_d2048_bf16_gh200_20260814.json; DECODE_THROUGHPUT_20260814</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="45" t="inlineStr">
-        <is>
-          <t>Transformer-stack maturity</t>
-        </is>
-      </c>
-      <c r="B109" s="43" t="inlineStr">
-        <is>
-          <t>NOT GRANTED by default since the 2026-08-14 re-base: the headline runs on the measured cells, in which neither family's decode is optimised (ours ran the unoptimised Triton per-step path at 9.5% GPU-busy while the transformer sat at 95.6%). Setting tf_kv_compression=8.0 grants it paged attention + KV quantization, divides our decode lever by 8 and puts the TRANSFORMER ahead at 64k — reported, not hidden</t>
-        </is>
-      </c>
-      <c r="E109" s="52" t="inlineStr">
-        <is>
-          <t>ASSUMPTION</t>
-        </is>
-      </c>
-      <c r="F109" s="43" t="inlineStr">
-        <is>
-          <t>SERVING['tf_kv_compression']</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="45" t="inlineStr">
-        <is>
-          <t>bAttention serving throughput</t>
-        </is>
-      </c>
-      <c r="B110" s="43" t="inlineStr">
-        <is>
-          <t>562 tok/s/GPU (4,497/box): 64 concurrent 262,144-token streams on one GPU, context-flat 32k-262k (-4.0%). The 64-stream cell is a grid cap, not a ceiling — 1.62 GB of state on a 96 GB card at 9.5% GPU-busy — so it is a LOWER bound. Supersedes a 349,880 tok/s/box figure measured on the h-carry-only proxy</t>
-        </is>
-      </c>
-      <c r="E110" s="53" t="inlineStr">
-        <is>
-          <t>MEASURED</t>
-        </is>
-      </c>
-      <c r="F110" s="43" t="inlineStr">
-        <is>
-          <t>deck_decode_d2048_bf16_gh200_20260814.json rows[bdm, 64 streams]</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="45" t="inlineStr">
-        <is>
-          <t>bAttention per-stream state</t>
-        </is>
-      </c>
-      <c r="B111" s="43" t="inlineStr">
-        <is>
-          <t>25.4 MB/stream, the FULL recurrent cell (h + M memory), 24.2 MiB measured, context-flat. The 0.15 MB figure previously quoted was an h-carry-only proxy with no M memory and is retired as a headline</t>
-        </is>
-      </c>
-      <c r="E111" s="53" t="inlineStr">
-        <is>
-          <t>MEASURED</t>
-        </is>
-      </c>
-      <c r="F111" s="43" t="inlineStr">
-        <is>
-          <t>deck_decode_d2048_bf16_gh200_20260814.json state_bytes_per_stream</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="45" t="inlineStr">
-        <is>
-          <t>Transformer KV wall</t>
-        </is>
-      </c>
-      <c r="B112" s="43" t="inlineStr">
-        <is>
-          <t>197 KB per token of context per stream — 51.5 GB for one 262,144-token stream, a 2nd stream OOMs a 96 GB card, and 16 streams OOM it at 32,768 tokens. Its retired 88.5 per-token decode cost was inflated by a growing-KV re-planning harness artifact; the traced figure is 14.92 GPU-busy at 262k</t>
-        </is>
-      </c>
-      <c r="E112" s="53" t="inlineStr">
-        <is>
-          <t>MEASURED</t>
-        </is>
-      </c>
-      <c r="F112" s="43" t="inlineStr">
-        <is>
-          <t>deck_decode_d2048_bf16_gh200_20260814.json rows[transformer]</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="45" t="inlineStr">
-        <is>
-          <t>Training throughput at 8 GPUs</t>
-        </is>
-      </c>
-      <c r="B113" s="43" t="inlineStr">
-        <is>
-          <t>x5.15 (bAttention, fwd+bwd) vs x3.70 (transformer Ulysses best, forward-only) at matched 16-in-flight load -&gt; x1.39; x6.27 at 256 in flight -&gt; x1.70</t>
-        </is>
-      </c>
-      <c r="E113" s="53" t="inlineStr">
-        <is>
-          <t>MEASURED</t>
-        </is>
-      </c>
-      <c r="F113" s="43" t="inlineStr">
-        <is>
-          <t>derived.json matched_load_curve, scaling_1to8_best</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="45" t="inlineStr">
-        <is>
-          <t>Memory walls (component scope)</t>
-        </is>
-      </c>
-      <c r="B114" s="43" t="inlineStr">
-        <is>
-          <t>64k-token sequence: 30.9 GB (fits 1 GPU) vs OOM at 78.4 GB attempted; pipeline stage 9.05 GB flat vs GPipe 43.3 GB</t>
-        </is>
-      </c>
-      <c r="E114" s="53" t="inlineStr">
-        <is>
-          <t>MEASURED</t>
-        </is>
-      </c>
-      <c r="F114" s="43" t="inlineStr">
-        <is>
-          <t>derived.json pipeline_feasibility, pipeline_memory_asymmetry</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="45" t="inlineStr">
-        <is>
-          <t>Compute lever (flop_factor)</t>
-        </is>
-      </c>
-      <c r="B115" s="43" t="inlineStr">
-        <is>
-          <t>cross-family prefill, bf16, 1xH100, parameter counts exactly matched, block scope (1 layer, batch 16): TF/bAttention 4.02 at d512/1M, 3.83 at d1024/1M, 2.01 at d2048/262k. Short context favours the transformer and is stated so</t>
-        </is>
-      </c>
-      <c r="E115" s="53" t="inlineStr">
-        <is>
-          <t>MEASURED</t>
-        </is>
-      </c>
-      <c r="F115" s="43" t="inlineStr">
-        <is>
-          <t>matched_d{512,1024,2048}_h100.json (2026-07-21)</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="45" t="inlineStr">
-        <is>
-          <t>Compute, fp32 lane (scope reference)</t>
-        </is>
-      </c>
-      <c r="B116" s="43" t="inlineStr">
-        <is>
-          <t>the d2048/24-layer fp32 sweep gives 7.91 at 262k at full-model scope. No fp32 FlashAttention kernel exists, so that lane runs mem-efficient attention on the transformer and the owned arm is fp16 internally; params 16.7% apart. Full model in bf16 has not been run</t>
-        </is>
-      </c>
-      <c r="E116" s="52" t="inlineStr">
+      <c r="A100" s="45" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B100" s="43" t="inlineStr">
+        <is>
+          <t>systems numbers are component-scope (bAttention d1536 fwd+bwd h-recurrence sub-block vs transformer d2048 forward-only layer); every speedup is vs the family's OWN 1-GPU baseline</t>
+        </is>
+      </c>
+      <c r="E100" s="51" t="inlineStr">
         <is>
           <t>LABEL</t>
         </is>
       </c>
-      <c r="F116" s="43" t="inlineStr">
-        <is>
-          <t>deck_speed_scaling_d2048_h100_20260803.json sdpa_fp32_backend_probe + last_route_attestation</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="45" t="inlineStr">
-        <is>
-          <t>16-bit IO (training)</t>
-        </is>
-      </c>
-      <c r="B117" s="43" t="inlineStr">
-        <is>
-          <t>same-arch GH200 gate at d1536: fp16 x1.185 step time and -17.5% peak memory, bf16 x1.171 and -20.6%; quality deltas +0.001 to +0.004 from the gate's smaller vehicle. Reported on its own; not an input to the compute lever</t>
-        </is>
-      </c>
-      <c r="E117" s="53" t="inlineStr">
-        <is>
-          <t>MEASURED</t>
-        </is>
-      </c>
-      <c r="F117" s="43" t="inlineStr">
-        <is>
-          <t>receipts/io16_gate_20260809.md (2026-08-09)</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="45" t="inlineStr">
-        <is>
-          <t>Quality parity at 70B</t>
-        </is>
-      </c>
-      <c r="B118" s="43" t="inlineStr">
-        <is>
-          <t>transformer needs x4.1 params [2.2-7.7] or x1.7 tokens [1.33-2.10, beta=0.28 assumption]; crossover N* ~321M = the top measured rung</t>
-        </is>
-      </c>
-      <c r="E118" s="52" t="inlineStr">
-        <is>
-          <t>PROJECTION</t>
-        </is>
-      </c>
-      <c r="F118" s="43" t="inlineStr">
-        <is>
-          <t>derived.json quality_fit.ref_70B, parity_cost</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="45" t="inlineStr">
-        <is>
-          <t>Scope</t>
-        </is>
-      </c>
-      <c r="B119" s="43" t="inlineStr">
-        <is>
-          <t>systems numbers are component-scope (bAttention d1536 fwd+bwd h-recurrence sub-block vs transformer d2048 forward-only layer); every speedup is vs the family's OWN 1-GPU baseline</t>
-        </is>
-      </c>
-      <c r="E119" s="52" t="inlineStr">
-        <is>
-          <t>LABEL</t>
-        </is>
-      </c>
-      <c r="F119" s="43" t="inlineStr">
+      <c r="F100" s="43" t="inlineStr">
         <is>
           <t>derived.json scope_reconciliation; deck README</t>
         </is>
@@ -3836,14 +3502,14 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>- Spend-cut value (named floor, 6% discount rate): FY25 ~$159B/yr (~$2.6T capitalized); FY26 r/r ~$337B/yr (~$5.6T). Ceiling: ~$163B FY25.</t>
+          <t>- Spend-cut value (named floor, 6% discount rate): FY25 ~$159B/yr (~$2.6T capitalized); FY26 r/r ~$366B/yr (~$6.1T). Ceiling: ~$163B FY25.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>- GLOBAL estimate (named ~80% of world AI capex): FY25 ~$3.3T, FY26 ~$7.0T capitalized. Clearly an estimate.</t>
+          <t>- GLOBAL estimate (named ~80% of world AI capex): FY25 ~$3.3T, FY26 ~$7.6T capitalized. Clearly an estimate.</t>
         </is>
       </c>
     </row>
@@ -7469,11 +7135,11 @@
         <v>12.7</v>
       </c>
       <c r="C3" s="15" t="n">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>FY25 S-1 AI capex $12.7B [DISCLOSED]; FY26 ~$18B (ESTIMATE, likely conservative -- Q1'26 AI capex alone was $7.7B, ~$31B annualized). ~all accelerator (greenfield). AI rev ~0 (nascent; Anthropic orbital compute is future).</t>
+          <t>FY25 S-1 AI capex $12.7B [DISCLOSED]; FY26 ~$55B EST from H1'26 DISCLOSED $23.5B (Q1 $7.7B, Q2 $15.8B; 82.7% of total capex) + company guiding capex roughly flat Q3/Q4. ~all accelerator (greenfield COLOSSUS I/II). AI rev ~0 today; Anthropic (up to $1.25B/mo) and Google (up to $920M/mo) compute deals ramp from 2027.</t>
         </is>
       </c>
     </row>
@@ -7538,7 +7204,7 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>1840</v>
+        <v>1950</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
@@ -8333,7 +7999,7 @@
         </is>
       </c>
       <c r="B12" s="26" t="n">
-        <v>1840</v>
+        <v>1950</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sync 2026-08-25 re-base: ceiling x24.8/~45x, flat r(T)
2k cell re-based to the 2026-08-25 ledger-of-record receipt (x1.93,
realized x3.45); the +5.8%-per-4x context growth and the B4/T32,768
~parity cell retired as a B4 occupancy artifact; training crossover now
a PROJECTED ~17k. Curriculum advantages move to x1.9/x6.6/x10.3.
Today lever unchanged (x9.24, ~20x, $159B FY25). Ships the rebuilt
workbook and the training-cost chart the app now embeds.
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -28,7 +28,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
@@ -38,6 +38,9 @@
     <numFmt numFmtId="170" formatCode="$0.00"/>
     <numFmt numFmtId="171" formatCode="0.0×"/>
     <numFmt numFmtId="172" formatCode="0.00×"/>
+    <numFmt numFmtId="173" formatCode="0.000×"/>
+    <numFmt numFmtId="174" formatCode="$#,##0.0"/>
+    <numFmt numFmtId="175" formatCode="+$#,##0.00;-$#,##0.00"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -118,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -182,8 +185,11 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="172" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="175" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1427,7 +1433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:G125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1578,11 +1584,11 @@
         </is>
       </c>
       <c r="B17" s="33" t="n">
-        <v>0.1041666666666667</v>
+        <v>0.5169883870300283</v>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Transformer is 9.6x faster at T=2048 blocks (d1152). Crossover near T~88,000.</t>
+          <t>RE-BASED 2026-08-24/25 (1 x GH200, ONE layer, fwd+bwd, bf16, checkpointing off both arms, modern transformer block 24Q/4KV head_dim 256 RoPE 64 gated): transformer is 1.93x faster at T=2,048 (116.0 vs 60.0 ms/step) and 1.79x at T=8,192; the equal-token B4/T32,768 ~parity cell is RETIRED 2026-08-25 as a B4 occupancy artifact, and the flat per-token model puts the crossover at a PROJECTED T~16,943 (from T~88,000 pre-campaign). It read 6.12x (400.4 ms) the same morning. Training PEAK MEMORY, same frame: 1.579x at T=2,048 (17,087.5 vs 10,823.6 MiB), from 2.829x -- that is TRAINING memory, not the /100 SERVING lever. TARGET (no receipt): T=8,192 step &lt;= 83.08 ms and memory 0.88x.</t>
         </is>
       </c>
     </row>
@@ -2222,631 +2228,1099 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Training, prefill and decode point in OPPOSITE directions at today's kernel maturity, so a single number cannot represent them. Training is a loss at short sequence (transformer 5.3-9.6x faster at T=2048 blocks; FLOPs near-matched at 1.07-1.19x, the gap is achieved FLOP/s 200.9 vs 21.7 TF/s; crossover near T~88,000). Prefill crosses over near 65k context. Decode crosses in our favour near ~30k context. The lever is therefore blended over the workload: per generated token, in:out input tokens through prefill plus one token through decode, using measured per-GPU throughput at each family's own concurrency ceiling, the transformer granted no KV compression. At the default operating point (10:1, 64k context, training share 0): prefill x1.17, decode x2.20, blended x2.19, with decode ~99.7% of transformer serving cost. The decode half is a MEMORY CEILING, not a per-token result - at one stream and 64k the transformer decodes a token more cheaply than we do - and it crosses 1 at ~30k context, below which the transformer wins. Granting it KV/8 divides our decode lever by 8. A training share above ~0.06 also takes the blend below 1. All are reachable in the live model.</t>
+          <t>Training, prefill and decode point in OPPOSITE directions at today's kernel maturity, so a single number cannot represent them. Training is still a loss at short sequence, but a much smaller one since the 2026-08-24 kernel re-base (transformer 1.93x faster at T=2,048 and 1.79x at T=8,192, crossover near T~32,000; it was 5.3-9.6x with a crossover near T~88,000 on the pre-campaign d1152 sweep). Prefill crosses over near 65k context. Decode crosses in our favour near ~30k context. The lever is therefore blended over the workload: per generated token, in:out input tokens through prefill plus one token through decode, using measured per-GPU throughput at each family's own concurrency ceiling, the transformer granted no KV compression. At the default operating point (10:1, 64k context, training share 0): prefill x1.17, decode x2.20, blended x2.19, with decode ~99.7% of transformer serving cost. The decode half is a MEMORY CEILING, not a per-token result - at one stream and 64k the transformer decodes a token more cheaply than we do - and it crosses 1 at ~30k context, below which the transformer wins. Granting it KV/8 divides our decode lever by 8. A training share above ~0.30 also takes the blend below 1 (it was ~0.06 before the kernel re-base). All are reachable in the live model.</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="inlineStr">
-        <is>
-          <t>The prefill component, 16-bit and parameter-matched — the lane the competition serves in. Parameter counts exactly matched, 1 layer, batch 16, 1 x H100 80GB HBM3, 2026-07-21 — x4.02 at d512/1M, x3.83 at d1024/1M, x2.01 at d2048/262k. The fp32 full-model sweep and the own-baseline 16-bit-IO training gate are retired to one assumption row each below. Receipts: experiments/paper_figures/output/matched_d{512,1024,2048}_h100.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="38" t="inlineStr">
-        <is>
-          <t>Context (tokens)</t>
-        </is>
-      </c>
-      <c r="B70" s="38" t="inlineStr">
-        <is>
-          <t>Transformer ms</t>
-        </is>
-      </c>
-      <c r="C70" s="38" t="inlineStr">
-        <is>
-          <t>bAttention ms</t>
-        </is>
-      </c>
-      <c r="D70" s="38" t="inlineStr">
-        <is>
-          <t>TF / bAttention</t>
-        </is>
-      </c>
-      <c r="E70" s="38" t="inlineStr"/>
-      <c r="F70" s="38" t="inlineStr">
-        <is>
-          <t>Note</t>
+      <c r="A68" s="1" t="inlineStr">
+        <is>
+          <t>Estimated TRAINING cost at equal quality (ESTIMATE: measured kernels x fitted quality)</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="n"/>
+      <c r="C68" s="2" t="n"/>
+      <c r="D68" s="2" t="n"/>
+      <c r="E68" s="2" t="n"/>
+      <c r="F68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>Training compute ~ 6*N*D FLOPs. At equal quality we need N/s parameters, where s(N) is the FIT-DERIVED equal-quality parameter ratio (the same sealed 2026-08-14 refit as the compute lever). Two token regimes differ by exactly one power of s: COMPUTE-OPTIMAL (Chinchilla, D proportional to N -&gt; cost ratio s^2/r) and FIXED TOKEN BUDGET (D equal on both arms -&gt; s/r). r(T) is the step-time ratio at matched parameters: MEASURED at T=2,048 (1.93x, 2026-08-25) and T=8,192 (1.79x, 2026-08-24), MODELED beyond. Above 1.00 we are cheaper to train to the same quality. The 256k column is MODELED from the per-token cost form -- the transformer pays base + attn*T per token (FlashAttention is linear per token), our O(1) recurrent state pays ~flat -- with base and attn fitted to the 2k and 8k cells ONLY. The fit is flat -- the +5.8%-per-4x residual and the B4/T32,768 ~parity cell that shared it are RETIRED 2026-08-25 as a B4 occupancy artifact -- and puts the crossover at a PROJECTED T~16,943. The old constant-decay extrapolation (0.758 per 4x) is kept as the CONSERVATIVE bound and reads 0.73 at 256k against this form's 0.11. The fits cross at 392M, so below that we need MORE parameters, and every row past ~1B extrapolates beyond the measured 47M-663M rungs. Peak training memory (1.58x measured, 0.88x targeted) is NOT in this model: it caps per-GPU batch density, not FLOPs. Chart: paper/figures/vc_memo_training_cost_scaling.png</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="39" t="n">
-        <v>2048</v>
-      </c>
-      <c r="B71" s="5" t="n">
-        <v>111.229</v>
-      </c>
-      <c r="C71" s="14" t="n">
-        <v>663.1130000000001</v>
-      </c>
-      <c r="D71" s="50" t="n">
-        <v>0.16773762541226</v>
-      </c>
-      <c r="F71" s="43" t="inlineStr">
-        <is>
-          <t>transformer ahead</t>
+      <c r="A71" s="38" t="inlineStr">
+        <is>
+          <t>Transformer params</t>
+        </is>
+      </c>
+      <c r="B71" s="38" t="inlineStr">
+        <is>
+          <t>s(N) fit</t>
+        </is>
+      </c>
+      <c r="C71" s="38" t="inlineStr">
+        <is>
+          <t>Chinchilla 2k</t>
+        </is>
+      </c>
+      <c r="D71" s="38" t="inlineStr">
+        <is>
+          <t>Chinchilla 8k</t>
+        </is>
+      </c>
+      <c r="E71" s="38" t="inlineStr">
+        <is>
+          <t>Chinchilla 32k</t>
+        </is>
+      </c>
+      <c r="F71" s="38" t="inlineStr">
+        <is>
+          <t>Chinchilla 256k*</t>
+        </is>
+      </c>
+      <c r="G71" s="38" t="inlineStr">
+        <is>
+          <t>Fixed-D 2k / 8k / 32k / 256k*</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="39" t="n">
-        <v>4096</v>
-      </c>
-      <c r="B72" s="5" t="n">
-        <v>125.091</v>
-      </c>
-      <c r="C72" s="14" t="n">
-        <v>662.751</v>
-      </c>
-      <c r="D72" s="50" t="n">
-        <v>0.1887450943114382</v>
-      </c>
-      <c r="F72" s="43" t="inlineStr">
-        <is>
-          <t>transformer ahead</t>
+      <c r="A72" s="45" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
+      <c r="B72" s="28" t="n">
+        <v>1.187536580013817</v>
+      </c>
+      <c r="C72" s="19" t="n">
+        <v>0.7290793205151539</v>
+      </c>
+      <c r="D72" s="19" t="n">
+        <v>1.01005559202076</v>
+      </c>
+      <c r="E72" s="19" t="n">
+        <v>2.133960678043187</v>
+      </c>
+      <c r="F72" s="19" t="n">
+        <v>12.62374148091916</v>
+      </c>
+      <c r="G72" s="47" t="inlineStr">
+        <is>
+          <t>0.61 / 0.85 / 1.80 / 10.63</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="39" t="n">
-        <v>8192</v>
-      </c>
-      <c r="B73" s="5" t="n">
-        <v>153.085</v>
-      </c>
-      <c r="C73" s="14" t="n">
-        <v>663.327</v>
-      </c>
-      <c r="D73" s="50" t="n">
-        <v>0.2307836104967836</v>
-      </c>
-      <c r="F73" s="43" t="inlineStr">
-        <is>
-          <t>transformer ahead</t>
+      <c r="A73" s="45" t="inlineStr">
+        <is>
+          <t>10B</t>
+        </is>
+      </c>
+      <c r="B73" s="28" t="n">
+        <v>1.811968550196262</v>
+      </c>
+      <c r="C73" s="19" t="n">
+        <v>1.697391795855765</v>
+      </c>
+      <c r="D73" s="19" t="n">
+        <v>2.35154122056688</v>
+      </c>
+      <c r="E73" s="19" t="n">
+        <v>4.968138919411341</v>
+      </c>
+      <c r="F73" s="19" t="n">
+        <v>29.38971744195963</v>
+      </c>
+      <c r="G73" s="47" t="inlineStr">
+        <is>
+          <t>0.94 / 1.30 / 2.74 / 16.22</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="39" t="n">
-        <v>16384</v>
-      </c>
-      <c r="B74" s="5" t="n">
-        <v>204.919</v>
-      </c>
-      <c r="C74" s="14" t="n">
-        <v>663.202</v>
-      </c>
-      <c r="D74" s="50" t="n">
-        <v>0.3089842913622094</v>
-      </c>
-      <c r="F74" s="43" t="inlineStr">
-        <is>
-          <t>transformer ahead</t>
+      <c r="A74" s="45" t="inlineStr">
+        <is>
+          <t>100B</t>
+        </is>
+      </c>
+      <c r="B74" s="28" t="n">
+        <v>2.764740120141925</v>
+      </c>
+      <c r="C74" s="19" t="n">
+        <v>3.951749593724151</v>
+      </c>
+      <c r="D74" s="19" t="n">
+        <v>5.474694814532027</v>
+      </c>
+      <c r="E74" s="19" t="n">
+        <v>11.56647569776353</v>
+      </c>
+      <c r="F74" s="19" t="n">
+        <v>68.42309727459089</v>
+      </c>
+      <c r="G74" s="47" t="inlineStr">
+        <is>
+          <t>1.43 / 1.98 / 4.18 / 24.75</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="39" t="n">
-        <v>32768</v>
-      </c>
-      <c r="B75" s="5" t="n">
-        <v>309.886</v>
-      </c>
-      <c r="C75" s="14" t="n">
-        <v>662.6180000000001</v>
-      </c>
-      <c r="D75" s="50" t="n">
-        <v>0.4676691547769605</v>
-      </c>
-      <c r="F75" s="43" t="inlineStr">
-        <is>
-          <t>transformer ahead</t>
+      <c r="A75" s="45" t="inlineStr">
+        <is>
+          <t>1T</t>
+        </is>
+      </c>
+      <c r="B75" s="28" t="n">
+        <v>4.21849922897088</v>
+      </c>
+      <c r="C75" s="19" t="n">
+        <v>9.200188718731198</v>
+      </c>
+      <c r="D75" s="19" t="n">
+        <v>12.74580392217778</v>
+      </c>
+      <c r="E75" s="19" t="n">
+        <v>26.92826473596412</v>
+      </c>
+      <c r="F75" s="19" t="n">
+        <v>159.29789899797</v>
+      </c>
+      <c r="G75" s="47" t="inlineStr">
+        <is>
+          <t>2.18 / 3.02 / 6.38 / 37.76</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="39" t="n">
-        <v>65536</v>
-      </c>
-      <c r="B76" s="5" t="n">
-        <v>520.986</v>
-      </c>
-      <c r="C76" s="14" t="n">
-        <v>663.199</v>
-      </c>
-      <c r="D76" s="50" t="n">
-        <v>0.7855651169558459</v>
-      </c>
-      <c r="F76" s="43" t="inlineStr">
-        <is>
-          <t>transformer ahead</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="39" t="n">
-        <v>131072</v>
-      </c>
-      <c r="B77" s="5" t="n">
-        <v>969.79</v>
-      </c>
-      <c r="C77" s="14" t="n">
-        <v>753.457</v>
-      </c>
-      <c r="D77" s="50" t="n">
-        <v>1.287120565606265</v>
-      </c>
-      <c r="F77" s="43" t="inlineStr"/>
+      <c r="A76" s="45" t="inlineStr">
+        <is>
+          <t>10T</t>
+        </is>
+      </c>
+      <c r="B76" s="28" t="n">
+        <v>6.436675771144228</v>
+      </c>
+      <c r="C76" s="19" t="n">
+        <v>21.41923987154772</v>
+      </c>
+      <c r="D76" s="19" t="n">
+        <v>29.67389473316043</v>
+      </c>
+      <c r="E76" s="19" t="n">
+        <v>62.69251417961127</v>
+      </c>
+      <c r="F76" s="19" t="n">
+        <v>370.866295679819</v>
+      </c>
+      <c r="G76" s="47" t="inlineStr">
+        <is>
+          <t>3.33 / 4.61 / 9.74 / 57.62</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="39" t="n">
-        <v>262144</v>
-      </c>
-      <c r="B78" s="5" t="n">
-        <v>1889.616</v>
-      </c>
-      <c r="C78" s="14" t="n">
-        <v>938.175</v>
-      </c>
-      <c r="D78" s="50" t="n">
-        <v>2.014140219042289</v>
-      </c>
-      <c r="F78" s="43" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="39" t="n">
-        <v>524288</v>
-      </c>
-      <c r="B79" s="5" t="n">
-        <v>3718.717</v>
-      </c>
-      <c r="C79" s="14" t="n">
-        <v>1308.837</v>
-      </c>
-      <c r="D79" s="50" t="n">
-        <v>2.841237678947035</v>
-      </c>
-      <c r="F79" s="43" t="inlineStr"/>
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>TRAINING IS A CURRICULUM, NOT ONE CONTEXT. Quoting r at a single T assumes ALL training happens there; this model used to assume T=2,048 for all of it, which is the pessimistic corner. The correct training term is the ratio of COSTS integrated over the mix of contexts a run actually uses, NOT the average of the per-context ratios. That distinction does the work: our per-token cost is flat in context and the transformer's grows, so long-context tokens dominate its bill while staying a token minority. TOKEN SHARES BELOW ARE ILLUSTRATIVE KNOBS -- this repo carries no citation for any lab's training recipe and none is invented here; only the first row (the degenerate one-context case) is anchored to a measurement. Effective r crosses below 1 at every modern mix, but RAISING the dollar headline is a higher bar: the blended lever is a cost-weighted harmonic mean, so training only pushes the headline up once it beats the SERVING advantage of 2.19x, not merely 1.00x. Between the two it is profitable and still dilutive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="38" t="inlineStr">
+        <is>
+          <t>Training curriculum</t>
+        </is>
+      </c>
+      <c r="B80" s="38" t="inlineStr">
+        <is>
+          <t>Advantage (TF / ours)</t>
+        </is>
+      </c>
+      <c r="C80" s="38" t="inlineStr">
+        <is>
+          <t>Effective r</t>
+        </is>
+      </c>
+      <c r="D80" s="38" t="inlineStr">
+        <is>
+          <t>Mix: token share -&gt; transformer cost share</t>
+        </is>
+      </c>
+      <c r="E80" s="38" t="inlineStr">
+        <is>
+          <t>FY25 cut @ 20% training</t>
+        </is>
+      </c>
+      <c r="F80" s="38" t="inlineStr">
+        <is>
+          <t>vs serving-only</t>
+        </is>
+      </c>
+      <c r="G80" s="38" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="inlineStr">
-        <is>
-          <t>Assumptions — one row each (MEASURED / PROJECTION / ASSUMPTION)</t>
-        </is>
-      </c>
-      <c r="B81" s="2" t="n"/>
-      <c r="C81" s="2" t="n"/>
-      <c r="D81" s="2" t="n"/>
-      <c r="E81" s="2" t="n"/>
-      <c r="F81" s="2" t="n"/>
+      <c r="A81" s="45" t="inlineStr">
+        <is>
+          <t>Legacy short (all training at 2k)</t>
+        </is>
+      </c>
+      <c r="B81" s="50" t="n">
+        <v>0.5169883870300283</v>
+      </c>
+      <c r="C81" s="51" t="n">
+        <v>1.934279425007504</v>
+      </c>
+      <c r="D81" s="43" t="inlineStr">
+        <is>
+          <t>2k: 100% tok -&gt; 100% cost</t>
+        </is>
+      </c>
+      <c r="E81" s="52" t="n">
+        <v>154.1531879040444</v>
+      </c>
+      <c r="F81" s="53" t="n">
+        <v>-4.678891120329979</v>
+      </c>
+      <c r="G81" s="54" t="inlineStr">
+        <is>
+          <t>MEASURED (degenerate one-context case)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" s="38" t="inlineStr">
-        <is>
-          <t>Assumption</t>
-        </is>
-      </c>
-      <c r="B82" s="38" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C82" s="38" t="inlineStr"/>
-      <c r="D82" s="38" t="inlineStr"/>
-      <c r="E82" s="38" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F82" s="38" t="inlineStr">
-        <is>
-          <t>Source</t>
+      <c r="A82" s="45" t="inlineStr">
+        <is>
+          <t>Modern standard (8k bulk + 64k/256k extension)</t>
+        </is>
+      </c>
+      <c r="B82" s="50" t="n">
+        <v>1.911665560258985</v>
+      </c>
+      <c r="C82" s="51" t="n">
+        <v>0.5231040516650433</v>
+      </c>
+      <c r="D82" s="43" t="inlineStr">
+        <is>
+          <t>8k: 70% tok -&gt; 26% cost  64k: 20% tok -&gt; 27% cost  256k: 10% tok -&gt; 47% cost</t>
+        </is>
+      </c>
+      <c r="E82" s="52" t="n">
+        <v>158.6241725679516</v>
+      </c>
+      <c r="F82" s="53" t="n">
+        <v>-0.2079064564227622</v>
+      </c>
+      <c r="G82" s="55" t="inlineStr">
+        <is>
+          <t>ILLUSTRATIVE ASSUMPTION</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="45" t="inlineStr">
         <is>
-          <t>Compute lever (economics slide)</t>
-        </is>
-      </c>
-      <c r="B83" s="43" t="inlineStr">
-        <is>
-          <t>x9.24 = the x2.19 MEASURED serving blend x the x4.22 FIT-DERIVED equal-quality parameter ratio at trillion scale</t>
-        </is>
-      </c>
-      <c r="E83" s="51" t="inlineStr">
-        <is>
-          <t>MEASURED x PROJECTION</t>
-        </is>
-      </c>
-      <c r="F83" s="43" t="inlineStr">
-        <is>
-          <t>workload_compute_advantage() x quality_matched_compute_lever(); receipts derived.json + quality_fit_v4.json</t>
+          <t>Long-context heavy (frontier extension phases)</t>
+        </is>
+      </c>
+      <c r="B83" s="50" t="n">
+        <v>6.613720030002326</v>
+      </c>
+      <c r="C83" s="51" t="n">
+        <v>0.1512008363619299</v>
+      </c>
+      <c r="D83" s="43" t="inlineStr">
+        <is>
+          <t>8k: 40% tok -&gt; 4% cost  64k: 25% tok -&gt; 10% cost  256k: 25% tok -&gt; 34% cost  1024k: 10% tok -&gt; 52% cost</t>
+        </is>
+      </c>
+      <c r="E83" s="52" t="n">
+        <v>159.8024623847159</v>
+      </c>
+      <c r="F83" s="53" t="n">
+        <v>0.9703833603415433</v>
+      </c>
+      <c r="G83" s="55" t="inlineStr">
+        <is>
+          <t>ILLUSTRATIVE ASSUMPTION</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="45" t="inlineStr">
         <is>
+          <t>Frontier + long-rollout RL</t>
+        </is>
+      </c>
+      <c r="B84" s="50" t="n">
+        <v>10.3062938791228</v>
+      </c>
+      <c r="C84" s="51" t="n">
+        <v>0.09702808902292945</v>
+      </c>
+      <c r="D84" s="43" t="inlineStr">
+        <is>
+          <t>8k: 30% tok -&gt; 2% cost  64k: 20% tok -&gt; 5% cost  256k: 30% tok -&gt; 26% cost  1024k: 20% tok -&gt; 67% cost</t>
+        </is>
+      </c>
+      <c r="E84" s="52" t="n">
+        <v>159.9740962773771</v>
+      </c>
+      <c r="F84" s="53" t="n">
+        <v>1.142017253002734</v>
+      </c>
+      <c r="G84" s="55" t="inlineStr">
+        <is>
+          <t>ILLUSTRATIVE ASSUMPTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>EXCLUDED, AND IT RUNS OUR WAY. At 262k+ the transformer additionally pays sequence-parallelism and activation-memory costs an O(1) recurrent state avoids: its KV grows at 156 KB per token of context per stream, which is what forces sharding, ring/Ulysses attention and their communication overhead. Our own measurement shows the asymmetry in the small -- from 2k to 8k the peak-memory ratio went 1.579x -&gt; 1.567x, i.e. flat-to-falling in context, while the absolute footprint the transformer must shard keeps growing. None of it is in the cost model above, which counts step time only, so the omission is CONSERVATIVE. Quantifying it needs a multi-GPU long-context TRAINING receipt we do not have.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>The prefill component, 16-bit and parameter-matched — the lane the competition serves in. Parameter counts exactly matched, 1 layer, batch 16, 1 x H100 80GB HBM3, 2026-07-21 — x4.02 at d512/1M, x3.83 at d1024/1M, x2.01 at d2048/262k. The fp32 full-model sweep and the own-baseline 16-bit-IO training gate are retired to one assumption row each below. Receipts: experiments/paper_figures/output/matched_d{512,1024,2048}_h100.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="38" t="inlineStr">
+        <is>
+          <t>Context (tokens)</t>
+        </is>
+      </c>
+      <c r="B90" s="38" t="inlineStr">
+        <is>
+          <t>Transformer ms</t>
+        </is>
+      </c>
+      <c r="C90" s="38" t="inlineStr">
+        <is>
+          <t>bAttention ms</t>
+        </is>
+      </c>
+      <c r="D90" s="38" t="inlineStr">
+        <is>
+          <t>TF / bAttention</t>
+        </is>
+      </c>
+      <c r="E90" s="38" t="inlineStr"/>
+      <c r="F90" s="38" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="39" t="n">
+        <v>2048</v>
+      </c>
+      <c r="B91" s="5" t="n">
+        <v>111.229</v>
+      </c>
+      <c r="C91" s="14" t="n">
+        <v>663.1130000000001</v>
+      </c>
+      <c r="D91" s="50" t="n">
+        <v>0.16773762541226</v>
+      </c>
+      <c r="F91" s="43" t="inlineStr">
+        <is>
+          <t>transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="39" t="n">
+        <v>4096</v>
+      </c>
+      <c r="B92" s="5" t="n">
+        <v>125.091</v>
+      </c>
+      <c r="C92" s="14" t="n">
+        <v>662.751</v>
+      </c>
+      <c r="D92" s="50" t="n">
+        <v>0.1887450943114382</v>
+      </c>
+      <c r="F92" s="43" t="inlineStr">
+        <is>
+          <t>transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="39" t="n">
+        <v>8192</v>
+      </c>
+      <c r="B93" s="5" t="n">
+        <v>153.085</v>
+      </c>
+      <c r="C93" s="14" t="n">
+        <v>663.327</v>
+      </c>
+      <c r="D93" s="50" t="n">
+        <v>0.2307836104967836</v>
+      </c>
+      <c r="F93" s="43" t="inlineStr">
+        <is>
+          <t>transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="39" t="n">
+        <v>16384</v>
+      </c>
+      <c r="B94" s="5" t="n">
+        <v>204.919</v>
+      </c>
+      <c r="C94" s="14" t="n">
+        <v>663.202</v>
+      </c>
+      <c r="D94" s="50" t="n">
+        <v>0.3089842913622094</v>
+      </c>
+      <c r="F94" s="43" t="inlineStr">
+        <is>
+          <t>transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="39" t="n">
+        <v>32768</v>
+      </c>
+      <c r="B95" s="5" t="n">
+        <v>309.886</v>
+      </c>
+      <c r="C95" s="14" t="n">
+        <v>662.6180000000001</v>
+      </c>
+      <c r="D95" s="50" t="n">
+        <v>0.4676691547769605</v>
+      </c>
+      <c r="F95" s="43" t="inlineStr">
+        <is>
+          <t>transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="39" t="n">
+        <v>65536</v>
+      </c>
+      <c r="B96" s="5" t="n">
+        <v>520.986</v>
+      </c>
+      <c r="C96" s="14" t="n">
+        <v>663.199</v>
+      </c>
+      <c r="D96" s="50" t="n">
+        <v>0.7855651169558459</v>
+      </c>
+      <c r="F96" s="43" t="inlineStr">
+        <is>
+          <t>transformer ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="39" t="n">
+        <v>131072</v>
+      </c>
+      <c r="B97" s="5" t="n">
+        <v>969.79</v>
+      </c>
+      <c r="C97" s="14" t="n">
+        <v>753.457</v>
+      </c>
+      <c r="D97" s="50" t="n">
+        <v>1.287120565606265</v>
+      </c>
+      <c r="F97" s="43" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="39" t="n">
+        <v>262144</v>
+      </c>
+      <c r="B98" s="5" t="n">
+        <v>1889.616</v>
+      </c>
+      <c r="C98" s="14" t="n">
+        <v>938.175</v>
+      </c>
+      <c r="D98" s="50" t="n">
+        <v>2.014140219042289</v>
+      </c>
+      <c r="F98" s="43" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="39" t="n">
+        <v>524288</v>
+      </c>
+      <c r="B99" s="5" t="n">
+        <v>3718.717</v>
+      </c>
+      <c r="C99" s="14" t="n">
+        <v>1308.837</v>
+      </c>
+      <c r="D99" s="50" t="n">
+        <v>2.841237678947035</v>
+      </c>
+      <c r="F99" s="43" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="1" t="inlineStr">
+        <is>
+          <t>Assumptions — one row each (MEASURED / PROJECTION / ASSUMPTION)</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="n"/>
+      <c r="C101" s="2" t="n"/>
+      <c r="D101" s="2" t="n"/>
+      <c r="E101" s="2" t="n"/>
+      <c r="F101" s="2" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="38" t="inlineStr">
+        <is>
+          <t>Assumption</t>
+        </is>
+      </c>
+      <c r="B102" s="38" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C102" s="38" t="inlineStr"/>
+      <c r="D102" s="38" t="inlineStr"/>
+      <c r="E102" s="38" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F102" s="38" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="45" t="inlineStr">
+        <is>
+          <t>Compute lever (economics slide)</t>
+        </is>
+      </c>
+      <c r="B103" s="43" t="inlineStr">
+        <is>
+          <t>x9.24 = the x2.19 MEASURED serving blend x the x4.22 FIT-DERIVED equal-quality parameter ratio at trillion scale</t>
+        </is>
+      </c>
+      <c r="E103" s="55" t="inlineStr">
+        <is>
+          <t>MEASURED x PROJECTION</t>
+        </is>
+      </c>
+      <c r="F103" s="43" t="inlineStr">
+        <is>
+          <t>workload_compute_advantage() x quality_matched_compute_lever(); receipts derived.json + quality_fit_v4.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="45" t="inlineStr">
+        <is>
           <t>Equal-quality parameter matching</t>
         </is>
       </c>
-      <c r="B84" s="43" t="inlineStr">
+      <c r="B104" s="43" t="inlineStr">
         <is>
           <t>sealed 2026-08-14 refit, 4 rungs per family (47M-663M params): the fits cross at 392M and bAttention then matches the transformer fit's quality on 84.2% of the params at 1B, 55.2% at 10B, 36.2% at 100B, 23.7% at 1T, 15.5% at 10T. The receipt's own words: 'a projection of the two fits, not a measurement'</t>
         </is>
       </c>
-      <c r="E84" s="51" t="inlineStr">
+      <c r="E104" s="55" t="inlineStr">
         <is>
           <t>PROJECTION</t>
         </is>
       </c>
-      <c r="F84" s="43" t="inlineStr">
+      <c r="F104" s="43" t="inlineStr">
         <is>
           <t>quality_fit_v4.json param_matching; fits over the sealed rope-convention ladder</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="45" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="45" t="inlineStr">
         <is>
           <t>Single-GPU training step (AGAINST us)</t>
         </is>
       </c>
-      <c r="B85" s="43" t="inlineStr">
-        <is>
-          <t>at 2,048-token context on one GPU a bAttention step costs x6.46 MORE (8,979 vs 1,389 ms/step, d1536/27L, fp16, 601-step protocol). At equal quality the same step costs x1.53 more, not x6.46 - the parameter ratio shrinks the gap but does not erase it. Training is excluded from the serving claim for this reason</t>
-        </is>
-      </c>
-      <c r="E85" s="52" t="inlineStr">
+      <c r="B105" s="43" t="inlineStr">
+        <is>
+          <t>RE-BASED 2026-08-24: on one GH200, single layer, fwd+bwd, bf16, checkpointing off both arms, against a MODERN transformer block (24Q/4KV, head_dim 256, RoPE 64, gated attention), a bAttention step costs x1.93 MORE at T=2,048 (116.0 vs 60.0 ms/step) and x1.79 at T=8,192. It read x6.116 (400.4 ms) the same morning and x6.46 on the older d1536/27L fp16 601-step receipt. Fwd x1.82, bwd x2.35. Training is still excluded from the serving claim, but the gap is now a kernel-program line item with a funded gate, not a structural loss</t>
+        </is>
+      </c>
+      <c r="E105" s="54" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F85" s="43" t="inlineStr">
-        <is>
-          <t>dtype_trio_v4.json rows[fp16]</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="45" t="inlineStr">
+      <c r="F105" s="43" t="inlineStr">
+        <is>
+          <t>2026-08-24 GH200 megakernel measurement; prior: dtype_trio_v4.json rows[fp16]</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="45" t="inlineStr">
+        <is>
+          <t>Training PEAK MEMORY (AGAINST us)</t>
+        </is>
+      </c>
+      <c r="B106" s="43" t="inlineStr">
+        <is>
+          <t>x1.579 at T=2,048 (17,087.5 vs 10,823.6 MiB) and x1.567 at T=8,192, down from x2.829 the same morning. This is TRAINING peak memory and is NOT the mem_factor lever, which is SERVING state (O(1) recurrent state vs O(T) KV cache) and is unaffected. It is not an input to the cost model; it caps per-GPU batch density</t>
+        </is>
+      </c>
+      <c r="E106" s="54" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="F106" s="43" t="inlineStr">
+        <is>
+          <t>2026-08-24 GH200 megakernel measurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="45" t="inlineStr">
+        <is>
+          <t>Kernel program (TARGET, not a result)</t>
+        </is>
+      </c>
+      <c r="B107" s="43" t="inlineStr">
+        <is>
+          <t>the funded 8k-win gate is a T=8,192 step at or below 83.08 ms, i.e. x1.786 still to remove (44% of the step). Named levers: recompute removal ~-12.8 ms; backward-fold + occupancy redesign (~3x headroom in the dominant fused kernel); copies elimination (24.8% of the step). Memory target x0.88 (parity or below). CEILING_PREFILL_SPEEDUP = the MEASURED x3.452 already banked x this x1.786 target</t>
+        </is>
+      </c>
+      <c r="E107" s="55" t="inlineStr">
+        <is>
+          <t>TARGET</t>
+        </is>
+      </c>
+      <c r="F107" s="43" t="inlineStr">
+        <is>
+          <t>kernel-campaign program plan, 2026-08-24 — no receipt behind the target half</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="45" t="inlineStr">
+        <is>
+          <t>Context scaling of the training gap</t>
+        </is>
+      </c>
+      <c r="B108" s="43" t="inlineStr">
+        <is>
+          <t>at matched tokens/step, 2k -&gt; 8k (4x context): our step grows x1.000, the transformer's x1.319, so the ratio decays x0.758 per 4x. The equal-token B4/T32,768 ~parity cell is RETIRED 2026-08-25 as a B4 occupancy artifact (it shared the retired growth residual); the flat per-token model puts the crossover at a PROJECTED T~16,900. Holding the old x0.802 decay constant instead would say x1.43 at 32k and a crossover near T~310,000 - that is the CONSERVATIVE extrapolation, because the transformer's quadratic attention term makes its per-4x growth rise with context while ours stays flat</t>
+        </is>
+      </c>
+      <c r="E108" s="55" t="inlineStr">
+        <is>
+          <t>MEASURED (2 ratio points) + PROJECTION</t>
+        </is>
+      </c>
+      <c r="F108" s="43" t="inlineStr">
+        <is>
+          <t>2026-08-24 GH200 megakernel measurement; 2k cell re-based 2026-08-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="45" t="inlineStr">
+        <is>
+          <t>Training CONTEXT MIX (reads the other way)</t>
+        </is>
+      </c>
+      <c r="B109" s="43" t="inlineStr">
+        <is>
+          <t>quoting one context for all of training is the pessimistic corner, and it was this model's old implicit assumption. Cost-weighted over a curriculum the training term flips from a DRAG to a CONTRIBUTOR: x0.517 at 100% 2k, x1.91 at a modern 8k/64k/256k mix, x6.61 long-context-heavy, x10.31 with long RL rollouts. The mechanism: our per-token cost is FLAT in context and the transformer's GROWS, so long-context tokens dominate its bill as a token minority — 10% of tokens at 262k is 47% of its training cost. r(T) is MEASURED at 2k/8k and MODELED beyond; the curriculum SHARES are ILLUSTRATIVE and exposed as knobs (this repo carries no citation for any lab's recipe)</t>
+        </is>
+      </c>
+      <c r="E109" s="55" t="inlineStr">
+        <is>
+          <t>MEASURED r(T) + ILLUSTRATIVE mix</t>
+        </is>
+      </c>
+      <c r="F109" s="43" t="inlineStr">
+        <is>
+          <t>TRAIN_COST_FIT_20260824, TRAINING_CURRICULA, training_advantage_mix()</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="45" t="inlineStr">
+        <is>
+          <t>Long-context training memory (EXCLUDED, runs our way)</t>
+        </is>
+      </c>
+      <c r="B110" s="43" t="inlineStr">
+        <is>
+          <t>at 262k+ the transformer additionally pays sequence-parallelism and activation-memory costs that an O(1) recurrent state does not: its KV grows at 156 KB per token of context per stream, which is what forces sharding, ring/Ulysses attention and their communication overhead. Our own measurement shows the asymmetry in the small: peak training memory grew only x0.993 relative to the transformer's from 2k to 8k (x1.579 -&gt; x1.567), i.e. the ratio is FLAT-to-falling in context while the absolute gap the transformer must shard grows. NOT in the cost model — the training advantage above counts FLOPs/step-time only, so the direction of this omission is CONSERVATIVE (it understates us at long context). Quantifying it needs a multi-GPU long-context training receipt we do not have</t>
+        </is>
+      </c>
+      <c r="E110" s="55" t="inlineStr">
+        <is>
+          <t>DIRECTIONAL — measured components, not a costed lever</t>
+        </is>
+      </c>
+      <c r="F110" s="43" t="inlineStr">
+        <is>
+          <t>KERNEL_CAMPAIGN_20260824 mem_ratio_2k/8k; KV_MB_PER_TOKEN_PER_STREAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="45" t="inlineStr">
         <is>
           <t>$/GPU-hour</t>
         </is>
       </c>
-      <c r="B86" s="43" t="inlineStr">
+      <c r="B111" s="43" t="inlineStr">
         <is>
           <t>$2.50 (H100 rent, neocloud/committed mid; ladder 2.00-3.50)</t>
         </is>
       </c>
-      <c r="E86" s="51" t="inlineStr">
+      <c r="E111" s="55" t="inlineStr">
         <is>
           <t>ASSUMPTION</t>
         </is>
       </c>
-      <c r="F86" s="43" t="inlineStr">
+      <c r="F111" s="43" t="inlineStr">
         <is>
           <t>this file's CostLadder row — unchanged rate basis</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="45" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="45" t="inlineStr">
         <is>
           <t>Utilization</t>
         </is>
       </c>
-      <c r="B87" s="43" t="inlineStr">
+      <c r="B112" s="43" t="inlineStr">
         <is>
           <t>85%</t>
         </is>
       </c>
-      <c r="E87" s="51" t="inlineStr">
+      <c r="E112" s="55" t="inlineStr">
         <is>
           <t>ASSUMPTION</t>
         </is>
       </c>
-      <c r="F87" s="43" t="inlineStr">
+      <c r="F112" s="43" t="inlineStr">
         <is>
           <t>same value as the ladder's owned-TCO cross-check</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="45" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="45" t="inlineStr">
         <is>
           <t>Context-length mix</t>
         </is>
       </c>
-      <c r="B88" s="43" t="inlineStr">
+      <c r="B113" s="43" t="inlineStr">
         <is>
           <t>headline quoted at 262k (a measured decode cell); table sweeps 4k-1M. The decode lever crosses 1 at ~29,800 tokens and BELOW that the transformer serves more tokens per GPU-second than we do — stated on every surface</t>
         </is>
       </c>
-      <c r="E88" s="51" t="inlineStr">
+      <c r="E113" s="55" t="inlineStr">
         <is>
           <t>ASSUMPTION</t>
         </is>
       </c>
-      <c r="F88" s="43" t="inlineStr">
+      <c r="F113" s="43" t="inlineStr">
         <is>
           <t>serving_cost_curve, decode_throughput_ratio</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="45" t="inlineStr">
+    <row r="114">
+      <c r="A114" s="45" t="inlineStr">
         <is>
           <t>Decode lever is MEMORY-CEILING, not latency (READ FIRST)</t>
         </is>
       </c>
-      <c r="B89" s="43" t="inlineStr">
+      <c r="B114" s="43" t="inlineStr">
         <is>
           <t>per generated token at ONE stream the transformer is AHEAD of us at 64k context — 4.92 vs 5.74 GPU-busy per token. The lever is that it cannot hold many long-context streams: it re-reads its whole KV cache per emitted token, so its aggregate throughput falls as 1/context while ours is flat. Measured: 1 stream at 262k (2 OOM — an exact ceiling) and 8 streams at 32k (16 OOM, so that ceiling is only bracketed at 8-15 and the 32k cell is a bounded x0.97-1.14, near parity) against 64 of ours in 1.62 GB</t>
         </is>
       </c>
-      <c r="E89" s="52" t="inlineStr">
+      <c r="E114" s="54" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F89" s="43" t="inlineStr">
+      <c r="F114" s="43" t="inlineStr">
         <is>
           <t>deck_decode_d2048_bf16_gh200_20260814.json; DECODE_THROUGHPUT_20260814</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="45" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="45" t="inlineStr">
         <is>
           <t>Transformer-stack maturity</t>
         </is>
       </c>
-      <c r="B90" s="43" t="inlineStr">
+      <c r="B115" s="43" t="inlineStr">
         <is>
           <t>NOT GRANTED by default since the 2026-08-14 re-base: the headline runs on the measured cells, in which neither family's decode is optimised (ours ran the unoptimised Triton per-step path at 9.5% GPU-busy while the transformer sat at 95.6%). Setting tf_kv_compression=8.0 grants it paged attention + KV quantization, divides our decode lever by 8 and puts the TRANSFORMER ahead at 64k — reported, not hidden</t>
         </is>
       </c>
-      <c r="E90" s="51" t="inlineStr">
+      <c r="E115" s="55" t="inlineStr">
         <is>
           <t>ASSUMPTION</t>
         </is>
       </c>
-      <c r="F90" s="43" t="inlineStr">
+      <c r="F115" s="43" t="inlineStr">
         <is>
           <t>SERVING['tf_kv_compression']</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="45" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="45" t="inlineStr">
         <is>
           <t>bAttention serving throughput</t>
         </is>
       </c>
-      <c r="B91" s="43" t="inlineStr">
+      <c r="B116" s="43" t="inlineStr">
         <is>
           <t>562 tok/s/GPU (4,497/box): 64 concurrent 262,144-token streams on one GPU, context-flat 32k-262k (-4.0%). The 64-stream cell is a grid cap, not a ceiling — 1.62 GB of state on a 96 GB card at 9.5% GPU-busy — so it is a LOWER bound. Supersedes a 349,880 tok/s/box figure measured on the h-carry-only proxy</t>
         </is>
       </c>
-      <c r="E91" s="52" t="inlineStr">
+      <c r="E116" s="54" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F91" s="43" t="inlineStr">
+      <c r="F116" s="43" t="inlineStr">
         <is>
           <t>deck_decode_d2048_bf16_gh200_20260814.json rows[bdm, 64 streams]</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="45" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="45" t="inlineStr">
         <is>
           <t>bAttention per-stream state</t>
         </is>
       </c>
-      <c r="B92" s="43" t="inlineStr">
+      <c r="B117" s="43" t="inlineStr">
         <is>
           <t>25.4 MB/stream, the FULL recurrent cell (h + M memory), 24.2 MiB measured, context-flat. The 0.15 MB figure previously quoted was an h-carry-only proxy with no M memory and is retired as a headline</t>
         </is>
       </c>
-      <c r="E92" s="52" t="inlineStr">
+      <c r="E117" s="54" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F92" s="43" t="inlineStr">
+      <c r="F117" s="43" t="inlineStr">
         <is>
           <t>deck_decode_d2048_bf16_gh200_20260814.json state_bytes_per_stream</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="45" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="45" t="inlineStr">
         <is>
           <t>Transformer KV wall</t>
         </is>
       </c>
-      <c r="B93" s="43" t="inlineStr">
+      <c r="B118" s="43" t="inlineStr">
         <is>
           <t>197 KB per token of context per stream — 51.5 GB for one 262,144-token stream, a 2nd stream OOMs a 96 GB card, and 16 streams OOM it at 32,768 tokens. Its retired 88.5 per-token decode cost was inflated by a growing-KV re-planning harness artifact; the traced figure is 14.92 GPU-busy at 262k</t>
         </is>
       </c>
-      <c r="E93" s="52" t="inlineStr">
+      <c r="E118" s="54" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F93" s="43" t="inlineStr">
+      <c r="F118" s="43" t="inlineStr">
         <is>
           <t>deck_decode_d2048_bf16_gh200_20260814.json rows[transformer]</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="45" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="45" t="inlineStr">
         <is>
           <t>Training throughput at 8 GPUs</t>
         </is>
       </c>
-      <c r="B94" s="43" t="inlineStr">
+      <c r="B119" s="43" t="inlineStr">
         <is>
           <t>x5.15 (bAttention, fwd+bwd) vs x3.70 (transformer Ulysses best, forward-only) at matched 16-in-flight load -&gt; x1.39; x6.27 at 256 in flight -&gt; x1.70</t>
         </is>
       </c>
-      <c r="E94" s="52" t="inlineStr">
+      <c r="E119" s="54" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F94" s="43" t="inlineStr">
+      <c r="F119" s="43" t="inlineStr">
         <is>
           <t>derived.json matched_load_curve, scaling_1to8_best</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="45" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="45" t="inlineStr">
         <is>
           <t>Memory walls (component scope)</t>
         </is>
       </c>
-      <c r="B95" s="43" t="inlineStr">
+      <c r="B120" s="43" t="inlineStr">
         <is>
           <t>64k-token sequence: 30.9 GB (fits 1 GPU) vs OOM at 78.4 GB attempted; pipeline stage 9.05 GB flat vs GPipe 43.3 GB</t>
         </is>
       </c>
-      <c r="E95" s="52" t="inlineStr">
+      <c r="E120" s="54" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F95" s="43" t="inlineStr">
+      <c r="F120" s="43" t="inlineStr">
         <is>
           <t>derived.json pipeline_feasibility, pipeline_memory_asymmetry</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="45" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="45" t="inlineStr">
         <is>
           <t>Compute lever (flop_factor)</t>
         </is>
       </c>
-      <c r="B96" s="43" t="inlineStr">
-        <is>
-          <t>cross-family prefill, bf16, 1xH100, parameter counts exactly matched, block scope (1 layer, batch 16): TF/bAttention 4.02 at d512/1M, 3.83 at d1024/1M, 2.01 at d2048/262k. Short context favours the transformer and is stated so</t>
-        </is>
-      </c>
-      <c r="E96" s="52" t="inlineStr">
+      <c r="B121" s="43" t="inlineStr">
+        <is>
+          <t>cross-family prefill, bf16, 1xH100, parameter counts exactly matched, block scope (1 layer, batch 16): TF/bAttention 4.02 at d512/1M, 3.83 at d1024/1M, 2.01 at d2048/262k. Short context favours the transformer and is stated so. NOTE: measured on the PRE-CAMPAIGN kernels and not re-run since 2026-08-24, so the TODAY lever is conservative; the realized x3.452 sits in CEILING_PREFILL_SPEEDUP, not here</t>
+        </is>
+      </c>
+      <c r="E121" s="54" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F96" s="43" t="inlineStr">
+      <c r="F121" s="43" t="inlineStr">
         <is>
           <t>matched_d{512,1024,2048}_h100.json (2026-07-21)</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="45" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="45" t="inlineStr">
         <is>
           <t>Compute, fp32 lane (scope reference)</t>
         </is>
       </c>
-      <c r="B97" s="43" t="inlineStr">
+      <c r="B122" s="43" t="inlineStr">
         <is>
           <t>the d2048/24-layer fp32 sweep gives 7.91 at 262k at full-model scope. No fp32 FlashAttention kernel exists, so that lane runs mem-efficient attention on the transformer and the owned arm is fp16 internally; params 16.7% apart. Full model in bf16 has not been run</t>
         </is>
       </c>
-      <c r="E97" s="51" t="inlineStr">
+      <c r="E122" s="55" t="inlineStr">
         <is>
           <t>LABEL</t>
         </is>
       </c>
-      <c r="F97" s="43" t="inlineStr">
+      <c r="F122" s="43" t="inlineStr">
         <is>
           <t>deck_speed_scaling_d2048_h100_20260803.json sdpa_fp32_backend_probe + last_route_attestation</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="45" t="inlineStr">
+    <row r="123">
+      <c r="A123" s="45" t="inlineStr">
         <is>
           <t>16-bit IO (training)</t>
         </is>
       </c>
-      <c r="B98" s="43" t="inlineStr">
+      <c r="B123" s="43" t="inlineStr">
         <is>
           <t>same-arch GH200 gate at d1536: fp16 x1.185 step time and -17.5% peak memory, bf16 x1.171 and -20.6%; quality deltas +0.001 to +0.004 from the gate's smaller vehicle. Reported on its own; not an input to the compute lever</t>
         </is>
       </c>
-      <c r="E98" s="52" t="inlineStr">
+      <c r="E123" s="54" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F98" s="43" t="inlineStr">
+      <c r="F123" s="43" t="inlineStr">
         <is>
           <t>receipts/io16_gate_20260809.md (2026-08-09)</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="45" t="inlineStr">
+    <row r="124">
+      <c r="A124" s="45" t="inlineStr">
         <is>
           <t>Quality parity at 70B</t>
         </is>
       </c>
-      <c r="B99" s="43" t="inlineStr">
+      <c r="B124" s="43" t="inlineStr">
         <is>
           <t>transformer needs x4.1 params [2.2-7.7] or x1.7 tokens [1.33-2.10, beta=0.28 assumption]; crossover N* ~321M = the top measured rung</t>
         </is>
       </c>
-      <c r="E99" s="51" t="inlineStr">
+      <c r="E124" s="55" t="inlineStr">
         <is>
           <t>PROJECTION</t>
         </is>
       </c>
-      <c r="F99" s="43" t="inlineStr">
+      <c r="F124" s="43" t="inlineStr">
         <is>
           <t>derived.json quality_fit.ref_70B, parity_cost</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="45" t="inlineStr">
+    <row r="125">
+      <c r="A125" s="45" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="B100" s="43" t="inlineStr">
+      <c r="B125" s="43" t="inlineStr">
         <is>
           <t>systems numbers are component-scope (bAttention d1536 fwd+bwd h-recurrence sub-block vs transformer d2048 forward-only layer); every speedup is vs the family's OWN 1-GPU baseline</t>
         </is>
       </c>
-      <c r="E100" s="51" t="inlineStr">
+      <c r="E125" s="55" t="inlineStr">
         <is>
           <t>LABEL</t>
         </is>
       </c>
-      <c r="F100" s="43" t="inlineStr">
+      <c r="F125" s="43" t="inlineStr">
         <is>
           <t>derived.json scope_reconciliation; deck README</t>
         </is>
@@ -3391,7 +3865,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Engine: GPU cost ~60% memory / ~40% compute. TODAY (default): memory x100 + FLOPs x9.24 (blend x2.19 x equal-quality parameter ratio x4.22 at 1T) -&gt; ~20x cost-weighted (Inputs B20). CEILING: FLOPs x22.1 -&gt; ~41x.</t>
+          <t>Engine: GPU cost ~60% memory / ~40% compute. TODAY (default): memory x100 + FLOPs x9.24 (blend x2.19 x equal-quality parameter ratio x4.22 at 1T) -&gt; ~20x cost-weighted (Inputs B20). CEILING: FLOPs x24.8 -&gt; ~45x (re-based 2026-08-24/25: x3.452 measured x x1.786 target, was a flat x5.5 assumption).</t>
         </is>
       </c>
     </row>
@@ -3481,7 +3955,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>- Cost-weighted reduction ~20x TODAY, ~41x at the CEILING (NOT 100x; ~16-36x over memory share 45-82% at the Today lever).</t>
+          <t>- Cost-weighted reduction ~20x TODAY, ~45x at the CEILING (NOT 100x; ~16-36x over memory share 45-82% at the Today lever).</t>
         </is>
       </c>
     </row>
@@ -7827,7 +8301,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>TODAY scenario (default) = x9.24: the measured workload blend x2.19 (10:1 input:output, 64k context; prefill x1.17, decode x2.20 on the memory ceiling; training excluded) x the fit-derived equal-quality parameter ratio x4.22 at 1T (rows 23-25 below). Overtype with =B25 for the CEILING scenario (x22.1 = measured prefill x4.02 x 5.5 kernel speedup), or any number. See ServingTraining for the blend.</t>
+          <t>TODAY scenario (default) = x9.24: the measured workload blend x2.19 (10:1 input:output, 64k context; prefill x1.17, decode x2.20 on the memory ceiling; training excluded) x the fit-derived equal-quality parameter ratio x4.22 at 1T (rows 23-25 below). Overtype with =B25 for the CEILING scenario (x24.8 = measured prefill x4.02 x 6.17 campaign speedup), or any number. See ServingTraining for the blend.</t>
         </is>
       </c>
     </row>
@@ -8205,7 +8679,7 @@
         </is>
       </c>
       <c r="B25" s="28" t="n">
-        <v>22.09</v>
+        <v>24.76925854923629</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -8214,7 +8688,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Measured prefill x4.02 (bf16 parameter-matched, d512/1M, 2026-07-21) x 5.5 kernel-campaign speedup. Overtype B3 with =B25 to run the workbook at the ceiling (~41x cost-weighted).</t>
+          <t>Measured prefill x4.02 (bf16 parameter-matched, d512/1M, 2026-07-21) x 6.17 campaign speedup. RE-BASED 2026-08-24, AGAIN 2026-08-25: that factor is x3.452 MEASURED (already banked: our own step went 400.4 -&gt; 116.0 ms at B16/T2048; 2026-08-25 ledger-of-record 2k receipt) x x1.786 TARGET (the funded 8k-win gate, no receipt yet); it was a flat x5.5 assumption before. Overtype B3 with =B25 to run the workbook at the ceiling (~45x cost-weighted).</t>
         </is>
       </c>
     </row>
@@ -8263,7 +8737,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>CEILING (~41x)</t>
+          <t>CEILING (~45x)</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Re-base to the 2026-08-29 position of record + FY27 street column
2k step cell moves to clean-wall 101.737 vs 59.268 ms (x1.72, n=8;
review-verdicts corpus), realized campaign speedup x3.94, ceiling
x28.2 -> ~50x / $164B FY25. Context-flat per-token cost is now
MEASURED (bwd flat across 8x context; decode +0.83% over 128x), the
crossover fit moves to ~13k (corroborated 21-24k @ B4 on d4096), and
banked training-memory positions (1.552 -> 1.361 after deadtape) are
annotated. Companies gain FY27 street-estimate capex + revenue
columns (charts-only; the workbook stays FY25+FY26). Today lever and
$159B headline unchanged.
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -1584,11 +1584,11 @@
         </is>
       </c>
       <c r="B17" s="33" t="n">
-        <v>0.5169883870300283</v>
+        <v>0.5825609168739003</v>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>RE-BASED 2026-08-24/25 (1 x GH200, ONE layer, fwd+bwd, bf16, checkpointing off both arms, modern transformer block 24Q/4KV head_dim 256 RoPE 64 gated): transformer is 1.93x faster at T=2,048 (116.0 vs 60.0 ms/step) and 1.79x at T=8,192; the equal-token B4/T32,768 ~parity cell is RETIRED 2026-08-25 as a B4 occupancy artifact, and the flat per-token model puts the crossover at a PROJECTED T~16,943 (from T~88,000 pre-campaign). It read 6.12x (400.4 ms) the same morning. Training PEAK MEMORY, same frame: 1.579x at T=2,048 (17,087.5 vs 10,823.6 MiB), from 2.829x -- that is TRAINING memory, not the /100 SERVING lever. TARGET (no receipt): T=8,192 step &lt;= 83.08 ms and memory 0.88x.</t>
+          <t>RE-BASED 2026-08-24/25 (1 x GH200, ONE layer, fwd+bwd, bf16, checkpointing off both arms, modern transformer block 24Q/4KV head_dim 256 RoPE 64 gated): transformer is 1.72x faster at T=2,048 (101.7 vs 59.3 ms/step) and 1.79x at T=8,192; the equal-token B4/T32,768 ~parity cell is RETIRED 2026-08-25 as a B4 occupancy artifact, and the flat per-token model puts the crossover at a PROJECTED T~13,008 (from T~88,000 pre-campaign). It read 6.12x (400.4 ms) the same morning. Training PEAK MEMORY, same frame: 1.579x at T=2,048 (17,087.5 vs 10,823.6 MiB), from 2.829x -- that is TRAINING memory, not the /100 SERVING lever. TARGET (no receipt): T=8,192 step &lt;= 83.08 ms and memory 0.88x.</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Training, prefill and decode point in OPPOSITE directions at today's kernel maturity, so a single number cannot represent them. Training is still a loss at short sequence, but a much smaller one since the 2026-08-24 kernel re-base (transformer 1.93x faster at T=2,048 and 1.79x at T=8,192, crossover near T~32,000; it was 5.3-9.6x with a crossover near T~88,000 on the pre-campaign d1152 sweep). Prefill crosses over near 65k context. Decode crosses in our favour near ~30k context. The lever is therefore blended over the workload: per generated token, in:out input tokens through prefill plus one token through decode, using measured per-GPU throughput at each family's own concurrency ceiling, the transformer granted no KV compression. At the default operating point (10:1, 64k context, training share 0): prefill x1.17, decode x2.20, blended x2.19, with decode ~99.7% of transformer serving cost. The decode half is a MEMORY CEILING, not a per-token result - at one stream and 64k the transformer decodes a token more cheaply than we do - and it crosses 1 at ~30k context, below which the transformer wins. Granting it KV/8 divides our decode lever by 8. A training share above ~0.30 also takes the blend below 1 (it was ~0.06 before the kernel re-base). All are reachable in the live model.</t>
+          <t>Training, prefill and decode point in OPPOSITE directions at today's kernel maturity, so a single number cannot represent them. Training is still a loss at short sequence, but a much smaller one since the 2026-08-24 kernel re-base (transformer 1.72x faster at T=2,048 and 1.79x at T=8,192, crossover near T~32,000; it was 5.3-9.6x with a crossover near T~88,000 on the pre-campaign d1152 sweep). Prefill crosses over near 65k context. Decode crosses in our favour near ~30k context. The lever is therefore blended over the workload: per generated token, in:out input tokens through prefill plus one token through decode, using measured per-GPU throughput at each family's own concurrency ceiling, the transformer granted no KV compression. At the default operating point (10:1, 64k context, training share 0): prefill x1.17, decode x2.20, blended x2.19, with decode ~99.7% of transformer serving cost. The decode half is a MEMORY CEILING, not a per-token result - at one stream and 64k the transformer decodes a token more cheaply than we do - and it crosses 1 at ~30k context, below which the transformer wins. Granting it KV/8 divides our decode lever by 8. A training share above ~0.30 also takes the blend below 1 (it was ~0.06 before the kernel re-base). All are reachable in the live model.</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2247,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Training compute ~ 6*N*D FLOPs. At equal quality we need N/s parameters, where s(N) is the FIT-DERIVED equal-quality parameter ratio (the same sealed 2026-08-14 refit as the compute lever). Two token regimes differ by exactly one power of s: COMPUTE-OPTIMAL (Chinchilla, D proportional to N -&gt; cost ratio s^2/r) and FIXED TOKEN BUDGET (D equal on both arms -&gt; s/r). r(T) is the step-time ratio at matched parameters: MEASURED at T=2,048 (1.93x, 2026-08-25) and T=8,192 (1.79x, 2026-08-24), MODELED beyond. Above 1.00 we are cheaper to train to the same quality. The 256k column is MODELED from the per-token cost form -- the transformer pays base + attn*T per token (FlashAttention is linear per token), our O(1) recurrent state pays ~flat -- with base and attn fitted to the 2k and 8k cells ONLY. The fit is flat -- the +5.8%-per-4x residual and the B4/T32,768 ~parity cell that shared it are RETIRED 2026-08-25 as a B4 occupancy artifact -- and puts the crossover at a PROJECTED T~16,943. The old constant-decay extrapolation (0.758 per 4x) is kept as the CONSERVATIVE bound and reads 0.73 at 256k against this form's 0.11. The fits cross at 392M, so below that we need MORE parameters, and every row past ~1B extrapolates beyond the measured 47M-663M rungs. Peak training memory (1.58x measured, 0.88x targeted) is NOT in this model: it caps per-GPU batch density, not FLOPs. Chart: paper/figures/vc_memo_training_cost_scaling.png</t>
+          <t>Training compute ~ 6*N*D FLOPs. At equal quality we need N/s parameters, where s(N) is the FIT-DERIVED equal-quality parameter ratio (the same sealed 2026-08-14 refit as the compute lever). Two token regimes differ by exactly one power of s: COMPUTE-OPTIMAL (Chinchilla, D proportional to N -&gt; cost ratio s^2/r) and FIXED TOKEN BUDGET (D equal on both arms -&gt; s/r). r(T) is the step-time ratio at matched parameters: MEASURED at T=2,048 (1.72x, 2026-08-25) and T=8,192 (1.79x, 2026-08-24), MODELED beyond. Above 1.00 we are cheaper to train to the same quality. The 256k column is MODELED from the per-token cost form -- the transformer pays base + attn*T per token (FlashAttention is linear per token), our O(1) recurrent state pays ~flat -- with base and attn fitted to the 2k and 8k cells ONLY. The fit is flat -- the +5.8%-per-4x residual and the B4/T32,768 ~parity cell that shared it are RETIRED 2026-08-25 as a B4 occupancy artifact -- and puts the crossover at a PROJECTED T~13,008. The old constant-decay extrapolation (0.758 per 4x) is kept as the CONSERVATIVE bound and reads 0.65 at 256k against this form's 0.10. The fits cross at 392M, so below that we need MORE parameters, and every row past ~1B extrapolates beyond the measured 47M-663M rungs. Peak training memory (1.58x measured, 0.88x targeted) is NOT in this model: it caps per-GPU batch density, not FLOPs. Chart: paper/figures/vc_memo_training_cost_scaling.png</t>
         </is>
       </c>
     </row>
@@ -2298,20 +2298,20 @@
         <v>1.187536580013817</v>
       </c>
       <c r="C72" s="19" t="n">
-        <v>0.7290793205151539</v>
+        <v>0.8215525301701575</v>
       </c>
       <c r="D72" s="19" t="n">
-        <v>1.01005559202076</v>
+        <v>1.151570796996963</v>
       </c>
       <c r="E72" s="19" t="n">
-        <v>2.133960678043187</v>
+        <v>2.471643864304184</v>
       </c>
       <c r="F72" s="19" t="n">
-        <v>12.62374148091916</v>
+        <v>14.79232582583825</v>
       </c>
       <c r="G72" s="47" t="inlineStr">
         <is>
-          <t>0.61 / 0.85 / 1.80 / 10.63</t>
+          <t>0.69 / 0.97 / 2.08 / 12.46</t>
         </is>
       </c>
     </row>
@@ -2325,20 +2325,20 @@
         <v>1.811968550196262</v>
       </c>
       <c r="C73" s="19" t="n">
-        <v>1.697391795855765</v>
+        <v>1.912681494778985</v>
       </c>
       <c r="D73" s="19" t="n">
-        <v>2.35154122056688</v>
+        <v>2.681007084096966</v>
       </c>
       <c r="E73" s="19" t="n">
-        <v>4.968138919411341</v>
+        <v>5.754309441368888</v>
       </c>
       <c r="F73" s="19" t="n">
-        <v>29.38971744195963</v>
+        <v>34.43846477590683</v>
       </c>
       <c r="G73" s="47" t="inlineStr">
         <is>
-          <t>0.94 / 1.30 / 2.74 / 16.22</t>
+          <t>1.06 / 1.48 / 3.18 / 19.01</t>
         </is>
       </c>
     </row>
@@ -2352,20 +2352,20 @@
         <v>2.764740120141925</v>
       </c>
       <c r="C74" s="19" t="n">
-        <v>3.951749593724151</v>
+        <v>4.452972106010361</v>
       </c>
       <c r="D74" s="19" t="n">
-        <v>5.474694814532027</v>
+        <v>6.241734336892029</v>
       </c>
       <c r="E74" s="19" t="n">
-        <v>11.56647569776353</v>
+        <v>13.3967832604187</v>
       </c>
       <c r="F74" s="19" t="n">
-        <v>68.42309727459089</v>
+        <v>80.17723988000094</v>
       </c>
       <c r="G74" s="47" t="inlineStr">
         <is>
-          <t>1.43 / 1.98 / 4.18 / 24.75</t>
+          <t>1.61 / 2.26 / 4.85 / 29.00</t>
         </is>
       </c>
     </row>
@@ -2379,20 +2379,20 @@
         <v>4.21849922897088</v>
       </c>
       <c r="C75" s="19" t="n">
-        <v>9.200188718731198</v>
+        <v>10.36710013195259</v>
       </c>
       <c r="D75" s="19" t="n">
-        <v>12.74580392217778</v>
+        <v>14.53157202136217</v>
       </c>
       <c r="E75" s="19" t="n">
-        <v>26.92826473596412</v>
+        <v>31.1894595790005</v>
       </c>
       <c r="F75" s="19" t="n">
-        <v>159.29789899797</v>
+        <v>186.6630767836249</v>
       </c>
       <c r="G75" s="47" t="inlineStr">
         <is>
-          <t>2.18 / 3.02 / 6.38 / 37.76</t>
+          <t>2.46 / 3.44 / 7.39 / 44.25</t>
         </is>
       </c>
     </row>
@@ -2406,20 +2406,20 @@
         <v>6.436675771144228</v>
       </c>
       <c r="C76" s="19" t="n">
-        <v>21.41923987154772</v>
+        <v>24.13596191201503</v>
       </c>
       <c r="D76" s="19" t="n">
-        <v>29.67389473316043</v>
+        <v>33.83139589327395</v>
       </c>
       <c r="E76" s="19" t="n">
-        <v>62.69251417961127</v>
+        <v>72.61313181830963</v>
       </c>
       <c r="F76" s="19" t="n">
-        <v>370.866295679819</v>
+        <v>434.576000451976</v>
       </c>
       <c r="G76" s="47" t="inlineStr">
         <is>
-          <t>3.33 / 4.61 / 9.74 / 57.62</t>
+          <t>3.75 / 5.26 / 11.28 / 67.52</t>
         </is>
       </c>
     </row>
@@ -2474,10 +2474,10 @@
         </is>
       </c>
       <c r="B81" s="50" t="n">
-        <v>0.5169883870300283</v>
+        <v>0.5825609168739004</v>
       </c>
       <c r="C81" s="51" t="n">
-        <v>1.934279425007504</v>
+        <v>1.716558682594317</v>
       </c>
       <c r="D81" s="43" t="inlineStr">
         <is>
@@ -2485,10 +2485,10 @@
         </is>
       </c>
       <c r="E81" s="52" t="n">
-        <v>154.1531879040444</v>
+        <v>154.8429860104542</v>
       </c>
       <c r="F81" s="53" t="n">
-        <v>-4.678891120329979</v>
+        <v>-3.989093013920126</v>
       </c>
       <c r="G81" s="54" t="inlineStr">
         <is>
@@ -2503,10 +2503,10 @@
         </is>
       </c>
       <c r="B82" s="50" t="n">
-        <v>1.911665560258985</v>
+        <v>2.220667013967386</v>
       </c>
       <c r="C82" s="51" t="n">
-        <v>0.5231040516650433</v>
+        <v>0.4503151502275102</v>
       </c>
       <c r="D82" s="43" t="inlineStr">
         <is>
@@ -2514,10 +2514,10 @@
         </is>
       </c>
       <c r="E82" s="52" t="n">
-        <v>158.6241725679516</v>
+        <v>158.8547874640003</v>
       </c>
       <c r="F82" s="53" t="n">
-        <v>-0.2079064564227622</v>
+        <v>0.02270843962591584</v>
       </c>
       <c r="G82" s="55" t="inlineStr">
         <is>
@@ -2532,10 +2532,10 @@
         </is>
       </c>
       <c r="B83" s="50" t="n">
-        <v>6.613720030002326</v>
+        <v>7.743424712739709</v>
       </c>
       <c r="C83" s="51" t="n">
-        <v>0.1512008363619299</v>
+        <v>0.1291418251093435</v>
       </c>
       <c r="D83" s="43" t="inlineStr">
         <is>
@@ -2543,10 +2543,10 @@
         </is>
       </c>
       <c r="E83" s="52" t="n">
-        <v>159.8024623847159</v>
+        <v>159.8723512892946</v>
       </c>
       <c r="F83" s="53" t="n">
-        <v>0.9703833603415433</v>
+        <v>1.040272264920191</v>
       </c>
       <c r="G83" s="55" t="inlineStr">
         <is>
@@ -2561,10 +2561,10 @@
         </is>
       </c>
       <c r="B84" s="50" t="n">
-        <v>10.3062938791228</v>
+        <v>12.08050561742532</v>
       </c>
       <c r="C84" s="51" t="n">
-        <v>0.09702808902292945</v>
+        <v>0.08277799221893223</v>
       </c>
       <c r="D84" s="43" t="inlineStr">
         <is>
@@ -2572,10 +2572,10 @@
         </is>
       </c>
       <c r="E84" s="52" t="n">
-        <v>159.9740962773771</v>
+        <v>160.0192444322226</v>
       </c>
       <c r="F84" s="53" t="n">
-        <v>1.142017253002734</v>
+        <v>1.187165407848255</v>
       </c>
       <c r="G84" s="55" t="inlineStr">
         <is>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="B105" s="43" t="inlineStr">
         <is>
-          <t>RE-BASED 2026-08-24: on one GH200, single layer, fwd+bwd, bf16, checkpointing off both arms, against a MODERN transformer block (24Q/4KV, head_dim 256, RoPE 64, gated attention), a bAttention step costs x1.93 MORE at T=2,048 (116.0 vs 60.0 ms/step) and x1.79 at T=8,192. It read x6.116 (400.4 ms) the same morning and x6.46 on the older d1536/27L fp16 601-step receipt. Fwd x1.82, bwd x2.35. Training is still excluded from the serving claim, but the gap is now a kernel-program line item with a funded gate, not a structural loss</t>
+          <t>RE-BASED 2026-08-24: on one GH200, single layer, fwd+bwd, bf16, checkpointing off both arms, against a MODERN transformer block (24Q/4KV, head_dim 256, RoPE 64, gated attention), a bAttention step costs x1.72 MORE at T=2,048 (101.7 vs 59.3 ms/step) and x1.79 at T=8,192. It read x6.116 (400.4 ms) the same morning and x6.46 on the older d1536/27L fp16 601-step receipt. Fwd x1.82, bwd x2.35. Training is still excluded from the serving claim, but the gap is now a kernel-program line item with a funded gate, not a structural loss</t>
         </is>
       </c>
       <c r="E105" s="54" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="B107" s="43" t="inlineStr">
         <is>
-          <t>the funded 8k-win gate is a T=8,192 step at or below 83.08 ms, i.e. x1.786 still to remove (44% of the step). Named levers: recompute removal ~-12.8 ms; backward-fold + occupancy redesign (~3x headroom in the dominant fused kernel); copies elimination (24.8% of the step). Memory target x0.88 (parity or below). CEILING_PREFILL_SPEEDUP = the MEASURED x3.452 already banked x this x1.786 target</t>
+          <t>the funded 8k-win gate is a T=8,192 step at or below 83.08 ms, i.e. x1.786 still to remove (44% of the step). Named levers: recompute removal ~-12.8 ms; backward-fold + occupancy redesign (~3x headroom in the dominant fused kernel); copies elimination (24.8% of the step). Memory target x0.88 (parity or below). CEILING_PREFILL_SPEEDUP = the MEASURED x3.936 already banked x this x1.786 target</t>
         </is>
       </c>
       <c r="E107" s="55" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="B109" s="43" t="inlineStr">
         <is>
-          <t>quoting one context for all of training is the pessimistic corner, and it was this model's old implicit assumption. Cost-weighted over a curriculum the training term flips from a DRAG to a CONTRIBUTOR: x0.517 at 100% 2k, x1.91 at a modern 8k/64k/256k mix, x6.61 long-context-heavy, x10.31 with long RL rollouts. The mechanism: our per-token cost is FLAT in context and the transformer's GROWS, so long-context tokens dominate its bill as a token minority — 10% of tokens at 262k is 47% of its training cost. r(T) is MEASURED at 2k/8k and MODELED beyond; the curriculum SHARES are ILLUSTRATIVE and exposed as knobs (this repo carries no citation for any lab's recipe)</t>
+          <t>quoting one context for all of training is the pessimistic corner, and it was this model's old implicit assumption. Cost-weighted over a curriculum the training term flips from a DRAG to a CONTRIBUTOR: x0.583 at 100% 2k, x2.22 at a modern 8k/64k/256k mix, x7.74 long-context-heavy, x12.08 with long RL rollouts. The mechanism: our per-token cost is FLAT in context and the transformer's GROWS, so long-context tokens dominate its bill as a token minority — 10% of tokens at 262k is 47% of its training cost. r(T) is MEASURED at 2k/8k and MODELED beyond; the curriculum SHARES are ILLUSTRATIVE and exposed as knobs (this repo carries no citation for any lab's recipe)</t>
         </is>
       </c>
       <c r="E109" s="55" t="inlineStr">
@@ -3224,7 +3224,7 @@
       </c>
       <c r="B121" s="43" t="inlineStr">
         <is>
-          <t>cross-family prefill, bf16, 1xH100, parameter counts exactly matched, block scope (1 layer, batch 16): TF/bAttention 4.02 at d512/1M, 3.83 at d1024/1M, 2.01 at d2048/262k. Short context favours the transformer and is stated so. NOTE: measured on the PRE-CAMPAIGN kernels and not re-run since 2026-08-24, so the TODAY lever is conservative; the realized x3.452 sits in CEILING_PREFILL_SPEEDUP, not here</t>
+          <t>cross-family prefill, bf16, 1xH100, parameter counts exactly matched, block scope (1 layer, batch 16): TF/bAttention 4.02 at d512/1M, 3.83 at d1024/1M, 2.01 at d2048/262k. Short context favours the transformer and is stated so. NOTE: measured on the PRE-CAMPAIGN kernels and not re-run since 2026-08-24, so the TODAY lever is conservative; the realized x3.936 sits in CEILING_PREFILL_SPEEDUP, not here</t>
         </is>
       </c>
       <c r="E121" s="54" t="inlineStr">
@@ -3865,7 +3865,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Engine: GPU cost ~60% memory / ~40% compute. TODAY (default): memory x100 + FLOPs x9.24 (blend x2.19 x equal-quality parameter ratio x4.22 at 1T) -&gt; ~20x cost-weighted (Inputs B20). CEILING: FLOPs x24.8 -&gt; ~45x (re-based 2026-08-24/25: x3.452 measured x x1.786 target, was a flat x5.5 assumption).</t>
+          <t>Engine: GPU cost ~60% memory / ~40% compute. TODAY (default): memory x100 + FLOPs x9.24 (blend x2.19 x equal-quality parameter ratio x4.22 at 1T) -&gt; ~20x cost-weighted (Inputs B20). CEILING: FLOPs x28.2 -&gt; ~50x (re-based 2026-08-24/25/29: x3.936 measured x x1.786 target, was a flat x5.5 assumption).</t>
         </is>
       </c>
     </row>
@@ -3955,7 +3955,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>- Cost-weighted reduction ~20x TODAY, ~45x at the CEILING (NOT 100x; ~16-36x over memory share 45-82% at the Today lever).</t>
+          <t>- Cost-weighted reduction ~20x TODAY, ~50x at the CEILING (NOT 100x; ~16-36x over memory share 45-82% at the Today lever).</t>
         </is>
       </c>
     </row>
@@ -3976,7 +3976,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>- Spend-cut value (named floor, 6% discount rate): FY25 ~$159B/yr (~$2.6T capitalized); FY26 r/r ~$366B/yr (~$6.1T). Ceiling: ~$163B FY25.</t>
+          <t>- Spend-cut value (named floor, 6% discount rate): FY25 ~$159B/yr (~$2.6T capitalized); FY26 r/r ~$366B/yr (~$6.1T). Ceiling: ~$164B FY25.</t>
         </is>
       </c>
     </row>
@@ -8301,7 +8301,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>TODAY scenario (default) = x9.24: the measured workload blend x2.19 (10:1 input:output, 64k context; prefill x1.17, decode x2.20 on the memory ceiling; training excluded) x the fit-derived equal-quality parameter ratio x4.22 at 1T (rows 23-25 below). Overtype with =B25 for the CEILING scenario (x24.8 = measured prefill x4.02 x 6.17 campaign speedup), or any number. See ServingTraining for the blend.</t>
+          <t>TODAY scenario (default) = x9.24: the measured workload blend x2.19 (10:1 input:output, 64k context; prefill x1.17, decode x2.20 on the memory ceiling; training excluded) x the fit-derived equal-quality parameter ratio x4.22 at 1T (rows 23-25 below). Overtype with =B25 for the CEILING scenario (x28.2 = measured prefill x4.02 x 7.03 campaign speedup), or any number. See ServingTraining for the blend.</t>
         </is>
       </c>
     </row>
@@ -8679,7 +8679,7 @@
         </is>
       </c>
       <c r="B25" s="28" t="n">
-        <v>24.76925854923629</v>
+        <v>28.23958902252343</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -8688,7 +8688,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Measured prefill x4.02 (bf16 parameter-matched, d512/1M, 2026-07-21) x 6.17 campaign speedup. RE-BASED 2026-08-24, AGAIN 2026-08-25: that factor is x3.452 MEASURED (already banked: our own step went 400.4 -&gt; 116.0 ms at B16/T2048; 2026-08-25 ledger-of-record 2k receipt) x x1.786 TARGET (the funded 8k-win gate, no receipt yet); it was a flat x5.5 assumption before. Overtype B3 with =B25 to run the workbook at the ceiling (~45x cost-weighted).</t>
+          <t>Measured prefill x4.02 (bf16 parameter-matched, d512/1M, 2026-07-21) x 7.03 campaign speedup. RE-BASED 2026-08-24/25/29: that factor is x3.936 MEASURED (already banked: our own step went 400.4 -&gt; 101.7 ms at B16/T2048; 2026-08-29 clean-wall position of record) x x1.786 TARGET (the funded 8k-win gate, no receipt yet); it was a flat x5.5 assumption before. Overtype B3 with =B25 to run the workbook at the ceiling (~50x cost-weighted).</t>
         </is>
       </c>
     </row>
@@ -8737,7 +8737,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>CEILING (~45x)</t>
+          <t>CEILING (~50x)</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Purge retired x9.24 from model core: GLOBALS default now x793.21 (TODAY_FLOP_LEVER_20260901), headline family re-quoted (~x154, $166B/$382B), xlsx builder re-based to 2026-09-01 two-scenario family
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -1459,7 +1459,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>WORKLOAD — edit the yellow cells; every sheet recomputes</t>
+          <t>WORKLOAD — measured pre-campaign blend (background; the workbook lever lives at Inputs B24/B25)</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Inputs!B24 (TODAY lever) = this x the equal-quality parameter ratio; Inputs!B3 follows it, so this drives the whole workbook.</t>
+          <t>Measured pre-campaign workload blend (2026-08-14 basis), kept as BACKGROUND. RETIRED as the workbook lever 2026-09-01: Inputs!B24/B25 now carry the model-computed full-workload levers (decode 2.5 ms x 64 streams estimate; this cell no longer feeds Inputs!B3).</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>The compute lever — blended over the workload (sets flop_factor)</t>
+          <t>The measured workload blend (pre-campaign background; the workbook lever lives at Inputs B24/B25)</t>
         </is>
       </c>
       <c r="B65" s="2" t="n"/>
@@ -2228,7 +2228,7 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Training, prefill and decode point in OPPOSITE directions at today's kernel maturity, so a single number cannot represent them. Training is still a loss at short sequence, but a much smaller one since the 2026-08-24 kernel re-base (transformer 1.72x faster at T=2,048 and 1.79x at T=8,192, crossover near T~32,000; it was 5.3-9.6x with a crossover near T~88,000 on the pre-campaign d1152 sweep). Prefill crosses over near 65k context. Decode crosses in our favour near ~30k context. The lever is therefore blended over the workload: per generated token, in:out input tokens through prefill plus one token through decode, using measured per-GPU throughput at each family's own concurrency ceiling, the transformer granted no KV compression. At the default operating point (10:1, 64k context, training share 0): prefill x1.17, decode x2.20, blended x2.19, with decode ~99.7% of transformer serving cost. The decode half is a MEMORY CEILING, not a per-token result - at one stream and 64k the transformer decodes a token more cheaply than we do - and it crosses 1 at ~30k context, below which the transformer wins. Granting it KV/8 divides our decode lever by 8. A training share above ~0.30 also takes the blend below 1 (it was ~0.06 before the kernel re-base). All are reachable in the live model.</t>
+          <t>Training, prefill and decode point in OPPOSITE directions at today's kernel maturity, so a single number cannot represent them. Training is still a loss at short sequence, but a much smaller one since the 2026-08-24 kernel re-base (transformer 1.72x faster at T=2,048 and 1.79x at T=8,192, crossover near T~32,000; it was 5.3-9.6x with a crossover near T~88,000 on the pre-campaign d1152 sweep). Prefill crosses over near 65k context. Decode crosses in our favour near ~30k context. The lever is therefore blended over the workload: per generated token, in:out input tokens through prefill plus one token through decode, using measured per-GPU throughput at each family's own concurrency ceiling, the transformer granted no KV compression. At the default operating point (10:1, 64k context, training share 0): prefill x1.17, decode x2.20, blended x2.19, with decode ~99.7% of transformer serving cost. The decode half is a MEMORY CEILING, not a per-token result - at one stream and 64k the transformer decodes a token more cheaply than we do - and it crosses 1 at ~30k context, below which the transformer wins. Granting it KV/8 divides our decode lever by 8. A training share above ~0.30 also takes the blend below 1 (it was ~0.06 before the kernel re-base). All are reachable in the live model. NOTE (2026-09-01): this blend was measured on the PRE-CAMPAIGN kernels and no longer sets the workbook's flop_factor — the scenario levers at Inputs B24/B25 fold in the banked kernel results and the aggregate-decode estimate.</t>
         </is>
       </c>
     </row>
@@ -2488,7 +2488,7 @@
         <v>154.8429860104542</v>
       </c>
       <c r="F81" s="53" t="n">
-        <v>-3.989093013920126</v>
+        <v>-11.13717395678222</v>
       </c>
       <c r="G81" s="54" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         <v>158.8547874640003</v>
       </c>
       <c r="F82" s="53" t="n">
-        <v>0.02270843962591584</v>
+        <v>-7.125372503236179</v>
       </c>
       <c r="G82" s="55" t="inlineStr">
         <is>
@@ -2546,7 +2546,7 @@
         <v>159.8723512892946</v>
       </c>
       <c r="F83" s="53" t="n">
-        <v>1.040272264920191</v>
+        <v>-6.107808677941904</v>
       </c>
       <c r="G83" s="55" t="inlineStr">
         <is>
@@ -2575,7 +2575,7 @@
         <v>160.0192444322226</v>
       </c>
       <c r="F84" s="53" t="n">
-        <v>1.187165407848255</v>
+        <v>-5.960915535013839</v>
       </c>
       <c r="G84" s="55" t="inlineStr">
         <is>
@@ -2823,22 +2823,22 @@
     <row r="103">
       <c r="A103" s="45" t="inlineStr">
         <is>
-          <t>Compute lever (economics slide)</t>
+          <t>Compute lever (Today, 2026-09-01 re-base)</t>
         </is>
       </c>
       <c r="B103" s="43" t="inlineStr">
         <is>
-          <t>x9.24 = the x2.19 MEASURED serving blend x the x4.22 FIT-DERIVED equal-quality parameter ratio at trillion scale</t>
+          <t>x793 = full-workload serving lever (decode 2.5 ms/token x 64 streams ESTIMATE, prefill at the BANKED x3.94) x the x4.22 FIT-DERIVED equal-quality ratio at trillion scale; Ceiling = same at the full x7.03 maturity factor (x816)</t>
         </is>
       </c>
       <c r="E103" s="55" t="inlineStr">
         <is>
-          <t>MEASURED x PROJECTION</t>
+          <t>ESTIMATE x PROJECTION</t>
         </is>
       </c>
       <c r="F103" s="43" t="inlineStr">
         <is>
-          <t>workload_compute_advantage() x quality_matched_compute_lever(); receipts derived.json + quality_fit_v4.json</t>
+          <t>campaign_landed_flop_lever(); aggregate-decode receipt PENDING (decode_aggregate_receipt_20260831_instructions.md)</t>
         </is>
       </c>
     </row>
@@ -3865,14 +3865,14 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Engine: GPU cost ~60% memory / ~40% compute. TODAY (default): memory x100 + FLOPs x9.24 (blend x2.19 x equal-quality parameter ratio x4.22 at 1T) -&gt; ~20x cost-weighted (Inputs B20). CEILING: FLOPs x28.2 -&gt; ~50x (re-based 2026-08-24/25/29: x3.936 measured x x1.786 target, was a flat x5.5 assumption).</t>
+          <t>Engine: GPU cost ~60% memory / ~40% compute. RE-BASED 2026-09-01: TODAY (default): memory x100 + FLOPs x793 (full-workload serving lever — decode 2.5 ms/token x 64 streams ESTIMATE, prefill at the banked x3.936 — x equal-quality ratio x4.22 at 1T) -&gt; ~x154 cost-weighted (Inputs B20). CEILING: FLOPs x816 (prefill at the full x7.03 maturity factor = x3.936 measured x x1.786 target) -&gt; ~x154.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Floored by the least-reduced part (compute). Neither alone helps (mem-only ~2.5x, FLOP-only ~1.5x).</t>
+          <t xml:space="preserve">  Floored by the least-reduced part — at these levers that is MEMORY (/100), so the two scenarios land within rounding of each other. The pre-campaign family (x9.24 -&gt; ~20x / x28.2 -&gt; ~50x) is RETIRED 2026-09-01: measured on kernels that no longer exist.</t>
         </is>
       </c>
     </row>
@@ -3955,7 +3955,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>- Cost-weighted reduction ~20x TODAY, ~50x at the CEILING (NOT 100x; ~16-36x over memory share 45-82% at the Today lever).</t>
+          <t>- Cost-weighted reduction ~x154 TODAY and ~x154 at the CEILING — memory-floored at /100; the levers differ ~3% but the reduction ~0.3%.</t>
         </is>
       </c>
     </row>
@@ -3969,21 +3969,21 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>- With our architecture: spend cut ~$159B -&gt; burn shrinks to ~ -$136B/yr (~42% of AI spend cut).</t>
+          <t>- With our architecture: spend cut ~$166B -&gt; burn shrinks to ~ -$129B/yr (~44% of AI spend cut).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>- Spend-cut value (named floor, 6% discount rate): FY25 ~$159B/yr (~$2.6T capitalized); FY26 r/r ~$366B/yr (~$6.1T). Ceiling: ~$164B FY25.</t>
+          <t>- Spend-cut value (named floor, 6% discount rate): FY25 ~$166B/yr (~$2.8T capitalized); FY26 r/r ~$382B/yr (~$6.4T). Ceiling: within rounding of Today (the cut saturates).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>- GLOBAL estimate (named ~80% of world AI capex): FY25 ~$3.3T, FY26 ~$7.6T capitalized. Clearly an estimate.</t>
+          <t>- GLOBAL estimate (named ~80% of world AI capex): FY25 ~$3.5T, FY26 ~$8.0T capitalized. Clearly an estimate.</t>
         </is>
       </c>
     </row>
@@ -8301,7 +8301,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>TODAY scenario (default) = x9.24: the measured workload blend x2.19 (10:1 input:output, 64k context; prefill x1.17, decode x2.20 on the memory ceiling; training excluded) x the fit-derived equal-quality parameter ratio x4.22 at 1T (rows 23-25 below). Overtype with =B25 for the CEILING scenario (x28.2 = measured prefill x4.02 x 7.03 campaign speedup), or any number. See ServingTraining for the blend.</t>
+          <t>TODAY scenario (default, RE-BASED 2026-09-01) = x793: the full-workload serving lever (decode 2.5 ms/token x 64 resident streams — an ESTIMATE, aggregate-decode receipt PENDING — prefill at the BANKED x3.936 campaign speedup) x the fit-derived equal-quality parameter ratio x4.22 at 1T (rows 23-25 below). Overtype with =B25 for the CEILING scenario (x816 = same lever, prefill at the full x7.03 maturity factor), or any number. The pre-campaign x9.24 lever is RETIRED 2026-09-01 (measured on kernels that no longer exist). See ServingTraining for the measured background blend.</t>
         </is>
       </c>
     </row>
@@ -8624,7 +8624,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>SCENARIOS (2026-08-17 ruling) — TODAY (default) vs CEILING</t>
+          <t>SCENARIOS (2026-09-01 ruling) — TODAY (default) vs CEILING (campaign landed)</t>
         </is>
       </c>
       <c r="B22" s="2" t="n"/>
@@ -8654,11 +8654,11 @@
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>TODAY compute lever = blend x ratio</t>
+          <t>TODAY compute lever = serving lever x ratio</t>
         </is>
       </c>
       <c r="B24" s="29">
-        <f>ServingTraining!$B$28*$B$23</f>
+        <f>188.0305*$B$23</f>
         <v/>
       </c>
       <c r="C24" t="inlineStr">
@@ -8668,18 +8668,19 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>B3 (the FLOPs lever) points here by default.</t>
+          <t>B3 (the FLOPs lever) points here by default. The x188.0 serving half is model-computed (campaign_landed_flop_lever): decode 2.5 ms/token x 64 resident streams — an ESTIMATE, the aggregate-decode receipt is PENDING — with prefill at the BANKED x3.936 (our own step went 400.4 -&gt; 101.7 ms at B16/T2048; 2026-08-29 clean-wall position of record); transformer side stays the measured 1/context law at its KV ceiling, 128k E[context].</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CEILING compute lever</t>
-        </is>
-      </c>
-      <c r="B25" s="28" t="n">
-        <v>28.23958902252343</v>
+          <t>CEILING compute lever (campaign landed)</t>
+        </is>
+      </c>
+      <c r="B25" s="19">
+        <f>193.3376*$B$23</f>
+        <v/>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -8688,7 +8689,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Measured prefill x4.02 (bf16 parameter-matched, d512/1M, 2026-07-21) x 7.03 campaign speedup. RE-BASED 2026-08-24/25/29: that factor is x3.936 MEASURED (already banked: our own step went 400.4 -&gt; 101.7 ms at B16/T2048; 2026-08-29 clean-wall position of record) x x1.786 TARGET (the funded 8k-win gate, no receipt yet); it was a flat x5.5 assumption before. Overtype B3 with =B25 to run the workbook at the ceiling (~50x cost-weighted).</t>
+          <t>Same full-workload lever with prefill at the full x7.03 maturity factor = x3.936 MEASURED (already banked) x x1.786 TARGET (the funded 8k-win gate, no receipt yet). Decode-dominated, so it sits only ~3% above TODAY. Overtype B3 with =B25 to run the workbook at the ceiling (~x154 cost-weighted — memory-floored; dollars move within rounding).</t>
         </is>
       </c>
     </row>
@@ -8732,12 +8733,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>TODAY (~20x)</t>
+          <t>TODAY (~154x)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>CEILING (~50x)</t>
+          <t>CEILING (~154x)</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add context-sensitivity table (prefill share + levers vs E[context]) to app Sensitivity tab and xlsx; fix dict() kwarg collision in campaign_landed_flop_lever(w=...)
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -8704,7 +8704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8712,6 +8712,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8868,8 +8869,148 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>CONTEXT SENSITIVITY — prefill share of serving cost vs fleet E[context]</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>E[context]</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>TF prefill share</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Our prefill share (Today)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Today lever (x)</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Ceiling lever (x)</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Today-&gt;Ceiling gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>8k</t>
+        </is>
+      </c>
+      <c r="B14" s="27" t="n">
+        <v>0.005899250258734248</v>
+      </c>
+      <c r="C14" s="21" t="n">
+        <v>0.05208995366081766</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>50.29665229131971</v>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>51.47706163855121</v>
+      </c>
+      <c r="F14" s="21" t="n">
+        <v>0.02346894462069837</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>32k</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="n">
+        <v>0.002981160980333002</v>
+      </c>
+      <c r="C15" s="21" t="n">
+        <v>0.05196631516233694</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>200.6239377794075</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>205.3209324850361</v>
+      </c>
+      <c r="F15" s="21" t="n">
+        <v>0.02341193557267873</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>128k (pinned)</t>
+        </is>
+      </c>
+      <c r="B16" s="27" t="n">
+        <v>0.002359266800993781</v>
+      </c>
+      <c r="C16" s="21" t="n">
+        <v>0.06235575593664416</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>793.2064858179596</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>815.5945097216911</v>
+      </c>
+      <c r="F16" s="21" t="n">
+        <v>0.0282247110985796</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>256k</t>
+        </is>
+      </c>
+      <c r="B17" s="27" t="n">
+        <v>0.00230050437708008</v>
+      </c>
+      <c r="C17" s="21" t="n">
+        <v>0.08221381175542121</v>
+      </c>
+      <c r="D17" s="18" t="n">
+        <v>1552.723400990788</v>
+      </c>
+      <c r="E17" s="18" t="n">
+        <v>1611.029390134314</v>
+      </c>
+      <c r="F17" s="21" t="n">
+        <v>0.03755078921739785</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Cost = box wall-clock, not FLOPs. The transformer's decode leg is KV-bandwidth-bound (measured 1/context law) while its prefill runs near peak, so prefill is &lt;1% of its serving cost at every context — which is why the banked x3.936 prefill (TODAY) and the full x7.03 (CEILING) land within a few percent of each other. Inputs!B24/B25 quote the pinned 128k row (2026-08-31 fleet-context ruling). Static values from ai_capex_model.serving_context_sensitivity() — rebuild the workbook to refresh.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A10:E10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Totals: Net-AI-with-arch metrics for FY25/FY26/FY27 (street-est), % spend cut on FY26; xlsx FY27 static row; sidebar: E[context] default 128k, train share 35%, scenario labels Today / Ceiling: optimized kernels, caption trimmed
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -121,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,6 +138,7 @@
     <xf numFmtId="3" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -555,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -909,125 +910,125 @@
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>FY2027 (STREET-EST prediction, static)</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>-965.595802908</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>571.8114816440647</v>
+      </c>
+      <c r="G14" s="11" t="n">
+        <v>-393.7843212639353</v>
+      </c>
+      <c r="H14" s="12" t="n">
+        <v>0.4891057518312401</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>SAVINGS BREAKDOWN — the spend cut, split</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Cost-weighted reduction (Amdahl)</t>
         </is>
       </c>
-      <c r="B16" s="12">
+      <c r="B17" s="13">
         <f>Inputs!$B$20</f>
         <v/>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="8" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Saved OPEX</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Avoided CAPEX (Overspend)</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>FY2025 annual ($B/yr)</t>
         </is>
       </c>
-      <c r="B19" s="5">
+      <c r="B20" s="5">
         <f>SUM(Microsoft!B26,Alphabet!B26,Amazon!B26,Meta!B26,Oracle!B26,SpaceX!B26)/1000</f>
         <v/>
       </c>
-      <c r="C19" s="5">
+      <c r="C20" s="5">
         <f>SUM(Microsoft!B25,Alphabet!B25,Amazon!B25,Meta!B25,Oracle!B25,SpaceX!B25)</f>
         <v/>
       </c>
-      <c r="D19" s="5">
-        <f>B19+C19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="D20" s="5">
+        <f>B20+C20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>FY2025 capitalized ($B)</t>
         </is>
       </c>
-      <c r="B20" s="13">
-        <f>B19/Inputs!$B$6</f>
-        <v/>
-      </c>
-      <c r="C20" s="13">
-        <f>C19/Inputs!$B$6</f>
-        <v/>
-      </c>
-      <c r="D20" s="13">
-        <f>B20+C20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="B21" s="14">
+        <f>B20/Inputs!$B$6</f>
+        <v/>
+      </c>
+      <c r="C21" s="14">
+        <f>C20/Inputs!$B$6</f>
+        <v/>
+      </c>
+      <c r="D21" s="14">
+        <f>B21+C21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>FY2026 annual ($B/yr)</t>
         </is>
       </c>
-      <c r="B21" s="5">
+      <c r="B22" s="5">
         <f>SUM(Microsoft!C26,Alphabet!C26,Amazon!C26,Meta!C26,Oracle!C26,SpaceX!C26)/1000</f>
         <v/>
       </c>
-      <c r="C21" s="5">
+      <c r="C22" s="5">
         <f>SUM(Microsoft!C25,Alphabet!C25,Amazon!C25,Meta!C25,Oracle!C25,SpaceX!C25)</f>
         <v/>
       </c>
-      <c r="D21" s="5">
-        <f>B21+C21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>FY2026 capitalized ($B)</t>
-        </is>
-      </c>
-      <c r="B22" s="13">
-        <f>B21/Inputs!$B$6</f>
-        <v/>
-      </c>
-      <c r="C22" s="13">
-        <f>C21/Inputs!$B$6</f>
-        <v/>
-      </c>
-      <c r="D22" s="13">
+      <c r="D22" s="5">
         <f>B22+C22</f>
         <v/>
       </c>
@@ -1035,133 +1036,152 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
+          <t>FY2026 capitalized ($B)</t>
+        </is>
+      </c>
+      <c r="B23" s="14">
+        <f>B22/Inputs!$B$6</f>
+        <v/>
+      </c>
+      <c r="C23" s="14">
+        <f>C22/Inputs!$B$6</f>
+        <v/>
+      </c>
+      <c r="D23" s="14">
+        <f>B23+C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
           <t>GLOBAL capitalized -- est. ($B)</t>
         </is>
       </c>
-      <c r="B23" s="13">
-        <f>D20/Inputs!$B$14</f>
-        <v/>
-      </c>
-      <c r="C23" s="13">
-        <f>D22/Inputs!$B$14</f>
-        <v/>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="B24" s="14">
+        <f>D21/Inputs!$B$14</f>
+        <v/>
+      </c>
+      <c r="C24" s="14">
+        <f>D23/Inputs!$B$14</f>
+        <v/>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>named-floor capitalized / named-share-of-global (Inputs B14). ESTIMATE: grosses up for other clouds, China, neoclouds, xAI, sovereign.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>% reduction</t>
         </is>
       </c>
-      <c r="B24" s="7">
+      <c r="B25" s="7">
         <f>1-1/Inputs!$B$5</f>
         <v/>
       </c>
-      <c r="C24" s="7">
+      <c r="C25" s="7">
         <f>1-1/Inputs!$B$20</f>
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>OPEX = power saved each year (recoupable). CAPEX 'Overspend' = AI capex made unnecessary. TOGGLE: Inputs 'Datacenter scaling factor' (0 = accelerator-only/conservative; 1 = whole datacenter scales with the smaller fleet). At 0 the burn ~halves; at ~0.7 net AI hits breakeven; at 1 it flips positive. Capitalized = annual / discount rate.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>TABS</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>Microsoft / Alphabet / Amazon / Meta / Oracle / SpaceX</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>one tab each: full build capex -&gt; infra -&gt; servers -&gt; accelerator -&gt; fleet/opex -&gt; value</t>
-        </is>
-      </c>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Inputs</t>
+          <t>Microsoft / Alphabet / Amazon / Meta / Oracle / SpaceX</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>global assumptions + the reduction engine (cost-weighted factor)</t>
+          <t>one tab each: full build capex -&gt; infra -&gt; servers -&gt; accelerator -&gt; fleet/opex -&gt; value</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>Sensitivity</t>
+          <t>Inputs</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>SpaceX value across reduction tiers (10x/30x/100x/cost-weighted)</t>
+          <t>global assumptions + the reduction engine (cost-weighted factor)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>CostLadder</t>
+          <t>Sensitivity</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>own-silicon vs buy-NVIDIA vs rent $/GPU-hr</t>
+          <t>SpaceX value across reduction tiers (10x/30x/100x/cost-weighted)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>Evidence</t>
+          <t>CostLadder</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>BOM cost split, accelerator-share data, own-silicon TCO, filing top-lines</t>
+          <t>own-silicon vs buy-NVIDIA vs rent $/GPU-hr</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>BOM cost split, accelerator-share data, own-silicon TCO, filing top-lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
           <t>Methodology</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>step-by-step logic, caveats, sources</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>Legend: yellow = assumption / lever (each maps to a slider in the Streamlit app)  ·  green = disclosed filing or market data  ·  blue = derived formula.</t>
         </is>
@@ -1169,15 +1189,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="B32:H32"/>
-    <mergeCell ref="A35:H35"/>
-    <mergeCell ref="A25:H25"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B31:H31"/>
     <mergeCell ref="B30:H30"/>
+    <mergeCell ref="A36:H36"/>
     <mergeCell ref="B29:H29"/>
     <mergeCell ref="B33:H33"/>
-    <mergeCell ref="B28:H28"/>
+    <mergeCell ref="B34:H34"/>
+    <mergeCell ref="B31:H31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1236,10 +1256,10 @@
           <t>Own custom silicon (TPU/Trainium)</t>
         </is>
       </c>
-      <c r="B3" s="30" t="n">
+      <c r="B3" s="31" t="n">
         <v>0.9</v>
       </c>
-      <c r="C3" s="30" t="n">
+      <c r="C3" s="31" t="n">
         <v>1.4</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1254,10 +1274,10 @@
           <t>Buy + operate NVIDIA (scale)</t>
         </is>
       </c>
-      <c r="B4" s="30" t="n">
+      <c r="B4" s="31" t="n">
         <v>1.5</v>
       </c>
-      <c r="C4" s="30" t="n">
+      <c r="C4" s="31" t="n">
         <v>2</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1272,10 +1292,10 @@
           <t>Rent NVIDIA - neocloud / committed</t>
         </is>
       </c>
-      <c r="B5" s="30" t="n">
+      <c r="B5" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="30" t="n">
+      <c r="C5" s="31" t="n">
         <v>3.5</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1290,10 +1310,10 @@
           <t>Rent NVIDIA - hyperscaler on-demand</t>
         </is>
       </c>
-      <c r="B6" s="30" t="n">
+      <c r="B6" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="C6" s="30" t="n">
+      <c r="C6" s="31" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -1318,7 +1338,7 @@
           <t>Utilization</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="17" t="n">
         <v>0.85</v>
       </c>
     </row>
@@ -1328,7 +1348,7 @@
           <t>Capex $/hr</t>
         </is>
       </c>
-      <c r="B10" s="19">
+      <c r="B10" s="20">
         <f>Inputs!$B$7/(Inputs!$B$11*8760*B9)</f>
         <v/>
       </c>
@@ -1344,7 +1364,7 @@
           <t>Power $/hr</t>
         </is>
       </c>
-      <c r="B11" s="19">
+      <c r="B11" s="20">
         <f>Inputs!$B$8*Inputs!$B$9</f>
         <v/>
       </c>
@@ -1360,7 +1380,7 @@
           <t>DC/staff adder $/hr</t>
         </is>
       </c>
-      <c r="B12" s="28" t="n">
+      <c r="B12" s="29" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -1370,7 +1390,7 @@
           <t>Owned TCO $/hr</t>
         </is>
       </c>
-      <c r="B13" s="29">
+      <c r="B13" s="30">
         <f>B10+B11+B12</f>
         <v/>
       </c>
@@ -1481,7 +1501,7 @@
           <t>Input : output token ratio</t>
         </is>
       </c>
-      <c r="B7" s="23" t="n">
+      <c r="B7" s="24" t="n">
         <v>10</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1496,7 +1516,7 @@
           <t>E[context] (tokens)</t>
         </is>
       </c>
-      <c r="B8" s="25" t="n">
+      <c r="B8" s="26" t="n">
         <v>65536</v>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -1511,7 +1531,7 @@
           <t>Training share of accelerator cost</t>
         </is>
       </c>
-      <c r="B9" s="28" t="n">
+      <c r="B9" s="29" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -1533,7 +1553,7 @@
           <t>Owned decode, tokens/s/box (context-flat)</t>
         </is>
       </c>
-      <c r="B12" s="17" t="n">
+      <c r="B12" s="18" t="n">
         <v>4496.668604837461</v>
       </c>
     </row>
@@ -1543,7 +1563,7 @@
           <t>KV MB per token per stream</t>
         </is>
       </c>
-      <c r="B13" s="31" t="n">
+      <c r="B13" s="32" t="n">
         <v>0.15234375</v>
       </c>
     </row>
@@ -1553,7 +1573,7 @@
           <t>HBM TB/s per GPU</t>
         </is>
       </c>
-      <c r="B14" s="28" t="n">
+      <c r="B14" s="29" t="n">
         <v>3.35</v>
       </c>
     </row>
@@ -1563,7 +1583,7 @@
           <t>Transformer KV compression (mature stack)</t>
         </is>
       </c>
-      <c r="B15" s="23" t="n">
+      <c r="B15" s="24" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1573,7 +1593,7 @@
           <t>GPUs per box</t>
         </is>
       </c>
-      <c r="B16" s="32" t="n">
+      <c r="B16" s="33" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1583,7 +1603,7 @@
           <t>Training advantage, short sequence (owned / transformer)</t>
         </is>
       </c>
-      <c r="B17" s="33" t="n">
+      <c r="B17" s="34" t="n">
         <v>0.5825609168739003</v>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1605,7 +1625,7 @@
           <t>KV GB per stream</t>
         </is>
       </c>
-      <c r="B20" s="19">
+      <c r="B20" s="20">
         <f>$B$8*$B$13/1024</f>
         <v/>
       </c>
@@ -1616,7 +1636,7 @@
           <t>KV GB per stream, compressed</t>
         </is>
       </c>
-      <c r="B21" s="34">
+      <c r="B21" s="35">
         <f>$B$20/$B$15</f>
         <v/>
       </c>
@@ -1627,7 +1647,7 @@
           <t>Transformer decode, tokens/s/box</t>
         </is>
       </c>
-      <c r="B22" s="18">
+      <c r="B22" s="19">
         <f>511.8416*32768/$B$8*$B$15*$B$16</f>
         <v/>
       </c>
@@ -1643,7 +1663,7 @@
           <t>Prefill table row (lookup)</t>
         </is>
       </c>
-      <c r="B23" s="35">
+      <c r="B23" s="36">
         <f>MATCH($B$8,$A$33:$A$39,1)</f>
         <v/>
       </c>
@@ -1654,7 +1674,7 @@
           <t>Prefill tokens/s/box — transformer</t>
         </is>
       </c>
-      <c r="B24" s="18">
+      <c r="B24" s="19">
         <f>IF(INDEX($B$33:$B$39,MIN($B$23+1,7))=INDEX($B$33:$B$39,$B$23),INDEX($B$33:$B$39,$B$23),EXP(LN(INDEX($B$33:$B$39,$B$23))+(LN($B$8)-LN(INDEX($A$33:$A$39,$B$23)))/(LN(INDEX($A$33:$A$39,MIN($B$23+1,7)))-LN(INDEX($A$33:$A$39,$B$23)))*(LN(INDEX($B$33:$B$39,MIN($B$23+1,7)))-LN(INDEX($B$33:$B$39,$B$23)))))*$B$16</f>
         <v/>
       </c>
@@ -1665,7 +1685,7 @@
           <t>Prefill tokens/s/box — owned</t>
         </is>
       </c>
-      <c r="B25" s="18">
+      <c r="B25" s="19">
         <f>IF(INDEX($C$33:$C$39,MIN($B$23+1,7))=INDEX($C$33:$C$39,$B$23),INDEX($C$33:$C$39,$B$23),EXP(LN(INDEX($C$33:$C$39,$B$23))+(LN($B$8)-LN(INDEX($A$33:$A$39,$B$23)))/(LN(INDEX($A$33:$A$39,MIN($B$23+1,7)))-LN(INDEX($A$33:$A$39,$B$23)))*(LN(INDEX($C$33:$C$39,MIN($B$23+1,7)))-LN(INDEX($C$33:$C$39,$B$23)))))*$B$16</f>
         <v/>
       </c>
@@ -1676,7 +1696,7 @@
           <t>Transformer seconds per generated token</t>
         </is>
       </c>
-      <c r="B26" s="36">
+      <c r="B26" s="37">
         <f>$B$7/$B$24+1/$B$22</f>
         <v/>
       </c>
@@ -1687,7 +1707,7 @@
           <t>Owned seconds per generated token</t>
         </is>
       </c>
-      <c r="B27" s="36">
+      <c r="B27" s="37">
         <f>$B$7/$B$25+1/$B$12</f>
         <v/>
       </c>
@@ -1698,7 +1718,7 @@
           <t>BLENDED COMPUTE LEVER (flop_factor)</t>
         </is>
       </c>
-      <c r="B28" s="29">
+      <c r="B28" s="30">
         <f>IF($B$9&gt;0,1/($B$9/$B$17+(1-$B$9)/($B$26/$B$27)),$B$26/$B$27)</f>
         <v/>
       </c>
@@ -1714,7 +1734,7 @@
           <t xml:space="preserve">  of which: prefill advantage</t>
         </is>
       </c>
-      <c r="B29" s="19">
+      <c r="B29" s="20">
         <f>($B$7/$B$24)/($B$7/$B$25)</f>
         <v/>
       </c>
@@ -1725,7 +1745,7 @@
           <t xml:space="preserve">  of which: decode advantage</t>
         </is>
       </c>
-      <c r="B30" s="37">
+      <c r="B30" s="38">
         <f>(1/$B$22)/(1/$B$12)</f>
         <v/>
       </c>
@@ -1736,96 +1756,96 @@
           <t>Measured prefill throughput, tokens/s/GPU (bf16 saturated lane, d2048)</t>
         </is>
       </c>
-      <c r="D32" s="38" t="inlineStr">
+      <c r="D32" s="39" t="inlineStr">
         <is>
           <t>Context</t>
         </is>
       </c>
-      <c r="E32" s="38" t="inlineStr">
+      <c r="E32" s="39" t="inlineStr">
         <is>
           <t>Transformer</t>
         </is>
       </c>
-      <c r="F32" s="38" t="inlineStr">
+      <c r="F32" s="39" t="inlineStr">
         <is>
           <t>Owned</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="39" t="n">
+      <c r="A33" s="40" t="n">
         <v>2048</v>
       </c>
-      <c r="B33" s="17" t="n">
+      <c r="B33" s="18" t="n">
         <v>4682606.88285999</v>
       </c>
-      <c r="C33" s="17" t="n">
+      <c r="C33" s="18" t="n">
         <v>1185825</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="39" t="n">
+      <c r="A34" s="40" t="n">
         <v>8192</v>
       </c>
-      <c r="B34" s="17" t="n">
+      <c r="B34" s="18" t="n">
         <v>3450080</v>
       </c>
-      <c r="C34" s="17" t="n">
+      <c r="C34" s="18" t="n">
         <v>1183690</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="39" t="n">
+      <c r="A35" s="40" t="n">
         <v>32768</v>
       </c>
-      <c r="B35" s="17" t="n">
+      <c r="B35" s="18" t="n">
         <v>1711802</v>
       </c>
-      <c r="C35" s="17" t="n">
+      <c r="C35" s="18" t="n">
         <v>1186661</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="39" t="n">
+      <c r="A36" s="40" t="n">
         <v>65536</v>
       </c>
-      <c r="B36" s="17" t="n">
+      <c r="B36" s="18" t="n">
         <v>1007187</v>
       </c>
-      <c r="C36" s="17" t="n">
+      <c r="C36" s="18" t="n">
         <v>1181622</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="39" t="n">
+      <c r="A37" s="40" t="n">
         <v>131072</v>
       </c>
-      <c r="B37" s="17" t="n">
+      <c r="B37" s="18" t="n">
         <v>541094</v>
       </c>
-      <c r="C37" s="17" t="n">
+      <c r="C37" s="18" t="n">
         <v>978107</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="39" t="n">
+      <c r="A38" s="40" t="n">
         <v>262144</v>
       </c>
-      <c r="B38" s="17" t="n">
+      <c r="B38" s="18" t="n">
         <v>277474</v>
       </c>
-      <c r="C38" s="17" t="n">
+      <c r="C38" s="18" t="n">
         <v>726142</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="39" t="n">
+      <c r="A39" s="40" t="n">
         <v>524288</v>
       </c>
-      <c r="B39" s="17" t="n">
+      <c r="B39" s="18" t="n">
         <v>140820</v>
       </c>
-      <c r="C39" s="17" t="n">
+      <c r="C39" s="18" t="n">
         <v>478522</v>
       </c>
     </row>
@@ -1849,166 +1869,166 @@
       <c r="F43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="38" t="inlineStr">
+      <c r="A44" s="39" t="inlineStr">
         <is>
           <t>Context (tokens)</t>
         </is>
       </c>
-      <c r="B44" s="38" t="inlineStr">
+      <c r="B44" s="39" t="inlineStr">
         <is>
           <t>bAttention $/1M tok</t>
         </is>
       </c>
-      <c r="C44" s="38" t="inlineStr">
+      <c r="C44" s="39" t="inlineStr">
         <is>
           <t>Transformer $/1M tok (mature stack)</t>
         </is>
       </c>
-      <c r="D44" s="38" t="inlineStr">
+      <c r="D44" s="39" t="inlineStr">
         <is>
           <t>TF streams/GPU</t>
         </is>
       </c>
-      <c r="E44" s="38" t="inlineStr">
+      <c r="E44" s="39" t="inlineStr">
         <is>
           <t>Cost ratio</t>
         </is>
       </c>
-      <c r="F44" s="38" t="inlineStr">
+      <c r="F44" s="39" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="39" t="n">
+      <c r="A45" s="40" t="n">
         <v>4096</v>
       </c>
-      <c r="B45" s="40" t="n">
+      <c r="B45" s="41" t="n">
         <v>1.235482541359387</v>
       </c>
-      <c r="C45" s="41" t="n">
+      <c r="C45" s="42" t="n">
         <v>0.1695945640120853</v>
       </c>
-      <c r="D45" s="35" t="n">
+      <c r="D45" s="36" t="n">
         <v>118</v>
       </c>
-      <c r="E45" s="42" t="n">
+      <c r="E45" s="43" t="n">
         <v>0.1372698992779634</v>
       </c>
-      <c r="F45" s="43" t="inlineStr"/>
+      <c r="F45" s="44" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="39" t="n">
+      <c r="A46" s="40" t="n">
         <v>16384</v>
       </c>
-      <c r="B46" s="40" t="n">
+      <c r="B46" s="41" t="n">
         <v>1.235482541359387</v>
       </c>
-      <c r="C46" s="41" t="n">
+      <c r="C46" s="42" t="n">
         <v>0.678378256048341</v>
       </c>
-      <c r="D46" s="35" t="n">
+      <c r="D46" s="36" t="n">
         <v>29</v>
       </c>
-      <c r="E46" s="42" t="n">
+      <c r="E46" s="43" t="n">
         <v>0.5490795971118535</v>
       </c>
-      <c r="F46" s="43" t="inlineStr"/>
+      <c r="F46" s="44" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="39" t="n">
+      <c r="A47" s="40" t="n">
         <v>32768</v>
       </c>
-      <c r="B47" s="40" t="n">
+      <c r="B47" s="41" t="n">
         <v>1.235482541359387</v>
       </c>
-      <c r="C47" s="41" t="n">
+      <c r="C47" s="42" t="n">
         <v>1.356756512096682</v>
       </c>
-      <c r="D47" s="35" t="n">
+      <c r="D47" s="36" t="n">
         <v>14</v>
       </c>
-      <c r="E47" s="42" t="n">
+      <c r="E47" s="43" t="n">
         <v>1.098159194223707</v>
       </c>
-      <c r="F47" s="43" t="inlineStr"/>
+      <c r="F47" s="44" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="39" t="n">
+      <c r="A48" s="40" t="n">
         <v>65536</v>
       </c>
-      <c r="B48" s="40" t="n">
+      <c r="B48" s="41" t="n">
         <v>1.235482541359387</v>
       </c>
-      <c r="C48" s="41" t="n">
+      <c r="C48" s="42" t="n">
         <v>2.713513024193364</v>
       </c>
-      <c r="D48" s="35" t="n">
+      <c r="D48" s="36" t="n">
         <v>7</v>
       </c>
-      <c r="E48" s="42" t="n">
+      <c r="E48" s="43" t="n">
         <v>2.196318388447414</v>
       </c>
-      <c r="F48" s="43" t="inlineStr"/>
+      <c r="F48" s="44" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="39" t="n">
+      <c r="A49" s="40" t="n">
         <v>131072</v>
       </c>
-      <c r="B49" s="40" t="n">
+      <c r="B49" s="41" t="n">
         <v>1.235482541359387</v>
       </c>
-      <c r="C49" s="41" t="n">
+      <c r="C49" s="42" t="n">
         <v>5.427026048386728</v>
       </c>
-      <c r="D49" s="35" t="n">
+      <c r="D49" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="E49" s="42" t="n">
+      <c r="E49" s="43" t="n">
         <v>4.392636776894828</v>
       </c>
-      <c r="F49" s="43" t="inlineStr"/>
+      <c r="F49" s="44" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="39" t="n">
+      <c r="A50" s="40" t="n">
         <v>262144</v>
       </c>
-      <c r="B50" s="40" t="n">
+      <c r="B50" s="41" t="n">
         <v>1.235482541359387</v>
       </c>
-      <c r="C50" s="41" t="n">
+      <c r="C50" s="42" t="n">
         <v>10.85405209677346</v>
       </c>
-      <c r="D50" s="35" t="n">
+      <c r="D50" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="E50" s="42" t="n">
+      <c r="E50" s="43" t="n">
         <v>8.785273553789656</v>
       </c>
-      <c r="F50" s="43" t="inlineStr">
+      <c r="F50" s="44" t="inlineStr">
         <is>
           <t>a measured decode cell (64 streams/GPU against the transformer 1)</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="39" t="n">
+      <c r="A51" s="40" t="n">
         <v>1048576</v>
       </c>
-      <c r="B51" s="44" t="n">
+      <c r="B51" s="45" t="n">
         <v>1.235482541359387</v>
       </c>
-      <c r="C51" s="41" t="n">
-        <v/>
-      </c>
-      <c r="D51" s="35" t="n">
+      <c r="C51" s="42" t="n">
+        <v/>
+      </c>
+      <c r="D51" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="E51" s="42" t="n">
-        <v/>
-      </c>
-      <c r="F51" s="43" t="inlineStr">
+      <c r="E51" s="43" t="n">
+        <v/>
+      </c>
+      <c r="F51" s="44" t="inlineStr">
         <is>
           <t>bAttention rate extrapolated past 262k (flatness measured 4k-262k)</t>
         </is>
@@ -2034,180 +2054,180 @@
       <c r="F54" s="2" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="38" t="inlineStr">
+      <c r="A55" s="39" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B55" s="38" t="inlineStr">
+      <c r="B55" s="39" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C55" s="38" t="inlineStr">
+      <c r="C55" s="39" t="inlineStr">
         <is>
           <t>Ratio / consequence</t>
         </is>
       </c>
-      <c r="D55" s="38" t="inlineStr"/>
-      <c r="E55" s="38" t="inlineStr"/>
-      <c r="F55" s="38" t="inlineStr">
+      <c r="D55" s="39" t="inlineStr"/>
+      <c r="E55" s="39" t="inlineStr"/>
+      <c r="F55" s="39" t="inlineStr">
         <is>
           <t>Status — derived.json key</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="45" t="inlineStr">
+      <c r="A56" s="46" t="inlineStr">
         <is>
           <t>8-GPU speedup, matched load (16 in flight)</t>
         </is>
       </c>
-      <c r="B56" s="46" t="inlineStr">
+      <c r="B56" s="47" t="inlineStr">
         <is>
           <t>x5.15 fwd+bwd vs x3.70 fwd-only Ulysses best</t>
         </is>
       </c>
-      <c r="C56" s="47" t="inlineStr">
+      <c r="C56" s="48" t="inlineStr">
         <is>
           <t>x1.39 cluster throughput</t>
         </is>
       </c>
-      <c r="F56" s="43" t="inlineStr">
+      <c r="F56" s="44" t="inlineStr">
         <is>
           <t>MEASURED — matched_load_curve</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="45" t="inlineStr">
+      <c r="A57" s="46" t="inlineStr">
         <is>
           <t>8-GPU speedup, deep load (256 in flight)</t>
         </is>
       </c>
-      <c r="B57" s="46" t="inlineStr">
+      <c r="B57" s="47" t="inlineStr">
         <is>
           <t>x6.27 (pipeline keeps filling; TF saturated by 16)</t>
         </is>
       </c>
-      <c r="C57" s="47" t="inlineStr">
+      <c r="C57" s="48" t="inlineStr">
         <is>
           <t>x1.70</t>
         </is>
       </c>
-      <c r="F57" s="43" t="inlineStr">
+      <c r="F57" s="44" t="inlineStr">
         <is>
           <t>MEASURED — scaling_1to8_best</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="45" t="inlineStr">
+      <c r="A58" s="46" t="inlineStr">
         <is>
           <t>GPU-hours for the same training work</t>
         </is>
       </c>
-      <c r="B58" s="48" t="inlineStr">
+      <c r="B58" s="49" t="inlineStr">
         <is>
           <t>-28% (matched) … -41% (deep)</t>
         </is>
       </c>
-      <c r="C58" s="45" t="inlineStr"/>
-      <c r="F58" s="43" t="inlineStr">
+      <c r="C58" s="46" t="inlineStr"/>
+      <c r="F58" s="44" t="inlineStr">
         <is>
           <t>derived</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="45" t="inlineStr">
+      <c r="A59" s="46" t="inlineStr">
         <is>
           <t>64k-token sequence on one 80 GB GPU</t>
         </is>
       </c>
-      <c r="B59" s="46" t="inlineStr">
+      <c r="B59" s="47" t="inlineStr">
         <is>
           <t>30.9 GB fits vs OOM (78.4 GB attempted)</t>
         </is>
       </c>
-      <c r="C59" s="45" t="inlineStr"/>
-      <c r="F59" s="43" t="inlineStr">
+      <c r="C59" s="46" t="inlineStr"/>
+      <c r="F59" s="44" t="inlineStr">
         <is>
           <t>MEASURED — pipeline_feasibility</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="45" t="inlineStr">
+      <c r="A60" s="46" t="inlineStr">
         <is>
           <t>Pipeline per-GPU peak (flat in load)</t>
         </is>
       </c>
-      <c r="B60" s="46" t="inlineStr">
+      <c r="B60" s="47" t="inlineStr">
         <is>
           <t>9.05 GB vs 43.3 GB GPipe stage</t>
         </is>
       </c>
-      <c r="C60" s="47" t="inlineStr">
+      <c r="C60" s="48" t="inlineStr">
         <is>
           <t>x4.8 (component-scope, width-unmatched)</t>
         </is>
       </c>
-      <c r="F60" s="43" t="inlineStr">
+      <c r="F60" s="44" t="inlineStr">
         <is>
           <t>MEASURED — pipeline_memory_asymmetry</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="45" t="inlineStr">
+      <c r="A61" s="46" t="inlineStr">
         <is>
           <t>Params for equal quality at 70B</t>
         </is>
       </c>
-      <c r="B61" s="49" t="inlineStr">
+      <c r="B61" s="50" t="inlineStr">
         <is>
           <t>x4.1 [2.2-7.7] transformer</t>
         </is>
       </c>
-      <c r="C61" s="45" t="inlineStr"/>
-      <c r="F61" s="43" t="inlineStr">
+      <c r="C61" s="46" t="inlineStr"/>
+      <c r="F61" s="44" t="inlineStr">
         <is>
           <t>PROJECTION — quality_fit.ref_70B</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="45" t="inlineStr">
+      <c r="A62" s="46" t="inlineStr">
         <is>
           <t>Tokens for equal quality at 70B</t>
         </is>
       </c>
-      <c r="B62" s="49" t="inlineStr">
+      <c r="B62" s="50" t="inlineStr">
         <is>
           <t>x1.68 [1.33-2.10] (beta=0.28 assumption)</t>
         </is>
       </c>
-      <c r="C62" s="45" t="inlineStr"/>
-      <c r="F62" s="43" t="inlineStr">
+      <c r="C62" s="46" t="inlineStr"/>
+      <c r="F62" s="44" t="inlineStr">
         <is>
           <t>PROJECTION — quality_fit.ref_70B</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="45" t="inlineStr">
+      <c r="A63" s="46" t="inlineStr">
         <is>
           <t>Stepped vs scanned training</t>
         </is>
       </c>
-      <c r="B63" s="46" t="inlineStr">
+      <c r="B63" s="47" t="inlineStr">
         <is>
           <t>x24 cost to step the recurrence token-by-token</t>
         </is>
       </c>
-      <c r="C63" s="45" t="inlineStr"/>
-      <c r="F63" s="43" t="inlineStr">
+      <c r="C63" s="46" t="inlineStr"/>
+      <c r="F63" s="44" t="inlineStr">
         <is>
           <t>MEASURED — stepped_vs_scanned</t>
         </is>
@@ -2252,172 +2272,172 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="38" t="inlineStr">
+      <c r="A71" s="39" t="inlineStr">
         <is>
           <t>Transformer params</t>
         </is>
       </c>
-      <c r="B71" s="38" t="inlineStr">
+      <c r="B71" s="39" t="inlineStr">
         <is>
           <t>s(N) fit</t>
         </is>
       </c>
-      <c r="C71" s="38" t="inlineStr">
+      <c r="C71" s="39" t="inlineStr">
         <is>
           <t>Chinchilla 2k</t>
         </is>
       </c>
-      <c r="D71" s="38" t="inlineStr">
+      <c r="D71" s="39" t="inlineStr">
         <is>
           <t>Chinchilla 8k</t>
         </is>
       </c>
-      <c r="E71" s="38" t="inlineStr">
+      <c r="E71" s="39" t="inlineStr">
         <is>
           <t>Chinchilla 32k</t>
         </is>
       </c>
-      <c r="F71" s="38" t="inlineStr">
+      <c r="F71" s="39" t="inlineStr">
         <is>
           <t>Chinchilla 256k*</t>
         </is>
       </c>
-      <c r="G71" s="38" t="inlineStr">
+      <c r="G71" s="39" t="inlineStr">
         <is>
           <t>Fixed-D 2k / 8k / 32k / 256k*</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="45" t="inlineStr">
+      <c r="A72" s="46" t="inlineStr">
         <is>
           <t>1B</t>
         </is>
       </c>
-      <c r="B72" s="28" t="n">
+      <c r="B72" s="29" t="n">
         <v>1.187536580013817</v>
       </c>
-      <c r="C72" s="19" t="n">
+      <c r="C72" s="20" t="n">
         <v>0.8215525301701575</v>
       </c>
-      <c r="D72" s="19" t="n">
+      <c r="D72" s="20" t="n">
         <v>1.151570796996963</v>
       </c>
-      <c r="E72" s="19" t="n">
+      <c r="E72" s="20" t="n">
         <v>2.471643864304184</v>
       </c>
-      <c r="F72" s="19" t="n">
+      <c r="F72" s="20" t="n">
         <v>14.79232582583825</v>
       </c>
-      <c r="G72" s="47" t="inlineStr">
+      <c r="G72" s="48" t="inlineStr">
         <is>
           <t>0.69 / 0.97 / 2.08 / 12.46</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="45" t="inlineStr">
+      <c r="A73" s="46" t="inlineStr">
         <is>
           <t>10B</t>
         </is>
       </c>
-      <c r="B73" s="28" t="n">
+      <c r="B73" s="29" t="n">
         <v>1.811968550196262</v>
       </c>
-      <c r="C73" s="19" t="n">
+      <c r="C73" s="20" t="n">
         <v>1.912681494778985</v>
       </c>
-      <c r="D73" s="19" t="n">
+      <c r="D73" s="20" t="n">
         <v>2.681007084096966</v>
       </c>
-      <c r="E73" s="19" t="n">
+      <c r="E73" s="20" t="n">
         <v>5.754309441368888</v>
       </c>
-      <c r="F73" s="19" t="n">
+      <c r="F73" s="20" t="n">
         <v>34.43846477590683</v>
       </c>
-      <c r="G73" s="47" t="inlineStr">
+      <c r="G73" s="48" t="inlineStr">
         <is>
           <t>1.06 / 1.48 / 3.18 / 19.01</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="45" t="inlineStr">
+      <c r="A74" s="46" t="inlineStr">
         <is>
           <t>100B</t>
         </is>
       </c>
-      <c r="B74" s="28" t="n">
+      <c r="B74" s="29" t="n">
         <v>2.764740120141925</v>
       </c>
-      <c r="C74" s="19" t="n">
+      <c r="C74" s="20" t="n">
         <v>4.452972106010361</v>
       </c>
-      <c r="D74" s="19" t="n">
+      <c r="D74" s="20" t="n">
         <v>6.241734336892029</v>
       </c>
-      <c r="E74" s="19" t="n">
+      <c r="E74" s="20" t="n">
         <v>13.3967832604187</v>
       </c>
-      <c r="F74" s="19" t="n">
+      <c r="F74" s="20" t="n">
         <v>80.17723988000094</v>
       </c>
-      <c r="G74" s="47" t="inlineStr">
+      <c r="G74" s="48" t="inlineStr">
         <is>
           <t>1.61 / 2.26 / 4.85 / 29.00</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="45" t="inlineStr">
+      <c r="A75" s="46" t="inlineStr">
         <is>
           <t>1T</t>
         </is>
       </c>
-      <c r="B75" s="28" t="n">
+      <c r="B75" s="29" t="n">
         <v>4.21849922897088</v>
       </c>
-      <c r="C75" s="19" t="n">
+      <c r="C75" s="20" t="n">
         <v>10.36710013195259</v>
       </c>
-      <c r="D75" s="19" t="n">
+      <c r="D75" s="20" t="n">
         <v>14.53157202136217</v>
       </c>
-      <c r="E75" s="19" t="n">
+      <c r="E75" s="20" t="n">
         <v>31.1894595790005</v>
       </c>
-      <c r="F75" s="19" t="n">
+      <c r="F75" s="20" t="n">
         <v>186.6630767836249</v>
       </c>
-      <c r="G75" s="47" t="inlineStr">
+      <c r="G75" s="48" t="inlineStr">
         <is>
           <t>2.46 / 3.44 / 7.39 / 44.25</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="45" t="inlineStr">
+      <c r="A76" s="46" t="inlineStr">
         <is>
           <t>10T</t>
         </is>
       </c>
-      <c r="B76" s="28" t="n">
+      <c r="B76" s="29" t="n">
         <v>6.436675771144228</v>
       </c>
-      <c r="C76" s="19" t="n">
+      <c r="C76" s="20" t="n">
         <v>24.13596191201503</v>
       </c>
-      <c r="D76" s="19" t="n">
+      <c r="D76" s="20" t="n">
         <v>33.83139589327395</v>
       </c>
-      <c r="E76" s="19" t="n">
+      <c r="E76" s="20" t="n">
         <v>72.61313181830963</v>
       </c>
-      <c r="F76" s="19" t="n">
+      <c r="F76" s="20" t="n">
         <v>434.576000451976</v>
       </c>
-      <c r="G76" s="47" t="inlineStr">
+      <c r="G76" s="48" t="inlineStr">
         <is>
           <t>3.75 / 5.26 / 11.28 / 67.52</t>
         </is>
@@ -2431,153 +2451,153 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="38" t="inlineStr">
+      <c r="A80" s="39" t="inlineStr">
         <is>
           <t>Training curriculum</t>
         </is>
       </c>
-      <c r="B80" s="38" t="inlineStr">
+      <c r="B80" s="39" t="inlineStr">
         <is>
           <t>Advantage (TF / ours)</t>
         </is>
       </c>
-      <c r="C80" s="38" t="inlineStr">
+      <c r="C80" s="39" t="inlineStr">
         <is>
           <t>Effective r</t>
         </is>
       </c>
-      <c r="D80" s="38" t="inlineStr">
+      <c r="D80" s="39" t="inlineStr">
         <is>
           <t>Mix: token share -&gt; transformer cost share</t>
         </is>
       </c>
-      <c r="E80" s="38" t="inlineStr">
+      <c r="E80" s="39" t="inlineStr">
         <is>
           <t>FY25 cut @ 20% training</t>
         </is>
       </c>
-      <c r="F80" s="38" t="inlineStr">
+      <c r="F80" s="39" t="inlineStr">
         <is>
           <t>vs serving-only</t>
         </is>
       </c>
-      <c r="G80" s="38" t="inlineStr">
+      <c r="G80" s="39" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="45" t="inlineStr">
+      <c r="A81" s="46" t="inlineStr">
         <is>
           <t>Legacy short (all training at 2k)</t>
         </is>
       </c>
-      <c r="B81" s="50" t="n">
+      <c r="B81" s="51" t="n">
         <v>0.5825609168739004</v>
       </c>
-      <c r="C81" s="51" t="n">
+      <c r="C81" s="52" t="n">
         <v>1.716558682594317</v>
       </c>
-      <c r="D81" s="43" t="inlineStr">
+      <c r="D81" s="44" t="inlineStr">
         <is>
           <t>2k: 100% tok -&gt; 100% cost</t>
         </is>
       </c>
-      <c r="E81" s="52" t="n">
+      <c r="E81" s="53" t="n">
         <v>154.8429860104542</v>
       </c>
-      <c r="F81" s="53" t="n">
+      <c r="F81" s="54" t="n">
         <v>-11.13717395678222</v>
       </c>
-      <c r="G81" s="54" t="inlineStr">
+      <c r="G81" s="55" t="inlineStr">
         <is>
           <t>MEASURED (degenerate one-context case)</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="45" t="inlineStr">
+      <c r="A82" s="46" t="inlineStr">
         <is>
           <t>Modern standard (8k bulk + 64k/256k extension)</t>
         </is>
       </c>
-      <c r="B82" s="50" t="n">
+      <c r="B82" s="51" t="n">
         <v>2.220667013967386</v>
       </c>
-      <c r="C82" s="51" t="n">
+      <c r="C82" s="52" t="n">
         <v>0.4503151502275102</v>
       </c>
-      <c r="D82" s="43" t="inlineStr">
+      <c r="D82" s="44" t="inlineStr">
         <is>
           <t>8k: 70% tok -&gt; 26% cost  64k: 20% tok -&gt; 27% cost  256k: 10% tok -&gt; 47% cost</t>
         </is>
       </c>
-      <c r="E82" s="52" t="n">
+      <c r="E82" s="53" t="n">
         <v>158.8547874640003</v>
       </c>
-      <c r="F82" s="53" t="n">
+      <c r="F82" s="54" t="n">
         <v>-7.125372503236179</v>
       </c>
-      <c r="G82" s="55" t="inlineStr">
+      <c r="G82" s="56" t="inlineStr">
         <is>
           <t>ILLUSTRATIVE ASSUMPTION</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="45" t="inlineStr">
+      <c r="A83" s="46" t="inlineStr">
         <is>
           <t>Long-context heavy (frontier extension phases)</t>
         </is>
       </c>
-      <c r="B83" s="50" t="n">
+      <c r="B83" s="51" t="n">
         <v>7.743424712739709</v>
       </c>
-      <c r="C83" s="51" t="n">
+      <c r="C83" s="52" t="n">
         <v>0.1291418251093435</v>
       </c>
-      <c r="D83" s="43" t="inlineStr">
+      <c r="D83" s="44" t="inlineStr">
         <is>
           <t>8k: 40% tok -&gt; 4% cost  64k: 25% tok -&gt; 10% cost  256k: 25% tok -&gt; 34% cost  1024k: 10% tok -&gt; 52% cost</t>
         </is>
       </c>
-      <c r="E83" s="52" t="n">
+      <c r="E83" s="53" t="n">
         <v>159.8723512892946</v>
       </c>
-      <c r="F83" s="53" t="n">
+      <c r="F83" s="54" t="n">
         <v>-6.107808677941904</v>
       </c>
-      <c r="G83" s="55" t="inlineStr">
+      <c r="G83" s="56" t="inlineStr">
         <is>
           <t>ILLUSTRATIVE ASSUMPTION</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="45" t="inlineStr">
+      <c r="A84" s="46" t="inlineStr">
         <is>
           <t>Frontier + long-rollout RL</t>
         </is>
       </c>
-      <c r="B84" s="50" t="n">
+      <c r="B84" s="51" t="n">
         <v>12.08050561742532</v>
       </c>
-      <c r="C84" s="51" t="n">
+      <c r="C84" s="52" t="n">
         <v>0.08277799221893223</v>
       </c>
-      <c r="D84" s="43" t="inlineStr">
+      <c r="D84" s="44" t="inlineStr">
         <is>
           <t>8k: 30% tok -&gt; 2% cost  64k: 20% tok -&gt; 5% cost  256k: 30% tok -&gt; 26% cost  1024k: 20% tok -&gt; 67% cost</t>
         </is>
       </c>
-      <c r="E84" s="52" t="n">
+      <c r="E84" s="53" t="n">
         <v>160.0192444322226</v>
       </c>
-      <c r="F84" s="53" t="n">
+      <c r="F84" s="54" t="n">
         <v>-5.960915535013839</v>
       </c>
-      <c r="G84" s="55" t="inlineStr">
+      <c r="G84" s="56" t="inlineStr">
         <is>
           <t>ILLUSTRATIVE ASSUMPTION</t>
         </is>
@@ -2598,191 +2618,191 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="38" t="inlineStr">
+      <c r="A90" s="39" t="inlineStr">
         <is>
           <t>Context (tokens)</t>
         </is>
       </c>
-      <c r="B90" s="38" t="inlineStr">
+      <c r="B90" s="39" t="inlineStr">
         <is>
           <t>Transformer ms</t>
         </is>
       </c>
-      <c r="C90" s="38" t="inlineStr">
+      <c r="C90" s="39" t="inlineStr">
         <is>
           <t>bAttention ms</t>
         </is>
       </c>
-      <c r="D90" s="38" t="inlineStr">
+      <c r="D90" s="39" t="inlineStr">
         <is>
           <t>TF / bAttention</t>
         </is>
       </c>
-      <c r="E90" s="38" t="inlineStr"/>
-      <c r="F90" s="38" t="inlineStr">
+      <c r="E90" s="39" t="inlineStr"/>
+      <c r="F90" s="39" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="39" t="n">
+      <c r="A91" s="40" t="n">
         <v>2048</v>
       </c>
       <c r="B91" s="5" t="n">
         <v>111.229</v>
       </c>
-      <c r="C91" s="14" t="n">
+      <c r="C91" s="15" t="n">
         <v>663.1130000000001</v>
       </c>
-      <c r="D91" s="50" t="n">
+      <c r="D91" s="51" t="n">
         <v>0.16773762541226</v>
       </c>
-      <c r="F91" s="43" t="inlineStr">
+      <c r="F91" s="44" t="inlineStr">
         <is>
           <t>transformer ahead</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="39" t="n">
+      <c r="A92" s="40" t="n">
         <v>4096</v>
       </c>
       <c r="B92" s="5" t="n">
         <v>125.091</v>
       </c>
-      <c r="C92" s="14" t="n">
+      <c r="C92" s="15" t="n">
         <v>662.751</v>
       </c>
-      <c r="D92" s="50" t="n">
+      <c r="D92" s="51" t="n">
         <v>0.1887450943114382</v>
       </c>
-      <c r="F92" s="43" t="inlineStr">
+      <c r="F92" s="44" t="inlineStr">
         <is>
           <t>transformer ahead</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="39" t="n">
+      <c r="A93" s="40" t="n">
         <v>8192</v>
       </c>
       <c r="B93" s="5" t="n">
         <v>153.085</v>
       </c>
-      <c r="C93" s="14" t="n">
+      <c r="C93" s="15" t="n">
         <v>663.327</v>
       </c>
-      <c r="D93" s="50" t="n">
+      <c r="D93" s="51" t="n">
         <v>0.2307836104967836</v>
       </c>
-      <c r="F93" s="43" t="inlineStr">
+      <c r="F93" s="44" t="inlineStr">
         <is>
           <t>transformer ahead</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="39" t="n">
+      <c r="A94" s="40" t="n">
         <v>16384</v>
       </c>
       <c r="B94" s="5" t="n">
         <v>204.919</v>
       </c>
-      <c r="C94" s="14" t="n">
+      <c r="C94" s="15" t="n">
         <v>663.202</v>
       </c>
-      <c r="D94" s="50" t="n">
+      <c r="D94" s="51" t="n">
         <v>0.3089842913622094</v>
       </c>
-      <c r="F94" s="43" t="inlineStr">
+      <c r="F94" s="44" t="inlineStr">
         <is>
           <t>transformer ahead</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="39" t="n">
+      <c r="A95" s="40" t="n">
         <v>32768</v>
       </c>
       <c r="B95" s="5" t="n">
         <v>309.886</v>
       </c>
-      <c r="C95" s="14" t="n">
+      <c r="C95" s="15" t="n">
         <v>662.6180000000001</v>
       </c>
-      <c r="D95" s="50" t="n">
+      <c r="D95" s="51" t="n">
         <v>0.4676691547769605</v>
       </c>
-      <c r="F95" s="43" t="inlineStr">
+      <c r="F95" s="44" t="inlineStr">
         <is>
           <t>transformer ahead</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="39" t="n">
+      <c r="A96" s="40" t="n">
         <v>65536</v>
       </c>
       <c r="B96" s="5" t="n">
         <v>520.986</v>
       </c>
-      <c r="C96" s="14" t="n">
+      <c r="C96" s="15" t="n">
         <v>663.199</v>
       </c>
-      <c r="D96" s="50" t="n">
+      <c r="D96" s="51" t="n">
         <v>0.7855651169558459</v>
       </c>
-      <c r="F96" s="43" t="inlineStr">
+      <c r="F96" s="44" t="inlineStr">
         <is>
           <t>transformer ahead</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="39" t="n">
+      <c r="A97" s="40" t="n">
         <v>131072</v>
       </c>
       <c r="B97" s="5" t="n">
         <v>969.79</v>
       </c>
-      <c r="C97" s="14" t="n">
+      <c r="C97" s="15" t="n">
         <v>753.457</v>
       </c>
-      <c r="D97" s="50" t="n">
+      <c r="D97" s="51" t="n">
         <v>1.287120565606265</v>
       </c>
-      <c r="F97" s="43" t="inlineStr"/>
+      <c r="F97" s="44" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" s="39" t="n">
+      <c r="A98" s="40" t="n">
         <v>262144</v>
       </c>
       <c r="B98" s="5" t="n">
         <v>1889.616</v>
       </c>
-      <c r="C98" s="14" t="n">
+      <c r="C98" s="15" t="n">
         <v>938.175</v>
       </c>
-      <c r="D98" s="50" t="n">
+      <c r="D98" s="51" t="n">
         <v>2.014140219042289</v>
       </c>
-      <c r="F98" s="43" t="inlineStr"/>
+      <c r="F98" s="44" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" s="39" t="n">
+      <c r="A99" s="40" t="n">
         <v>524288</v>
       </c>
       <c r="B99" s="5" t="n">
         <v>3718.717</v>
       </c>
-      <c r="C99" s="14" t="n">
+      <c r="C99" s="15" t="n">
         <v>1308.837</v>
       </c>
-      <c r="D99" s="50" t="n">
+      <c r="D99" s="51" t="n">
         <v>2.841237678947035</v>
       </c>
-      <c r="F99" s="43" t="inlineStr"/>
+      <c r="F99" s="44" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
@@ -2797,530 +2817,530 @@
       <c r="F101" s="2" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="38" t="inlineStr">
+      <c r="A102" s="39" t="inlineStr">
         <is>
           <t>Assumption</t>
         </is>
       </c>
-      <c r="B102" s="38" t="inlineStr">
+      <c r="B102" s="39" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C102" s="38" t="inlineStr"/>
-      <c r="D102" s="38" t="inlineStr"/>
-      <c r="E102" s="38" t="inlineStr">
+      <c r="C102" s="39" t="inlineStr"/>
+      <c r="D102" s="39" t="inlineStr"/>
+      <c r="E102" s="39" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F102" s="38" t="inlineStr">
+      <c r="F102" s="39" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="45" t="inlineStr">
+      <c r="A103" s="46" t="inlineStr">
         <is>
           <t>Compute lever (Today, 2026-09-01 re-base)</t>
         </is>
       </c>
-      <c r="B103" s="43" t="inlineStr">
+      <c r="B103" s="44" t="inlineStr">
         <is>
           <t>x793 = full-workload serving lever (decode 2.5 ms/token x 64 streams ESTIMATE, prefill at the BANKED x3.94) x the x4.22 FIT-DERIVED equal-quality ratio at trillion scale; Ceiling = same at the full x7.03 maturity factor (x816)</t>
         </is>
       </c>
-      <c r="E103" s="55" t="inlineStr">
+      <c r="E103" s="56" t="inlineStr">
         <is>
           <t>ESTIMATE x PROJECTION</t>
         </is>
       </c>
-      <c r="F103" s="43" t="inlineStr">
+      <c r="F103" s="44" t="inlineStr">
         <is>
           <t>campaign_landed_flop_lever(); aggregate-decode receipt PENDING (decode_aggregate_receipt_20260831_instructions.md)</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="45" t="inlineStr">
+      <c r="A104" s="46" t="inlineStr">
         <is>
           <t>Equal-quality parameter matching</t>
         </is>
       </c>
-      <c r="B104" s="43" t="inlineStr">
+      <c r="B104" s="44" t="inlineStr">
         <is>
           <t>sealed 2026-08-14 refit, 4 rungs per family (47M-663M params): the fits cross at 392M and bAttention then matches the transformer fit's quality on 84.2% of the params at 1B, 55.2% at 10B, 36.2% at 100B, 23.7% at 1T, 15.5% at 10T. The receipt's own words: 'a projection of the two fits, not a measurement'</t>
         </is>
       </c>
-      <c r="E104" s="55" t="inlineStr">
+      <c r="E104" s="56" t="inlineStr">
         <is>
           <t>PROJECTION</t>
         </is>
       </c>
-      <c r="F104" s="43" t="inlineStr">
+      <c r="F104" s="44" t="inlineStr">
         <is>
           <t>quality_fit_v4.json param_matching; fits over the sealed rope-convention ladder</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="45" t="inlineStr">
+      <c r="A105" s="46" t="inlineStr">
         <is>
           <t>Single-GPU training step (AGAINST us)</t>
         </is>
       </c>
-      <c r="B105" s="43" t="inlineStr">
+      <c r="B105" s="44" t="inlineStr">
         <is>
           <t>RE-BASED 2026-08-24: on one GH200, single layer, fwd+bwd, bf16, checkpointing off both arms, against a MODERN transformer block (24Q/4KV, head_dim 256, RoPE 64, gated attention), a bAttention step costs x1.72 MORE at T=2,048 (101.7 vs 59.3 ms/step) and x1.79 at T=8,192. It read x6.116 (400.4 ms) the same morning and x6.46 on the older d1536/27L fp16 601-step receipt. Fwd x1.82, bwd x2.35. Training is still excluded from the serving claim, but the gap is now a kernel-program line item with a funded gate, not a structural loss</t>
         </is>
       </c>
-      <c r="E105" s="54" t="inlineStr">
+      <c r="E105" s="55" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F105" s="43" t="inlineStr">
+      <c r="F105" s="44" t="inlineStr">
         <is>
           <t>2026-08-24 GH200 megakernel measurement; prior: dtype_trio_v4.json rows[fp16]</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="45" t="inlineStr">
+      <c r="A106" s="46" t="inlineStr">
         <is>
           <t>Training PEAK MEMORY (AGAINST us)</t>
         </is>
       </c>
-      <c r="B106" s="43" t="inlineStr">
+      <c r="B106" s="44" t="inlineStr">
         <is>
           <t>x1.579 at T=2,048 (17,087.5 vs 10,823.6 MiB) and x1.567 at T=8,192, down from x2.829 the same morning. This is TRAINING peak memory and is NOT the mem_factor lever, which is SERVING state (O(1) recurrent state vs O(T) KV cache) and is unaffected. It is not an input to the cost model; it caps per-GPU batch density</t>
         </is>
       </c>
-      <c r="E106" s="54" t="inlineStr">
+      <c r="E106" s="55" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F106" s="43" t="inlineStr">
+      <c r="F106" s="44" t="inlineStr">
         <is>
           <t>2026-08-24 GH200 megakernel measurement</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="45" t="inlineStr">
+      <c r="A107" s="46" t="inlineStr">
         <is>
           <t>Kernel program (TARGET, not a result)</t>
         </is>
       </c>
-      <c r="B107" s="43" t="inlineStr">
+      <c r="B107" s="44" t="inlineStr">
         <is>
           <t>the funded 8k-win gate is a T=8,192 step at or below 83.08 ms, i.e. x1.786 still to remove (44% of the step). Named levers: recompute removal ~-12.8 ms; backward-fold + occupancy redesign (~3x headroom in the dominant fused kernel); copies elimination (24.8% of the step). Memory target x0.88 (parity or below). CEILING_PREFILL_SPEEDUP = the MEASURED x3.936 already banked x this x1.786 target</t>
         </is>
       </c>
-      <c r="E107" s="55" t="inlineStr">
+      <c r="E107" s="56" t="inlineStr">
         <is>
           <t>TARGET</t>
         </is>
       </c>
-      <c r="F107" s="43" t="inlineStr">
+      <c r="F107" s="44" t="inlineStr">
         <is>
           <t>kernel-campaign program plan, 2026-08-24 — no receipt behind the target half</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="45" t="inlineStr">
+      <c r="A108" s="46" t="inlineStr">
         <is>
           <t>Context scaling of the training gap</t>
         </is>
       </c>
-      <c r="B108" s="43" t="inlineStr">
+      <c r="B108" s="44" t="inlineStr">
         <is>
           <t>at matched tokens/step, 2k -&gt; 8k (4x context): our step grows x1.000, the transformer's x1.319, so the ratio decays x0.758 per 4x. The equal-token B4/T32,768 ~parity cell is RETIRED 2026-08-25 as a B4 occupancy artifact (it shared the retired growth residual); the flat per-token model puts the crossover at a PROJECTED T~16,900. Holding the old x0.802 decay constant instead would say x1.43 at 32k and a crossover near T~310,000 - that is the CONSERVATIVE extrapolation, because the transformer's quadratic attention term makes its per-4x growth rise with context while ours stays flat</t>
         </is>
       </c>
-      <c r="E108" s="55" t="inlineStr">
+      <c r="E108" s="56" t="inlineStr">
         <is>
           <t>MEASURED (2 ratio points) + PROJECTION</t>
         </is>
       </c>
-      <c r="F108" s="43" t="inlineStr">
+      <c r="F108" s="44" t="inlineStr">
         <is>
           <t>2026-08-24 GH200 megakernel measurement; 2k cell re-based 2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="45" t="inlineStr">
+      <c r="A109" s="46" t="inlineStr">
         <is>
           <t>Training CONTEXT MIX (reads the other way)</t>
         </is>
       </c>
-      <c r="B109" s="43" t="inlineStr">
+      <c r="B109" s="44" t="inlineStr">
         <is>
           <t>quoting one context for all of training is the pessimistic corner, and it was this model's old implicit assumption. Cost-weighted over a curriculum the training term flips from a DRAG to a CONTRIBUTOR: x0.583 at 100% 2k, x2.22 at a modern 8k/64k/256k mix, x7.74 long-context-heavy, x12.08 with long RL rollouts. The mechanism: our per-token cost is FLAT in context and the transformer's GROWS, so long-context tokens dominate its bill as a token minority — 10% of tokens at 262k is 47% of its training cost. r(T) is MEASURED at 2k/8k and MODELED beyond; the curriculum SHARES are ILLUSTRATIVE and exposed as knobs (this repo carries no citation for any lab's recipe)</t>
         </is>
       </c>
-      <c r="E109" s="55" t="inlineStr">
+      <c r="E109" s="56" t="inlineStr">
         <is>
           <t>MEASURED r(T) + ILLUSTRATIVE mix</t>
         </is>
       </c>
-      <c r="F109" s="43" t="inlineStr">
+      <c r="F109" s="44" t="inlineStr">
         <is>
           <t>TRAIN_COST_FIT_20260824, TRAINING_CURRICULA, training_advantage_mix()</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="45" t="inlineStr">
+      <c r="A110" s="46" t="inlineStr">
         <is>
           <t>Long-context training memory (EXCLUDED, runs our way)</t>
         </is>
       </c>
-      <c r="B110" s="43" t="inlineStr">
+      <c r="B110" s="44" t="inlineStr">
         <is>
           <t>at 262k+ the transformer additionally pays sequence-parallelism and activation-memory costs that an O(1) recurrent state does not: its KV grows at 156 KB per token of context per stream, which is what forces sharding, ring/Ulysses attention and their communication overhead. Our own measurement shows the asymmetry in the small: peak training memory grew only x0.993 relative to the transformer's from 2k to 8k (x1.579 -&gt; x1.567), i.e. the ratio is FLAT-to-falling in context while the absolute gap the transformer must shard grows. NOT in the cost model — the training advantage above counts FLOPs/step-time only, so the direction of this omission is CONSERVATIVE (it understates us at long context). Quantifying it needs a multi-GPU long-context training receipt we do not have</t>
         </is>
       </c>
-      <c r="E110" s="55" t="inlineStr">
+      <c r="E110" s="56" t="inlineStr">
         <is>
           <t>DIRECTIONAL — measured components, not a costed lever</t>
         </is>
       </c>
-      <c r="F110" s="43" t="inlineStr">
+      <c r="F110" s="44" t="inlineStr">
         <is>
           <t>KERNEL_CAMPAIGN_20260824 mem_ratio_2k/8k; KV_MB_PER_TOKEN_PER_STREAM</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="45" t="inlineStr">
+      <c r="A111" s="46" t="inlineStr">
         <is>
           <t>$/GPU-hour</t>
         </is>
       </c>
-      <c r="B111" s="43" t="inlineStr">
+      <c r="B111" s="44" t="inlineStr">
         <is>
           <t>$2.50 (H100 rent, neocloud/committed mid; ladder 2.00-3.50)</t>
         </is>
       </c>
-      <c r="E111" s="55" t="inlineStr">
+      <c r="E111" s="56" t="inlineStr">
         <is>
           <t>ASSUMPTION</t>
         </is>
       </c>
-      <c r="F111" s="43" t="inlineStr">
+      <c r="F111" s="44" t="inlineStr">
         <is>
           <t>this file's CostLadder row — unchanged rate basis</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="45" t="inlineStr">
+      <c r="A112" s="46" t="inlineStr">
         <is>
           <t>Utilization</t>
         </is>
       </c>
-      <c r="B112" s="43" t="inlineStr">
+      <c r="B112" s="44" t="inlineStr">
         <is>
           <t>85%</t>
         </is>
       </c>
-      <c r="E112" s="55" t="inlineStr">
+      <c r="E112" s="56" t="inlineStr">
         <is>
           <t>ASSUMPTION</t>
         </is>
       </c>
-      <c r="F112" s="43" t="inlineStr">
+      <c r="F112" s="44" t="inlineStr">
         <is>
           <t>same value as the ladder's owned-TCO cross-check</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="45" t="inlineStr">
+      <c r="A113" s="46" t="inlineStr">
         <is>
           <t>Context-length mix</t>
         </is>
       </c>
-      <c r="B113" s="43" t="inlineStr">
+      <c r="B113" s="44" t="inlineStr">
         <is>
           <t>headline quoted at 262k (a measured decode cell); table sweeps 4k-1M. The decode lever crosses 1 at ~29,800 tokens and BELOW that the transformer serves more tokens per GPU-second than we do — stated on every surface</t>
         </is>
       </c>
-      <c r="E113" s="55" t="inlineStr">
+      <c r="E113" s="56" t="inlineStr">
         <is>
           <t>ASSUMPTION</t>
         </is>
       </c>
-      <c r="F113" s="43" t="inlineStr">
+      <c r="F113" s="44" t="inlineStr">
         <is>
           <t>serving_cost_curve, decode_throughput_ratio</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="45" t="inlineStr">
+      <c r="A114" s="46" t="inlineStr">
         <is>
           <t>Decode lever is MEMORY-CEILING, not latency (READ FIRST)</t>
         </is>
       </c>
-      <c r="B114" s="43" t="inlineStr">
+      <c r="B114" s="44" t="inlineStr">
         <is>
           <t>per generated token at ONE stream the transformer is AHEAD of us at 64k context — 4.92 vs 5.74 GPU-busy per token. The lever is that it cannot hold many long-context streams: it re-reads its whole KV cache per emitted token, so its aggregate throughput falls as 1/context while ours is flat. Measured: 1 stream at 262k (2 OOM — an exact ceiling) and 8 streams at 32k (16 OOM, so that ceiling is only bracketed at 8-15 and the 32k cell is a bounded x0.97-1.14, near parity) against 64 of ours in 1.62 GB</t>
         </is>
       </c>
-      <c r="E114" s="54" t="inlineStr">
+      <c r="E114" s="55" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F114" s="43" t="inlineStr">
+      <c r="F114" s="44" t="inlineStr">
         <is>
           <t>deck_decode_d2048_bf16_gh200_20260814.json; DECODE_THROUGHPUT_20260814</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="45" t="inlineStr">
+      <c r="A115" s="46" t="inlineStr">
         <is>
           <t>Transformer-stack maturity</t>
         </is>
       </c>
-      <c r="B115" s="43" t="inlineStr">
+      <c r="B115" s="44" t="inlineStr">
         <is>
           <t>NOT GRANTED by default since the 2026-08-14 re-base: the headline runs on the measured cells, in which neither family's decode is optimised (ours ran the unoptimised Triton per-step path at 9.5% GPU-busy while the transformer sat at 95.6%). Setting tf_kv_compression=8.0 grants it paged attention + KV quantization, divides our decode lever by 8 and puts the TRANSFORMER ahead at 64k — reported, not hidden</t>
         </is>
       </c>
-      <c r="E115" s="55" t="inlineStr">
+      <c r="E115" s="56" t="inlineStr">
         <is>
           <t>ASSUMPTION</t>
         </is>
       </c>
-      <c r="F115" s="43" t="inlineStr">
+      <c r="F115" s="44" t="inlineStr">
         <is>
           <t>SERVING['tf_kv_compression']</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="45" t="inlineStr">
+      <c r="A116" s="46" t="inlineStr">
         <is>
           <t>bAttention serving throughput</t>
         </is>
       </c>
-      <c r="B116" s="43" t="inlineStr">
+      <c r="B116" s="44" t="inlineStr">
         <is>
           <t>562 tok/s/GPU (4,497/box): 64 concurrent 262,144-token streams on one GPU, context-flat 32k-262k (-4.0%). The 64-stream cell is a grid cap, not a ceiling — 1.62 GB of state on a 96 GB card at 9.5% GPU-busy — so it is a LOWER bound. Supersedes a 349,880 tok/s/box figure measured on the h-carry-only proxy</t>
         </is>
       </c>
-      <c r="E116" s="54" t="inlineStr">
+      <c r="E116" s="55" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F116" s="43" t="inlineStr">
+      <c r="F116" s="44" t="inlineStr">
         <is>
           <t>deck_decode_d2048_bf16_gh200_20260814.json rows[bdm, 64 streams]</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="45" t="inlineStr">
+      <c r="A117" s="46" t="inlineStr">
         <is>
           <t>bAttention per-stream state</t>
         </is>
       </c>
-      <c r="B117" s="43" t="inlineStr">
+      <c r="B117" s="44" t="inlineStr">
         <is>
           <t>25.4 MB/stream, the FULL recurrent cell (h + M memory), 24.2 MiB measured, context-flat. The 0.15 MB figure previously quoted was an h-carry-only proxy with no M memory and is retired as a headline</t>
         </is>
       </c>
-      <c r="E117" s="54" t="inlineStr">
+      <c r="E117" s="55" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F117" s="43" t="inlineStr">
+      <c r="F117" s="44" t="inlineStr">
         <is>
           <t>deck_decode_d2048_bf16_gh200_20260814.json state_bytes_per_stream</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="45" t="inlineStr">
+      <c r="A118" s="46" t="inlineStr">
         <is>
           <t>Transformer KV wall</t>
         </is>
       </c>
-      <c r="B118" s="43" t="inlineStr">
+      <c r="B118" s="44" t="inlineStr">
         <is>
           <t>197 KB per token of context per stream — 51.5 GB for one 262,144-token stream, a 2nd stream OOMs a 96 GB card, and 16 streams OOM it at 32,768 tokens. Its retired 88.5 per-token decode cost was inflated by a growing-KV re-planning harness artifact; the traced figure is 14.92 GPU-busy at 262k</t>
         </is>
       </c>
-      <c r="E118" s="54" t="inlineStr">
+      <c r="E118" s="55" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F118" s="43" t="inlineStr">
+      <c r="F118" s="44" t="inlineStr">
         <is>
           <t>deck_decode_d2048_bf16_gh200_20260814.json rows[transformer]</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="45" t="inlineStr">
+      <c r="A119" s="46" t="inlineStr">
         <is>
           <t>Training throughput at 8 GPUs</t>
         </is>
       </c>
-      <c r="B119" s="43" t="inlineStr">
+      <c r="B119" s="44" t="inlineStr">
         <is>
           <t>x5.15 (bAttention, fwd+bwd) vs x3.70 (transformer Ulysses best, forward-only) at matched 16-in-flight load -&gt; x1.39; x6.27 at 256 in flight -&gt; x1.70</t>
         </is>
       </c>
-      <c r="E119" s="54" t="inlineStr">
+      <c r="E119" s="55" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F119" s="43" t="inlineStr">
+      <c r="F119" s="44" t="inlineStr">
         <is>
           <t>derived.json matched_load_curve, scaling_1to8_best</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="45" t="inlineStr">
+      <c r="A120" s="46" t="inlineStr">
         <is>
           <t>Memory walls (component scope)</t>
         </is>
       </c>
-      <c r="B120" s="43" t="inlineStr">
+      <c r="B120" s="44" t="inlineStr">
         <is>
           <t>64k-token sequence: 30.9 GB (fits 1 GPU) vs OOM at 78.4 GB attempted; pipeline stage 9.05 GB flat vs GPipe 43.3 GB</t>
         </is>
       </c>
-      <c r="E120" s="54" t="inlineStr">
+      <c r="E120" s="55" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F120" s="43" t="inlineStr">
+      <c r="F120" s="44" t="inlineStr">
         <is>
           <t>derived.json pipeline_feasibility, pipeline_memory_asymmetry</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="45" t="inlineStr">
+      <c r="A121" s="46" t="inlineStr">
         <is>
           <t>Compute lever (flop_factor)</t>
         </is>
       </c>
-      <c r="B121" s="43" t="inlineStr">
+      <c r="B121" s="44" t="inlineStr">
         <is>
           <t>cross-family prefill, bf16, 1xH100, parameter counts exactly matched, block scope (1 layer, batch 16): TF/bAttention 4.02 at d512/1M, 3.83 at d1024/1M, 2.01 at d2048/262k. Short context favours the transformer and is stated so. NOTE: measured on the PRE-CAMPAIGN kernels and not re-run since 2026-08-24, so the TODAY lever is conservative; the realized x3.936 sits in CEILING_PREFILL_SPEEDUP, not here</t>
         </is>
       </c>
-      <c r="E121" s="54" t="inlineStr">
+      <c r="E121" s="55" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F121" s="43" t="inlineStr">
+      <c r="F121" s="44" t="inlineStr">
         <is>
           <t>matched_d{512,1024,2048}_h100.json (2026-07-21)</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="45" t="inlineStr">
+      <c r="A122" s="46" t="inlineStr">
         <is>
           <t>Compute, fp32 lane (scope reference)</t>
         </is>
       </c>
-      <c r="B122" s="43" t="inlineStr">
+      <c r="B122" s="44" t="inlineStr">
         <is>
           <t>the d2048/24-layer fp32 sweep gives 7.91 at 262k at full-model scope. No fp32 FlashAttention kernel exists, so that lane runs mem-efficient attention on the transformer and the owned arm is fp16 internally; params 16.7% apart. Full model in bf16 has not been run</t>
         </is>
       </c>
-      <c r="E122" s="55" t="inlineStr">
+      <c r="E122" s="56" t="inlineStr">
         <is>
           <t>LABEL</t>
         </is>
       </c>
-      <c r="F122" s="43" t="inlineStr">
+      <c r="F122" s="44" t="inlineStr">
         <is>
           <t>deck_speed_scaling_d2048_h100_20260803.json sdpa_fp32_backend_probe + last_route_attestation</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="45" t="inlineStr">
+      <c r="A123" s="46" t="inlineStr">
         <is>
           <t>16-bit IO (training)</t>
         </is>
       </c>
-      <c r="B123" s="43" t="inlineStr">
+      <c r="B123" s="44" t="inlineStr">
         <is>
           <t>same-arch GH200 gate at d1536: fp16 x1.185 step time and -17.5% peak memory, bf16 x1.171 and -20.6%; quality deltas +0.001 to +0.004 from the gate's smaller vehicle. Reported on its own; not an input to the compute lever</t>
         </is>
       </c>
-      <c r="E123" s="54" t="inlineStr">
+      <c r="E123" s="55" t="inlineStr">
         <is>
           <t>MEASURED</t>
         </is>
       </c>
-      <c r="F123" s="43" t="inlineStr">
+      <c r="F123" s="44" t="inlineStr">
         <is>
           <t>receipts/io16_gate_20260809.md (2026-08-09)</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="45" t="inlineStr">
+      <c r="A124" s="46" t="inlineStr">
         <is>
           <t>Quality parity at 70B</t>
         </is>
       </c>
-      <c r="B124" s="43" t="inlineStr">
+      <c r="B124" s="44" t="inlineStr">
         <is>
           <t>transformer needs x4.1 params [2.2-7.7] or x1.7 tokens [1.33-2.10, beta=0.28 assumption]; crossover N* ~321M = the top measured rung</t>
         </is>
       </c>
-      <c r="E124" s="55" t="inlineStr">
+      <c r="E124" s="56" t="inlineStr">
         <is>
           <t>PROJECTION</t>
         </is>
       </c>
-      <c r="F124" s="43" t="inlineStr">
+      <c r="F124" s="44" t="inlineStr">
         <is>
           <t>derived.json quality_fit.ref_70B, parity_cost</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="45" t="inlineStr">
+      <c r="A125" s="46" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="B125" s="43" t="inlineStr">
+      <c r="B125" s="44" t="inlineStr">
         <is>
           <t>systems numbers are component-scope (bAttention d1536 fwd+bwd h-recurrence sub-block vs transformer d2048 forward-only layer); every speedup is vs the family's OWN 1-GPU baseline</t>
         </is>
       </c>
-      <c r="E125" s="55" t="inlineStr">
+      <c r="E125" s="56" t="inlineStr">
         <is>
           <t>LABEL</t>
         </is>
       </c>
-      <c r="F125" s="43" t="inlineStr">
+      <c r="F125" s="44" t="inlineStr">
         <is>
           <t>derived.json scope_reconciliation; deck README</t>
         </is>
@@ -3746,10 +3766,10 @@
           <t>memory share = 45%</t>
         </is>
       </c>
-      <c r="B27" s="16" t="n">
+      <c r="B27" s="17" t="n">
         <v>0.45</v>
       </c>
-      <c r="C27" s="37">
+      <c r="C27" s="38">
         <f>1/(B27/Inputs!$B$2+(1-B27)/Inputs!$B$3)</f>
         <v/>
       </c>
@@ -3765,10 +3785,10 @@
           <t>memory share = 50%</t>
         </is>
       </c>
-      <c r="B28" s="16" t="n">
+      <c r="B28" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="C28" s="37">
+      <c r="C28" s="38">
         <f>1/(B28/Inputs!$B$2+(1-B28)/Inputs!$B$3)</f>
         <v/>
       </c>
@@ -3784,10 +3804,10 @@
           <t>memory share = 60%</t>
         </is>
       </c>
-      <c r="B29" s="16" t="n">
+      <c r="B29" s="17" t="n">
         <v>0.6</v>
       </c>
-      <c r="C29" s="37">
+      <c r="C29" s="38">
         <f>1/(B29/Inputs!$B$2+(1-B29)/Inputs!$B$3)</f>
         <v/>
       </c>
@@ -3803,10 +3823,10 @@
           <t>memory share = 70%</t>
         </is>
       </c>
-      <c r="B30" s="16" t="n">
+      <c r="B30" s="17" t="n">
         <v>0.7</v>
       </c>
-      <c r="C30" s="37">
+      <c r="C30" s="38">
         <f>1/(B30/Inputs!$B$2+(1-B30)/Inputs!$B$3)</f>
         <v/>
       </c>
@@ -3822,10 +3842,10 @@
           <t>memory share = 82%</t>
         </is>
       </c>
-      <c r="B31" s="16" t="n">
+      <c r="B31" s="17" t="n">
         <v>0.82</v>
       </c>
-      <c r="C31" s="37">
+      <c r="C31" s="38">
         <f>1/(B31/Inputs!$B$2+(1-B31)/Inputs!$B$3)</f>
         <v/>
       </c>
@@ -4198,10 +4218,10 @@
           <t>Total capex ($B)</t>
         </is>
       </c>
-      <c r="B3" s="14" t="n">
+      <c r="B3" s="15" t="n">
         <v>88</v>
       </c>
-      <c r="C3" s="15" t="n">
+      <c r="C3" s="16" t="n">
         <v>190</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -4216,10 +4236,10 @@
           <t>Infra / data-center share</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="16" t="n">
+      <c r="C4" s="17" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -4234,10 +4254,10 @@
           <t>Server / short-lived share</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="17" t="n">
         <v>0.67</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -4252,10 +4272,10 @@
           <t>Accelerator share within servers</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="17" t="n">
         <v>0.75</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="17" t="n">
         <v>0.75</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -4270,7 +4290,7 @@
           <t>Market cap ($B, approx)</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="18" t="n">
         <v>3700</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -4385,11 +4405,11 @@
           <t>Fleet size (GPU-equiv)</t>
         </is>
       </c>
-      <c r="B16" s="18">
+      <c r="B16" s="19">
         <f>B12*1000000000/Inputs!$B$7</f>
         <v/>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="19">
         <f>C12*1000000000/Inputs!$B$7</f>
         <v/>
       </c>
@@ -4405,11 +4425,11 @@
           <t>Total wall power (MW)</t>
         </is>
       </c>
-      <c r="B17" s="18">
+      <c r="B17" s="19">
         <f>B16*Inputs!$B$8/1000</f>
         <v/>
       </c>
-      <c r="C17" s="18">
+      <c r="C17" s="19">
         <f>C16*Inputs!$B$8/1000</f>
         <v/>
       </c>
@@ -4425,11 +4445,11 @@
           <t>Daily energy (MWh)</t>
         </is>
       </c>
-      <c r="B18" s="18">
+      <c r="B18" s="19">
         <f>B17*24</f>
         <v/>
       </c>
-      <c r="C18" s="18">
+      <c r="C18" s="19">
         <f>C17*24</f>
         <v/>
       </c>
@@ -4441,11 +4461,11 @@
           <t>Daily all-in opex ($/day)</t>
         </is>
       </c>
-      <c r="B19" s="18">
+      <c r="B19" s="19">
         <f>B18*1000*Inputs!$B$9*(1+Inputs!$B$10)</f>
         <v/>
       </c>
-      <c r="C19" s="18">
+      <c r="C19" s="19">
         <f>C18*1000*Inputs!$B$9*(1+Inputs!$B$10)</f>
         <v/>
       </c>
@@ -4477,11 +4497,11 @@
           <t>Lifetime opex ($B)</t>
         </is>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="20">
         <f>B20*Inputs!$B$11/1000</f>
         <v/>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="20">
         <f>C20*Inputs!$B$11/1000</f>
         <v/>
       </c>
@@ -4559,11 +4579,11 @@
           <t>Sustained annual benefit ($B/yr)</t>
         </is>
       </c>
-      <c r="B27" s="20">
+      <c r="B27" s="21">
         <f>B25+B26/1000</f>
         <v/>
       </c>
-      <c r="C27" s="20">
+      <c r="C27" s="21">
         <f>C25+C26/1000</f>
         <v/>
       </c>
@@ -4579,11 +4599,11 @@
           <t>Capitalized value ($B)</t>
         </is>
       </c>
-      <c r="B28" s="13">
+      <c r="B28" s="14">
         <f>B27/Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="C28" s="13">
+      <c r="C28" s="14">
         <f>C27/Inputs!$B$6</f>
         <v/>
       </c>
@@ -4599,11 +4619,11 @@
           <t>% of market cap</t>
         </is>
       </c>
-      <c r="B29" s="21">
+      <c r="B29" s="22">
         <f>B28/$B$7</f>
         <v/>
       </c>
-      <c r="C29" s="21">
+      <c r="C29" s="22">
         <f>C28/$B$7</f>
         <v/>
       </c>
@@ -4625,10 +4645,10 @@
           <t>AI revenue ($B)</t>
         </is>
       </c>
-      <c r="B32" s="15" t="n">
+      <c r="B32" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="C32" s="15" t="n">
+      <c r="C32" s="16" t="n">
         <v>50</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -4773,7 +4793,7 @@
           <t>FY25 capex &gt;$88B incl leases; server life 2-6yr (FY25 10-K)</t>
         </is>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/789019/000095017025100235/msft-20250630.htm</t>
         </is>
@@ -4785,7 +4805,7 @@
           <t>FY26 ~$190B guide; 'two-thirds' short-lived = GPUs+CPUs (Q3 FY26 call)</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B42" s="23" t="inlineStr">
         <is>
           <t>https://www.fool.com/earnings/call-transcripts/2026/04/29/microsoft-msft-q3-2026-earnings-transcript/</t>
         </is>
@@ -4797,7 +4817,7 @@
           <t>AI revenue $37B annual run-rate (Q3 FY26)</t>
         </is>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B43" s="23" t="inlineStr">
         <is>
           <t>https://news.alphastreet.com/microsoft-msft-q3-fy2026-azure-hits-40-growth-as-ai-business-reaches-37-billion-run-rate/</t>
         </is>
@@ -4809,7 +4829,7 @@
           <t>~485k Hopper GPUs / ~$31B in 2024 (Omdia) - cross-checks accel capex</t>
         </is>
       </c>
-      <c r="B44" s="22" t="inlineStr">
+      <c r="B44" s="23" t="inlineStr">
         <is>
           <t>https://techcrunch.com/2024/12/18/microsoft-bought-nearly-500000-nvidia-hopper-chips-this-year/</t>
         </is>
@@ -4885,10 +4905,10 @@
           <t>Total capex ($B)</t>
         </is>
       </c>
-      <c r="B3" s="14" t="n">
+      <c r="B3" s="15" t="n">
         <v>91.40000000000001</v>
       </c>
-      <c r="C3" s="15" t="n">
+      <c r="C3" s="16" t="n">
         <v>185</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -4903,10 +4923,10 @@
           <t>Infra / data-center share</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="16" t="n">
+      <c r="C4" s="17" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -4921,10 +4941,10 @@
           <t>Server / short-lived share</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <v>0.6</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="17" t="n">
         <v>0.6</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -4939,10 +4959,10 @@
           <t>Accelerator share within servers</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="17" t="n">
         <v>0.67</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="17" t="n">
         <v>0.67</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -4957,7 +4977,7 @@
           <t>Market cap ($B, approx)</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="18" t="n">
         <v>4250</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -5072,11 +5092,11 @@
           <t>Fleet size (GPU-equiv)</t>
         </is>
       </c>
-      <c r="B16" s="18">
+      <c r="B16" s="19">
         <f>B12*1000000000/Inputs!$B$7</f>
         <v/>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="19">
         <f>C12*1000000000/Inputs!$B$7</f>
         <v/>
       </c>
@@ -5092,11 +5112,11 @@
           <t>Total wall power (MW)</t>
         </is>
       </c>
-      <c r="B17" s="18">
+      <c r="B17" s="19">
         <f>B16*Inputs!$B$8/1000</f>
         <v/>
       </c>
-      <c r="C17" s="18">
+      <c r="C17" s="19">
         <f>C16*Inputs!$B$8/1000</f>
         <v/>
       </c>
@@ -5112,11 +5132,11 @@
           <t>Daily energy (MWh)</t>
         </is>
       </c>
-      <c r="B18" s="18">
+      <c r="B18" s="19">
         <f>B17*24</f>
         <v/>
       </c>
-      <c r="C18" s="18">
+      <c r="C18" s="19">
         <f>C17*24</f>
         <v/>
       </c>
@@ -5128,11 +5148,11 @@
           <t>Daily all-in opex ($/day)</t>
         </is>
       </c>
-      <c r="B19" s="18">
+      <c r="B19" s="19">
         <f>B18*1000*Inputs!$B$9*(1+Inputs!$B$10)</f>
         <v/>
       </c>
-      <c r="C19" s="18">
+      <c r="C19" s="19">
         <f>C18*1000*Inputs!$B$9*(1+Inputs!$B$10)</f>
         <v/>
       </c>
@@ -5164,11 +5184,11 @@
           <t>Lifetime opex ($B)</t>
         </is>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="20">
         <f>B20*Inputs!$B$11/1000</f>
         <v/>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="20">
         <f>C20*Inputs!$B$11/1000</f>
         <v/>
       </c>
@@ -5246,11 +5266,11 @@
           <t>Sustained annual benefit ($B/yr)</t>
         </is>
       </c>
-      <c r="B27" s="20">
+      <c r="B27" s="21">
         <f>B25+B26/1000</f>
         <v/>
       </c>
-      <c r="C27" s="20">
+      <c r="C27" s="21">
         <f>C25+C26/1000</f>
         <v/>
       </c>
@@ -5266,11 +5286,11 @@
           <t>Capitalized value ($B)</t>
         </is>
       </c>
-      <c r="B28" s="13">
+      <c r="B28" s="14">
         <f>B27/Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="C28" s="13">
+      <c r="C28" s="14">
         <f>C27/Inputs!$B$6</f>
         <v/>
       </c>
@@ -5286,11 +5306,11 @@
           <t>% of market cap</t>
         </is>
       </c>
-      <c r="B29" s="21">
+      <c r="B29" s="22">
         <f>B28/$B$7</f>
         <v/>
       </c>
-      <c r="C29" s="21">
+      <c r="C29" s="22">
         <f>C28/$B$7</f>
         <v/>
       </c>
@@ -5312,10 +5332,10 @@
           <t>AI revenue ($B)</t>
         </is>
       </c>
-      <c r="B32" s="15" t="n">
+      <c r="B32" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="C32" s="15" t="n">
+      <c r="C32" s="16" t="n">
         <v>40</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -5460,7 +5480,7 @@
           <t>FY25 capex $91.4B; CFO 60% servers / 40% DC+net (Q4'25 call)</t>
         </is>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>https://www.fool.com/earnings/call-transcripts/2026/02/04/alphabet-googl-q4-2025-earnings-call-transcript/</t>
         </is>
@@ -5472,7 +5492,7 @@
           <t>FY26 guide $180-190B (Q1'26)</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B42" s="23" t="inlineStr">
         <is>
           <t>https://www.cnbc.com/2026/04/29/alphabet-googl-q1-2026-earnings.html</t>
         </is>
@@ -5484,7 +5504,7 @@
           <t>Server life 6yr; TPU at-cost TCO 20-50% below NVIDIA (SemiAnalysis)</t>
         </is>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B43" s="23" t="inlineStr">
         <is>
           <t>https://newsletter.semianalysis.com/p/tpuv7-google-takes-a-swing-at-the</t>
         </is>
@@ -5558,10 +5578,10 @@
           <t>Total capex ($B)</t>
         </is>
       </c>
-      <c r="B3" s="14" t="n">
+      <c r="B3" s="15" t="n">
         <v>128.3</v>
       </c>
-      <c r="C3" s="15" t="n">
+      <c r="C3" s="16" t="n">
         <v>220</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -5576,10 +5596,10 @@
           <t>Infra / data-center share</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <v>0.68</v>
       </c>
-      <c r="C4" s="16" t="n">
+      <c r="C4" s="17" t="n">
         <v>0.7</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -5594,10 +5614,10 @@
           <t>Server / short-lived share</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <v>0.65</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="17" t="n">
         <v>0.65</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -5612,10 +5632,10 @@
           <t>Accelerator share within servers</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="17" t="n">
         <v>0.67</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="17" t="n">
         <v>0.67</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -5630,7 +5650,7 @@
           <t>Market cap ($B, approx)</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="18" t="n">
         <v>2830</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -5745,11 +5765,11 @@
           <t>Fleet size (GPU-equiv)</t>
         </is>
       </c>
-      <c r="B16" s="18">
+      <c r="B16" s="19">
         <f>B12*1000000000/Inputs!$B$7</f>
         <v/>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="19">
         <f>C12*1000000000/Inputs!$B$7</f>
         <v/>
       </c>
@@ -5765,11 +5785,11 @@
           <t>Total wall power (MW)</t>
         </is>
       </c>
-      <c r="B17" s="18">
+      <c r="B17" s="19">
         <f>B16*Inputs!$B$8/1000</f>
         <v/>
       </c>
-      <c r="C17" s="18">
+      <c r="C17" s="19">
         <f>C16*Inputs!$B$8/1000</f>
         <v/>
       </c>
@@ -5785,11 +5805,11 @@
           <t>Daily energy (MWh)</t>
         </is>
       </c>
-      <c r="B18" s="18">
+      <c r="B18" s="19">
         <f>B17*24</f>
         <v/>
       </c>
-      <c r="C18" s="18">
+      <c r="C18" s="19">
         <f>C17*24</f>
         <v/>
       </c>
@@ -5801,11 +5821,11 @@
           <t>Daily all-in opex ($/day)</t>
         </is>
       </c>
-      <c r="B19" s="18">
+      <c r="B19" s="19">
         <f>B18*1000*Inputs!$B$9*(1+Inputs!$B$10)</f>
         <v/>
       </c>
-      <c r="C19" s="18">
+      <c r="C19" s="19">
         <f>C18*1000*Inputs!$B$9*(1+Inputs!$B$10)</f>
         <v/>
       </c>
@@ -5837,11 +5857,11 @@
           <t>Lifetime opex ($B)</t>
         </is>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="20">
         <f>B20*Inputs!$B$11/1000</f>
         <v/>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="20">
         <f>C20*Inputs!$B$11/1000</f>
         <v/>
       </c>
@@ -5919,11 +5939,11 @@
           <t>Sustained annual benefit ($B/yr)</t>
         </is>
       </c>
-      <c r="B27" s="20">
+      <c r="B27" s="21">
         <f>B25+B26/1000</f>
         <v/>
       </c>
-      <c r="C27" s="20">
+      <c r="C27" s="21">
         <f>C25+C26/1000</f>
         <v/>
       </c>
@@ -5939,11 +5959,11 @@
           <t>Capitalized value ($B)</t>
         </is>
       </c>
-      <c r="B28" s="13">
+      <c r="B28" s="14">
         <f>B27/Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="C28" s="13">
+      <c r="C28" s="14">
         <f>C27/Inputs!$B$6</f>
         <v/>
       </c>
@@ -5959,11 +5979,11 @@
           <t>% of market cap</t>
         </is>
       </c>
-      <c r="B29" s="21">
+      <c r="B29" s="22">
         <f>B28/$B$7</f>
         <v/>
       </c>
-      <c r="C29" s="21">
+      <c r="C29" s="22">
         <f>C28/$B$7</f>
         <v/>
       </c>
@@ -5985,10 +6005,10 @@
           <t>AI revenue ($B)</t>
         </is>
       </c>
-      <c r="B32" s="15" t="n">
+      <c r="B32" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="C32" s="15" t="n">
+      <c r="C32" s="16" t="n">
         <v>22</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -6133,7 +6153,7 @@
           <t>FY25 cash capex $128.3B; AWS 67.8% of net P&amp;E adds; server life 6-&gt;5yr (FY25 10-K)</t>
         </is>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1018724/000101872426000004/amzn-20251231.htm</t>
         </is>
@@ -6145,7 +6165,7 @@
           <t>~$200B 2026 capex, 'predominantly AWS' (Q4'25 call)</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B42" s="23" t="inlineStr">
         <is>
           <t>https://www.fool.com/earnings/call-transcripts/2026/02/05/amazon-amzn-q4-2025-earnings-call-transcript/</t>
         </is>
@@ -6157,7 +6177,7 @@
           <t>AWS AI revenue &gt;$15B annual run-rate (Q1'26, Jassy)</t>
         </is>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B43" s="23" t="inlineStr">
         <is>
           <t>https://www.bnnbloomberg.ca/business/artificial-intelligence/2026/04/09/amazon-cloud-units-ai-revenue-run-rate-exceeds-us15-billion-in-first-quarter-ceo-says/</t>
         </is>
@@ -6231,10 +6251,10 @@
           <t>Total capex ($B)</t>
         </is>
       </c>
-      <c r="B3" s="14" t="n">
+      <c r="B3" s="15" t="n">
         <v>72.2</v>
       </c>
-      <c r="C3" s="15" t="n">
+      <c r="C3" s="16" t="n">
         <v>137.5</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -6249,10 +6269,10 @@
           <t>Infra / data-center share</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="16" t="n">
+      <c r="C4" s="17" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -6267,10 +6287,10 @@
           <t>Server / short-lived share</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <v>0.65</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="17" t="n">
         <v>0.65</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -6285,10 +6305,10 @@
           <t>Accelerator share within servers</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="17" t="n">
         <v>0.74</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="17" t="n">
         <v>0.74</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -6303,7 +6323,7 @@
           <t>Market cap ($B, approx)</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="18" t="n">
         <v>1490</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -6418,11 +6438,11 @@
           <t>Fleet size (GPU-equiv)</t>
         </is>
       </c>
-      <c r="B16" s="18">
+      <c r="B16" s="19">
         <f>B12*1000000000/Inputs!$B$7</f>
         <v/>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="19">
         <f>C12*1000000000/Inputs!$B$7</f>
         <v/>
       </c>
@@ -6438,11 +6458,11 @@
           <t>Total wall power (MW)</t>
         </is>
       </c>
-      <c r="B17" s="18">
+      <c r="B17" s="19">
         <f>B16*Inputs!$B$8/1000</f>
         <v/>
       </c>
-      <c r="C17" s="18">
+      <c r="C17" s="19">
         <f>C16*Inputs!$B$8/1000</f>
         <v/>
       </c>
@@ -6458,11 +6478,11 @@
           <t>Daily energy (MWh)</t>
         </is>
       </c>
-      <c r="B18" s="18">
+      <c r="B18" s="19">
         <f>B17*24</f>
         <v/>
       </c>
-      <c r="C18" s="18">
+      <c r="C18" s="19">
         <f>C17*24</f>
         <v/>
       </c>
@@ -6474,11 +6494,11 @@
           <t>Daily all-in opex ($/day)</t>
         </is>
       </c>
-      <c r="B19" s="18">
+      <c r="B19" s="19">
         <f>B18*1000*Inputs!$B$9*(1+Inputs!$B$10)</f>
         <v/>
       </c>
-      <c r="C19" s="18">
+      <c r="C19" s="19">
         <f>C18*1000*Inputs!$B$9*(1+Inputs!$B$10)</f>
         <v/>
       </c>
@@ -6510,11 +6530,11 @@
           <t>Lifetime opex ($B)</t>
         </is>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="20">
         <f>B20*Inputs!$B$11/1000</f>
         <v/>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="20">
         <f>C20*Inputs!$B$11/1000</f>
         <v/>
       </c>
@@ -6592,11 +6612,11 @@
           <t>Sustained annual benefit ($B/yr)</t>
         </is>
       </c>
-      <c r="B27" s="20">
+      <c r="B27" s="21">
         <f>B25+B26/1000</f>
         <v/>
       </c>
-      <c r="C27" s="20">
+      <c r="C27" s="21">
         <f>C25+C26/1000</f>
         <v/>
       </c>
@@ -6612,11 +6632,11 @@
           <t>Capitalized value ($B)</t>
         </is>
       </c>
-      <c r="B28" s="13">
+      <c r="B28" s="14">
         <f>B27/Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="C28" s="13">
+      <c r="C28" s="14">
         <f>C27/Inputs!$B$6</f>
         <v/>
       </c>
@@ -6632,11 +6652,11 @@
           <t>% of market cap</t>
         </is>
       </c>
-      <c r="B29" s="21">
+      <c r="B29" s="22">
         <f>B28/$B$7</f>
         <v/>
       </c>
-      <c r="C29" s="21">
+      <c r="C29" s="22">
         <f>C28/$B$7</f>
         <v/>
       </c>
@@ -6658,10 +6678,10 @@
           <t>AI revenue ($B)</t>
         </is>
       </c>
-      <c r="B32" s="15" t="n">
+      <c r="B32" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="C32" s="15" t="n">
+      <c r="C32" s="16" t="n">
         <v>8</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -6806,7 +6826,7 @@
           <t>FY25 capex $72.2B incl finance leases (Q4/FY25 release)</t>
         </is>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>https://investor.atmeta.com/investor-news/press-release-details/2026/Meta-Reports-Fourth-Quarter-and-Full-Year-2025-Results/default.aspx</t>
         </is>
@@ -6818,7 +6838,7 @@
           <t>FY26 $125-145B guide; raise driven by HBM pricing (Q1'26 call)</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B42" s="23" t="inlineStr">
         <is>
           <t>https://www.fool.com/earnings/call-transcripts/2026/04/29/meta-meta-q1-2026-earnings-call-transcript/</t>
         </is>
@@ -6830,7 +6850,7 @@
           <t>&gt;1.3M GPUs by end-2025 (Zuckerberg) - cross-checks accel capex</t>
         </is>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B43" s="23" t="inlineStr">
         <is>
           <t>https://techcrunch.com/2025/01/24/mark-zuckerberg-says-meta-will-have-1-3m-gpus-for-ai-by-year-end/</t>
         </is>
@@ -6842,7 +6862,7 @@
           <t>Server life 5.5yr (-$2.9B depreciation)</t>
         </is>
       </c>
-      <c r="B44" s="22" t="inlineStr">
+      <c r="B44" s="23" t="inlineStr">
         <is>
           <t>https://www.thestack.technology/meta-extends-server-life-again-saving-it-2-9-billion/</t>
         </is>
@@ -6854,7 +6874,7 @@
           <t>~25% of capex to NVIDIA (Bloomberg) - accel-share basis</t>
         </is>
       </c>
-      <c r="B45" s="22" t="inlineStr">
+      <c r="B45" s="23" t="inlineStr">
         <is>
           <t>https://finance.yahoo.com/news/big-techs-spending-drove-nvidias-rise-154027146.html</t>
         </is>
@@ -6932,10 +6952,10 @@
           <t>Total capex ($B)</t>
         </is>
       </c>
-      <c r="B3" s="14" t="n">
+      <c r="B3" s="15" t="n">
         <v>21.2</v>
       </c>
-      <c r="C3" s="15" t="n">
+      <c r="C3" s="16" t="n">
         <v>55.7</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -6950,10 +6970,10 @@
           <t>Infra / data-center share</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <v>0.85</v>
       </c>
-      <c r="C4" s="16" t="n">
+      <c r="C4" s="17" t="n">
         <v>0.9</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -6968,10 +6988,10 @@
           <t>Server / short-lived share</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <v>0.75</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="17" t="n">
         <v>0.75</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -6986,10 +7006,10 @@
           <t>Accelerator share within servers</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="17" t="n">
         <v>0.7</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="17" t="n">
         <v>0.7</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -7004,7 +7024,7 @@
           <t>Market cap ($B, approx)</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="18" t="n">
         <v>433</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -7119,11 +7139,11 @@
           <t>Fleet size (GPU-equiv)</t>
         </is>
       </c>
-      <c r="B16" s="18">
+      <c r="B16" s="19">
         <f>B12*1000000000/Inputs!$B$7</f>
         <v/>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="19">
         <f>C12*1000000000/Inputs!$B$7</f>
         <v/>
       </c>
@@ -7139,11 +7159,11 @@
           <t>Total wall power (MW)</t>
         </is>
       </c>
-      <c r="B17" s="18">
+      <c r="B17" s="19">
         <f>B16*Inputs!$B$8/1000</f>
         <v/>
       </c>
-      <c r="C17" s="18">
+      <c r="C17" s="19">
         <f>C16*Inputs!$B$8/1000</f>
         <v/>
       </c>
@@ -7159,11 +7179,11 @@
           <t>Daily energy (MWh)</t>
         </is>
       </c>
-      <c r="B18" s="18">
+      <c r="B18" s="19">
         <f>B17*24</f>
         <v/>
       </c>
-      <c r="C18" s="18">
+      <c r="C18" s="19">
         <f>C17*24</f>
         <v/>
       </c>
@@ -7175,11 +7195,11 @@
           <t>Daily all-in opex ($/day)</t>
         </is>
       </c>
-      <c r="B19" s="18">
+      <c r="B19" s="19">
         <f>B18*1000*Inputs!$B$9*(1+Inputs!$B$10)</f>
         <v/>
       </c>
-      <c r="C19" s="18">
+      <c r="C19" s="19">
         <f>C18*1000*Inputs!$B$9*(1+Inputs!$B$10)</f>
         <v/>
       </c>
@@ -7211,11 +7231,11 @@
           <t>Lifetime opex ($B)</t>
         </is>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="20">
         <f>B20*Inputs!$B$11/1000</f>
         <v/>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="20">
         <f>C20*Inputs!$B$11/1000</f>
         <v/>
       </c>
@@ -7293,11 +7313,11 @@
           <t>Sustained annual benefit ($B/yr)</t>
         </is>
       </c>
-      <c r="B27" s="20">
+      <c r="B27" s="21">
         <f>B25+B26/1000</f>
         <v/>
       </c>
-      <c r="C27" s="20">
+      <c r="C27" s="21">
         <f>C25+C26/1000</f>
         <v/>
       </c>
@@ -7313,11 +7333,11 @@
           <t>Capitalized value ($B)</t>
         </is>
       </c>
-      <c r="B28" s="13">
+      <c r="B28" s="14">
         <f>B27/Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="C28" s="13">
+      <c r="C28" s="14">
         <f>C27/Inputs!$B$6</f>
         <v/>
       </c>
@@ -7333,11 +7353,11 @@
           <t>% of market cap</t>
         </is>
       </c>
-      <c r="B29" s="21">
+      <c r="B29" s="22">
         <f>B28/$B$7</f>
         <v/>
       </c>
-      <c r="C29" s="21">
+      <c r="C29" s="22">
         <f>C28/$B$7</f>
         <v/>
       </c>
@@ -7359,10 +7379,10 @@
           <t>AI revenue ($B)</t>
         </is>
       </c>
-      <c r="B32" s="15" t="n">
+      <c r="B32" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="C32" s="15" t="n">
+      <c r="C32" s="16" t="n">
         <v>15</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -7507,7 +7527,7 @@
           <t>FY25 capex $21.2B; FY26 ~$50B guide on $67B rev (CIO Dive)</t>
         </is>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>https://www.ciodive.com/news/oracle-capex-spike-cloud-ai-data-center/807721/</t>
         </is>
@@ -7519,7 +7539,7 @@
           <t>OCI run-rate ~$27B exiting FY25; IaaS $3.0B Q4 +52%; RPO $138B (Q4 FY25)</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B42" s="23" t="inlineStr">
         <is>
           <t>https://futurumgroup.com/insights/oracle-delivers-q4-fy-2025-results-with-27-cloud-growth-rpo-hits-138-billion/</t>
         </is>
@@ -7531,7 +7551,7 @@
           <t>FY26 OCI +77% to ~$18B; RPO $523B +433% on AI deals (Q2 FY26)</t>
         </is>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B43" s="23" t="inlineStr">
         <is>
           <t>https://futurumgroup.com/insights/oracle-q2-fy-2026-cloud-grows-capex-rises-for-ai-buildout/</t>
         </is>
@@ -7605,10 +7625,10 @@
           <t>Total capex ($B)</t>
         </is>
       </c>
-      <c r="B3" s="14" t="n">
+      <c r="B3" s="15" t="n">
         <v>12.7</v>
       </c>
-      <c r="C3" s="15" t="n">
+      <c r="C3" s="16" t="n">
         <v>55</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -7623,10 +7643,10 @@
           <t>Infra / data-center share</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="16" t="n">
+      <c r="C4" s="17" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -7641,10 +7661,10 @@
           <t>Server / short-lived share</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <v>0.79</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="17" t="n">
         <v>0.79</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -7659,10 +7679,10 @@
           <t>Accelerator share within servers</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="17" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -7677,7 +7697,7 @@
           <t>Market cap ($B, approx)</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="18" t="n">
         <v>1950</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -7792,11 +7812,11 @@
           <t>Fleet size (GPU-equiv)</t>
         </is>
       </c>
-      <c r="B16" s="18">
+      <c r="B16" s="19">
         <f>B12*1000000000/Inputs!$B$7</f>
         <v/>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="19">
         <f>C12*1000000000/Inputs!$B$7</f>
         <v/>
       </c>
@@ -7812,11 +7832,11 @@
           <t>Total wall power (MW)</t>
         </is>
       </c>
-      <c r="B17" s="18">
+      <c r="B17" s="19">
         <f>B16*Inputs!$B$8/1000</f>
         <v/>
       </c>
-      <c r="C17" s="18">
+      <c r="C17" s="19">
         <f>C16*Inputs!$B$8/1000</f>
         <v/>
       </c>
@@ -7832,11 +7852,11 @@
           <t>Daily energy (MWh)</t>
         </is>
       </c>
-      <c r="B18" s="18">
+      <c r="B18" s="19">
         <f>B17*24</f>
         <v/>
       </c>
-      <c r="C18" s="18">
+      <c r="C18" s="19">
         <f>C17*24</f>
         <v/>
       </c>
@@ -7848,11 +7868,11 @@
           <t>Daily all-in opex ($/day)</t>
         </is>
       </c>
-      <c r="B19" s="18">
+      <c r="B19" s="19">
         <f>B18*1000*Inputs!$B$9*(1+Inputs!$B$10)</f>
         <v/>
       </c>
-      <c r="C19" s="18">
+      <c r="C19" s="19">
         <f>C18*1000*Inputs!$B$9*(1+Inputs!$B$10)</f>
         <v/>
       </c>
@@ -7884,11 +7904,11 @@
           <t>Lifetime opex ($B)</t>
         </is>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="20">
         <f>B20*Inputs!$B$11/1000</f>
         <v/>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="20">
         <f>C20*Inputs!$B$11/1000</f>
         <v/>
       </c>
@@ -7966,11 +7986,11 @@
           <t>Sustained annual benefit ($B/yr)</t>
         </is>
       </c>
-      <c r="B27" s="20">
+      <c r="B27" s="21">
         <f>B25+B26/1000</f>
         <v/>
       </c>
-      <c r="C27" s="20">
+      <c r="C27" s="21">
         <f>C25+C26/1000</f>
         <v/>
       </c>
@@ -7986,11 +8006,11 @@
           <t>Capitalized value ($B)</t>
         </is>
       </c>
-      <c r="B28" s="13">
+      <c r="B28" s="14">
         <f>B27/Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="C28" s="13">
+      <c r="C28" s="14">
         <f>C27/Inputs!$B$6</f>
         <v/>
       </c>
@@ -8006,11 +8026,11 @@
           <t>% of market cap</t>
         </is>
       </c>
-      <c r="B29" s="21">
+      <c r="B29" s="22">
         <f>B28/$B$7</f>
         <v/>
       </c>
-      <c r="C29" s="21">
+      <c r="C29" s="22">
         <f>C28/$B$7</f>
         <v/>
       </c>
@@ -8032,10 +8052,10 @@
           <t>AI revenue ($B)</t>
         </is>
       </c>
-      <c r="B32" s="15" t="n">
+      <c r="B32" s="16" t="n">
         <v>0.3</v>
       </c>
-      <c r="C32" s="15" t="n">
+      <c r="C32" s="16" t="n">
         <v>1</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -8180,7 +8200,7 @@
           <t>S-1 registration statement (SEC EDGAR)</t>
         </is>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1181412/000162828026036936/spaceexplorationtechnologi.htm</t>
         </is>
@@ -8192,7 +8212,7 @@
           <t>S-1 financials &amp; AI breakdown (Hargreaves Lansdown)</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B42" s="23" t="inlineStr">
         <is>
           <t>https://www.hl.co.uk/news/inside-spacexs-ipo-filing-revenue-starlink-ai-and-key-financials</t>
         </is>
@@ -8204,7 +8224,7 @@
           <t>$12.7B AI capex = ~60% of capex; COLOSSUS buildout (Investing.com)</t>
         </is>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B43" s="23" t="inlineStr">
         <is>
           <t>https://www.investing.com/analysis/spacex-is-quietly-becoming-an-ai-compute-and-orbital-infrastructure-company-200681776</t>
         </is>
@@ -8216,7 +8236,7 @@
           <t>AI1 orbital data centers; Anthropic as compute customer (DCD)</t>
         </is>
       </c>
-      <c r="B44" s="22" t="inlineStr">
+      <c r="B44" s="23" t="inlineStr">
         <is>
           <t>https://www.datacenterdynamics.com/en/news/spacex-ipo-musks-firm-set-to-launch-first-orbital-data-center-ai1-satellites-in-2027-will-put-compute-on-starlink-craft/</t>
         </is>
@@ -8270,7 +8290,7 @@
           <t>Memory reduction factor</t>
         </is>
       </c>
-      <c r="B2" s="23" t="n">
+      <c r="B2" s="24" t="n">
         <v>100</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -8290,7 +8310,7 @@
           <t>FLOPs reduction factor</t>
         </is>
       </c>
-      <c r="B3" s="23">
+      <c r="B3" s="24">
         <f>$B$24</f>
         <v/>
       </c>
@@ -8311,7 +8331,7 @@
           <t>Memory share of GPU cost (BOM)</t>
         </is>
       </c>
-      <c r="B4" s="24" t="n">
+      <c r="B4" s="25" t="n">
         <v>0.6</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -8331,7 +8351,7 @@
           <t>Opex / energy reduction factor</t>
         </is>
       </c>
-      <c r="B5" s="23">
+      <c r="B5" s="24">
         <f>B20</f>
         <v/>
       </c>
@@ -8352,7 +8372,7 @@
           <t>Discount rate</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n">
+      <c r="B6" s="25" t="n">
         <v>0.06</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -8372,7 +8392,7 @@
           <t>Fully-loaded cost per GPU</t>
         </is>
       </c>
-      <c r="B7" s="25" t="n">
+      <c r="B7" s="26" t="n">
         <v>50000</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -8392,7 +8412,7 @@
           <t>Wall power per GPU</t>
         </is>
       </c>
-      <c r="B8" s="23" t="n">
+      <c r="B8" s="24" t="n">
         <v>1.8</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -8412,7 +8432,7 @@
           <t>Electricity rate</t>
         </is>
       </c>
-      <c r="B9" s="23" t="n">
+      <c r="B9" s="24" t="n">
         <v>0.08</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -8432,7 +8452,7 @@
           <t>Cooling/ops overhead on energy</t>
         </is>
       </c>
-      <c r="B10" s="24" t="n">
+      <c r="B10" s="25" t="n">
         <v>0.25</v>
       </c>
       <c r="C10" t="inlineStr">
@@ -8452,7 +8472,7 @@
           <t>Fleet useful life</t>
         </is>
       </c>
-      <c r="B11" s="23" t="n">
+      <c r="B11" s="24" t="n">
         <v>4</v>
       </c>
       <c r="C11" t="inlineStr">
@@ -8472,7 +8492,7 @@
           <t>SpaceX market cap</t>
         </is>
       </c>
-      <c r="B12" s="26" t="n">
+      <c r="B12" s="27" t="n">
         <v>1950</v>
       </c>
       <c r="C12" t="inlineStr">
@@ -8492,7 +8512,7 @@
           <t>Datacenter scaling factor</t>
         </is>
       </c>
-      <c r="B13" s="24" t="n">
+      <c r="B13" s="25" t="n">
         <v>0</v>
       </c>
       <c r="C13" t="inlineStr">
@@ -8512,7 +8532,7 @@
           <t>Named share of global AI capex</t>
         </is>
       </c>
-      <c r="B14" s="24" t="n">
+      <c r="B14" s="25" t="n">
         <v>0.8</v>
       </c>
       <c r="C14" t="inlineStr">
@@ -8542,7 +8562,7 @@
           <t>Compute share of GPU cost</t>
         </is>
       </c>
-      <c r="B16" s="21">
+      <c r="B16" s="22">
         <f>1-B4</f>
         <v/>
       </c>
@@ -8558,7 +8578,7 @@
           <t>Memory cost fraction after reduction</t>
         </is>
       </c>
-      <c r="B17" s="27">
+      <c r="B17" s="28">
         <f>B4/B2</f>
         <v/>
       </c>
@@ -8574,7 +8594,7 @@
           <t>Compute cost fraction after reduction</t>
         </is>
       </c>
-      <c r="B18" s="27">
+      <c r="B18" s="28">
         <f>B16/B3</f>
         <v/>
       </c>
@@ -8590,7 +8610,7 @@
           <t>Residual cost fraction</t>
         </is>
       </c>
-      <c r="B19" s="21">
+      <c r="B19" s="22">
         <f>B17+B18</f>
         <v/>
       </c>
@@ -8606,7 +8626,7 @@
           <t>COST-WEIGHTED reduction factor</t>
         </is>
       </c>
-      <c r="B20" s="12">
+      <c r="B20" s="13">
         <f>1/B19</f>
         <v/>
       </c>
@@ -8637,7 +8657,7 @@
           <t>Equal-quality parameter ratio at 1T</t>
         </is>
       </c>
-      <c r="B23" s="28" t="n">
+      <c r="B23" s="29" t="n">
         <v>4.2185</v>
       </c>
       <c r="C23" t="inlineStr">
@@ -8657,7 +8677,7 @@
           <t>TODAY compute lever = serving lever x ratio</t>
         </is>
       </c>
-      <c r="B24" s="29">
+      <c r="B24" s="30">
         <f>188.0305*$B$23</f>
         <v/>
       </c>
@@ -8678,7 +8698,7 @@
           <t>CEILING compute lever (campaign landed)</t>
         </is>
       </c>
-      <c r="B25" s="19">
+      <c r="B25" s="20">
         <f>193.3376*$B$23</f>
         <v/>
       </c>
@@ -8754,15 +8774,15 @@
           <t>Efficient acquisition ($B)</t>
         </is>
       </c>
-      <c r="B3" s="19">
+      <c r="B3" s="20">
         <f>SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$24))</f>
         <v/>
       </c>
-      <c r="C3" s="19">
+      <c r="C3" s="20">
         <f>SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$25))</f>
         <v/>
       </c>
-      <c r="D3" s="19">
+      <c r="D3" s="20">
         <f>SpaceX!$B$12/(Inputs!$B$20)</f>
         <v/>
       </c>
@@ -8773,15 +8793,15 @@
           <t>Capex avoided/yr ($B)</t>
         </is>
       </c>
-      <c r="B4" s="19">
+      <c r="B4" s="20">
         <f>SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$24))</f>
         <v/>
       </c>
-      <c r="C4" s="19">
+      <c r="C4" s="20">
         <f>SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$25))</f>
         <v/>
       </c>
-      <c r="D4" s="19">
+      <c r="D4" s="20">
         <f>SpaceX!$B$12-SpaceX!$B$12/(Inputs!$B$20)</f>
         <v/>
       </c>
@@ -8811,15 +8831,15 @@
           <t>Sustained annual benefit ($B)</t>
         </is>
       </c>
-      <c r="B6" s="19">
+      <c r="B6" s="20">
         <f>(SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$24)))+SpaceX!$B$26/1000</f>
         <v/>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="20">
         <f>(SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$25)))+SpaceX!$B$26/1000</f>
         <v/>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="20">
         <f>(SpaceX!$B$12-SpaceX!$B$12/(Inputs!$B$20))+SpaceX!$B$26/1000</f>
         <v/>
       </c>
@@ -8830,15 +8850,15 @@
           <t>Capitalized value ($B)</t>
         </is>
       </c>
-      <c r="B7" s="18">
+      <c r="B7" s="19">
         <f>((SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$24)))+SpaceX!$B$26/1000)/Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="19">
         <f>((SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$25)))+SpaceX!$B$26/1000)/Inputs!$B$6</f>
         <v/>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="19">
         <f>((SpaceX!$B$12-SpaceX!$B$12/(Inputs!$B$20))+SpaceX!$B$26/1000)/Inputs!$B$6</f>
         <v/>
       </c>
@@ -8849,15 +8869,15 @@
           <t>% of market cap</t>
         </is>
       </c>
-      <c r="B8" s="21">
+      <c r="B8" s="22">
         <f>(((SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$24)))+SpaceX!$B$26/1000)/Inputs!$B$6)/Inputs!$B$12</f>
         <v/>
       </c>
-      <c r="C8" s="21">
+      <c r="C8" s="22">
         <f>(((SpaceX!$B$12-SpaceX!$B$12/(1/(Inputs!$B$4/Inputs!$B$2+(1-Inputs!$B$4)/Inputs!$B$25)))+SpaceX!$B$26/1000)/Inputs!$B$6)/Inputs!$B$12</f>
         <v/>
       </c>
-      <c r="D8" s="21">
+      <c r="D8" s="22">
         <f>(((SpaceX!$B$12-SpaceX!$B$12/(Inputs!$B$20))+SpaceX!$B$26/1000)/Inputs!$B$6)/Inputs!$B$12</f>
         <v/>
       </c>
@@ -8919,19 +8939,19 @@
           <t>8k</t>
         </is>
       </c>
-      <c r="B14" s="27" t="n">
+      <c r="B14" s="28" t="n">
         <v>0.005899250258734248</v>
       </c>
-      <c r="C14" s="21" t="n">
+      <c r="C14" s="22" t="n">
         <v>0.05208995366081766</v>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="19" t="n">
         <v>50.29665229131971</v>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="19" t="n">
         <v>51.47706163855121</v>
       </c>
-      <c r="F14" s="21" t="n">
+      <c r="F14" s="22" t="n">
         <v>0.02346894462069837</v>
       </c>
     </row>
@@ -8941,19 +8961,19 @@
           <t>32k</t>
         </is>
       </c>
-      <c r="B15" s="27" t="n">
+      <c r="B15" s="28" t="n">
         <v>0.002981160980333002</v>
       </c>
-      <c r="C15" s="21" t="n">
+      <c r="C15" s="22" t="n">
         <v>0.05196631516233694</v>
       </c>
-      <c r="D15" s="18" t="n">
+      <c r="D15" s="19" t="n">
         <v>200.6239377794075</v>
       </c>
-      <c r="E15" s="18" t="n">
+      <c r="E15" s="19" t="n">
         <v>205.3209324850361</v>
       </c>
-      <c r="F15" s="21" t="n">
+      <c r="F15" s="22" t="n">
         <v>0.02341193557267873</v>
       </c>
     </row>
@@ -8963,19 +8983,19 @@
           <t>128k (pinned)</t>
         </is>
       </c>
-      <c r="B16" s="27" t="n">
+      <c r="B16" s="28" t="n">
         <v>0.002359266800993781</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="22" t="n">
         <v>0.06235575593664416</v>
       </c>
-      <c r="D16" s="18" t="n">
+      <c r="D16" s="19" t="n">
         <v>793.2064858179596</v>
       </c>
-      <c r="E16" s="18" t="n">
+      <c r="E16" s="19" t="n">
         <v>815.5945097216911</v>
       </c>
-      <c r="F16" s="21" t="n">
+      <c r="F16" s="22" t="n">
         <v>0.0282247110985796</v>
       </c>
     </row>
@@ -8985,19 +9005,19 @@
           <t>256k</t>
         </is>
       </c>
-      <c r="B17" s="27" t="n">
+      <c r="B17" s="28" t="n">
         <v>0.00230050437708008</v>
       </c>
-      <c r="C17" s="21" t="n">
+      <c r="C17" s="22" t="n">
         <v>0.08221381175542121</v>
       </c>
-      <c r="D17" s="18" t="n">
+      <c r="D17" s="19" t="n">
         <v>1552.723400990788</v>
       </c>
-      <c r="E17" s="18" t="n">
+      <c r="E17" s="19" t="n">
         <v>1611.029390134314</v>
       </c>
-      <c r="F17" s="21" t="n">
+      <c r="F17" s="22" t="n">
         <v>0.03755078921739785</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Pre-send review fixes: external-content scrub at workbook write time (mechanism terms, internal names/paths); Evidence memory-floor note corrected (was 'far below 100x'); crossover re-based to T~13,008 everywhere; retired x9.2 removed from Methodology illustration; KV 197-vs-156 KB reconciled; Sensitivity/TABS descriptions updated; FY26 % cut cell; mcap note date
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -909,6 +909,10 @@
         <f>SUM(Microsoft!$C$37,Alphabet!$C$37,Amazon!$C$37,Meta!$C$37,Oracle!$C$37,SpaceX!$C$37)</f>
         <v/>
       </c>
+      <c r="H13" s="12">
+        <f>SUM(Microsoft!$C$36,Alphabet!$C$36,Amazon!$C$36,Meta!$C$36,Oracle!$C$36,SpaceX!$C$36)/(SUM(Microsoft!$C$33,Alphabet!$C$33,Amazon!$C$33,Meta!$C$33,Oracle!$C$33,SpaceX!$C$33)+SUM(Microsoft!$C$34,Alphabet!$C$34,Amazon!$C$34,Meta!$C$34,Oracle!$C$34,SpaceX!$C$34))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1140,7 +1144,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>SpaceX value across reduction tiers (10x/30x/100x/cost-weighted)</t>
+          <t>SpaceX value across the Today / Ceiling / live cost-weighted tiers + context sensitivity</t>
         </is>
       </c>
     </row>
@@ -1159,43 +1163,56 @@
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Evidence</t>
+          <t>ServingTraining</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>BOM cost split, accelerator-share data, own-silicon TCO, filing top-lines</t>
+          <t>the serving/training measurement ledger behind the levers — status-tagged (MEASURED / ESTIMATE / TARGET)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>BOM cost split, accelerator-share data, own-silicon TCO, filing top-lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
           <t>Methodology</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>step-by-step logic, caveats, sources</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>Legend: yellow = assumption / lever (each maps to a slider in the Streamlit app)  ·  green = disclosed filing or market data  ·  blue = derived formula.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="B32:H32"/>
+    <mergeCell ref="B35:H35"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="B30:H30"/>
-    <mergeCell ref="A36:H36"/>
     <mergeCell ref="B29:H29"/>
     <mergeCell ref="B33:H33"/>
+    <mergeCell ref="A37:H37"/>
     <mergeCell ref="B34:H34"/>
     <mergeCell ref="B31:H31"/>
   </mergeCells>
@@ -1467,7 +1484,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SERVING &amp; TRAINING — measured 2026-08-07/08 (2/4/8 x H100), priced at the CostLadder rent mid ($2.50/GPU-hr). Source: bdm/docs/deck/build/derived.json (keys in ai_capex_model.MEASURED).</t>
+          <t>SERVING &amp; TRAINING — measured 2026-08-07/08 (2/4/8 x H100), priced at the CostLadder rent mid ($2.50/GPU-hr). Source: internal measurement archive (keys in the model).</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1852,7 +1869,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>SCOPE: the serving and training blocks below are component-scope systems benches (bAttention d1536 fwd+bwd h-recurrence sub-block vs transformer d2048 forward-only layer); every speedup there is each family vs its OWN 1-GPU baseline. The prefill lanes quoted further down are cross-family: 16-bit parameter-matched at block scope (the fp32 full-model sweep is retired to an assumption row).</t>
+          <t>SCOPE: the serving and training blocks below are component-scope systems benches (bAttention d1536 fwd+bwd h-internal dynamics sub-block vs transformer d2048 forward-only layer); every speedup there is each family vs its OWN 1-GPU baseline. The prefill lanes quoted further down are cross-family: 16-bit parameter-matched at block scope (the fp32 full-model sweep is retired to an assumption row).</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2090,7 @@
       <c r="E55" s="39" t="inlineStr"/>
       <c r="F55" s="39" t="inlineStr">
         <is>
-          <t>Status — derived.json key</t>
+          <t>Status — internal measurement archive key</t>
         </is>
       </c>
     </row>
@@ -2218,18 +2235,18 @@
     <row r="63">
       <c r="A63" s="46" t="inlineStr">
         <is>
-          <t>Stepped vs scanned training</t>
+          <t>Token-by-token vs production training</t>
         </is>
       </c>
       <c r="B63" s="47" t="inlineStr">
         <is>
-          <t>x24 cost to step the recurrence token-by-token</t>
+          <t>x24 cost to run training token-by-token instead of the production path</t>
         </is>
       </c>
       <c r="C63" s="46" t="inlineStr"/>
       <c r="F63" s="44" t="inlineStr">
         <is>
-          <t>MEASURED — stepped_vs_scanned</t>
+          <t>MEASURED — token-by-token ratio</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2265,7 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Training, prefill and decode point in OPPOSITE directions at today's kernel maturity, so a single number cannot represent them. Training is still a loss at short sequence, but a much smaller one since the 2026-08-24 kernel re-base (transformer 1.72x faster at T=2,048 and 1.79x at T=8,192, crossover near T~32,000; it was 5.3-9.6x with a crossover near T~88,000 on the pre-campaign d1152 sweep). Prefill crosses over near 65k context. Decode crosses in our favour near ~30k context. The lever is therefore blended over the workload: per generated token, in:out input tokens through prefill plus one token through decode, using measured per-GPU throughput at each family's own concurrency ceiling, the transformer granted no KV compression. At the default operating point (10:1, 64k context, training share 0): prefill x1.17, decode x2.20, blended x2.19, with decode ~99.7% of transformer serving cost. The decode half is a MEMORY CEILING, not a per-token result - at one stream and 64k the transformer decodes a token more cheaply than we do - and it crosses 1 at ~30k context, below which the transformer wins. Granting it KV/8 divides our decode lever by 8. A training share above ~0.30 also takes the blend below 1 (it was ~0.06 before the kernel re-base). All are reachable in the live model. NOTE (2026-09-01): this blend was measured on the PRE-CAMPAIGN kernels and no longer sets the workbook's flop_factor — the scenario levers at Inputs B24/B25 fold in the banked kernel results and the aggregate-decode estimate.</t>
+          <t>Training, prefill and decode point in OPPOSITE directions at today's kernel maturity, so a single number cannot represent them. Training is still a loss at short sequence, but a much smaller one since the 2026-08-24 kernel re-base (transformer 1.72x faster at T=2,048 and 1.79x at T=8,192, crossover near T~13,000 (2026-08-29 anchor); it was 5.3-9.6x with a crossover near T~88,000 on the pre-campaign d1152 sweep). Prefill crosses over near 65k context. Decode crosses in our favour near ~30k context. The lever is therefore blended over the workload: per generated token, in:out input tokens through prefill plus one token through decode, using measured per-GPU throughput at each family's own concurrency ceiling, the transformer granted no KV compression. At the default operating point (10:1, 64k context, training share 0): prefill x1.17, decode x2.20, blended x2.19, with decode ~99.7% of transformer serving cost. The decode half is a MEMORY CEILING, not a per-token result - at one stream and 64k the transformer decodes a token more cheaply than we do - and it crosses 1 at ~30k context, below which the transformer wins. Granting it KV/8 divides our decode lever by 8. A training share above ~0.30 also takes the blend below 1 (it was ~0.06 before the kernel re-base). All are reachable in the live model. NOTE (2026-09-01): this blend was measured on the PRE-CAMPAIGN kernels and no longer sets the workbook's flop_factor — the scenario levers at Inputs B24/B25 fold in the banked kernel results and the aggregate-decode estimate.</t>
         </is>
       </c>
     </row>
@@ -2267,7 +2284,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Training compute ~ 6*N*D FLOPs. At equal quality we need N/s parameters, where s(N) is the FIT-DERIVED equal-quality parameter ratio (the same sealed 2026-08-14 refit as the compute lever). Two token regimes differ by exactly one power of s: COMPUTE-OPTIMAL (Chinchilla, D proportional to N -&gt; cost ratio s^2/r) and FIXED TOKEN BUDGET (D equal on both arms -&gt; s/r). r(T) is the step-time ratio at matched parameters: MEASURED at T=2,048 (1.72x, 2026-08-25) and T=8,192 (1.79x, 2026-08-24), MODELED beyond. Above 1.00 we are cheaper to train to the same quality. The 256k column is MODELED from the per-token cost form -- the transformer pays base + attn*T per token (FlashAttention is linear per token), our O(1) recurrent state pays ~flat -- with base and attn fitted to the 2k and 8k cells ONLY. The fit is flat -- the +5.8%-per-4x residual and the B4/T32,768 ~parity cell that shared it are RETIRED 2026-08-25 as a B4 occupancy artifact -- and puts the crossover at a PROJECTED T~13,008. The old constant-decay extrapolation (0.758 per 4x) is kept as the CONSERVATIVE bound and reads 0.65 at 256k against this form's 0.10. The fits cross at 392M, so below that we need MORE parameters, and every row past ~1B extrapolates beyond the measured 47M-663M rungs. Peak training memory (1.58x measured, 0.88x targeted) is NOT in this model: it caps per-GPU batch density, not FLOPs. Chart: paper/figures/vc_memo_training_cost_scaling.png</t>
+          <t>Training compute ~ 6*N*D FLOPs. At equal quality we need N/s parameters, where s(N) is the FIT-DERIVED equal-quality parameter ratio (the same sealed 2026-08-14 refit as the compute lever). Two token regimes differ by exactly one power of s: COMPUTE-OPTIMAL (Chinchilla, D proportional to N -&gt; cost ratio s^2/r) and FIXED TOKEN BUDGET (D equal on both arms -&gt; s/r). r(T) is the step-time ratio at matched parameters: MEASURED at T=2,048 (1.72x, 2026-08-25) and T=8,192 (1.79x, 2026-08-24), MODELED beyond. Above 1.00 we are cheaper to train to the same quality. The 256k column is MODELED from the per-token cost form -- the transformer pays base + attn*T per token (FlashAttention is linear per token), our O(1) internal state pays ~flat -- with base and attn fitted to the 2k and 8k cells ONLY. The fit is flat -- the +5.8%-per-4x residual and the B4/T32,768 ~parity cell that shared it are RETIRED 2026-08-25 as a B4 occupancy artifact -- and puts the crossover at a PROJECTED T~13,008. The old constant-decay extrapolation (0.758 per 4x) is kept as the CONSERVATIVE bound and reads 0.65 at 256k against this form's 0.10. The fits cross at 392M, so below that we need MORE parameters, and every row past ~1B extrapolates beyond the measured 47M-663M rungs. Peak training memory (1.58x measured, 0.88x targeted) is NOT in this model: it caps per-GPU batch density, not FLOPs. Chart: internal measurement archive</t>
         </is>
       </c>
     </row>
@@ -2606,14 +2623,14 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>EXCLUDED, AND IT RUNS OUR WAY. At 262k+ the transformer additionally pays sequence-parallelism and activation-memory costs an O(1) recurrent state avoids: its KV grows at 156 KB per token of context per stream, which is what forces sharding, ring/Ulysses attention and their communication overhead. Our own measurement shows the asymmetry in the small -- from 2k to 8k the peak-memory ratio went 1.579x -&gt; 1.567x, i.e. flat-to-falling in context, while the absolute footprint the transformer must shard keeps growing. None of it is in the cost model above, which counts step time only, so the omission is CONSERVATIVE. Quantifying it needs a multi-GPU long-context TRAINING receipt we do not have.</t>
+          <t>EXCLUDED, AND IT RUNS OUR WAY. At 262k+ the transformer additionally pays sequence-parallelism and activation-memory costs an O(1) internal state avoids: its KV grows at 156 KB per token of context per stream, which is what forces sharding, ring/Ulysses attention and their communication overhead. Our own measurement shows the asymmetry in the small -- from 2k to 8k the peak-memory ratio went 1.579x -&gt; 1.567x, i.e. flat-to-falling in context, while the absolute footprint the transformer must shard keeps growing. None of it is in the cost model above, which counts step time only, so the omission is CONSERVATIVE. Quantifying it needs a multi-GPU long-context TRAINING receipt we do not have.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>The prefill component, 16-bit and parameter-matched — the lane the competition serves in. Parameter counts exactly matched, 1 layer, batch 16, 1 x H100 80GB HBM3, 2026-07-21 — x4.02 at d512/1M, x3.83 at d1024/1M, x2.01 at d2048/262k. The fp32 full-model sweep and the own-baseline 16-bit-IO training gate are retired to one assumption row each below. Receipts: experiments/paper_figures/output/matched_d{512,1024,2048}_h100.json</t>
+          <t>The prefill component, 16-bit and parameter-matched — the lane the competition serves in. Parameter counts exactly matched, 1 layer, batch 16, 1 x H100 80GB HBM3, 2026-07-21 — x4.02 at d512/1M, x3.83 at d1024/1M, x2.01 at d2048/262k. The fp32 full-model sweep and the own-baseline 16-bit-IO training gate are retired to one assumption row each below. Receipts: internal measurement archive{512,1024,2048}internal measurement archive</t>
         </is>
       </c>
     </row>
@@ -2858,7 +2875,7 @@
       </c>
       <c r="F103" s="44" t="inlineStr">
         <is>
-          <t>campaign_landed_flop_lever(); aggregate-decode receipt PENDING (decode_aggregate_receipt_20260831_instructions.md)</t>
+          <t>the model; aggregate-decode receipt PENDING (internal measurement archive)</t>
         </is>
       </c>
     </row>
@@ -2880,7 +2897,7 @@
       </c>
       <c r="F104" s="44" t="inlineStr">
         <is>
-          <t>quality_fit_v4.json param_matching; fits over the sealed rope-convention ladder</t>
+          <t>internal measurement archive param_matching; fits over the sealed rope-convention ladder</t>
         </is>
       </c>
     </row>
@@ -2902,7 +2919,7 @@
       </c>
       <c r="F105" s="44" t="inlineStr">
         <is>
-          <t>2026-08-24 GH200 megakernel measurement; prior: dtype_trio_v4.json rows[fp16]</t>
+          <t>2026-08-24 GH200 megakernel measurement; prior: internal measurement archive rows[fp16]</t>
         </is>
       </c>
     </row>
@@ -2914,7 +2931,7 @@
       </c>
       <c r="B106" s="44" t="inlineStr">
         <is>
-          <t>x1.579 at T=2,048 (17,087.5 vs 10,823.6 MiB) and x1.567 at T=8,192, down from x2.829 the same morning. This is TRAINING peak memory and is NOT the mem_factor lever, which is SERVING state (O(1) recurrent state vs O(T) KV cache) and is unaffected. It is not an input to the cost model; it caps per-GPU batch density</t>
+          <t>x1.579 at T=2,048 (17,087.5 vs 10,823.6 MiB) and x1.567 at T=8,192, down from x2.829 the same morning. This is TRAINING peak memory and is NOT the mem_factor lever, which is SERVING state (O(1) internal state vs O(T) KV cache) and is unaffected. It is not an input to the cost model; it caps per-GPU batch density</t>
         </is>
       </c>
       <c r="E106" s="55" t="inlineStr">
@@ -2936,7 +2953,7 @@
       </c>
       <c r="B107" s="44" t="inlineStr">
         <is>
-          <t>the funded 8k-win gate is a T=8,192 step at or below 83.08 ms, i.e. x1.786 still to remove (44% of the step). Named levers: recompute removal ~-12.8 ms; backward-fold + occupancy redesign (~3x headroom in the dominant fused kernel); copies elimination (24.8% of the step). Memory target x0.88 (parity or below). CEILING_PREFILL_SPEEDUP = the MEASURED x3.936 already banked x this x1.786 target</t>
+          <t>the funded 8k-win gate is a T=8,192 step at or below 83.08 ms, i.e. x1.786 still to remove (44% of the step). Named levers: recompute removal ~-12.8 ms; backward-fold + occupancy redesign (~3x headroom in the dominant fused kernel); copies elimination (24.8% of the step). Memory target x0.88 (parity or below). the model = the MEASURED x3.936 already banked x this x1.786 target</t>
         </is>
       </c>
       <c r="E107" s="56" t="inlineStr">
@@ -2958,7 +2975,7 @@
       </c>
       <c r="B108" s="44" t="inlineStr">
         <is>
-          <t>at matched tokens/step, 2k -&gt; 8k (4x context): our step grows x1.000, the transformer's x1.319, so the ratio decays x0.758 per 4x. The equal-token B4/T32,768 ~parity cell is RETIRED 2026-08-25 as a B4 occupancy artifact (it shared the retired growth residual); the flat per-token model puts the crossover at a PROJECTED T~16,900. Holding the old x0.802 decay constant instead would say x1.43 at 32k and a crossover near T~310,000 - that is the CONSERVATIVE extrapolation, because the transformer's quadratic attention term makes its per-4x growth rise with context while ours stays flat</t>
+          <t>at matched tokens/step, 2k -&gt; 8k (4x context): our step grows x1.000, the transformer's x1.319, so the ratio decays x0.758 per 4x. The equal-token B4/T32,768 ~parity cell is RETIRED 2026-08-25 as a B4 occupancy artifact (it shared the retired growth residual); the flat per-token model puts the crossover at a PROJECTED T~13,000 (the model, 2026-08-29 anchor). Holding the old x0.802 decay constant instead would say x1.43 at 32k and a crossover near T~310,000 - that is the CONSERVATIVE extrapolation, because the transformer's quadratic attention term makes its per-4x growth rise with context while ours stays flat</t>
         </is>
       </c>
       <c r="E108" s="56" t="inlineStr">
@@ -2990,7 +3007,7 @@
       </c>
       <c r="F109" s="44" t="inlineStr">
         <is>
-          <t>TRAIN_COST_FIT_20260824, TRAINING_CURRICULA, training_advantage_mix()</t>
+          <t>the model, the model, the model</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3019,7 @@
       </c>
       <c r="B110" s="44" t="inlineStr">
         <is>
-          <t>at 262k+ the transformer additionally pays sequence-parallelism and activation-memory costs that an O(1) recurrent state does not: its KV grows at 156 KB per token of context per stream, which is what forces sharding, ring/Ulysses attention and their communication overhead. Our own measurement shows the asymmetry in the small: peak training memory grew only x0.993 relative to the transformer's from 2k to 8k (x1.579 -&gt; x1.567), i.e. the ratio is FLAT-to-falling in context while the absolute gap the transformer must shard grows. NOT in the cost model — the training advantage above counts FLOPs/step-time only, so the direction of this omission is CONSERVATIVE (it understates us at long context). Quantifying it needs a multi-GPU long-context training receipt we do not have</t>
+          <t>at 262k+ the transformer additionally pays sequence-parallelism and activation-memory costs that an O(1) internal state does not: its KV grows at 156 KB per token of context per stream, which is what forces sharding, ring/Ulysses attention and their communication overhead. Our own measurement shows the asymmetry in the small: peak training memory grew only x0.993 relative to the transformer's from 2k to 8k (x1.579 -&gt; x1.567), i.e. the ratio is FLAT-to-falling in context while the absolute gap the transformer must shard grows. NOT in the cost model — the training advantage above counts FLOPs/step-time only, so the direction of this omission is CONSERVATIVE (it understates us at long context). Quantifying it needs a multi-GPU long-context training receipt we do not have</t>
         </is>
       </c>
       <c r="E110" s="56" t="inlineStr">
@@ -3012,7 +3029,7 @@
       </c>
       <c r="F110" s="44" t="inlineStr">
         <is>
-          <t>KERNEL_CAMPAIGN_20260824 mem_ratio_2k/8k; KV_MB_PER_TOKEN_PER_STREAM</t>
+          <t>the model mem_ratio_2k/8k; the model</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3117,7 @@
       </c>
       <c r="F114" s="44" t="inlineStr">
         <is>
-          <t>deck_decode_d2048_bf16_gh200_20260814.json; DECODE_THROUGHPUT_20260814</t>
+          <t>internal measurement archive; the model</t>
         </is>
       </c>
     </row>
@@ -3112,7 +3129,7 @@
       </c>
       <c r="B115" s="44" t="inlineStr">
         <is>
-          <t>NOT GRANTED by default since the 2026-08-14 re-base: the headline runs on the measured cells, in which neither family's decode is optimised (ours ran the unoptimised Triton per-step path at 9.5% GPU-busy while the transformer sat at 95.6%). Setting tf_kv_compression=8.0 grants it paged attention + KV quantization, divides our decode lever by 8 and puts the TRANSFORMER ahead at 64k — reported, not hidden</t>
+          <t>NOT GRANTED by default since the 2026-08-14 re-base: the headline runs on the measured cells, in which neither family's decode is optimised (ours ran the unoptimised per-step path at 9.5% GPU-busy while the transformer sat at 95.6%). Setting tf_kv_compression=8.0 grants it paged attention + KV quantization, divides our decode lever by 8 and puts the TRANSFORMER ahead at 64k — reported, not hidden</t>
         </is>
       </c>
       <c r="E115" s="56" t="inlineStr">
@@ -3122,7 +3139,7 @@
       </c>
       <c r="F115" s="44" t="inlineStr">
         <is>
-          <t>SERVING['tf_kv_compression']</t>
+          <t>the model</t>
         </is>
       </c>
     </row>
@@ -3144,7 +3161,7 @@
       </c>
       <c r="F116" s="44" t="inlineStr">
         <is>
-          <t>deck_decode_d2048_bf16_gh200_20260814.json rows[bdm, 64 streams]</t>
+          <t>internal measurement archive rows[bAttention, 64 streams]</t>
         </is>
       </c>
     </row>
@@ -3156,7 +3173,7 @@
       </c>
       <c r="B117" s="44" t="inlineStr">
         <is>
-          <t>25.4 MB/stream, the FULL recurrent cell (h + M memory), 24.2 MiB measured, context-flat. The 0.15 MB figure previously quoted was an h-carry-only proxy with no M memory and is retired as a headline</t>
+          <t>25.4 MB/stream, the FULL internal cell (h + M memory), 24.2 MiB measured, context-flat. The 0.15 MB figure previously quoted was an h-carry-only proxy with no M memory and is retired as a headline</t>
         </is>
       </c>
       <c r="E117" s="55" t="inlineStr">
@@ -3166,7 +3183,7 @@
       </c>
       <c r="F117" s="44" t="inlineStr">
         <is>
-          <t>deck_decode_d2048_bf16_gh200_20260814.json state_bytes_per_stream</t>
+          <t>internal measurement archive state_bytes_per_stream</t>
         </is>
       </c>
     </row>
@@ -3178,7 +3195,7 @@
       </c>
       <c r="B118" s="44" t="inlineStr">
         <is>
-          <t>197 KB per token of context per stream — 51.5 GB for one 262,144-token stream, a 2nd stream OOMs a 96 GB card, and 16 streams OOM it at 32,768 tokens. Its retired 88.5 per-token decode cost was inflated by a growing-KV re-planning harness artifact; the traced figure is 14.92 GPU-busy at 262k</t>
+          <t>197 KB per token of context per stream as reserved end-to-end (51.5 GB for one 262,144-token stream; the linear KV fit alone is 156 KB/token, the rest is workspace) — a 2nd stream OOMs a 96 GB card, and 16 streams OOM it at 32,768 tokens. Its retired 88.5 per-token decode cost was inflated by a growing-KV re-planning harness artifact; the traced figure is 14.92 GPU-busy at 262k</t>
         </is>
       </c>
       <c r="E118" s="55" t="inlineStr">
@@ -3188,7 +3205,7 @@
       </c>
       <c r="F118" s="44" t="inlineStr">
         <is>
-          <t>deck_decode_d2048_bf16_gh200_20260814.json rows[transformer]</t>
+          <t>internal measurement archive rows[transformer]</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3227,7 @@
       </c>
       <c r="F119" s="44" t="inlineStr">
         <is>
-          <t>derived.json matched_load_curve, scaling_1to8_best</t>
+          <t>internal measurement archive matched_load_curve, scaling_1to8_best</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3249,7 @@
       </c>
       <c r="F120" s="44" t="inlineStr">
         <is>
-          <t>derived.json pipeline_feasibility, pipeline_memory_asymmetry</t>
+          <t>internal measurement archive pipeline_feasibility, pipeline_memory_asymmetry</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3261,7 @@
       </c>
       <c r="B121" s="44" t="inlineStr">
         <is>
-          <t>cross-family prefill, bf16, 1xH100, parameter counts exactly matched, block scope (1 layer, batch 16): TF/bAttention 4.02 at d512/1M, 3.83 at d1024/1M, 2.01 at d2048/262k. Short context favours the transformer and is stated so. NOTE: measured on the PRE-CAMPAIGN kernels and not re-run since 2026-08-24, so the TODAY lever is conservative; the realized x3.936 sits in CEILING_PREFILL_SPEEDUP, not here</t>
+          <t>cross-family prefill, bf16, 1xH100, parameter counts exactly matched, block scope (1 layer, batch 16): TF/bAttention 4.02 at d512/1M, 3.83 at d1024/1M, 2.01 at d2048/262k. Short context favours the transformer and is stated so. NOTE: measured on the PRE-CAMPAIGN kernels and not re-run since 2026-08-24, so the TODAY lever is conservative; the realized x3.936 sits in the model, not here</t>
         </is>
       </c>
       <c r="E121" s="55" t="inlineStr">
@@ -3254,7 +3271,7 @@
       </c>
       <c r="F121" s="44" t="inlineStr">
         <is>
-          <t>matched_d{512,1024,2048}_h100.json (2026-07-21)</t>
+          <t>matched_d{512,1024,2048}internal measurement archive (2026-07-21)</t>
         </is>
       </c>
     </row>
@@ -3276,7 +3293,7 @@
       </c>
       <c r="F122" s="44" t="inlineStr">
         <is>
-          <t>deck_speed_scaling_d2048_h100_20260803.json sdpa_fp32_backend_probe + last_route_attestation</t>
+          <t>internal measurement archive sdpa_fp32_backend_probe + last_route_attestation</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3315,7 @@
       </c>
       <c r="F123" s="44" t="inlineStr">
         <is>
-          <t>receipts/io16_gate_20260809.md (2026-08-09)</t>
+          <t>internal measurement archive (2026-08-09)</t>
         </is>
       </c>
     </row>
@@ -3320,7 +3337,7 @@
       </c>
       <c r="F124" s="44" t="inlineStr">
         <is>
-          <t>derived.json quality_fit.ref_70B, parity_cost</t>
+          <t>internal measurement archive quality_fit.ref_70B, parity_cost</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3349,7 @@
       </c>
       <c r="B125" s="44" t="inlineStr">
         <is>
-          <t>systems numbers are component-scope (bAttention d1536 fwd+bwd h-recurrence sub-block vs transformer d2048 forward-only layer); every speedup is vs the family's OWN 1-GPU baseline</t>
+          <t>systems numbers are component-scope (bAttention d1536 fwd+bwd h-internal dynamics sub-block vs transformer d2048 forward-only layer); every speedup is vs the family's OWN 1-GPU baseline</t>
         </is>
       </c>
       <c r="E125" s="56" t="inlineStr">
@@ -3342,7 +3359,7 @@
       </c>
       <c r="F125" s="44" t="inlineStr">
         <is>
-          <t>derived.json scope_reconciliation; deck README</t>
+          <t>internal measurement archive scope_reconciliation; deck README</t>
         </is>
       </c>
     </row>
@@ -3775,7 +3792,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>compute term dominates -&gt; stays far below 100x</t>
+          <t>memory term dominates -&gt; pinned near the 100x memory lever</t>
         </is>
       </c>
     </row>
@@ -3794,7 +3811,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>compute term dominates -&gt; stays far below 100x</t>
+          <t>memory term dominates -&gt; pinned near the 100x memory lever</t>
         </is>
       </c>
     </row>
@@ -3813,7 +3830,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>compute term dominates -&gt; stays far below 100x</t>
+          <t>memory term dominates -&gt; pinned near the 100x memory lever</t>
         </is>
       </c>
     </row>
@@ -3832,7 +3849,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>compute term dominates -&gt; stays far below 100x</t>
+          <t>memory term dominates -&gt; pinned near the 100x memory lever</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3868,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>compute term dominates -&gt; stays far below 100x</t>
+          <t>memory term dominates -&gt; pinned near the 100x memory lever</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4079,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>- Multiplying the levers (100x * 9.2x ~ 900x) is NOT physical: cost is additive (Amdahl), not multiplicative.</t>
+          <t>- Multiplying the levers (100x * ~793x ~ 79,000x) is NOT physical: cost is additive (Amdahl), not multiplicative.</t>
         </is>
       </c>
     </row>
@@ -8300,7 +8317,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>1e-2 memory = 100x less (RNN O(1) state vs transformer O(T) KV cache).</t>
+          <t>1e-2 memory = 100x less (O(1) internal state vs transformer O(T) KV cache).</t>
         </is>
       </c>
     </row>
@@ -8502,7 +8519,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>~$1.84T Aug 2026; IPO 2026-06-12 at ~$1.77T (market data; used by Sensitivity).</t>
+          <t>~$1.95T Aug 2026; IPO 2026-06-12 at ~$1.77T (market data; used by Sensitivity).</t>
         </is>
       </c>
     </row>
@@ -9024,7 +9041,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Cost = box wall-clock, not FLOPs. The transformer's decode leg is KV-bandwidth-bound (measured 1/context law) while its prefill runs near peak, so prefill is &lt;1% of its serving cost at every context — which is why the banked x3.936 prefill (TODAY) and the full x7.03 (CEILING) land within a few percent of each other. Inputs!B24/B25 quote the pinned 128k row (2026-08-31 fleet-context ruling). Static values from ai_capex_model.serving_context_sensitivity() — rebuild the workbook to refresh.</t>
+          <t>Cost = box wall-clock, not FLOPs. The transformer's decode leg is KV-bandwidth-bound (measured 1/context law) while its prefill runs near peak, so prefill is &lt;1% of its serving cost at every context — which is why the banked x3.936 prefill (TODAY) and the full x7.03 (CEILING) land within a few percent of each other. Inputs!B24/B25 quote the pinned 128k row (2026-08-31 fleet-context ruling). Static values from the the model — rebuild the workbook to refresh.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Charts: one color per bar with value labels (app + workbook); ladder as horizontal bars
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -415,6 +415,70 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="2A78D6"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="EB6834"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="EB6834"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="2"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="1BAF7A"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="3"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="EDA100"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="EDA100"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dLbls>
+            <numFmt formatCode="&quot;$&quot;#,##0&quot;B&quot;"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Summary'!$A$16:$A$19</f>
@@ -426,15 +490,16 @@
             </numRef>
           </val>
         </ser>
-        <gapWidth val="150"/>
+        <gapWidth val="60"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
-          <orientation val="minMax"/>
+          <orientation val="maxMin"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -446,6 +511,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -466,6 +532,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -494,7 +561,7 @@
     </title>
     <plotArea>
       <barChart>
-        <barDir val="col"/>
+        <barDir val="bar"/>
         <grouping val="clustered"/>
         <ser>
           <idx val="0"/>
@@ -509,6 +576,84 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="A3A29C"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="A3A29C"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="2A78D6"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="2"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="EB6834"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="EB6834"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="3"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="1BAF7A"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="4"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="EDA100"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="EDA100"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dLbls>
+            <numFmt formatCode="&quot;$&quot;#,##0&quot;B&quot;"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Value Bridge'!$A$49:$A$53</f>
@@ -520,15 +665,16 @@
             </numRef>
           </val>
         </ser>
-        <gapWidth val="150"/>
+        <gapWidth val="60"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
-          <orientation val="minMax"/>
+          <orientation val="maxMin"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -540,6 +686,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -560,6 +707,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>

</xml_diff>

<commit_message>
Data-center shares from 10-K/10-Q filings; re-quote headline
Infra (data-center) share per company now comes from the property &
equipment notes (gross additions by asset class; offices, leasehold
improvements, furniture and equipment-and-other counted as
non-data-center) or segment notes:
- Microsoft 1.00 -> 0.97 (FY25 and FY26 10-K)
- Alphabet 1.00 -> 0.93 FY25 (10-K), 0.95 FY26 (Q2 2026 10-Q)
- Meta 1.00 -> 0.95 FY25 (10-K), 0.98 FY26 (Q2 2026 10-Q)
- Amazon FY26 0.70 -> 0.76 (AWS share of H1 2026 net P&E additions)
- Oracle, SpaceX unchanged
Each company tab cites its filing basis. Headline re-quoted: FY25
$166B -> $161B, FY26 $382B -> $380B (Totals); Value Bridge FY26
$379B -> $377B.
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -2122,16 +2122,16 @@
         </is>
       </c>
       <c r="E14" s="48" t="n">
-        <v>-965.5958029079999</v>
+        <v>-960.45442678288</v>
       </c>
       <c r="F14" s="48" t="n">
-        <v>571.8114816440648</v>
+        <v>569.1669985864507</v>
       </c>
       <c r="G14" s="48" t="n">
-        <v>-393.7843212639353</v>
+        <v>-391.2874281964292</v>
       </c>
       <c r="H14" s="49" t="n">
-        <v>0.4891057518312402</v>
+        <v>0.4889942299198121</v>
       </c>
     </row>
     <row r="16">
@@ -4518,10 +4518,10 @@
         </is>
       </c>
       <c r="E81" s="78" t="n">
-        <v>154.8429860104542</v>
+        <v>149.7773849697697</v>
       </c>
       <c r="F81" s="79" t="n">
-        <v>-11.13717395678219</v>
+        <v>-10.77282758605313</v>
       </c>
       <c r="G81" s="80" t="inlineStr">
         <is>
@@ -4547,10 +4547,10 @@
         </is>
       </c>
       <c r="E82" s="78" t="n">
-        <v>158.8547874640003</v>
+        <v>153.657942599222</v>
       </c>
       <c r="F82" s="79" t="n">
-        <v>-7.125372503236122</v>
+        <v>-6.892269956600785</v>
       </c>
       <c r="G82" s="81" t="inlineStr">
         <is>
@@ -4576,10 +4576,10 @@
         </is>
       </c>
       <c r="E83" s="78" t="n">
-        <v>159.8723512892945</v>
+        <v>154.6422173973205</v>
       </c>
       <c r="F83" s="79" t="n">
-        <v>-6.107808677941904</v>
+        <v>-5.907995158502331</v>
       </c>
       <c r="G83" s="81" t="inlineStr">
         <is>
@@ -4605,10 +4605,10 @@
         </is>
       </c>
       <c r="E84" s="78" t="n">
-        <v>160.0192444322226</v>
+        <v>154.784305013845</v>
       </c>
       <c r="F84" s="79" t="n">
-        <v>-5.960915535013811</v>
+        <v>-5.765907541977811</v>
       </c>
       <c r="G84" s="81" t="inlineStr">
         <is>
@@ -5924,7 +5924,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  infra share strips non-AI (Amazon AWS 68%); server share CFO-disclosed (MSFT ~50%, Google 60%); accel-within-server ~67-80% from BOM.</t>
+          <t xml:space="preserve">  infra (data-center) share from 10-K/10-Q P&amp;E and segment notes (MSFT 97%, Alphabet 93-95%, Meta 95-98%, Amazon AWS 68-76%); server share CFO-disclosed (MSFT ~50%, Google 60%); accel-within-server ~67-80% from BOM.</t>
         </is>
       </c>
     </row>
@@ -5997,28 +5997,28 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>- Net AI FY25: 6 named firms spend ~$375B (capex+opex) vs ~$79B AI revenue = ~ -$295B/yr cash burn.</t>
+          <t>- Net AI FY25: 6 named firms spend ~$362B (capex+opex) vs ~$79B AI revenue = ~ -$283B/yr cash burn.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>- With our architecture: spend cut ~$166B -&gt; burn shrinks to ~ -$129B/yr (~44% of AI spend cut).</t>
+          <t>- With our architecture: spend cut ~$161B -&gt; burn shrinks to ~ -$122B/yr (~44% of AI spend cut).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>- Spend-cut value (named floor, 6% discount rate): FY25 ~$166B/yr (~$2.8T capitalized); FY26 r/r ~$382B/yr (~$6.4T). Ceiling: within rounding of Today (the cut saturates).</t>
+          <t>- Spend-cut value (named floor, 6% discount rate): FY25 ~$161B/yr (~$2.7T capitalized); FY26 r/r ~$380B/yr (~$6.3T). Ceiling: within rounding of Today (the cut saturates).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>- GLOBAL estimate (named ~80% of world AI capex): FY25 ~$3.5T, FY26 ~$8.0T capitalized. Clearly an estimate.</t>
+          <t>- GLOBAL estimate (named ~80% of world AI capex): FY25 ~$3.3T, FY26 ~$7.9T capitalized. Clearly an estimate.</t>
         </is>
       </c>
     </row>
@@ -8953,14 +8953,14 @@
         </is>
       </c>
       <c r="B4" s="33" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
       <c r="C4" s="33" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>strips non-AI (Amazon = AWS only)</t>
+          <t>FILING: P&amp;E note (FY25/FY26 10-K). Leasehold improvements, the only non-datacenter class, are $2.5B of $86.6B (FY25) and $4.2B of $133.1B (FY26) of gross additions -&gt; 97%.</t>
         </is>
       </c>
     </row>
@@ -9641,14 +9641,14 @@
         </is>
       </c>
       <c r="B4" s="33" t="n">
-        <v>1</v>
+        <v>0.93</v>
       </c>
       <c r="C4" s="33" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>strips non-AI (Amazon = AWS only)</t>
+          <t>FILING: P&amp;E note. Technical infrastructure +$61.8B vs office space +$2.9B and corporate +$1.9B in 2025 (10-K) -&gt; 93%; +$43.5B vs +$2.3B office in H1 2026 (10-Q) -&gt; 95%.</t>
         </is>
       </c>
     </row>
@@ -10318,11 +10318,11 @@
         <v>0.68</v>
       </c>
       <c r="C4" s="33" t="n">
-        <v>0.7</v>
+        <v>0.76</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>strips non-AI (Amazon = AWS only)</t>
+          <t>FILING: segment note, AWS share of net P&amp;E additions. $96.5B of $142.4B in 2025 (10-K) -&gt; 68%; $90.1B of $118.6B in H1 2026 (10-Q) -&gt; 76%. Strips fulfillment/logistics.</t>
         </is>
       </c>
     </row>
@@ -10989,14 +10989,14 @@
         </is>
       </c>
       <c r="B4" s="33" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="C4" s="33" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>strips non-AI (Amazon = AWS only)</t>
+          <t>FILING: Note 6 P&amp;E. Leasehold improvements + equipment and other are $3.3B of $69.1B gross additions in 2025 (10-K) -&gt; 95%; $0.95B of $59.1B in H1 2026 (10-Q) -&gt; 98%.</t>
         </is>
       </c>
     </row>
@@ -11698,7 +11698,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>strips non-AI (Amazon = AWS only)</t>
+          <t>ESTIMATE: the P&amp;E note has no office line (buildings mix datacenters with the Nashville HQ build); capex growth is 'primarily due to the expansion of our data centers' (FY26 10-K).</t>
         </is>
       </c>
     </row>
@@ -12372,7 +12372,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>strips non-AI (Amazon = AWS only)</t>
+          <t>FILING: capex is the AI segment's own figure (S-1; Q2 2026 10-Q segment note, $23.6B in H1 2026).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Serving priced on whole GPUs; README rewritten to the current model
Summary / Value Bridge / Levers (workbook + app): serving memory and
serving compute merge into one Serving GPUs line. A GPU is bought
whole, so the serving fleet shrinks by the binding (smaller) of the
memory lever and the compute lever: x100 at the defaults. FY2026
bridge $377.2B -> $376.3B. The one-lever-at-a-time ladder now shows
the smaller model saving training only (serving GPUs stay memory-bound)
until fixed-size memory unlocks serving. Technical tabs keep the
memory/compute cost split (~154x); the Levers tab shows it for
reference.

README: headline, scenarios, data-center share table and engine
description updated to the current model; retired x9.24 / $159B
figures removed; measured serving cells kept as background.
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -33,7 +33,7 @@
     <definedName name="ServeThroughput">Levers!$C$11</definedName>
     <definedName name="TrainLever">Levers!$C$14</definedName>
     <definedName name="ServeComputeLever">Levers!$C$16</definedName>
-    <definedName name="MemShare">Levers!$C$17</definedName>
+    <definedName name="ServeGPULever">Levers!$C$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,20 +447,6 @@
             <idx val="2"/>
             <spPr>
               <a:solidFill>
-                <a:srgbClr val="1BAF7A"/>
-              </a:solidFill>
-              <a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="1BAF7A"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="3"/>
-            <spPr>
-              <a:solidFill>
                 <a:srgbClr val="EDA100"/>
               </a:solidFill>
               <a:ln>
@@ -481,12 +467,12 @@
           </dLbls>
           <cat>
             <numRef>
-              <f>'Summary'!$A$16:$A$19</f>
+              <f>'Summary'!$A$16:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$B$16:$B$19</f>
+              <f>'Summary'!$B$16:$B$18</f>
             </numRef>
           </val>
         </ser>
@@ -1272,7 +1258,7 @@
         <v/>
       </c>
       <c r="C16" s="14">
-        <f>B16/$B$20</f>
+        <f>B16/$B$19</f>
         <v/>
       </c>
       <c r="D16" s="3">
@@ -1283,7 +1269,7 @@
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Serving: memory</t>
+          <t>Serving GPUs</t>
         </is>
       </c>
       <c r="B17" s="6">
@@ -1291,70 +1277,51 @@
         <v/>
       </c>
       <c r="C17" s="14">
-        <f>B17/$B$20</f>
+        <f>B17/$B$19</f>
         <v/>
       </c>
       <c r="D17" s="3">
-        <f>"A transformer's memory grows with every token of every live conversation; Helarctos keeps a fixed-size state → ÷"&amp;TEXT(MemoryLever,"0")&amp;" memory per conversation (memory is ~60% of a GPU's cost)."</f>
+        <f>"A transformer's memory grows with every token of every live conversation; Helarctos keeps a fixed-size state (÷"&amp;TEXT(MemoryLever,"0")&amp;" memory) and does "&amp;TEXT(ServeComputeLever,"0")&amp;"× less compute per token. A GPU is bought whole, so the fleet shrinks by whichever limit binds: "&amp;TEXT(ServeGPULever,"0")&amp;"× fewer serving GPUs."</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Serving: compute</t>
+          <t>Power &amp; operations</t>
         </is>
       </c>
       <c r="B18" s="6">
-        <f>'Value Bridge'!H70</f>
+        <f>'Value Bridge'!K70</f>
         <v/>
       </c>
       <c r="C18" s="14">
-        <f>B18/$B$20</f>
-        <v/>
-      </c>
-      <c r="D18" s="3">
-        <f>"Smaller model ("&amp;TEXT(SmallerModel,"0.0")&amp;"×) × far more conversations per GPU ("&amp;TEXT(ServeThroughput,"0")&amp;"× at a 128k-token average) → "&amp;TEXT(ServeComputeLever,"0")&amp;"× less compute per token served."</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="46" customHeight="1">
+        <f>B18/$B$19</f>
+        <v/>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Fewer chips draw less power and need less cooling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>Power &amp; operations</t>
-        </is>
-      </c>
-      <c r="B19" s="6">
-        <f>'Value Bridge'!K70</f>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B19" s="15">
+        <f>SUM(B16:B18)</f>
         <v/>
       </c>
       <c r="C19" s="14">
-        <f>B19/$B$20</f>
-        <v/>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Fewer chips draw less power and need less cooling.</t>
-        </is>
+        <f>SUM(C16:C18)</f>
+        <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B20" s="15">
-        <f>SUM(B16:B19)</f>
-        <v/>
-      </c>
-      <c r="C20" s="14">
-        <f>SUM(C16:C19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Step-by-step build and the one-lever-at-a-time view: Value Bridge tab.</t>
         </is>
@@ -1643,7 +1610,7 @@
     <row r="34" ht="62" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Costs add; they don't multiply. A GPU's cost is ~60% memory and ~40% compute. Once Helarctos cuts the memory needed 100× and the compute needed hundreds of times, ~99% of the chip bill for the same AI output is gone — bigger multiples can only move the last 1%. So the dollars are set by how much these firms spend on chips, not by how large the multiple is. We report dollars.</t>
+          <t>Multiples don't multiply. A GPU is bought whole — memory and compute together — so a serving fleet shrinks by whichever need falls LEAST (here the conservative 100× memory cap), not by 100 × 793. Cutting a fleet 100× already removes 99% of it; bigger multiples can only move the last 1%. So the dollars are set by how much these firms spend on chips, not by how large the multiple is. We report dollars.</t>
         </is>
       </c>
     </row>
@@ -1728,19 +1695,18 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="14">
     <mergeCell ref="B38:G38"/>
     <mergeCell ref="D18:G18"/>
     <mergeCell ref="D17:G17"/>
     <mergeCell ref="B37:G37"/>
     <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A21:G21"/>
     <mergeCell ref="A34:G34"/>
     <mergeCell ref="D16:G16"/>
     <mergeCell ref="B41:G41"/>
+    <mergeCell ref="A20:G20"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="D15:G15"/>
-    <mergeCell ref="D19:G19"/>
     <mergeCell ref="B40:G40"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="B39:G39"/>
@@ -6516,29 +6482,17 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>STEP 4 — SERVING: less memory and more conversations per GPU → smaller serving fleet</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>$ today</t>
-        </is>
-      </c>
+          <t>STEP 4 — SERVING: less memory and more conversations per GPU → fewer serving GPUs</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n"/>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>falls by</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>$ needed</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>$ avoided</t>
-        </is>
-      </c>
+          <t>lever</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="5" t="n"/>
       <c r="F26" s="5" t="n"/>
       <c r="G26" s="5" t="n"/>
       <c r="H26" s="5" t="n"/>
@@ -6558,64 +6512,75 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Memory part of those chips (≈60% of cost)</t>
-        </is>
-      </c>
-      <c r="B28" s="6">
-        <f>B27*MemShare</f>
-        <v/>
+          <t>Memory needed per conversation falls by</t>
+        </is>
       </c>
       <c r="C28" s="23">
         <f>MemoryLever</f>
         <v/>
       </c>
-      <c r="D28" s="6">
-        <f>B28/C28</f>
-        <v/>
-      </c>
-      <c r="E28" s="6">
-        <f>B28-D28</f>
-        <v/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>fixed-size state (lever 4)</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Compute part of those chips (≈40% of cost)</t>
-        </is>
-      </c>
-      <c r="B29" s="6">
-        <f>B27*(1-MemShare)</f>
-        <v/>
+          <t>Compute needed per token falls by</t>
+        </is>
       </c>
       <c r="C29" s="21">
         <f>ServeComputeLever</f>
         <v/>
       </c>
-      <c r="D29" s="6">
-        <f>B29/C29</f>
-        <v/>
-      </c>
-      <c r="E29" s="6">
-        <f>B29-D29</f>
-        <v/>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>smaller model × more conversations per GPU (levers 1 × 5)</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="20" t="inlineStr">
         <is>
+          <t>GPUs needed fall by — whichever limit binds</t>
+        </is>
+      </c>
+      <c r="C30" s="22">
+        <f>ServeGPULever</f>
+        <v/>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>the smaller of the two: a GPU is bought whole</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Serving fleet needed with Helarctos</t>
+        </is>
+      </c>
+      <c r="B31" s="6">
+        <f>B27/C30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
           <t>SERVING CAPEX AVOIDED</t>
         </is>
       </c>
-      <c r="B30" s="15">
-        <f>E28+E29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="48" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>Memory: a transformer's memory grows with every token of every live conversation, so long conversations fill a GPU after one or two users; Helarctos keeps a fixed-size state (lever 4). Compute: the smaller model does less work per token and each GPU serves many more conversations at once (levers 1 × 5).</t>
+      <c r="B32" s="15">
+        <f>B27-B31</f>
+        <v/>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>A GPU brings memory and compute together; the fleet must cover whichever runs out first. Transformers at long context run out of MEMORY (the growing KV cache), so memory is the limit we relieve first; compute then binds only if it falls less than memory.</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6659,7 @@
         </is>
       </c>
       <c r="B39" s="6">
-        <f>B30</f>
+        <f>B32</f>
         <v/>
       </c>
     </row>
@@ -6743,7 +6708,7 @@
         </is>
       </c>
       <c r="B43" s="14">
-        <f>(B23+B30)/B7</f>
+        <f>(B23+B32)/B7</f>
         <v/>
       </c>
     </row>
@@ -6812,7 +6777,7 @@
       </c>
       <c r="E48" s="16" t="inlineStr">
         <is>
-          <t>Chip fleet cut</t>
+          <t>Chip fleet cut (serving GPUs fall by the smaller)</t>
         </is>
       </c>
       <c r="F48" s="16" t="inlineStr">
@@ -6842,7 +6807,7 @@
         <v>1</v>
       </c>
       <c r="E49" s="25">
-        <f>(D70*(1-1/B49)+E70*(MemShare*(1-1/C49)+(1-MemShare)*(1-1/D49)))/B70</f>
+        <f>(D70*(1-1/B49)+E70*(1-1/MIN(C49,D49)))/B70</f>
         <v/>
       </c>
       <c r="F49" s="18">
@@ -6872,7 +6837,7 @@
         <v/>
       </c>
       <c r="E50" s="25">
-        <f>(D70*(1-1/B50)+E70*(MemShare*(1-1/C50)+(1-MemShare)*(1-1/D50)))/B70</f>
+        <f>(D70*(1-1/B50)+E70*(1-1/MIN(C50,D50)))/B70</f>
         <v/>
       </c>
       <c r="F50" s="18">
@@ -6903,7 +6868,7 @@
         <v/>
       </c>
       <c r="E51" s="25">
-        <f>(D70*(1-1/B51)+E70*(MemShare*(1-1/C51)+(1-MemShare)*(1-1/D51)))/B70</f>
+        <f>(D70*(1-1/B51)+E70*(1-1/MIN(C51,D51)))/B70</f>
         <v/>
       </c>
       <c r="F51" s="18">
@@ -6934,7 +6899,7 @@
         <v/>
       </c>
       <c r="E52" s="25">
-        <f>(D70*(1-1/B52)+E70*(MemShare*(1-1/C52)+(1-MemShare)*(1-1/D52)))/B70</f>
+        <f>(D70*(1-1/B52)+E70*(1-1/MIN(C52,D52)))/B70</f>
         <v/>
       </c>
       <c r="F52" s="18">
@@ -6965,7 +6930,7 @@
         <v/>
       </c>
       <c r="E53" s="25">
-        <f>(D70*(1-1/B53)+E70*(MemShare*(1-1/C53)+(1-MemShare)*(1-1/D53)))/B70</f>
+        <f>(D70*(1-1/B53)+E70*(1-1/MIN(C53,D53)))/B70</f>
         <v/>
       </c>
       <c r="F53" s="18">
@@ -6980,7 +6945,7 @@
     <row r="55" ht="62" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Read this as: the smaller model alone removes about half the chip bill (and nearly all of the training bill, since fewer parameters AND fewer tokens compound). Fixed-size memory is the biggest single serving lever because memory is ~60% of what a GPU costs. The later levers have large multiples but add little, because by then over 90% of the cost is already gone: a cost can only fall to zero once. That is why this workbook reports dollars, not multiples. The order is the storyline; the end point does not depend on it.</t>
+          <t>Read this as: the smaller model alone removes nearly all of the TRAINING bill (fewer parameters AND fewer tokens compound) but no serving GPUs — at long context a transformer's serving GPUs are full of memory (the growing KV cache), not busy computing, and a smaller model doesn't change that. Fixed-size memory unlocks serving, until compute becomes the limit; many more conversations per GPU lifts that limit. The last levers have big multiples but add little, because by then over 95% of the cost is already gone: a cost can only fall to zero once. That is why this workbook reports dollars, not multiples. The order is the storyline; the end point does not depend on it.</t>
         </is>
       </c>
     </row>
@@ -7002,7 +6967,7 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Totals tab, FY2026 spend cut (whole fleet priced on serving levers)</t>
+          <t>Totals tab, FY2026 spend cut (memory and compute priced separately, ~154×)</t>
         </is>
       </c>
       <c r="B58" s="6">
@@ -7013,7 +6978,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>This bridge (training priced on its own lever)</t>
+          <t>This bridge (training on GPU-hours, serving on whole GPUs)</t>
         </is>
       </c>
       <c r="B59" s="6">
@@ -7093,12 +7058,12 @@
       </c>
       <c r="G63" s="16" t="inlineStr">
         <is>
-          <t>Serving memory avoided</t>
+          <t>Serving capex avoided</t>
         </is>
       </c>
       <c r="H63" s="16" t="inlineStr">
         <is>
-          <t>Serving compute avoided</t>
+          <t>Serving fleet needed</t>
         </is>
       </c>
       <c r="I63" s="16" t="inlineStr">
@@ -7174,15 +7139,15 @@
         <v/>
       </c>
       <c r="G64" s="6">
-        <f>E64*MemShare*(1-1/MemoryLever)</f>
-        <v/>
-      </c>
-      <c r="H64" s="6">
-        <f>E64*(1-MemShare)*(1-1/ServeComputeLever)</f>
+        <f>E64*(1-1/ServeGPULever)</f>
+        <v/>
+      </c>
+      <c r="H64" s="28">
+        <f>E64/ServeGPULever</f>
         <v/>
       </c>
       <c r="I64" s="6">
-        <f>F64+G64+H64</f>
+        <f>F64+G64</f>
         <v/>
       </c>
       <c r="J64" s="28">
@@ -7245,15 +7210,15 @@
         <v/>
       </c>
       <c r="G65" s="6">
-        <f>E65*MemShare*(1-1/MemoryLever)</f>
-        <v/>
-      </c>
-      <c r="H65" s="6">
-        <f>E65*(1-MemShare)*(1-1/ServeComputeLever)</f>
+        <f>E65*(1-1/ServeGPULever)</f>
+        <v/>
+      </c>
+      <c r="H65" s="28">
+        <f>E65/ServeGPULever</f>
         <v/>
       </c>
       <c r="I65" s="6">
-        <f>F65+G65+H65</f>
+        <f>F65+G65</f>
         <v/>
       </c>
       <c r="J65" s="28">
@@ -7316,15 +7281,15 @@
         <v/>
       </c>
       <c r="G66" s="6">
-        <f>E66*MemShare*(1-1/MemoryLever)</f>
-        <v/>
-      </c>
-      <c r="H66" s="6">
-        <f>E66*(1-MemShare)*(1-1/ServeComputeLever)</f>
+        <f>E66*(1-1/ServeGPULever)</f>
+        <v/>
+      </c>
+      <c r="H66" s="28">
+        <f>E66/ServeGPULever</f>
         <v/>
       </c>
       <c r="I66" s="6">
-        <f>F66+G66+H66</f>
+        <f>F66+G66</f>
         <v/>
       </c>
       <c r="J66" s="28">
@@ -7387,15 +7352,15 @@
         <v/>
       </c>
       <c r="G67" s="6">
-        <f>E67*MemShare*(1-1/MemoryLever)</f>
-        <v/>
-      </c>
-      <c r="H67" s="6">
-        <f>E67*(1-MemShare)*(1-1/ServeComputeLever)</f>
+        <f>E67*(1-1/ServeGPULever)</f>
+        <v/>
+      </c>
+      <c r="H67" s="28">
+        <f>E67/ServeGPULever</f>
         <v/>
       </c>
       <c r="I67" s="6">
-        <f>F67+G67+H67</f>
+        <f>F67+G67</f>
         <v/>
       </c>
       <c r="J67" s="28">
@@ -7458,15 +7423,15 @@
         <v/>
       </c>
       <c r="G68" s="6">
-        <f>E68*MemShare*(1-1/MemoryLever)</f>
-        <v/>
-      </c>
-      <c r="H68" s="6">
-        <f>E68*(1-MemShare)*(1-1/ServeComputeLever)</f>
+        <f>E68*(1-1/ServeGPULever)</f>
+        <v/>
+      </c>
+      <c r="H68" s="28">
+        <f>E68/ServeGPULever</f>
         <v/>
       </c>
       <c r="I68" s="6">
-        <f>F68+G68+H68</f>
+        <f>F68+G68</f>
         <v/>
       </c>
       <c r="J68" s="28">
@@ -7529,15 +7494,15 @@
         <v/>
       </c>
       <c r="G69" s="6">
-        <f>E69*MemShare*(1-1/MemoryLever)</f>
-        <v/>
-      </c>
-      <c r="H69" s="6">
-        <f>E69*(1-MemShare)*(1-1/ServeComputeLever)</f>
+        <f>E69*(1-1/ServeGPULever)</f>
+        <v/>
+      </c>
+      <c r="H69" s="28">
+        <f>E69/ServeGPULever</f>
         <v/>
       </c>
       <c r="I69" s="6">
-        <f>F69+G69+H69</f>
+        <f>F69+G69</f>
         <v/>
       </c>
       <c r="J69" s="28">
@@ -7603,7 +7568,7 @@
         <f>SUM(G64:G69)</f>
         <v/>
       </c>
-      <c r="H70" s="18">
+      <c r="H70" s="29">
         <f>SUM(H64:H69)</f>
         <v/>
       </c>
@@ -7700,12 +7665,12 @@
       </c>
       <c r="G74" s="16" t="inlineStr">
         <is>
-          <t>Serving memory avoided</t>
+          <t>Serving capex avoided</t>
         </is>
       </c>
       <c r="H74" s="16" t="inlineStr">
         <is>
-          <t>Serving compute avoided</t>
+          <t>Serving fleet needed</t>
         </is>
       </c>
       <c r="I74" s="16" t="inlineStr">
@@ -7781,15 +7746,15 @@
         <v/>
       </c>
       <c r="G75" s="6">
-        <f>E75*MemShare*(1-1/MemoryLever)</f>
-        <v/>
-      </c>
-      <c r="H75" s="6">
-        <f>E75*(1-MemShare)*(1-1/ServeComputeLever)</f>
+        <f>E75*(1-1/ServeGPULever)</f>
+        <v/>
+      </c>
+      <c r="H75" s="28">
+        <f>E75/ServeGPULever</f>
         <v/>
       </c>
       <c r="I75" s="6">
-        <f>F75+G75+H75</f>
+        <f>F75+G75</f>
         <v/>
       </c>
       <c r="J75" s="28">
@@ -7852,15 +7817,15 @@
         <v/>
       </c>
       <c r="G76" s="6">
-        <f>E76*MemShare*(1-1/MemoryLever)</f>
-        <v/>
-      </c>
-      <c r="H76" s="6">
-        <f>E76*(1-MemShare)*(1-1/ServeComputeLever)</f>
+        <f>E76*(1-1/ServeGPULever)</f>
+        <v/>
+      </c>
+      <c r="H76" s="28">
+        <f>E76/ServeGPULever</f>
         <v/>
       </c>
       <c r="I76" s="6">
-        <f>F76+G76+H76</f>
+        <f>F76+G76</f>
         <v/>
       </c>
       <c r="J76" s="28">
@@ -7923,15 +7888,15 @@
         <v/>
       </c>
       <c r="G77" s="6">
-        <f>E77*MemShare*(1-1/MemoryLever)</f>
-        <v/>
-      </c>
-      <c r="H77" s="6">
-        <f>E77*(1-MemShare)*(1-1/ServeComputeLever)</f>
+        <f>E77*(1-1/ServeGPULever)</f>
+        <v/>
+      </c>
+      <c r="H77" s="28">
+        <f>E77/ServeGPULever</f>
         <v/>
       </c>
       <c r="I77" s="6">
-        <f>F77+G77+H77</f>
+        <f>F77+G77</f>
         <v/>
       </c>
       <c r="J77" s="28">
@@ -7994,15 +7959,15 @@
         <v/>
       </c>
       <c r="G78" s="6">
-        <f>E78*MemShare*(1-1/MemoryLever)</f>
-        <v/>
-      </c>
-      <c r="H78" s="6">
-        <f>E78*(1-MemShare)*(1-1/ServeComputeLever)</f>
+        <f>E78*(1-1/ServeGPULever)</f>
+        <v/>
+      </c>
+      <c r="H78" s="28">
+        <f>E78/ServeGPULever</f>
         <v/>
       </c>
       <c r="I78" s="6">
-        <f>F78+G78+H78</f>
+        <f>F78+G78</f>
         <v/>
       </c>
       <c r="J78" s="28">
@@ -8065,15 +8030,15 @@
         <v/>
       </c>
       <c r="G79" s="6">
-        <f>E79*MemShare*(1-1/MemoryLever)</f>
-        <v/>
-      </c>
-      <c r="H79" s="6">
-        <f>E79*(1-MemShare)*(1-1/ServeComputeLever)</f>
+        <f>E79*(1-1/ServeGPULever)</f>
+        <v/>
+      </c>
+      <c r="H79" s="28">
+        <f>E79/ServeGPULever</f>
         <v/>
       </c>
       <c r="I79" s="6">
-        <f>F79+G79+H79</f>
+        <f>F79+G79</f>
         <v/>
       </c>
       <c r="J79" s="28">
@@ -8136,15 +8101,15 @@
         <v/>
       </c>
       <c r="G80" s="6">
-        <f>E80*MemShare*(1-1/MemoryLever)</f>
-        <v/>
-      </c>
-      <c r="H80" s="6">
-        <f>E80*(1-MemShare)*(1-1/ServeComputeLever)</f>
+        <f>E80*(1-1/ServeGPULever)</f>
+        <v/>
+      </c>
+      <c r="H80" s="28">
+        <f>E80/ServeGPULever</f>
         <v/>
       </c>
       <c r="I80" s="6">
-        <f>F80+G80+H80</f>
+        <f>F80+G80</f>
         <v/>
       </c>
       <c r="J80" s="28">
@@ -8210,7 +8175,7 @@
         <f>SUM(G75:G80)</f>
         <v/>
       </c>
-      <c r="H81" s="18">
+      <c r="H81" s="29">
         <f>SUM(H75:H80)</f>
         <v/>
       </c>
@@ -8252,25 +8217,28 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="21">
+    <mergeCell ref="D13:I13"/>
+    <mergeCell ref="D32:I32"/>
+    <mergeCell ref="D41:I41"/>
+    <mergeCell ref="A55:I55"/>
+    <mergeCell ref="D7:I7"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="D28:I28"/>
+    <mergeCell ref="D18:I18"/>
+    <mergeCell ref="D9:I9"/>
+    <mergeCell ref="D30:I30"/>
+    <mergeCell ref="D29:I29"/>
+    <mergeCell ref="D5:I5"/>
+    <mergeCell ref="D35:I35"/>
+    <mergeCell ref="D20:I20"/>
+    <mergeCell ref="D60:I60"/>
+    <mergeCell ref="A24:I24"/>
     <mergeCell ref="D19:I19"/>
     <mergeCell ref="D10:I10"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="D20:I20"/>
-    <mergeCell ref="D13:I13"/>
-    <mergeCell ref="D5:I5"/>
-    <mergeCell ref="D18:I18"/>
-    <mergeCell ref="D41:I41"/>
-    <mergeCell ref="D9:I9"/>
+    <mergeCell ref="D45:I45"/>
+    <mergeCell ref="D6:I6"/>
     <mergeCell ref="D21:I21"/>
-    <mergeCell ref="D45:I45"/>
-    <mergeCell ref="A31:I31"/>
-    <mergeCell ref="D35:I35"/>
-    <mergeCell ref="D6:I6"/>
-    <mergeCell ref="A55:I55"/>
-    <mergeCell ref="D60:I60"/>
-    <mergeCell ref="D7:I7"/>
-    <mergeCell ref="A24:I24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8527,7 +8495,7 @@
       </c>
       <c r="H10" s="24" t="inlineStr">
         <is>
-          <t>Serving memory (≈60% of a GPU's cost)</t>
+          <t>Serving GPUs (the memory limit)</t>
         </is>
       </c>
     </row>
@@ -8566,7 +8534,7 @@
       </c>
       <c r="H11" s="24" t="inlineStr">
         <is>
-          <t>Serving compute (≈40% of a GPU's cost)</t>
+          <t>Serving GPUs (the compute limit)</t>
         </is>
       </c>
     </row>
@@ -8603,7 +8571,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>Serving: memory needed falls by</t>
+          <t>Serving: memory needed per conversation falls by</t>
         </is>
       </c>
       <c r="C15" s="32">
@@ -8619,7 +8587,7 @@
     <row r="16" ht="30" customHeight="1">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>Serving: compute needed falls by</t>
+          <t>Serving: compute needed per token falls by</t>
         </is>
       </c>
       <c r="C16" s="22">
@@ -8635,32 +8603,32 @@
     <row r="17" ht="30" customHeight="1">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>Memory share of a GPU's cost</t>
-        </is>
-      </c>
-      <c r="C17" s="19">
-        <f>Inputs!$B$4</f>
+          <t>Serving: GPUs needed fall by</t>
+        </is>
+      </c>
+      <c r="C17" s="22">
+        <f>MIN(MemoryLever,ServeComputeLever)</f>
         <v/>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>HBM memory + its packaging ≈ 60%, the compute die ≈ 40% (chip teardowns; see Evidence).</t>
+          <t>A GPU is bought whole — memory and compute come together. The serving fleet has to cover whichever runs out first, so it shrinks by the SMALLER of the two levers (here the conservative ÷100 memory cap). Multiplying them (100 × 793 = 79,000×) would be wrong.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>Serving: fleet cost falls by (blended)</t>
+          <t>For reference: technical tabs' blended serving cut</t>
         </is>
       </c>
       <c r="C18" s="22">
-        <f>1/(MemShare/MemoryLever+(1-MemShare)/ServeComputeLever)</f>
+        <f>Inputs!$B$20</f>
         <v/>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Costs add, they don't multiply: the less-improved part (here memory) sets the floor. This is why 100× and 793× combine to ~154×, not 79,000×.</t>
+          <t>The technical appendix (Totals, company tabs) prices memory (~60% of a GPU's cost) and compute (~40%) separately and blends them (~154×). Same chip bill, under $1B apart on FY2026.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audience tabs: Training and Inference with power folded in; training speed at parity
- Summary / Value Bridge / app show two buckets, Training and Inference,
  each including the power its GPUs would have drawn (power scales with
  the fleet, so the split is exact). 'Serving' renamed 'Inference' on the
  reader-facing tabs.
- Training speed per token at the same model size is treated as roughly
  comparable to a transformer: no speed credit. Training GPU-hours fall
  x17.8 (smaller model x fewer tokens), was x40. The ladder drops the
  training-speed step.
- FY2026 bridge: Training $135B + Inference $237B = $372B (was $376B);
  FY2025 $157B. Technical Totals unchanged ($380B).
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -443,20 +443,6 @@
               </a:ln>
             </spPr>
           </dPt>
-          <dPt>
-            <idx val="2"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="EDA100"/>
-              </a:solidFill>
-              <a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="EDA100"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
           <dLbls>
             <numFmt formatCode="&quot;$&quot;#,##0&quot;B&quot;"/>
             <showLegendKey val="0"/>
@@ -467,12 +453,12 @@
           </dLbls>
           <cat>
             <numRef>
-              <f>'Summary'!$A$16:$A$18</f>
+              <f>'Summary'!$A$16:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$B$16:$B$18</f>
+              <f>'Summary'!$B$16:$B$17</f>
             </numRef>
           </val>
         </ser>
@@ -618,20 +604,6 @@
               </a:ln>
             </spPr>
           </dPt>
-          <dPt>
-            <idx val="4"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="EDA100"/>
-              </a:solidFill>
-              <a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="EDA100"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
           <dLbls>
             <numFmt formatCode="&quot;$&quot;#,##0&quot;B&quot;"/>
             <showLegendKey val="0"/>
@@ -642,12 +614,12 @@
           </dLbls>
           <cat>
             <numRef>
-              <f>'Value Bridge'!$A$49:$A$53</f>
+              <f>'Value Bridge'!$A$49:$A$52</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Value Bridge'!$F$49:$F$53</f>
+              <f>'Value Bridge'!$F$49:$F$52</f>
             </numRef>
           </val>
         </ser>
@@ -706,7 +678,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>8</col>
+      <col>9</col>
       <colOff>0</colOff>
       <row>4</row>
       <rowOff>0</rowOff>
@@ -1046,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1055,7 +1027,8 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1073,7 +1046,7 @@
     </row>
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="3">
-        <f>"In FY2026 the six largest AI spenders (Microsoft, Alphabet, Amazon, Meta, Oracle, SpaceX) will spend ~$"&amp;TEXT('Value Bridge'!M70,"#,##0")&amp;"B on AI and earn ~$"&amp;TEXT('Value Bridge'!O70,"#,##0")&amp;"B from it. Helarctos models do the same AI work — training and serving at the same quality — on a fraction of the hardware. This page shows how much of that spend becomes unnecessary, and where the savings come from."</f>
+        <f>"In FY2026 the six largest AI spenders (Microsoft, Alphabet, Amazon, Meta, Oracle, SpaceX) will spend ~$"&amp;TEXT('Value Bridge'!M70,"#,##0")&amp;"B on AI and earn ~$"&amp;TEXT('Value Bridge'!O70,"#,##0")&amp;"B from it. Helarctos models do the same AI work — training and inference at the same quality — on a fraction of the hardware. This page shows how much of that spend becomes unnecessary, and where the savings come from."</f>
         <v/>
       </c>
     </row>
@@ -1225,12 +1198,12 @@
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Where</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>$B / yr</t>
+          <t>$B / yr (capex + power)</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
@@ -1247,81 +1220,61 @@
       <c r="F15" s="12" t="n"/>
       <c r="G15" s="13" t="n"/>
     </row>
-    <row r="16" ht="46" customHeight="1">
+    <row r="16" ht="62" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Training clusters</t>
+          <t>Training</t>
         </is>
       </c>
       <c r="B16" s="6">
-        <f>'Value Bridge'!F70</f>
+        <f>'Value Bridge'!F70+'Value Bridge'!J70</f>
         <v/>
       </c>
       <c r="C16" s="14">
-        <f>B16/$B$19</f>
+        <f>B16/$B$18</f>
         <v/>
       </c>
       <c r="D16" s="3">
-        <f>"Same-quality model is "&amp;TEXT(SmallerModel,"0.0")&amp;"× smaller and needs "&amp;TEXT(FewerTokens,"0.0")&amp;"× fewer training tokens; each token trains "&amp;TEXT(TrainSpeed,"0.0")&amp;"× faster on long documents → "&amp;TEXT(TrainLever,"0")&amp;"× fewer GPU-hours → training clusters (and their capex) shrink."</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="46" customHeight="1">
+        <f>"Same-quality model is "&amp;TEXT(SmallerModel,"0.0")&amp;"× smaller and needs "&amp;TEXT(FewerTokens,"0.0")&amp;"× fewer training tokens (training speed per token is about the same) → "&amp;TEXT(TrainLever,"0")&amp;"× fewer GPU-hours → smaller training clusters, and the power they would draw."</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="62" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Serving GPUs</t>
+          <t>Inference</t>
         </is>
       </c>
       <c r="B17" s="6">
-        <f>'Value Bridge'!G70</f>
+        <f>'Value Bridge'!G70+'Value Bridge'!K70</f>
         <v/>
       </c>
       <c r="C17" s="14">
-        <f>B17/$B$19</f>
+        <f>B17/$B$18</f>
         <v/>
       </c>
       <c r="D17" s="3">
-        <f>"A transformer's memory grows with every token of every live conversation; Helarctos keeps a fixed-size state (÷"&amp;TEXT(MemoryLever,"0")&amp;" memory) and does "&amp;TEXT(ServeComputeLever,"0")&amp;"× less compute per token. A GPU is bought whole, so the fleet shrinks by whichever limit binds: "&amp;TEXT(ServeGPULever,"0")&amp;"× fewer serving GPUs."</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="46" customHeight="1">
+        <f>"A transformer's memory grows with every token of every live conversation; Helarctos keeps a fixed-size state (÷"&amp;TEXT(MemoryLever,"0")&amp;" memory) and does "&amp;TEXT(ServeComputeLever,"0")&amp;"× less compute per token. A GPU is bought whole, so the fleet shrinks by whichever limit binds: "&amp;TEXT(ServeGPULever,"0")&amp;"× fewer inference GPUs, and their power."</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Power &amp; operations</t>
-        </is>
-      </c>
-      <c r="B18" s="6">
-        <f>'Value Bridge'!K70</f>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B18" s="15">
+        <f>SUM(B16:B17)</f>
         <v/>
       </c>
       <c r="C18" s="14">
-        <f>B18/$B$19</f>
-        <v/>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>Fewer chips draw less power and need less cooling.</t>
-        </is>
+        <f>SUM(C16:C17)</f>
+        <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B19" s="15">
-        <f>SUM(B16:B18)</f>
-        <v/>
-      </c>
-      <c r="C19" s="14">
-        <f>SUM(C16:C18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Step-by-step build and the one-lever-at-a-time view: Value Bridge tab.</t>
         </is>
@@ -1339,6 +1292,7 @@
       <c r="E23" s="5" t="n"/>
       <c r="F23" s="5" t="n"/>
       <c r="G23" s="5" t="n"/>
+      <c r="H23" s="5" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
@@ -1353,25 +1307,30 @@
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
+          <t>Training saving</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Inference saving</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
           <t>Helarctos saving / yr</t>
         </is>
       </c>
-      <c r="D24" s="16" t="inlineStr">
+      <c r="F24" s="16" t="inlineStr">
         <is>
           <t>% of AI spend</t>
         </is>
       </c>
-      <c r="E24" s="16" t="inlineStr">
-        <is>
-          <t>…of which training</t>
-        </is>
-      </c>
-      <c r="F24" s="16" t="inlineStr">
+      <c r="G24" s="16" t="inlineStr">
         <is>
           <t>Net AI today</t>
         </is>
       </c>
-      <c r="G24" s="16" t="inlineStr">
+      <c r="H24" s="16" t="inlineStr">
         <is>
           <t>Net AI with Helarctos</t>
         </is>
@@ -1388,22 +1347,26 @@
         <v/>
       </c>
       <c r="C25" s="6">
+        <f>'Value Bridge'!F64+'Value Bridge'!J64</f>
+        <v/>
+      </c>
+      <c r="D25" s="6">
+        <f>'Value Bridge'!G64+'Value Bridge'!K64</f>
+        <v/>
+      </c>
+      <c r="E25" s="6">
         <f>'Value Bridge'!L64</f>
         <v/>
       </c>
-      <c r="D25" s="14">
+      <c r="F25" s="14">
         <f>'Value Bridge'!N64</f>
         <v/>
       </c>
-      <c r="E25" s="6">
-        <f>'Value Bridge'!F64</f>
-        <v/>
-      </c>
-      <c r="F25" s="6">
+      <c r="G25" s="6">
         <f>'Value Bridge'!P64</f>
         <v/>
       </c>
-      <c r="G25" s="6">
+      <c r="H25" s="6">
         <f>'Value Bridge'!Q64</f>
         <v/>
       </c>
@@ -1419,22 +1382,26 @@
         <v/>
       </c>
       <c r="C26" s="6">
+        <f>'Value Bridge'!F65+'Value Bridge'!J65</f>
+        <v/>
+      </c>
+      <c r="D26" s="6">
+        <f>'Value Bridge'!G65+'Value Bridge'!K65</f>
+        <v/>
+      </c>
+      <c r="E26" s="6">
         <f>'Value Bridge'!L65</f>
         <v/>
       </c>
-      <c r="D26" s="14">
+      <c r="F26" s="14">
         <f>'Value Bridge'!N65</f>
         <v/>
       </c>
-      <c r="E26" s="6">
-        <f>'Value Bridge'!F65</f>
-        <v/>
-      </c>
-      <c r="F26" s="6">
+      <c r="G26" s="6">
         <f>'Value Bridge'!P65</f>
         <v/>
       </c>
-      <c r="G26" s="6">
+      <c r="H26" s="6">
         <f>'Value Bridge'!Q65</f>
         <v/>
       </c>
@@ -1450,22 +1417,26 @@
         <v/>
       </c>
       <c r="C27" s="6">
+        <f>'Value Bridge'!F66+'Value Bridge'!J66</f>
+        <v/>
+      </c>
+      <c r="D27" s="6">
+        <f>'Value Bridge'!G66+'Value Bridge'!K66</f>
+        <v/>
+      </c>
+      <c r="E27" s="6">
         <f>'Value Bridge'!L66</f>
         <v/>
       </c>
-      <c r="D27" s="14">
+      <c r="F27" s="14">
         <f>'Value Bridge'!N66</f>
         <v/>
       </c>
-      <c r="E27" s="6">
-        <f>'Value Bridge'!F66</f>
-        <v/>
-      </c>
-      <c r="F27" s="6">
+      <c r="G27" s="6">
         <f>'Value Bridge'!P66</f>
         <v/>
       </c>
-      <c r="G27" s="6">
+      <c r="H27" s="6">
         <f>'Value Bridge'!Q66</f>
         <v/>
       </c>
@@ -1481,22 +1452,26 @@
         <v/>
       </c>
       <c r="C28" s="6">
+        <f>'Value Bridge'!F67+'Value Bridge'!J67</f>
+        <v/>
+      </c>
+      <c r="D28" s="6">
+        <f>'Value Bridge'!G67+'Value Bridge'!K67</f>
+        <v/>
+      </c>
+      <c r="E28" s="6">
         <f>'Value Bridge'!L67</f>
         <v/>
       </c>
-      <c r="D28" s="14">
+      <c r="F28" s="14">
         <f>'Value Bridge'!N67</f>
         <v/>
       </c>
-      <c r="E28" s="6">
-        <f>'Value Bridge'!F67</f>
-        <v/>
-      </c>
-      <c r="F28" s="6">
+      <c r="G28" s="6">
         <f>'Value Bridge'!P67</f>
         <v/>
       </c>
-      <c r="G28" s="6">
+      <c r="H28" s="6">
         <f>'Value Bridge'!Q67</f>
         <v/>
       </c>
@@ -1512,22 +1487,26 @@
         <v/>
       </c>
       <c r="C29" s="6">
+        <f>'Value Bridge'!F68+'Value Bridge'!J68</f>
+        <v/>
+      </c>
+      <c r="D29" s="6">
+        <f>'Value Bridge'!G68+'Value Bridge'!K68</f>
+        <v/>
+      </c>
+      <c r="E29" s="6">
         <f>'Value Bridge'!L68</f>
         <v/>
       </c>
-      <c r="D29" s="14">
+      <c r="F29" s="14">
         <f>'Value Bridge'!N68</f>
         <v/>
       </c>
-      <c r="E29" s="6">
-        <f>'Value Bridge'!F68</f>
-        <v/>
-      </c>
-      <c r="F29" s="6">
+      <c r="G29" s="6">
         <f>'Value Bridge'!P68</f>
         <v/>
       </c>
-      <c r="G29" s="6">
+      <c r="H29" s="6">
         <f>'Value Bridge'!Q68</f>
         <v/>
       </c>
@@ -1543,22 +1522,26 @@
         <v/>
       </c>
       <c r="C30" s="6">
+        <f>'Value Bridge'!F69+'Value Bridge'!J69</f>
+        <v/>
+      </c>
+      <c r="D30" s="6">
+        <f>'Value Bridge'!G69+'Value Bridge'!K69</f>
+        <v/>
+      </c>
+      <c r="E30" s="6">
         <f>'Value Bridge'!L69</f>
         <v/>
       </c>
-      <c r="D30" s="14">
+      <c r="F30" s="14">
         <f>'Value Bridge'!N69</f>
         <v/>
       </c>
-      <c r="E30" s="6">
-        <f>'Value Bridge'!F69</f>
-        <v/>
-      </c>
-      <c r="F30" s="6">
+      <c r="G30" s="6">
         <f>'Value Bridge'!P69</f>
         <v/>
       </c>
-      <c r="G30" s="6">
+      <c r="H30" s="6">
         <f>'Value Bridge'!Q69</f>
         <v/>
       </c>
@@ -1574,22 +1557,26 @@
         <v/>
       </c>
       <c r="C31" s="18">
+        <f>'Value Bridge'!F70+'Value Bridge'!J70</f>
+        <v/>
+      </c>
+      <c r="D31" s="18">
+        <f>'Value Bridge'!G70+'Value Bridge'!K70</f>
+        <v/>
+      </c>
+      <c r="E31" s="18">
         <f>'Value Bridge'!L70</f>
         <v/>
       </c>
-      <c r="D31" s="19">
+      <c r="F31" s="19">
         <f>'Value Bridge'!N70</f>
         <v/>
       </c>
-      <c r="E31" s="18">
-        <f>'Value Bridge'!F70</f>
-        <v/>
-      </c>
-      <c r="F31" s="18">
+      <c r="G31" s="18">
         <f>'Value Bridge'!P70</f>
         <v/>
       </c>
-      <c r="G31" s="18">
+      <c r="H31" s="18">
         <f>'Value Bridge'!Q70</f>
         <v/>
       </c>
@@ -1610,7 +1597,7 @@
     <row r="34" ht="62" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Multiples don't multiply. A GPU is bought whole — memory and compute together — so a serving fleet shrinks by whichever need falls LEAST (here the conservative 100× memory cap), not by 100 × 793. Cutting a fleet 100× already removes 99% of it; bigger multiples can only move the last 1%. So the dollars are set by how much these firms spend on chips, not by how large the multiple is. We report dollars.</t>
+          <t>Multiples don't multiply. A GPU is bought whole — memory and compute together — so an inference fleet shrinks by whichever need falls LEAST (here the conservative 100× memory cap), not by 100 × 793. Cutting a fleet 100× already removes 99% of it; bigger multiples can only move the last 1%. So the dollars are set by how much these firms spend on chips, not by how large the multiple is. We report dollars.</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1634,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>step by step from disclosed capex to the saving; training vs serving; where each lever moves the needle</t>
+          <t>step by step from disclosed capex to the saving; training vs inference; where each lever moves the needle</t>
         </is>
       </c>
     </row>
@@ -1695,20 +1682,19 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="13">
     <mergeCell ref="B38:G38"/>
-    <mergeCell ref="D18:G18"/>
     <mergeCell ref="D17:G17"/>
     <mergeCell ref="B37:G37"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A34:G34"/>
     <mergeCell ref="D16:G16"/>
     <mergeCell ref="B41:G41"/>
-    <mergeCell ref="A20:G20"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="D15:G15"/>
     <mergeCell ref="B40:G40"/>
     <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A19:G19"/>
     <mergeCell ref="B39:G39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6193,7 +6179,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Read top to bottom: what the six largest AI spenders spend, how their chip fleet splits between TRAINING models and SERVING users, what Helarctos changes in each, and the dollars that follow. Every cell is a live formula; the levers live on the Levers tab.</t>
+          <t>Read top to bottom: what the six largest AI spenders spend, how their chip fleet splits between TRAINING models and INFERENCE (serving users), what Helarctos changes in each, and the dollars that follow. Every cell is a live formula; the levers live on the Levers tab.</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6253,7 @@
         </is>
       </c>
       <c r="B8" s="6">
-        <f>J70</f>
+        <f>I70</f>
         <v/>
       </c>
     </row>
@@ -6345,7 +6331,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Serving fleet — answers users</t>
+          <t>Inference fleet — answers users</t>
         </is>
       </c>
       <c r="B14" s="6">
@@ -6360,7 +6346,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>STEP 3 — TRAINING: fewer GPU-hours per model → smaller training clusters → capex avoided</t>
+          <t>STEP 3 — TRAINING: fewer GPU-hours per model → smaller training clusters</t>
         </is>
       </c>
       <c r="B16" s="5" t="n"/>
@@ -6422,7 +6408,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>…and each token trains faster on long documents</t>
+          <t>…at about the same speed per token</t>
         </is>
       </c>
       <c r="C20" s="21">
@@ -6431,7 +6417,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>flat cost per token vs. rising (lever 3)</t>
+          <t>comparable at the same size — no speed credit taken (lever 3)</t>
         </is>
       </c>
     </row>
@@ -6463,157 +6449,153 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="inlineStr">
-        <is>
-          <t>TRAINING CAPEX AVOIDED</t>
-        </is>
-      </c>
-      <c r="B23" s="15">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Training capex avoided</t>
+        </is>
+      </c>
+      <c r="B23" s="6">
         <f>B17-B22</f>
         <v/>
       </c>
     </row>
-    <row r="24" ht="48" customHeight="1">
-      <c r="A24" s="3">
-        <f>"How training savings become capex savings: labs size their training clusters to the GPU-hours their training runs need. If every model of a given quality needs ~"&amp;TEXT(TrainLever,"0")&amp;"× fewer GPU-hours, the same training programme runs on a cluster ~"&amp;TEXT(TrainLever,"0")&amp;"× smaller — the GPUs that never have to be bought are capex avoided (and the power they would have drawn is opex avoided, Step 5)."</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>STEP 4 — SERVING: less memory and more conversations per GPU → fewer serving GPUs</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n"/>
-      <c r="C26" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Power &amp; operations those GPUs would have drawn</t>
+        </is>
+      </c>
+      <c r="B24" s="6">
+        <f>J70</f>
+        <v/>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>power scales with the fleet</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>TRAINING SAVING (capex + power)</t>
+        </is>
+      </c>
+      <c r="B25" s="15">
+        <f>B23+B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1">
+      <c r="A26" s="3">
+        <f>"How training savings become capex savings: labs size their training clusters to the GPU-hours their training runs need. If every model of a given quality needs ~"&amp;TEXT(TrainLever,"0")&amp;"× fewer GPU-hours, the same training programme runs on a cluster ~"&amp;TEXT(TrainLever,"0")&amp;"× smaller — the GPUs that never have to be bought are capex avoided, and the power they would have drawn is saved every year."</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>STEP 4 — INFERENCE: less memory and more conversations per GPU → fewer inference GPUs</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n"/>
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>lever</t>
         </is>
       </c>
-      <c r="D26" s="5" t="n"/>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="5" t="n"/>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="5" t="n"/>
-      <c r="I26" s="5" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>Serving fleet capex today</t>
-        </is>
-      </c>
-      <c r="B27" s="6">
-        <f>B14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Memory needed per conversation falls by</t>
-        </is>
-      </c>
-      <c r="C28" s="23">
-        <f>MemoryLever</f>
-        <v/>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>fixed-size state (lever 4)</t>
-        </is>
-      </c>
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
+      <c r="G28" s="5" t="n"/>
+      <c r="H28" s="5" t="n"/>
+      <c r="I28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
+          <t>Inference fleet capex today</t>
+        </is>
+      </c>
+      <c r="B29" s="6">
+        <f>B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Memory needed per conversation falls by</t>
+        </is>
+      </c>
+      <c r="C30" s="23">
+        <f>MemoryLever</f>
+        <v/>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>fixed-size state (lever 4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
           <t>Compute needed per token falls by</t>
         </is>
       </c>
-      <c r="C29" s="21">
+      <c r="C31" s="21">
         <f>ServeComputeLever</f>
         <v/>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>smaller model × more conversations per GPU (levers 1 × 5)</t>
         </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="20" t="inlineStr">
-        <is>
-          <t>GPUs needed fall by — whichever limit binds</t>
-        </is>
-      </c>
-      <c r="C30" s="22">
-        <f>ServeGPULever</f>
-        <v/>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>the smaller of the two: a GPU is bought whole</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Serving fleet needed with Helarctos</t>
-        </is>
-      </c>
-      <c r="B31" s="6">
-        <f>B27/C30</f>
-        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>SERVING CAPEX AVOIDED</t>
-        </is>
-      </c>
-      <c r="B32" s="15">
-        <f>B27-B31</f>
+          <t>GPUs needed fall by — whichever limit binds</t>
+        </is>
+      </c>
+      <c r="C32" s="22">
+        <f>ServeGPULever</f>
         <v/>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>A GPU brings memory and compute together; the fleet must cover whichever runs out first. Transformers at long context run out of MEMORY (the growing KV cache), so memory is the limit we relieve first; compute then binds only if it falls less than memory.</t>
+          <t>the smaller of the two: a GPU is bought whole</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>STEP 5 — Power &amp; operations shrink with the fleet</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="5" t="n"/>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="5" t="n"/>
-      <c r="I33" s="5" t="n"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Inference fleet needed with Helarctos</t>
+        </is>
+      </c>
+      <c r="B33" s="6">
+        <f>B29/C32</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Power &amp; operations for the chip fleet today</t>
+          <t>Inference capex avoided</t>
         </is>
       </c>
       <c r="B34" s="6">
-        <f>B8</f>
+        <f>B29-B33</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Power &amp; operations saved per year</t>
+          <t>Power &amp; operations those GPUs would have drawn</t>
         </is>
       </c>
       <c r="B35" s="6">
@@ -6622,55 +6604,60 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Same share as the chip fleet cut.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+          <t>power scales with the fleet</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="20" t="inlineStr">
+        <is>
+          <t>INFERENCE SAVING (capex + power)</t>
+        </is>
+      </c>
+      <c r="B36" s="15">
+        <f>B34+B35</f>
+        <v/>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>A GPU brings memory and compute together; the fleet must cover whichever runs out first. Transformers at long context run out of MEMORY (the growing KV cache) first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>RESULT — FY2026</t>
         </is>
       </c>
-      <c r="B37" s="5" t="n"/>
-      <c r="C37" s="5" t="n"/>
-      <c r="D37" s="5" t="n"/>
-      <c r="E37" s="5" t="n"/>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="5" t="n"/>
-      <c r="I37" s="5" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>Training capex avoided</t>
-        </is>
-      </c>
-      <c r="B38" s="6">
-        <f>B23</f>
-        <v/>
-      </c>
+      <c r="B38" s="5" t="n"/>
+      <c r="C38" s="5" t="n"/>
+      <c r="D38" s="5" t="n"/>
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="5" t="n"/>
+      <c r="G38" s="5" t="n"/>
+      <c r="H38" s="5" t="n"/>
+      <c r="I38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Serving capex avoided</t>
+          <t>Training (capex + power)</t>
         </is>
       </c>
       <c r="B39" s="6">
-        <f>B32</f>
+        <f>B25</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Power &amp; operations saved</t>
+          <t>Inference (capex + power)</t>
         </is>
       </c>
       <c r="B40" s="6">
-        <f>B35</f>
+        <f>B36</f>
         <v/>
       </c>
     </row>
@@ -6681,7 +6668,7 @@
         </is>
       </c>
       <c r="B41" s="15">
-        <f>B38+B39+B40</f>
+        <f>B39+B40</f>
         <v/>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -6708,7 +6695,7 @@
         </is>
       </c>
       <c r="B43" s="14">
-        <f>(B23+B32)/B7</f>
+        <f>(B23+B34)/B7</f>
         <v/>
       </c>
     </row>
@@ -6767,17 +6754,17 @@
       </c>
       <c r="C48" s="16" t="inlineStr">
         <is>
-          <t>Serving memory falls by</t>
+          <t>Inference memory falls by</t>
         </is>
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>Serving compute falls by</t>
+          <t>Inference compute falls by</t>
         </is>
       </c>
       <c r="E48" s="16" t="inlineStr">
         <is>
-          <t>Chip fleet cut (serving GPUs fall by the smaller)</t>
+          <t>Chip fleet cut (inference GPUs fall by the smaller)</t>
         </is>
       </c>
       <c r="F48" s="16" t="inlineStr">
@@ -6811,7 +6798,7 @@
         <v/>
       </c>
       <c r="F49" s="18">
-        <f>E49*(B70+J70)</f>
+        <f>E49*(B70+I70)</f>
         <v/>
       </c>
       <c r="G49" s="26">
@@ -6841,7 +6828,7 @@
         <v/>
       </c>
       <c r="F50" s="18">
-        <f>E50*(B70+J70)</f>
+        <f>E50*(B70+I70)</f>
         <v/>
       </c>
       <c r="G50" s="26">
@@ -6872,7 +6859,7 @@
         <v/>
       </c>
       <c r="F51" s="18">
-        <f>E51*(B70+J70)</f>
+        <f>E51*(B70+I70)</f>
         <v/>
       </c>
       <c r="G51" s="26">
@@ -6881,13 +6868,13 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="24" t="inlineStr">
+      <c r="A52" s="27" t="inlineStr">
         <is>
           <t>+ Many more conversations per GPU (lever 5)</t>
         </is>
       </c>
       <c r="B52" s="21">
-        <f>SmallerModel^2</f>
+        <f>TrainLever</f>
         <v/>
       </c>
       <c r="C52" s="23">
@@ -6903,7 +6890,7 @@
         <v/>
       </c>
       <c r="F52" s="18">
-        <f>E52*(B70+J70)</f>
+        <f>E52*(B70+I70)</f>
         <v/>
       </c>
       <c r="G52" s="26">
@@ -6911,41 +6898,10 @@
         <v/>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="27" t="inlineStr">
-        <is>
-          <t>+ Faster training on long documents (lever 3)</t>
-        </is>
-      </c>
-      <c r="B53" s="21">
-        <f>TrainLever</f>
-        <v/>
-      </c>
-      <c r="C53" s="23">
-        <f>MemoryLever</f>
-        <v/>
-      </c>
-      <c r="D53" s="21">
-        <f>ServeComputeLever</f>
-        <v/>
-      </c>
-      <c r="E53" s="25">
-        <f>(D70*(1-1/B53)+E70*(1-1/MIN(C53,D53)))/B70</f>
-        <v/>
-      </c>
-      <c r="F53" s="18">
-        <f>E53*(B70+J70)</f>
-        <v/>
-      </c>
-      <c r="G53" s="26">
-        <f>F53-F52</f>
-        <v/>
-      </c>
-    </row>
     <row r="55" ht="62" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Read this as: the smaller model alone removes nearly all of the TRAINING bill (fewer parameters AND fewer tokens compound) but no serving GPUs — at long context a transformer's serving GPUs are full of memory (the growing KV cache), not busy computing, and a smaller model doesn't change that. Fixed-size memory unlocks serving, until compute becomes the limit; many more conversations per GPU lifts that limit. The last levers have big multiples but add little, because by then over 95% of the cost is already gone: a cost can only fall to zero once. That is why this workbook reports dollars, not multiples. The order is the storyline; the end point does not depend on it.</t>
+          <t>Read this as: the smaller model alone removes nearly all of the TRAINING bill (fewer parameters AND fewer tokens compound) but no inference GPUs — at long context a transformer's inference GPUs are full of memory (the growing KV cache), not busy computing, and a smaller model doesn't change that. Fixed-size memory unlocks inference, until compute becomes the limit; many more conversations per GPU lifts that limit. By then ~99% of the chip bill is gone: bigger multiples can't add much, because a cost can only fall to zero once. That is why this workbook reports dollars, not multiples. The order is the storyline; the end point does not depend on it.</t>
         </is>
       </c>
     </row>
@@ -6978,7 +6934,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>This bridge (training on GPU-hours, serving on whole GPUs)</t>
+          <t>This bridge (training on GPU-hours, inference on whole GPUs)</t>
         </is>
       </c>
       <c r="B59" s="6">
@@ -7048,7 +7004,7 @@
       </c>
       <c r="E63" s="16" t="inlineStr">
         <is>
-          <t>Serving fleet</t>
+          <t>Inference fleet</t>
         </is>
       </c>
       <c r="F63" s="16" t="inlineStr">
@@ -7058,27 +7014,27 @@
       </c>
       <c r="G63" s="16" t="inlineStr">
         <is>
-          <t>Serving capex avoided</t>
+          <t>Inference capex avoided</t>
         </is>
       </c>
       <c r="H63" s="16" t="inlineStr">
         <is>
-          <t>Serving fleet needed</t>
+          <t>Chip capex avoided</t>
         </is>
       </c>
       <c r="I63" s="16" t="inlineStr">
         <is>
-          <t>Chip capex avoided</t>
+          <t>Power &amp; ops today</t>
         </is>
       </c>
       <c r="J63" s="16" t="inlineStr">
         <is>
-          <t>Power &amp; ops today</t>
+          <t>Training power saved</t>
         </is>
       </c>
       <c r="K63" s="16" t="inlineStr">
         <is>
-          <t>Power &amp; ops saved</t>
+          <t>Inference power saved</t>
         </is>
       </c>
       <c r="L63" s="16" t="inlineStr">
@@ -7142,28 +7098,28 @@
         <f>E64*(1-1/ServeGPULever)</f>
         <v/>
       </c>
-      <c r="H64" s="28">
-        <f>E64/ServeGPULever</f>
-        <v/>
-      </c>
-      <c r="I64" s="6">
+      <c r="H64" s="6">
         <f>F64+G64</f>
         <v/>
       </c>
+      <c r="I64" s="28">
+        <f>'Microsoft'!$C$34</f>
+        <v/>
+      </c>
       <c r="J64" s="28">
-        <f>'Microsoft'!$C$34</f>
+        <f>IF(B64&gt;0,I64*F64/B64,0)</f>
         <v/>
       </c>
       <c r="K64" s="28">
-        <f>IF(B64&gt;0,J64*I64/B64,0)</f>
+        <f>IF(B64&gt;0,I64*G64/B64,0)</f>
         <v/>
       </c>
       <c r="L64" s="18">
-        <f>I64+K64</f>
+        <f>H64+J64+K64</f>
         <v/>
       </c>
       <c r="M64" s="6">
-        <f>'Microsoft'!$C$10+J64</f>
+        <f>'Microsoft'!$C$10+I64</f>
         <v/>
       </c>
       <c r="N64" s="14">
@@ -7213,28 +7169,28 @@
         <f>E65*(1-1/ServeGPULever)</f>
         <v/>
       </c>
-      <c r="H65" s="28">
-        <f>E65/ServeGPULever</f>
-        <v/>
-      </c>
-      <c r="I65" s="6">
+      <c r="H65" s="6">
         <f>F65+G65</f>
         <v/>
       </c>
+      <c r="I65" s="28">
+        <f>'Alphabet'!$C$34</f>
+        <v/>
+      </c>
       <c r="J65" s="28">
-        <f>'Alphabet'!$C$34</f>
+        <f>IF(B65&gt;0,I65*F65/B65,0)</f>
         <v/>
       </c>
       <c r="K65" s="28">
-        <f>IF(B65&gt;0,J65*I65/B65,0)</f>
+        <f>IF(B65&gt;0,I65*G65/B65,0)</f>
         <v/>
       </c>
       <c r="L65" s="18">
-        <f>I65+K65</f>
+        <f>H65+J65+K65</f>
         <v/>
       </c>
       <c r="M65" s="6">
-        <f>'Alphabet'!$C$10+J65</f>
+        <f>'Alphabet'!$C$10+I65</f>
         <v/>
       </c>
       <c r="N65" s="14">
@@ -7284,28 +7240,28 @@
         <f>E66*(1-1/ServeGPULever)</f>
         <v/>
       </c>
-      <c r="H66" s="28">
-        <f>E66/ServeGPULever</f>
-        <v/>
-      </c>
-      <c r="I66" s="6">
+      <c r="H66" s="6">
         <f>F66+G66</f>
         <v/>
       </c>
+      <c r="I66" s="28">
+        <f>'Amazon'!$C$34</f>
+        <v/>
+      </c>
       <c r="J66" s="28">
-        <f>'Amazon'!$C$34</f>
+        <f>IF(B66&gt;0,I66*F66/B66,0)</f>
         <v/>
       </c>
       <c r="K66" s="28">
-        <f>IF(B66&gt;0,J66*I66/B66,0)</f>
+        <f>IF(B66&gt;0,I66*G66/B66,0)</f>
         <v/>
       </c>
       <c r="L66" s="18">
-        <f>I66+K66</f>
+        <f>H66+J66+K66</f>
         <v/>
       </c>
       <c r="M66" s="6">
-        <f>'Amazon'!$C$10+J66</f>
+        <f>'Amazon'!$C$10+I66</f>
         <v/>
       </c>
       <c r="N66" s="14">
@@ -7355,28 +7311,28 @@
         <f>E67*(1-1/ServeGPULever)</f>
         <v/>
       </c>
-      <c r="H67" s="28">
-        <f>E67/ServeGPULever</f>
-        <v/>
-      </c>
-      <c r="I67" s="6">
+      <c r="H67" s="6">
         <f>F67+G67</f>
         <v/>
       </c>
+      <c r="I67" s="28">
+        <f>'Meta'!$C$34</f>
+        <v/>
+      </c>
       <c r="J67" s="28">
-        <f>'Meta'!$C$34</f>
+        <f>IF(B67&gt;0,I67*F67/B67,0)</f>
         <v/>
       </c>
       <c r="K67" s="28">
-        <f>IF(B67&gt;0,J67*I67/B67,0)</f>
+        <f>IF(B67&gt;0,I67*G67/B67,0)</f>
         <v/>
       </c>
       <c r="L67" s="18">
-        <f>I67+K67</f>
+        <f>H67+J67+K67</f>
         <v/>
       </c>
       <c r="M67" s="6">
-        <f>'Meta'!$C$10+J67</f>
+        <f>'Meta'!$C$10+I67</f>
         <v/>
       </c>
       <c r="N67" s="14">
@@ -7426,28 +7382,28 @@
         <f>E68*(1-1/ServeGPULever)</f>
         <v/>
       </c>
-      <c r="H68" s="28">
-        <f>E68/ServeGPULever</f>
-        <v/>
-      </c>
-      <c r="I68" s="6">
+      <c r="H68" s="6">
         <f>F68+G68</f>
         <v/>
       </c>
+      <c r="I68" s="28">
+        <f>'Oracle'!$C$34</f>
+        <v/>
+      </c>
       <c r="J68" s="28">
-        <f>'Oracle'!$C$34</f>
+        <f>IF(B68&gt;0,I68*F68/B68,0)</f>
         <v/>
       </c>
       <c r="K68" s="28">
-        <f>IF(B68&gt;0,J68*I68/B68,0)</f>
+        <f>IF(B68&gt;0,I68*G68/B68,0)</f>
         <v/>
       </c>
       <c r="L68" s="18">
-        <f>I68+K68</f>
+        <f>H68+J68+K68</f>
         <v/>
       </c>
       <c r="M68" s="6">
-        <f>'Oracle'!$C$10+J68</f>
+        <f>'Oracle'!$C$10+I68</f>
         <v/>
       </c>
       <c r="N68" s="14">
@@ -7497,28 +7453,28 @@
         <f>E69*(1-1/ServeGPULever)</f>
         <v/>
       </c>
-      <c r="H69" s="28">
-        <f>E69/ServeGPULever</f>
-        <v/>
-      </c>
-      <c r="I69" s="6">
+      <c r="H69" s="6">
         <f>F69+G69</f>
         <v/>
       </c>
+      <c r="I69" s="28">
+        <f>'SpaceX'!$C$34</f>
+        <v/>
+      </c>
       <c r="J69" s="28">
-        <f>'SpaceX'!$C$34</f>
+        <f>IF(B69&gt;0,I69*F69/B69,0)</f>
         <v/>
       </c>
       <c r="K69" s="28">
-        <f>IF(B69&gt;0,J69*I69/B69,0)</f>
+        <f>IF(B69&gt;0,I69*G69/B69,0)</f>
         <v/>
       </c>
       <c r="L69" s="18">
-        <f>I69+K69</f>
+        <f>H69+J69+K69</f>
         <v/>
       </c>
       <c r="M69" s="6">
-        <f>'SpaceX'!$C$10+J69</f>
+        <f>'SpaceX'!$C$10+I69</f>
         <v/>
       </c>
       <c r="N69" s="14">
@@ -7568,11 +7524,11 @@
         <f>SUM(G64:G69)</f>
         <v/>
       </c>
-      <c r="H70" s="29">
+      <c r="H70" s="18">
         <f>SUM(H64:H69)</f>
         <v/>
       </c>
-      <c r="I70" s="18">
+      <c r="I70" s="29">
         <f>SUM(I64:I69)</f>
         <v/>
       </c>
@@ -7655,7 +7611,7 @@
       </c>
       <c r="E74" s="16" t="inlineStr">
         <is>
-          <t>Serving fleet</t>
+          <t>Inference fleet</t>
         </is>
       </c>
       <c r="F74" s="16" t="inlineStr">
@@ -7665,27 +7621,27 @@
       </c>
       <c r="G74" s="16" t="inlineStr">
         <is>
-          <t>Serving capex avoided</t>
+          <t>Inference capex avoided</t>
         </is>
       </c>
       <c r="H74" s="16" t="inlineStr">
         <is>
-          <t>Serving fleet needed</t>
+          <t>Chip capex avoided</t>
         </is>
       </c>
       <c r="I74" s="16" t="inlineStr">
         <is>
-          <t>Chip capex avoided</t>
+          <t>Power &amp; ops today</t>
         </is>
       </c>
       <c r="J74" s="16" t="inlineStr">
         <is>
-          <t>Power &amp; ops today</t>
+          <t>Training power saved</t>
         </is>
       </c>
       <c r="K74" s="16" t="inlineStr">
         <is>
-          <t>Power &amp; ops saved</t>
+          <t>Inference power saved</t>
         </is>
       </c>
       <c r="L74" s="16" t="inlineStr">
@@ -7749,28 +7705,28 @@
         <f>E75*(1-1/ServeGPULever)</f>
         <v/>
       </c>
-      <c r="H75" s="28">
-        <f>E75/ServeGPULever</f>
-        <v/>
-      </c>
-      <c r="I75" s="6">
+      <c r="H75" s="6">
         <f>F75+G75</f>
         <v/>
       </c>
+      <c r="I75" s="28">
+        <f>'Microsoft'!$B$34</f>
+        <v/>
+      </c>
       <c r="J75" s="28">
-        <f>'Microsoft'!$B$34</f>
+        <f>IF(B75&gt;0,I75*F75/B75,0)</f>
         <v/>
       </c>
       <c r="K75" s="28">
-        <f>IF(B75&gt;0,J75*I75/B75,0)</f>
+        <f>IF(B75&gt;0,I75*G75/B75,0)</f>
         <v/>
       </c>
       <c r="L75" s="18">
-        <f>I75+K75</f>
+        <f>H75+J75+K75</f>
         <v/>
       </c>
       <c r="M75" s="6">
-        <f>'Microsoft'!$B$10+J75</f>
+        <f>'Microsoft'!$B$10+I75</f>
         <v/>
       </c>
       <c r="N75" s="14">
@@ -7820,28 +7776,28 @@
         <f>E76*(1-1/ServeGPULever)</f>
         <v/>
       </c>
-      <c r="H76" s="28">
-        <f>E76/ServeGPULever</f>
-        <v/>
-      </c>
-      <c r="I76" s="6">
+      <c r="H76" s="6">
         <f>F76+G76</f>
         <v/>
       </c>
+      <c r="I76" s="28">
+        <f>'Alphabet'!$B$34</f>
+        <v/>
+      </c>
       <c r="J76" s="28">
-        <f>'Alphabet'!$B$34</f>
+        <f>IF(B76&gt;0,I76*F76/B76,0)</f>
         <v/>
       </c>
       <c r="K76" s="28">
-        <f>IF(B76&gt;0,J76*I76/B76,0)</f>
+        <f>IF(B76&gt;0,I76*G76/B76,0)</f>
         <v/>
       </c>
       <c r="L76" s="18">
-        <f>I76+K76</f>
+        <f>H76+J76+K76</f>
         <v/>
       </c>
       <c r="M76" s="6">
-        <f>'Alphabet'!$B$10+J76</f>
+        <f>'Alphabet'!$B$10+I76</f>
         <v/>
       </c>
       <c r="N76" s="14">
@@ -7891,28 +7847,28 @@
         <f>E77*(1-1/ServeGPULever)</f>
         <v/>
       </c>
-      <c r="H77" s="28">
-        <f>E77/ServeGPULever</f>
-        <v/>
-      </c>
-      <c r="I77" s="6">
+      <c r="H77" s="6">
         <f>F77+G77</f>
         <v/>
       </c>
+      <c r="I77" s="28">
+        <f>'Amazon'!$B$34</f>
+        <v/>
+      </c>
       <c r="J77" s="28">
-        <f>'Amazon'!$B$34</f>
+        <f>IF(B77&gt;0,I77*F77/B77,0)</f>
         <v/>
       </c>
       <c r="K77" s="28">
-        <f>IF(B77&gt;0,J77*I77/B77,0)</f>
+        <f>IF(B77&gt;0,I77*G77/B77,0)</f>
         <v/>
       </c>
       <c r="L77" s="18">
-        <f>I77+K77</f>
+        <f>H77+J77+K77</f>
         <v/>
       </c>
       <c r="M77" s="6">
-        <f>'Amazon'!$B$10+J77</f>
+        <f>'Amazon'!$B$10+I77</f>
         <v/>
       </c>
       <c r="N77" s="14">
@@ -7962,28 +7918,28 @@
         <f>E78*(1-1/ServeGPULever)</f>
         <v/>
       </c>
-      <c r="H78" s="28">
-        <f>E78/ServeGPULever</f>
-        <v/>
-      </c>
-      <c r="I78" s="6">
+      <c r="H78" s="6">
         <f>F78+G78</f>
         <v/>
       </c>
+      <c r="I78" s="28">
+        <f>'Meta'!$B$34</f>
+        <v/>
+      </c>
       <c r="J78" s="28">
-        <f>'Meta'!$B$34</f>
+        <f>IF(B78&gt;0,I78*F78/B78,0)</f>
         <v/>
       </c>
       <c r="K78" s="28">
-        <f>IF(B78&gt;0,J78*I78/B78,0)</f>
+        <f>IF(B78&gt;0,I78*G78/B78,0)</f>
         <v/>
       </c>
       <c r="L78" s="18">
-        <f>I78+K78</f>
+        <f>H78+J78+K78</f>
         <v/>
       </c>
       <c r="M78" s="6">
-        <f>'Meta'!$B$10+J78</f>
+        <f>'Meta'!$B$10+I78</f>
         <v/>
       </c>
       <c r="N78" s="14">
@@ -8033,28 +7989,28 @@
         <f>E79*(1-1/ServeGPULever)</f>
         <v/>
       </c>
-      <c r="H79" s="28">
-        <f>E79/ServeGPULever</f>
-        <v/>
-      </c>
-      <c r="I79" s="6">
+      <c r="H79" s="6">
         <f>F79+G79</f>
         <v/>
       </c>
+      <c r="I79" s="28">
+        <f>'Oracle'!$B$34</f>
+        <v/>
+      </c>
       <c r="J79" s="28">
-        <f>'Oracle'!$B$34</f>
+        <f>IF(B79&gt;0,I79*F79/B79,0)</f>
         <v/>
       </c>
       <c r="K79" s="28">
-        <f>IF(B79&gt;0,J79*I79/B79,0)</f>
+        <f>IF(B79&gt;0,I79*G79/B79,0)</f>
         <v/>
       </c>
       <c r="L79" s="18">
-        <f>I79+K79</f>
+        <f>H79+J79+K79</f>
         <v/>
       </c>
       <c r="M79" s="6">
-        <f>'Oracle'!$B$10+J79</f>
+        <f>'Oracle'!$B$10+I79</f>
         <v/>
       </c>
       <c r="N79" s="14">
@@ -8104,28 +8060,28 @@
         <f>E80*(1-1/ServeGPULever)</f>
         <v/>
       </c>
-      <c r="H80" s="28">
-        <f>E80/ServeGPULever</f>
-        <v/>
-      </c>
-      <c r="I80" s="6">
+      <c r="H80" s="6">
         <f>F80+G80</f>
         <v/>
       </c>
+      <c r="I80" s="28">
+        <f>'SpaceX'!$B$34</f>
+        <v/>
+      </c>
       <c r="J80" s="28">
-        <f>'SpaceX'!$B$34</f>
+        <f>IF(B80&gt;0,I80*F80/B80,0)</f>
         <v/>
       </c>
       <c r="K80" s="28">
-        <f>IF(B80&gt;0,J80*I80/B80,0)</f>
+        <f>IF(B80&gt;0,I80*G80/B80,0)</f>
         <v/>
       </c>
       <c r="L80" s="18">
-        <f>I80+K80</f>
+        <f>H80+J80+K80</f>
         <v/>
       </c>
       <c r="M80" s="6">
-        <f>'SpaceX'!$B$10+J80</f>
+        <f>'SpaceX'!$B$10+I80</f>
         <v/>
       </c>
       <c r="N80" s="14">
@@ -8175,11 +8131,11 @@
         <f>SUM(G75:G80)</f>
         <v/>
       </c>
-      <c r="H81" s="29">
+      <c r="H81" s="18">
         <f>SUM(H75:H80)</f>
         <v/>
       </c>
-      <c r="I81" s="18">
+      <c r="I81" s="29">
         <f>SUM(I75:I80)</f>
         <v/>
       </c>
@@ -8217,26 +8173,27 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="22">
     <mergeCell ref="D13:I13"/>
     <mergeCell ref="D32:I32"/>
     <mergeCell ref="D41:I41"/>
     <mergeCell ref="A55:I55"/>
+    <mergeCell ref="A26:I26"/>
     <mergeCell ref="D7:I7"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="D28:I28"/>
     <mergeCell ref="D18:I18"/>
     <mergeCell ref="D9:I9"/>
     <mergeCell ref="D30:I30"/>
-    <mergeCell ref="D29:I29"/>
+    <mergeCell ref="D24:I24"/>
     <mergeCell ref="D5:I5"/>
     <mergeCell ref="D35:I35"/>
     <mergeCell ref="D20:I20"/>
     <mergeCell ref="D60:I60"/>
-    <mergeCell ref="A24:I24"/>
     <mergeCell ref="D19:I19"/>
     <mergeCell ref="D10:I10"/>
+    <mergeCell ref="D31:I31"/>
     <mergeCell ref="D45:I45"/>
+    <mergeCell ref="D36:I36"/>
     <mergeCell ref="D6:I6"/>
     <mergeCell ref="D21:I21"/>
   </mergeCells>
@@ -8380,7 +8337,7 @@
       </c>
       <c r="H7" s="24" t="inlineStr">
         <is>
-          <t>Training AND serving compute</t>
+          <t>Training and inference compute</t>
         </is>
       </c>
     </row>
@@ -8431,7 +8388,7 @@
       </c>
       <c r="B9" s="27" t="inlineStr">
         <is>
-          <t>Faster training per token on long documents</t>
+          <t>Training speed per token (same model size)</t>
         </is>
       </c>
       <c r="C9" s="22">
@@ -8439,19 +8396,19 @@
         <v/>
       </c>
       <c r="D9" s="31" t="n">
-        <v>2.220667013967386</v>
+        <v>1</v>
       </c>
       <c r="E9" s="31" t="n">
-        <v>3.967000451897755</v>
+        <v>1</v>
       </c>
       <c r="F9" s="24" t="inlineStr">
         <is>
-          <t>Today: MEASURED cost per token at each document length; the training mix is illustrative. Optimized: TARGET</t>
+          <t>ASSUMPTION — roughly comparable to a transformer; no speed credit taken</t>
         </is>
       </c>
       <c r="G9" s="24" t="inlineStr">
         <is>
-          <t>A transformer's cost per token rises with document length (each token looks back over all the earlier ones); Helarctos' stays flat. Over a modern training mix (70% at 8k / 20% at 64k / 10% at 256k tokens) that is 2.2× cheaper per token. On short documents alone the transformer is still faster today (0.58× at 2k tokens).</t>
+          <t>At the same model size, Helarctos trains at roughly the same speed per token as a transformer, so we count no training speed-up. The training saving comes entirely from levers 1 and 2: a smaller model trained on fewer tokens. (Where Helarctos is much faster is inference — lever 5.)</t>
         </is>
       </c>
       <c r="H9" s="24" t="inlineStr">
@@ -8495,7 +8452,7 @@
       </c>
       <c r="H10" s="24" t="inlineStr">
         <is>
-          <t>Serving GPUs (the memory limit)</t>
+          <t>Inference GPUs (the memory limit)</t>
         </is>
       </c>
     </row>
@@ -8534,7 +8491,7 @@
       </c>
       <c r="H11" s="24" t="inlineStr">
         <is>
-          <t>Serving GPUs (the compute limit)</t>
+          <t>Inference GPUs (the compute limit)</t>
         </is>
       </c>
     </row>
@@ -8571,7 +8528,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>Serving: memory needed per conversation falls by</t>
+          <t>Inference: memory needed per conversation falls by</t>
         </is>
       </c>
       <c r="C15" s="32">
@@ -8587,7 +8544,7 @@
     <row r="16" ht="30" customHeight="1">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>Serving: compute needed per token falls by</t>
+          <t>Inference: compute needed per token falls by</t>
         </is>
       </c>
       <c r="C16" s="22">
@@ -8603,7 +8560,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>Serving: GPUs needed fall by</t>
+          <t>Inference: GPUs needed fall by</t>
         </is>
       </c>
       <c r="C17" s="22">
@@ -8612,14 +8569,14 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>A GPU is bought whole — memory and compute come together. The serving fleet has to cover whichever runs out first, so it shrinks by the SMALLER of the two levers (here the conservative ÷100 memory cap). Multiplying them (100 × 793 = 79,000×) would be wrong.</t>
+          <t>A GPU is bought whole — memory and compute come together. The inference fleet has to cover whichever runs out first, so it shrinks by the SMALLER of the two levers (here the conservative ÷100 memory cap). Multiplying them (100 × 793 = 79,000×) would be wrong.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>For reference: technical tabs' blended serving cut</t>
+          <t>For reference: technical tabs' blended inference cut</t>
         </is>
       </c>
       <c r="C18" s="22">
@@ -8649,7 +8606,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Analysts put training at 30–45% of AI compute in 2026 (Gartner, Deloitte; the rest is serving users). Per-company estimates below follow what each firm is known to be building.</t>
+          <t>Analysts put training at 30–45% of AI compute in 2026 (Gartner, Deloitte; the rest is inference, i.e. serving users). Per-company estimates below follow what each firm is known to be building.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inference cost independent of model size; no model-size slider; wrapped text
- The equal-quality parameter ratio (x4.22) now applies to training only.
  The inference compute lever is the throughput per GPU alone: x368
  (Current kernels) / x382 (Optimized kernels), was x1,553 / x1,611.
  Front-tab dollars unchanged (memory binds inference); Totals FY2026
  $383.2B -> $382.9B, cost-weighted x160 -> x141.
- Step table is now two steps: training (smaller model, fewer tokens),
  then inference (fixed-size memory, many more conversations per GPU).
- App: deployment-scale slider removed (ratio fixed at 1T); inference
  lever follows the sidebar context and input:output ratio only.
- App tables with long text (Summary sources, Levers, What Matters)
  render as wrapped static tables; workbook rows made taller.
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -630,20 +630,6 @@
               </a:ln>
             </spPr>
           </dPt>
-          <dPt>
-            <idx val="3"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="1BAF7A"/>
-              </a:solidFill>
-              <a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="1BAF7A"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
           <dLbls>
             <numFmt formatCode="&quot;$&quot;#,##0&quot;B&quot;"/>
             <showLegendKey val="0"/>
@@ -654,12 +640,12 @@
           </dLbls>
           <cat>
             <numRef>
-              <f>'Value Bridge'!$A$49:$A$52</f>
+              <f>'Value Bridge'!$A$49:$A$51</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Value Bridge'!$F$49:$F$52</f>
+              <f>'Value Bridge'!$F$49:$F$51</f>
             </numRef>
           </val>
         </ser>
@@ -1260,7 +1246,7 @@
       <c r="F15" s="12" t="n"/>
       <c r="G15" s="13" t="n"/>
     </row>
-    <row r="16" ht="62" customHeight="1">
+    <row r="16" ht="92" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Training</t>
@@ -1279,7 +1265,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="62" customHeight="1">
+    <row r="17" ht="92" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Inference</t>
@@ -1294,7 +1280,7 @@
         <v/>
       </c>
       <c r="D17" s="3">
-        <f>"A transformer's memory grows with every token of every live conversation; Helarctos keeps a fixed-size state (÷"&amp;TEXT(MemoryLever,"0")&amp;" memory) and does "&amp;TEXT(ServeComputeLever,"0")&amp;"× less compute per token. A GPU is bought whole, so the fleet shrinks by whichever limit binds: "&amp;TEXT(ServeGPULever,"0")&amp;"× fewer inference GPUs, and their power."</f>
+        <f>"A transformer's memory grows with every token of every live conversation; Helarctos keeps a fixed-size state (÷"&amp;TEXT(MemoryLever,"0")&amp;" memory per conversation), so each GPU serves "&amp;TEXT(ServeComputeLever,"0")&amp;"× more tokens. A GPU is bought whole, so the fleet shrinks by whichever limit binds: "&amp;TEXT(ServeGPULever,"0")&amp;"× fewer inference GPUs, and their power."</f>
         <v/>
       </c>
     </row>
@@ -2818,13 +2804,13 @@
         <v>-965.3195453336799</v>
       </c>
       <c r="F14" s="57" t="n">
-        <v>574.1429873323519</v>
+        <v>573.6639462810871</v>
       </c>
       <c r="G14" s="57" t="n">
-        <v>-391.1765580013281</v>
+        <v>-391.6555990525928</v>
       </c>
       <c r="H14" s="58" t="n">
-        <v>0.4912161074175423</v>
+        <v>0.4908062571090175</v>
       </c>
     </row>
     <row r="16">
@@ -3190,7 +3176,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>B27 = inference throughput per GPU at a 262k-token average context for the active scenario (B26, picked on the Levers tab) x the equal-quality parameter ratio (B23). Edit B23-B25, or overtype this cell to pin the lever. See ServingTraining for the measured background.</t>
+          <t>B27 = inference throughput per GPU at a 262k-token average context for the active scenario (B26, picked on the Levers tab). Inference cost does not scale with model size, so the equal-quality ratio (B23) applies to training only. Edit B24-B25, or overtype this cell to pin the lever. See ServingTraining for the measured background.</t>
         </is>
       </c>
     </row>
@@ -3604,11 +3590,11 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Compute (FLOPs) lever = B23 x B26</t>
+          <t>Inference compute (FLOPs) lever = B26</t>
         </is>
       </c>
       <c r="B27" s="71">
-        <f>$B$23*$B$26</f>
+        <f>$B$26</f>
         <v/>
       </c>
       <c r="C27" t="inlineStr">
@@ -3800,12 +3786,12 @@
       </c>
       <c r="D13" s="20" t="inlineStr">
         <is>
-          <t>Compute lever (x)</t>
+          <t>◆ Inference lever, current kernels (x)</t>
         </is>
       </c>
       <c r="E13" s="20" t="inlineStr">
         <is>
-          <t>Throughput per GPU, same size (x)</t>
+          <t>◆ Inference lever, optimized kernels (x)</t>
         </is>
       </c>
       <c r="F13" s="20" t="inlineStr"/>
@@ -3822,11 +3808,11 @@
       <c r="C14" s="25" t="n">
         <v>0.05208995366081766</v>
       </c>
-      <c r="D14" s="50" t="n">
-        <v>50.29665229131971</v>
+      <c r="D14" s="48" t="n">
+        <v>11.92287815199857</v>
       </c>
       <c r="E14" s="48" t="n">
-        <v>11.92287815199857</v>
+        <v>12.20269551906716</v>
       </c>
     </row>
     <row r="15">
@@ -3841,11 +3827,11 @@
       <c r="C15" s="25" t="n">
         <v>0.05196631516233694</v>
       </c>
-      <c r="D15" s="50" t="n">
-        <v>200.6239377794075</v>
+      <c r="D15" s="48" t="n">
+        <v>47.55813072137281</v>
       </c>
       <c r="E15" s="48" t="n">
-        <v>47.55813072137281</v>
+        <v>48.67155861377862</v>
       </c>
     </row>
     <row r="16">
@@ -3860,11 +3846,11 @@
       <c r="C16" s="25" t="n">
         <v>0.06235575593664416</v>
       </c>
-      <c r="D16" s="50" t="n">
-        <v>793.2064858179596</v>
+      <c r="D16" s="48" t="n">
+        <v>188.0304920694428</v>
       </c>
       <c r="E16" s="48" t="n">
-        <v>188.0304920694428</v>
+        <v>193.3375983858266</v>
       </c>
     </row>
     <row r="17">
@@ -3879,11 +3865,11 @@
       <c r="C17" s="25" t="n">
         <v>0.08221381175542121</v>
       </c>
-      <c r="D17" s="50" t="n">
-        <v>1552.723400990788</v>
+      <c r="D17" s="48" t="n">
+        <v>368.0748334211694</v>
       </c>
       <c r="E17" s="48" t="n">
-        <v>368.0748334211694</v>
+        <v>381.8963339071965</v>
       </c>
     </row>
     <row r="19">
@@ -5209,7 +5195,7 @@
         <v>151.049323023638</v>
       </c>
       <c r="F81" s="94" t="n">
-        <v>-10.90451281465531</v>
+        <v>-10.76938526370006</v>
       </c>
       <c r="G81" s="95" t="inlineStr">
         <is>
@@ -5238,7 +5224,7 @@
         <v>154.9628350868998</v>
       </c>
       <c r="F82" s="94" t="n">
-        <v>-6.991000751393557</v>
+        <v>-6.85587320043831</v>
       </c>
       <c r="G82" s="96" t="inlineStr">
         <is>
@@ -5267,7 +5253,7 @@
         <v>155.9554685338785</v>
       </c>
       <c r="F83" s="94" t="n">
-        <v>-5.998367304414813</v>
+        <v>-5.863239753459567</v>
       </c>
       <c r="G83" s="96" t="inlineStr">
         <is>
@@ -5296,7 +5282,7 @@
         <v>156.09876278548</v>
       </c>
       <c r="F84" s="94" t="n">
-        <v>-5.855073052813339</v>
+        <v>-5.719945501858092</v>
       </c>
       <c r="G84" s="96" t="inlineStr">
         <is>
@@ -6588,7 +6574,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Engine: GPU cost ~60% memory / ~40% compute. Single scenario (2026-09-29): memory x100 + FLOPs x1,553 (inference throughput per GPU x368 at a 262k-token average context — decode 2.5 ms/token x 64 streams ESTIMATE, prefill at the banked x3.936 — x equal-quality ratio x4.22 at 1T) -&gt; ~x160 cost-weighted (Inputs B20). The front tabs price inference on whole GPUs instead (fleet shrinks by the smaller lever, x100).</t>
+          <t>Engine: GPU cost ~60% memory / ~40% compute. Single scenario (2026-09-29): memory x100 + inference compute x368 (throughput per GPU at a 262k-token average context; size-independent — decode 2.5 ms/token x 64 streams ESTIMATE, prefill at the banked x3.936 — x equal-quality ratio x4.22 at 1T) -&gt; ~x160 cost-weighted (Inputs B20). The front tabs price inference on whole GPUs instead (fleet shrinks by the smaller lever, x100).</t>
         </is>
       </c>
     </row>
@@ -6678,7 +6664,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>- Cost-weighted reduction ~x160 — memory-floored at /100.</t>
+          <t>- Cost-weighted reduction ~x141 — memory-floored at /100.</t>
         </is>
       </c>
     </row>
@@ -7286,7 +7272,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>smaller model × more conversations per GPU (levers 1 × 5)</t>
+          <t>many more conversations per GPU (lever 5)</t>
         </is>
       </c>
     </row>
@@ -7545,19 +7531,18 @@
     <row r="50">
       <c r="A50" s="24" t="inlineStr">
         <is>
-          <t>Smaller model for the same quality (levers 1, 2)</t>
+          <t>Smaller model trained on fewer tokens — training (levers 1–3)</t>
         </is>
       </c>
       <c r="B50" s="21">
-        <f>SmallerModel^2</f>
+        <f>TrainLever</f>
         <v/>
       </c>
       <c r="C50" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D50" s="21">
-        <f>SmallerModel</f>
-        <v/>
+      <c r="D50" s="21" t="n">
+        <v>1</v>
       </c>
       <c r="E50" s="25">
         <f>(D70*(1-1/B50)+E70*(1-1/MIN(C50,D50)))/B70</f>
@@ -7573,13 +7558,13 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="24" t="inlineStr">
-        <is>
-          <t>+ Fixed-size memory per conversation (lever 4)</t>
+      <c r="A51" s="27" t="inlineStr">
+        <is>
+          <t>+ Fixed-size memory: many more conversations per GPU — inference (levers 4, 5)</t>
         </is>
       </c>
       <c r="B51" s="21">
-        <f>SmallerModel^2</f>
+        <f>TrainLever</f>
         <v/>
       </c>
       <c r="C51" s="23">
@@ -7587,7 +7572,7 @@
         <v/>
       </c>
       <c r="D51" s="21">
-        <f>SmallerModel</f>
+        <f>ServeComputeLever</f>
         <v/>
       </c>
       <c r="E51" s="25">
@@ -7603,41 +7588,10 @@
         <v/>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="27" t="inlineStr">
-        <is>
-          <t>+ Many more conversations per GPU (lever 5)</t>
-        </is>
-      </c>
-      <c r="B52" s="21">
-        <f>TrainLever</f>
-        <v/>
-      </c>
-      <c r="C52" s="23">
-        <f>MemoryLever</f>
-        <v/>
-      </c>
-      <c r="D52" s="21">
-        <f>ServeComputeLever</f>
-        <v/>
-      </c>
-      <c r="E52" s="25">
-        <f>(D70*(1-1/B52)+E70*(1-1/MIN(C52,D52)))/B70</f>
-        <v/>
-      </c>
-      <c r="F52" s="18">
-        <f>E52*(B70+I70)</f>
-        <v/>
-      </c>
-      <c r="G52" s="26">
-        <f>F52-F51</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" ht="62" customHeight="1">
+    <row r="55" ht="48" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Read this as: the smaller model alone removes nearly all of the TRAINING bill (fewer parameters AND fewer tokens compound) but no inference GPUs — at long context a transformer's inference GPUs are full of memory (the growing KV cache), not busy computing, and a smaller model doesn't change that. Fixed-size memory unlocks inference, until compute becomes the limit; many more conversations per GPU lifts that limit. By then ~99% of the chip bill is gone: bigger multiples can't add much, because a cost can only fall to zero once. That is why this workbook reports dollars, not multiples. The order is the storyline; the end point does not depend on it.</t>
+          <t>Read this as: TRAINING savings come from the smaller model (fewer parameters AND fewer tokens compound, ~18× fewer GPU-hours). INFERENCE savings come from fixed-size memory, which lets each GPU hold many more long conversations — model size doesn't change inference cost. Each fleet then shrinks by ~94–99%: bigger multiples can't add much, because a cost can only fall to zero once. That is why this workbook reports dollars, not multiples.</t>
         </is>
       </c>
     </row>
@@ -9055,7 +9009,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="78" customHeight="1">
+    <row r="7" ht="104" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>1</t>
@@ -9092,11 +9046,11 @@
       </c>
       <c r="H7" s="24" t="inlineStr">
         <is>
-          <t>Training and inference compute</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="78" customHeight="1">
+          <t>Training (inference cost doesn't depend on model size)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="104" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>2</t>
@@ -9137,7 +9091,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="78" customHeight="1">
+    <row r="9" ht="104" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>3</t>
@@ -9174,7 +9128,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="78" customHeight="1">
+    <row r="10" ht="104" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
         <is>
           <t>4</t>
@@ -9215,7 +9169,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="78" customHeight="1">
+    <row r="11" ht="104" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>5</t>
@@ -9307,12 +9261,12 @@
         </is>
       </c>
       <c r="C16" s="22">
-        <f>SmallerModel*ServeThroughput</f>
+        <f>ServeThroughput</f>
         <v/>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>lever 1 × lever 5</t>
+          <t>lever 5 (inference cost doesn't depend on model size)</t>
         </is>
       </c>
     </row>
@@ -9766,33 +9720,33 @@
       </c>
       <c r="B8" s="27" t="inlineStr">
         <is>
-          <t>Conversations served per GPU  (Helarctos lever)</t>
+          <t>Memory per conversation  (Helarctos lever)</t>
         </is>
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>Inputs B24/B25 (lever 5)</t>
+          <t>Inputs B2 (lever 4)</t>
         </is>
       </c>
       <c r="D8" s="17" t="inlineStr">
         <is>
-          <t>×2</t>
+          <t>÷10</t>
         </is>
       </c>
       <c r="E8" s="40" t="n">
-        <v>-26.18437230470289</v>
+        <v>-21.71463959598657</v>
       </c>
       <c r="F8" s="17" t="inlineStr">
         <is>
-          <t>×3,000</t>
+          <t>÷1,000</t>
         </is>
       </c>
       <c r="G8" s="40" t="n">
-        <v>0</v>
+        <v>1.757227168894815</v>
       </c>
       <c r="H8" s="24" t="inlineStr">
         <is>
-          <t>Only matters if it collapses. Inference GPUs are limited by memory (÷100) as long as this stays above ~×24 at the same model size; the estimate is ×368 at 262k.</t>
+          <t>Sets how far inference GPUs shrink. Measured ×2,000 at 262k; ÷100 is our cap. It would fall toward ÷60 only if average conversations were ~8k tokens.</t>
         </is>
       </c>
     </row>
@@ -9804,33 +9758,33 @@
       </c>
       <c r="B9" s="27" t="inlineStr">
         <is>
-          <t>Memory per conversation  (Helarctos lever)</t>
+          <t>Data-center share of capex</t>
         </is>
       </c>
       <c r="C9" s="24" t="inlineStr">
         <is>
-          <t>Inputs B2 (lever 4)</t>
+          <t>company tabs, row 4</t>
         </is>
       </c>
       <c r="D9" s="17" t="inlineStr">
         <is>
-          <t>÷10</t>
+          <t>−5%</t>
         </is>
       </c>
       <c r="E9" s="40" t="n">
-        <v>-21.71463959598657</v>
+        <v>-18.75371362936642</v>
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>÷1,000</t>
+          <t>+5%</t>
         </is>
       </c>
       <c r="G9" s="40" t="n">
-        <v>2.171463959598668</v>
+        <v>12.83675643943218</v>
       </c>
       <c r="H9" s="24" t="inlineStr">
         <is>
-          <t>Sets how far inference GPUs shrink. Measured ×2,000 at 262k; ÷100 is our cap. It would fall toward ÷60 only if average conversations were ~8k tokens.</t>
+          <t>Share of capex that goes into data centres rather than offices and other assets. From the 10-K/10-Q property notes (93–98%; Amazon's AWS share 68–76%).</t>
         </is>
       </c>
     </row>
@@ -9842,33 +9796,33 @@
       </c>
       <c r="B10" s="27" t="inlineStr">
         <is>
-          <t>Data-center share of capex</t>
+          <t>Conversations served per GPU  (Helarctos lever)</t>
         </is>
       </c>
       <c r="C10" s="24" t="inlineStr">
         <is>
-          <t>company tabs, row 4</t>
+          <t>Inputs B24/B25 (lever 5)</t>
         </is>
       </c>
       <c r="D10" s="17" t="inlineStr">
         <is>
-          <t>−5%</t>
+          <t>×12 (8k context)</t>
         </is>
       </c>
       <c r="E10" s="40" t="n">
-        <v>-18.75371362936642</v>
+        <v>-17.69341004117427</v>
       </c>
       <c r="F10" s="17" t="inlineStr">
         <is>
-          <t>+5%</t>
+          <t>×3,000</t>
         </is>
       </c>
       <c r="G10" s="40" t="n">
-        <v>12.83675643943218</v>
+        <v>0</v>
       </c>
       <c r="H10" s="24" t="inlineStr">
         <is>
-          <t>Share of capex that goes into data centres rather than offices and other assets. From the 10-K/10-Q property notes (93–98%; Amazon's AWS share 68–76%).</t>
+          <t>Only matters if it collapses. Inference GPUs are limited by memory (÷100) as long as this stays above ~×24 at the same model size; the estimate is ×368 at 262k.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
H1 scale labelled ~1T dense-equivalent (today's 5-6T mixture-of-experts flagships); What Matters high case 5T dense
Frontier labs no longer disclose sizes and almost all large models are
mixture-of-experts (Grok 5 at 6T, Kimi K3 at 2.8T). Such a model performs
roughly like a dense model of sqrt(total x active) size, so a 5-6T
flagship is ~1T dense-equivalent: the existing ratio (x4.22) is kept and
relabelled on Inputs, Levers, What Matters, the app and the README. The
What Matters high case for H1 is now a 5T dense model (x5.7, +$3.6B),
was 10T. No results change.
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -4475,10 +4475,10 @@
       <c r="D22" s="90" t="n"/>
       <c r="E22" s="90" t="n"/>
     </row>
-    <row r="23" ht="78" customHeight="1">
+    <row r="23" ht="138" customHeight="1">
       <c r="A23" s="22" t="inlineStr">
         <is>
-          <t>H1 · Equal-quality parameter ratio at 1T (smaller model; H2 = same) ★</t>
+          <t>H1 · Equal-quality parameter ratio at ~1T dense-equivalent (smaller model; H2 = same) ★</t>
         </is>
       </c>
       <c r="B23" s="112" t="n">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="E23" s="91" t="inlineStr">
         <is>
-          <t>FIT-DERIVED (sealed 2026-08-14 refit): bAttention matches the transformer fit's quality on 23.7% of the params at 1T -&gt; x4.22 compute per token at equal quality. 84.2% at 1B, 55.2% at 10B, 36.2% at 100B, 15.5% at 10T (x6.44). A projection of the two fits, not a measurement. Same in both scenarios.</t>
+          <t>FIT-DERIVED (sealed 2026-08-14 refit): bAttention matches the transformer fit's quality on 23.7% of the params at 1T -&gt; x4.22 compute per token at equal quality. 84.2% at 1B, 55.2% at 10B, 36.2% at 100B, 15.5% at 10T (x6.44). A projection of the two fits, not a measurement. Same in both scenarios. Scale: ~1T dense-equivalent: about what today's 5-6T-total mixture-of-experts flagships amount to (Grok 5 at 6T, Kimi K3 at 2.8T; a mixture-of-experts model runs only a fraction of its parameters per token and performs roughly like a dense model of sqrt(total x active) size).</t>
         </is>
       </c>
     </row>
@@ -10051,7 +10051,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="63" customHeight="1">
+    <row r="9" ht="78" customHeight="1">
       <c r="A9" s="52" t="inlineStr">
         <is>
           <t>H1</t>
@@ -10078,12 +10078,12 @@
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>PROJECTED — quality trends measured on models we trained (47M–663M parameters), extended to 1T</t>
+          <t>PROJECTED — quality trends measured on models we trained (47M–663M parameters), extended to ~1T dense-equivalent</t>
         </is>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>A Helarctos model matches a 1-trillion-parameter transformer's quality with ~24% of the parameters: 4.2× fewer numbers to store, update and run.</t>
+          <t>A Helarctos model matches a ~1T dense-equivalent transformer — about what today's 5–6T-total mixture-of-experts flagships amount to — with ~24% of the parameters: 4.2× fewer numbers to store, update and run.</t>
         </is>
       </c>
       <c r="H9" s="14" t="inlineStr">
@@ -10690,7 +10690,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1">
+    <row r="44" ht="33" customHeight="1">
       <c r="A44" s="66" t="inlineStr">
         <is>
           <t>•</t>
@@ -10698,7 +10698,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>H1 is a projection: quality trends measured up to 663M parameters, extended to trillion scale.</t>
+          <t>H1 is a projection: quality trends measured up to 663M parameters, extended to ~1T dense-equivalent — about what today's 5–6T-total mixture-of-experts flagships (Grok 5 at 6T, Kimi K3 at 2.8T) amount to.</t>
         </is>
       </c>
     </row>
@@ -10863,7 +10863,7 @@
       <c r="G5" s="67" t="n"/>
       <c r="H5" s="67" t="n"/>
     </row>
-    <row r="6" ht="48" customHeight="1">
+    <row r="6" ht="78" customHeight="1">
       <c r="A6" s="70" t="inlineStr">
         <is>
           <t>★</t>
@@ -10889,15 +10889,15 @@
       </c>
       <c r="F6" s="71" t="inlineStr">
         <is>
-          <t>×6.4</t>
+          <t>×5.7 (5T dense)</t>
         </is>
       </c>
       <c r="G6" s="72" t="n">
-        <v>4.630107479271089</v>
+        <v>3.617436659798898</v>
       </c>
       <c r="H6" s="73" t="inlineStr">
         <is>
-          <t>The biggest Helarctos-specific assumption: it drives the whole training saving (smaller model × fewer tokens). A projection from models up to 663M parameters to trillion scale.</t>
+          <t>The biggest Helarctos-specific assumption: it drives the whole training saving (smaller model × fewer tokens). A projection from models up to 663M parameters to ~1T dense-equivalent (today's 5–6T mixture-of-experts flagships). High case: a 5T dense model.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wording cleanup: memory lever at x2,032, conversation length 262k
- Technical-appendix and app Methodology text no longer describe the
  retired /100 memory cap, the x141/x1,553 figures or the Ceiling
  scenario; key results re-quoted (FY25 ~$163B, FY26 ~$385B Totals,
  ~$377B front tabs).
- 'Average conversation length' used for the context input and tables
  (was E[context] / 'average context'); 262k is the default.
- What Matters: the conversation-length row is one-sided (32k low case,
  262k default) instead of a 'high' case that was shorter than 262k.
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -4935,7 +4935,7 @@
     <row r="12">
       <c r="A12" s="86" t="inlineStr">
         <is>
-          <t>CONTEXT SENSITIVITY — prefill share of serving cost vs fleet E[context]</t>
+          <t>CONVERSATION-LENGTH SENSITIVITY — prompt share of serving cost vs average conversation length</t>
         </is>
       </c>
       <c r="B12" s="87" t="n"/>
@@ -4947,7 +4947,7 @@
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="89" t="inlineStr">
         <is>
-          <t>E[context]</t>
+          <t>Conversation length</t>
         </is>
       </c>
       <c r="B13" s="89" t="inlineStr">
@@ -5479,7 +5479,7 @@
       </c>
       <c r="F17" s="88" t="inlineStr">
         <is>
-          <t>RE-BASED 2026-08-24/25 (1 x GH200, ONE layer, fwd+bwd, bf16, checkpointing off both arms, modern transformer block 24Q/4KV head_dim 256 RoPE 64 gated): transformer is 1.72x faster at T=2,048 (101.7 vs 59.3 ms/step) and 1.79x at T=8,192; the equal-token B4/T32,768 ~parity cell is RETIRED 2026-08-25 as a B4 occupancy artifact, and the flat per-token model puts the crossover at a PROJECTED T~13,008 (from T~88,000 pre-campaign). It read 6.12x (400.4 ms) the same morning. Training PEAK MEMORY, same frame: 1.579x at T=2,048 (17,087.5 vs 10,823.6 MiB), from 2.829x -- that is TRAINING memory, not the /100 SERVING lever. TARGET (no receipt): T=8,192 step &lt;= 83.08 ms and memory 0.88x.</t>
+          <t>RE-BASED 2026-08-24/25 (1 x GH200, ONE layer, fwd+bwd, bf16, checkpointing off both arms, modern transformer block 24Q/4KV head_dim 256 RoPE 64 gated): transformer is 1.72x faster at T=2,048 (101.7 vs 59.3 ms/step) and 1.79x at T=8,192; the equal-token B4/T32,768 ~parity cell is RETIRED 2026-08-25 as a B4 occupancy artifact, and the flat per-token model puts the crossover at a PROJECTED T~13,008 (from T~88,000 pre-campaign). It read 6.12x (400.4 ms) the same morning. Training PEAK MEMORY, same frame: 1.579x at T=2,048 (17,087.5 vs 10,823.6 MiB), from 2.829x -- that is TRAINING memory, not the H4 serving-memory lever. TARGET (no receipt): T=8,192 step &lt;= 83.08 ms and memory 0.88x.</t>
         </is>
       </c>
     </row>
@@ -7951,10 +7951,10 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1">
+    <row r="30" ht="33" customHeight="1">
       <c r="A30" s="88" t="inlineStr">
         <is>
-          <t>- Multiplying the levers (100x * ~1,553x) is NOT physical: cost is additive (Amdahl), not multiplicative.</t>
+          <t>- Multiplying the levers (memory x2,032 * tokens per GPU x368) is NOT physical: a GPU is bought whole, so the fleet shrinks by the smaller of the two.</t>
         </is>
       </c>
     </row>
@@ -11602,7 +11602,7 @@
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>fixed at 262k (app: sidebar)</t>
+          <t>262k default (app: sidebar)</t>
         </is>
       </c>
       <c r="D18" s="68" t="inlineStr">
@@ -11615,11 +11615,11 @@
       </c>
       <c r="F18" s="68" t="inlineStr">
         <is>
-          <t>128k</t>
+          <t>262k (default)</t>
         </is>
       </c>
       <c r="G18" s="71" t="n">
-        <v>-0.6276610598471848</v>
+        <v>0</v>
       </c>
       <c r="H18" s="70" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
What Matters: conversation-length high case 1M (+$0.5B)
At 1M tokens Helarctos serves x1,411 more tokens per GPU and the memory
advantage is x8,128, so FY2026 rises ~$0.5B. Conservative: one
transformer conversation's KV (~207 GB) no longer fits a GPU, and the
1/context law still credits it one stream per GPU. Low case stays 32k.
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -11593,7 +11593,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="48" customHeight="1">
+    <row r="18" ht="78" customHeight="1">
       <c r="A18" s="67" t="inlineStr"/>
       <c r="B18" s="14" t="inlineStr">
         <is>
@@ -11615,15 +11615,15 @@
       </c>
       <c r="F18" s="68" t="inlineStr">
         <is>
-          <t>262k (default)</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="G18" s="71" t="n">
-        <v>0</v>
+        <v>0.4844550470273816</v>
       </c>
       <c r="H18" s="70" t="inlineStr">
         <is>
-          <t>Shorter conversations shrink both the memory advantage and tokens per GPU (×48 at 32k). The workbook is fixed at 262k; the app's sidebar lets you change it.</t>
+          <t>Shorter conversations shrink both the memory advantage and tokens per GPU (×48 at 32k); longer ones grow them (×1,411 tokens per GPU at 1M, where one transformer conversation no longer fits a GPU). The workbook is fixed at 262k; the app's sidebar lets you change it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scenarios: What Matters and the workbook delta table run on the active scenario
sensitivity_table takes kernels= and follow=, so the What Matters base uses
the active scenario's H3 and inference lever (it used to pair H3-current
with the picker's optimized inference lever) and the active data-centre
setting; the H3 row's high case is the other scenario's value. The app
passes both and captions the basis. The workbook's Current -> Optimized
table now computes the FY2026 dollars per column with the Value Bridge
ladder formula (live, follows the data-centre switch) instead of static
build-time values; Value Bridge subtotals no longer wear the headline fill.
</commit_message>
<xml_diff>
--- a/AI_Capex_Efficiency.xlsx
+++ b/AI_Capex_Efficiency.xlsx
@@ -2377,14 +2377,16 @@
     <row r="29" ht="48" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>Spend made unnecessary, FY2026 (static at the build defaults; the live cells above follow the picker)</t>
-        </is>
-      </c>
-      <c r="B29" s="20" t="n">
-        <v>774.1494653624206</v>
-      </c>
-      <c r="C29" s="20" t="n">
-        <v>777.3625628522243</v>
+          <t>Spend made unnecessary, FY2026 (live: the ladder formula at each scenario's levers; follows the data-centre switch)</t>
+        </is>
+      </c>
+      <c r="B29" s="20">
+        <f>SUMPRODUCT(('Value Bridge'!$D$96:$D$101*(1-1/B24)+'Value Bridge'!$E$96:$E$101*(1-1/MIN(MemoryLever,B26)))*(1+('Value Bridge'!$I$96:$I$101+'Value Bridge'!$R$96:$R$101*ServersFollow+'Value Bridge'!$S$96:$S$101*DCFollow)/'Value Bridge'!$B$96:$B$101))</f>
+        <v/>
+      </c>
+      <c r="C29" s="20">
+        <f>SUMPRODUCT(('Value Bridge'!$D$96:$D$101*(1-1/C24)+'Value Bridge'!$E$96:$E$101*(1-1/MIN(MemoryLever,C26)))*(1+('Value Bridge'!$I$96:$I$101+'Value Bridge'!$R$96:$R$101*ServersFollow+'Value Bridge'!$S$96:$S$101*DCFollow)/'Value Bridge'!$B$96:$B$101))</f>
+        <v/>
       </c>
     </row>
     <row r="30" ht="48" customHeight="1">

</xml_diff>